<commit_message>
Actualiza precios Facilito 2026-09-04 18:13 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$D$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$E$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,13 +440,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D164"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,6 +471,11 @@
           <t>2026-09-04 12:56</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04 13:13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -490,6 +496,9 @@
       <c r="D2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -510,6 +519,9 @@
       <c r="D3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -530,6 +542,9 @@
       <c r="D4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -550,6 +565,9 @@
       <c r="D5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -570,6 +588,9 @@
       <c r="D6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -590,6 +611,9 @@
       <c r="D7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -610,6 +634,9 @@
       <c r="D8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -630,6 +657,9 @@
       <c r="D9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -650,6 +680,9 @@
       <c r="D10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -670,6 +703,9 @@
       <c r="D11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -690,6 +726,9 @@
       <c r="D12" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -710,6 +749,9 @@
       <c r="D13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -730,6 +772,9 @@
       <c r="D14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -750,6 +795,9 @@
       <c r="D15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -770,6 +818,9 @@
       <c r="D16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -790,6 +841,9 @@
       <c r="D17" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -810,6 +864,9 @@
       <c r="D18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -830,6 +887,9 @@
       <c r="D19" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -850,6 +910,9 @@
       <c r="D20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -870,6 +933,9 @@
       <c r="D21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -890,6 +956,9 @@
       <c r="D22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -910,6 +979,9 @@
       <c r="D23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="E23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -930,6 +1002,9 @@
       <c r="D24" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="E24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -950,6 +1025,9 @@
       <c r="D25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="E25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -970,6 +1048,9 @@
       <c r="D26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="E26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -990,6 +1071,9 @@
       <c r="D27" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="E27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1010,6 +1094,9 @@
       <c r="D28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="E28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1030,6 +1117,9 @@
       <c r="D29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="E29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1050,6 +1140,9 @@
       <c r="D30" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="E30" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1070,6 +1163,9 @@
       <c r="D31" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="E31" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1090,6 +1186,9 @@
       <c r="D32" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="E32" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1110,6 +1209,9 @@
       <c r="D33" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="E33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1130,6 +1232,9 @@
       <c r="D34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="E34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1150,6 +1255,9 @@
       <c r="D35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="E35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1170,6 +1278,9 @@
       <c r="D36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="E36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1190,6 +1301,9 @@
       <c r="D37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="E37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1210,6 +1324,9 @@
       <c r="D38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="E38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1230,6 +1347,9 @@
       <c r="D39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="E39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1250,6 +1370,9 @@
       <c r="D40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1270,6 +1393,9 @@
       <c r="D41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1290,6 +1416,9 @@
       <c r="D42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1310,6 +1439,9 @@
       <c r="D43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1330,6 +1462,9 @@
       <c r="D44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1350,6 +1485,9 @@
       <c r="D45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="E45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1370,6 +1508,9 @@
       <c r="D46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="E46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1390,6 +1531,9 @@
       <c r="D47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="E47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1410,6 +1554,9 @@
       <c r="D48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="E48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1430,6 +1577,9 @@
       <c r="D49" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="E49" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1450,6 +1600,9 @@
       <c r="D50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="E50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1470,6 +1623,9 @@
       <c r="D51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="E51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1490,6 +1646,9 @@
       <c r="D52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="E52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1510,6 +1669,9 @@
       <c r="D53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="E53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1530,6 +1692,9 @@
       <c r="D54" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="E54" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1550,6 +1715,9 @@
       <c r="D55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="E55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1570,6 +1738,9 @@
       <c r="D56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="E56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1590,6 +1761,9 @@
       <c r="D57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="E57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1610,6 +1784,9 @@
       <c r="D58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="E58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1630,6 +1807,9 @@
       <c r="D59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="E59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1650,6 +1830,9 @@
       <c r="D60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="E60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1670,6 +1853,9 @@
       <c r="D61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="E61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1690,6 +1876,9 @@
       <c r="D62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="E62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1710,6 +1899,9 @@
       <c r="D63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="E63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1730,6 +1922,9 @@
       <c r="D64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="E64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1750,6 +1945,9 @@
       <c r="D65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1770,6 +1968,9 @@
       <c r="D66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1790,6 +1991,9 @@
       <c r="D67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1810,6 +2014,9 @@
       <c r="D68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1830,6 +2037,9 @@
       <c r="D69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1850,6 +2060,9 @@
       <c r="D70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1870,6 +2083,9 @@
       <c r="D71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1890,6 +2106,9 @@
       <c r="D72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1910,6 +2129,9 @@
       <c r="D73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1930,6 +2152,9 @@
       <c r="D74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1950,6 +2175,9 @@
       <c r="D75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1970,6 +2198,9 @@
       <c r="D76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -1990,6 +2221,9 @@
       <c r="D77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2010,6 +2244,9 @@
       <c r="D78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2030,6 +2267,9 @@
       <c r="D79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2050,6 +2290,9 @@
       <c r="D80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2070,6 +2313,9 @@
       <c r="D81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2090,6 +2336,9 @@
       <c r="D82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2110,6 +2359,9 @@
       <c r="D83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2130,6 +2382,9 @@
       <c r="D84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2150,6 +2405,9 @@
       <c r="D85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2170,6 +2428,9 @@
       <c r="D86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2190,6 +2451,9 @@
       <c r="D87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2210,6 +2474,9 @@
       <c r="D88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2230,6 +2497,9 @@
       <c r="D89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2250,6 +2520,9 @@
       <c r="D90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2270,6 +2543,9 @@
       <c r="D91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2290,6 +2566,9 @@
       <c r="D92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2310,6 +2589,9 @@
       <c r="D93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2330,6 +2612,9 @@
       <c r="D94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="E94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2350,6 +2635,9 @@
       <c r="D95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="E95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2370,6 +2658,9 @@
       <c r="D96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="E96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2390,6 +2681,9 @@
       <c r="D97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="E97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2410,6 +2704,9 @@
       <c r="D98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="E98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2430,6 +2727,9 @@
       <c r="D99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="E99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2450,6 +2750,9 @@
       <c r="D100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="E100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2470,6 +2773,9 @@
       <c r="D101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="E101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2490,6 +2796,9 @@
       <c r="D102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="E102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2510,6 +2819,9 @@
       <c r="D103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="E103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2530,6 +2842,9 @@
       <c r="D104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="E104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -2550,6 +2865,9 @@
       <c r="D105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="E105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -2570,6 +2888,9 @@
       <c r="D106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="E106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -2590,6 +2911,9 @@
       <c r="D107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="E107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -2610,6 +2934,9 @@
       <c r="D108" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="E108" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -2630,6 +2957,9 @@
       <c r="D109" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="E109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -2650,6 +2980,9 @@
       <c r="D110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="E110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -2670,6 +3003,9 @@
       <c r="D111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="E111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -2690,6 +3026,9 @@
       <c r="D112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="E112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -2710,6 +3049,9 @@
       <c r="D113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="E113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -2730,6 +3072,9 @@
       <c r="D114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="E114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2750,6 +3095,9 @@
       <c r="D115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="E115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -2770,6 +3118,9 @@
       <c r="D116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -2790,6 +3141,9 @@
       <c r="D117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -2810,6 +3164,9 @@
       <c r="D118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -2830,6 +3187,9 @@
       <c r="D119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -2850,6 +3210,9 @@
       <c r="D120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -2870,6 +3233,9 @@
       <c r="D121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="E121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -2890,6 +3256,9 @@
       <c r="D122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="E122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -2910,6 +3279,9 @@
       <c r="D123" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="E123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -2930,6 +3302,9 @@
       <c r="D124" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="E124" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -2950,6 +3325,9 @@
       <c r="D125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="E125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -2970,6 +3348,9 @@
       <c r="D126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="E126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -2990,6 +3371,9 @@
       <c r="D127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="E127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3010,6 +3394,9 @@
       <c r="D128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="E128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3030,6 +3417,9 @@
       <c r="D129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="E129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3050,6 +3440,9 @@
       <c r="D130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="E130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3070,6 +3463,9 @@
       <c r="D131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="E131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3090,6 +3486,9 @@
       <c r="D132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="E132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -3110,6 +3509,9 @@
       <c r="D133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="E133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3130,6 +3532,9 @@
       <c r="D134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="E134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3150,6 +3555,9 @@
       <c r="D135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="E135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3170,6 +3578,9 @@
       <c r="D136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="E136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -3190,6 +3601,9 @@
       <c r="D137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="E137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -3210,6 +3624,9 @@
       <c r="D138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="E138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -3230,6 +3647,9 @@
       <c r="D139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -3250,6 +3670,9 @@
       <c r="D140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -3270,6 +3693,9 @@
       <c r="D141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -3290,6 +3716,9 @@
       <c r="D142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -3310,6 +3739,9 @@
       <c r="D143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -3330,6 +3762,9 @@
       <c r="D144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="E144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -3350,6 +3785,9 @@
       <c r="D145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="E145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -3370,6 +3808,9 @@
       <c r="D146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="E146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -3390,6 +3831,9 @@
       <c r="D147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="E147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -3410,6 +3854,9 @@
       <c r="D148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="E148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -3430,6 +3877,9 @@
       <c r="D149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="E149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -3450,6 +3900,9 @@
       <c r="D150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="E150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -3470,6 +3923,9 @@
       <c r="D151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="E151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -3490,6 +3946,9 @@
       <c r="D152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="E152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -3510,6 +3969,9 @@
       <c r="D153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="E153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -3530,6 +3992,9 @@
       <c r="D154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="E154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -3550,6 +4015,9 @@
       <c r="D155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="E155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -3570,6 +4038,9 @@
       <c r="D156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="E156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -3590,6 +4061,9 @@
       <c r="D157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="E157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -3610,6 +4084,9 @@
       <c r="D158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="E158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -3630,6 +4107,9 @@
       <c r="D159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="E159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -3650,6 +4130,9 @@
       <c r="D160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="E160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -3670,6 +4153,9 @@
       <c r="D161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="E161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -3690,6 +4176,9 @@
       <c r="D162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="E162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -3710,6 +4199,9 @@
       <c r="D163" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="E163" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -3730,9 +4222,12 @@
       <c r="D164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="E164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D164"/>
+  <autoFilter ref="A1:E164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-04 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$E$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$F$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -448,6 +448,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,6 +477,11 @@
           <t>2026-09-04 13:13</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -499,6 +505,9 @@
       <c r="E2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="F2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -522,6 +531,9 @@
       <c r="E3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="F3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -545,6 +557,9 @@
       <c r="E4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="F4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -568,6 +583,9 @@
       <c r="E5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="F5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -591,6 +609,9 @@
       <c r="E6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="F6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -614,6 +635,9 @@
       <c r="E7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="F7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -637,6 +661,9 @@
       <c r="E8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="F8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -660,6 +687,9 @@
       <c r="E9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="F9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -683,6 +713,9 @@
       <c r="E10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="F10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -706,6 +739,9 @@
       <c r="E11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="F11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -729,6 +765,9 @@
       <c r="E12" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="F12" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -752,6 +791,9 @@
       <c r="E13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="F13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -775,6 +817,9 @@
       <c r="E14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="F14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -798,6 +843,9 @@
       <c r="E15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="F15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -821,6 +869,9 @@
       <c r="E16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="F16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -844,6 +895,9 @@
       <c r="E17" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="F17" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -867,6 +921,9 @@
       <c r="E18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="F18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -890,6 +947,9 @@
       <c r="E19" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="F19" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -913,6 +973,9 @@
       <c r="E20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="F20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -936,6 +999,9 @@
       <c r="E21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="F21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -959,6 +1025,9 @@
       <c r="E22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="F22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -982,6 +1051,9 @@
       <c r="E23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="F23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1005,6 +1077,9 @@
       <c r="E24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="F24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1028,6 +1103,9 @@
       <c r="E25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="F25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1051,6 +1129,9 @@
       <c r="E26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="F26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1074,6 +1155,9 @@
       <c r="E27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="F27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1097,6 +1181,9 @@
       <c r="E28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="F28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1120,6 +1207,9 @@
       <c r="E29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="F29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1143,6 +1233,9 @@
       <c r="E30" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="F30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1166,6 +1259,9 @@
       <c r="E31" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="F31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1189,6 +1285,9 @@
       <c r="E32" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="F32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1212,6 +1311,9 @@
       <c r="E33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="F33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1235,6 +1337,9 @@
       <c r="E34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="F34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1258,6 +1363,9 @@
       <c r="E35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="F35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1281,6 +1389,9 @@
       <c r="E36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="F36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1304,6 +1415,9 @@
       <c r="E37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="F37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1327,6 +1441,9 @@
       <c r="E38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="F38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1350,6 +1467,9 @@
       <c r="E39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="F39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1373,6 +1493,9 @@
       <c r="E40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1396,6 +1519,9 @@
       <c r="E41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1419,6 +1545,9 @@
       <c r="E42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1442,6 +1571,9 @@
       <c r="E43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1465,6 +1597,9 @@
       <c r="E44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1488,6 +1623,9 @@
       <c r="E45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="F45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1511,6 +1649,9 @@
       <c r="E46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="F46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1534,6 +1675,9 @@
       <c r="E47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="F47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1557,6 +1701,9 @@
       <c r="E48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="F48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1580,6 +1727,9 @@
       <c r="E49" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="F49" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1603,6 +1753,9 @@
       <c r="E50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="F50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1626,6 +1779,9 @@
       <c r="E51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="F51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1649,6 +1805,9 @@
       <c r="E52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="F52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1672,6 +1831,9 @@
       <c r="E53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="F53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1695,6 +1857,9 @@
       <c r="E54" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="F54" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1718,6 +1883,9 @@
       <c r="E55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="F55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1741,6 +1909,9 @@
       <c r="E56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="F56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1764,6 +1935,9 @@
       <c r="E57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1787,6 +1961,9 @@
       <c r="E58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="F58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1810,6 +1987,9 @@
       <c r="E59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="F59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1833,6 +2013,9 @@
       <c r="E60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="F60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1856,6 +2039,9 @@
       <c r="E61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="F61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1879,6 +2065,9 @@
       <c r="E62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="F62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1902,6 +2091,9 @@
       <c r="E63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="F63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1925,6 +2117,9 @@
       <c r="E64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="F64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1948,6 +2143,9 @@
       <c r="E65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1971,6 +2169,9 @@
       <c r="E66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1994,6 +2195,9 @@
       <c r="E67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2017,6 +2221,9 @@
       <c r="E68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2040,6 +2247,9 @@
       <c r="E69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2063,6 +2273,9 @@
       <c r="E70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2086,6 +2299,9 @@
       <c r="E71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2109,6 +2325,9 @@
       <c r="E72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2132,6 +2351,9 @@
       <c r="E73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2155,6 +2377,9 @@
       <c r="E74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2178,6 +2403,9 @@
       <c r="E75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2201,6 +2429,9 @@
       <c r="E76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2224,6 +2455,9 @@
       <c r="E77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2247,6 +2481,9 @@
       <c r="E78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2270,6 +2507,9 @@
       <c r="E79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2293,6 +2533,9 @@
       <c r="E80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2316,6 +2559,9 @@
       <c r="E81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2339,6 +2585,9 @@
       <c r="E82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2362,6 +2611,9 @@
       <c r="E83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2385,6 +2637,9 @@
       <c r="E84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2408,6 +2663,9 @@
       <c r="E85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2431,6 +2689,9 @@
       <c r="E86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2454,6 +2715,9 @@
       <c r="E87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2477,6 +2741,9 @@
       <c r="E88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2500,6 +2767,9 @@
       <c r="E89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2523,6 +2793,9 @@
       <c r="E90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2546,6 +2819,9 @@
       <c r="E91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2569,6 +2845,9 @@
       <c r="E92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2592,6 +2871,9 @@
       <c r="E93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2615,6 +2897,9 @@
       <c r="E94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2638,6 +2923,9 @@
       <c r="E95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="F95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2661,6 +2949,9 @@
       <c r="E96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="F96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2684,6 +2975,9 @@
       <c r="E97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="F97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2707,6 +3001,9 @@
       <c r="E98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="F98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2730,6 +3027,9 @@
       <c r="E99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="F99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2753,6 +3053,9 @@
       <c r="E100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="F100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2776,6 +3079,9 @@
       <c r="E101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="F101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2799,6 +3105,9 @@
       <c r="E102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="F102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2822,6 +3131,9 @@
       <c r="E103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="F103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2845,6 +3157,9 @@
       <c r="E104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="F104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -2868,6 +3183,9 @@
       <c r="E105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="F105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -2891,6 +3209,9 @@
       <c r="E106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="F106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -2914,6 +3235,9 @@
       <c r="E107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="F107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -2937,6 +3261,9 @@
       <c r="E108" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="F108" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -2960,6 +3287,9 @@
       <c r="E109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="F109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -2983,6 +3313,9 @@
       <c r="E110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="F110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -3006,6 +3339,9 @@
       <c r="E111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="F111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3029,6 +3365,9 @@
       <c r="E112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="F112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3052,6 +3391,9 @@
       <c r="E113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="F113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3075,6 +3417,9 @@
       <c r="E114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="F114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -3098,6 +3443,9 @@
       <c r="E115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="F115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3121,6 +3469,9 @@
       <c r="E116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3144,6 +3495,9 @@
       <c r="E117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3167,6 +3521,9 @@
       <c r="E118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3190,6 +3547,9 @@
       <c r="E119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3213,6 +3573,9 @@
       <c r="E120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3236,6 +3599,9 @@
       <c r="E121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="F121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3259,6 +3625,9 @@
       <c r="E122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="F122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3282,6 +3651,9 @@
       <c r="E123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="F123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3305,6 +3677,9 @@
       <c r="E124" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="F124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3328,6 +3703,9 @@
       <c r="E125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="F125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3351,6 +3729,9 @@
       <c r="E126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="F126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3374,6 +3755,9 @@
       <c r="E127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="F127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3397,6 +3781,9 @@
       <c r="E128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="F128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3420,6 +3807,9 @@
       <c r="E129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="F129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3443,6 +3833,9 @@
       <c r="E130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="F130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3466,6 +3859,9 @@
       <c r="E131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="F131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3489,6 +3885,9 @@
       <c r="E132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="F132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -3512,6 +3911,9 @@
       <c r="E133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="F133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3535,6 +3937,9 @@
       <c r="E134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="F134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3558,6 +3963,9 @@
       <c r="E135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="F135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3581,6 +3989,9 @@
       <c r="E136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="F136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -3604,6 +4015,9 @@
       <c r="E137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="F137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -3627,6 +4041,9 @@
       <c r="E138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="F138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -3650,6 +4067,9 @@
       <c r="E139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -3673,6 +4093,9 @@
       <c r="E140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -3696,6 +4119,9 @@
       <c r="E141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -3719,6 +4145,9 @@
       <c r="E142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -3742,6 +4171,9 @@
       <c r="E143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -3765,6 +4197,9 @@
       <c r="E144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="F144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -3788,6 +4223,9 @@
       <c r="E145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="F145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -3811,6 +4249,9 @@
       <c r="E146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="F146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -3834,6 +4275,9 @@
       <c r="E147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="F147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -3857,6 +4301,9 @@
       <c r="E148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="F148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -3880,6 +4327,9 @@
       <c r="E149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="F149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -3903,6 +4353,9 @@
       <c r="E150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="F150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -3926,6 +4379,9 @@
       <c r="E151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="F151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -3949,6 +4405,9 @@
       <c r="E152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="F152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -3972,6 +4431,9 @@
       <c r="E153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="F153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -3995,6 +4457,9 @@
       <c r="E154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="F154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -4018,6 +4483,9 @@
       <c r="E155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="F155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -4041,6 +4509,9 @@
       <c r="E156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="F156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -4064,6 +4535,9 @@
       <c r="E157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="F157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -4087,6 +4561,9 @@
       <c r="E158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="F158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -4110,6 +4587,9 @@
       <c r="E159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="F159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -4133,6 +4613,9 @@
       <c r="E160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="F160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -4156,6 +4639,9 @@
       <c r="E161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="F161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -4179,6 +4665,9 @@
       <c r="E162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="F162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -4202,6 +4691,9 @@
       <c r="E163" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="F163" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -4225,9 +4717,12 @@
       <c r="E164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="F164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E164"/>
+  <autoFilter ref="A1:F164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 00:15 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$F$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$G$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -449,6 +449,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,6 +483,11 @@
           <t>2026-09-04 16:08</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04 19:14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -508,6 +514,9 @@
       <c r="F2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="G2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -534,6 +543,9 @@
       <c r="F3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="G3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -560,6 +572,9 @@
       <c r="F4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="G4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -586,6 +601,9 @@
       <c r="F5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="G5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -612,6 +630,9 @@
       <c r="F6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="G6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -638,6 +659,9 @@
       <c r="F7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="G7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -664,6 +688,9 @@
       <c r="F8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="G8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -690,6 +717,9 @@
       <c r="F9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="G9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -716,6 +746,9 @@
       <c r="F10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="G10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -742,6 +775,9 @@
       <c r="F11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="G11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -768,6 +804,9 @@
       <c r="F12" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="G12" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -794,6 +833,9 @@
       <c r="F13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="G13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -820,6 +862,9 @@
       <c r="F14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="G14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -846,6 +891,9 @@
       <c r="F15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="G15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -872,6 +920,9 @@
       <c r="F16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="G16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -898,6 +949,9 @@
       <c r="F17" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="G17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -924,6 +978,9 @@
       <c r="F18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="G18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -950,6 +1007,9 @@
       <c r="F19" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="G19" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -976,6 +1036,9 @@
       <c r="F20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="G20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1002,6 +1065,9 @@
       <c r="F21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="G21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1028,6 +1094,9 @@
       <c r="F22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="G22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1054,6 +1123,9 @@
       <c r="F23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="G23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1080,6 +1152,9 @@
       <c r="F24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="G24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1106,6 +1181,9 @@
       <c r="F25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="G25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1132,6 +1210,9 @@
       <c r="F26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="G26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1158,6 +1239,9 @@
       <c r="F27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="G27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1184,6 +1268,9 @@
       <c r="F28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="G28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1210,6 +1297,9 @@
       <c r="F29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="G29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1236,6 +1326,9 @@
       <c r="F30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="G30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1262,6 +1355,9 @@
       <c r="F31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="G31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1288,6 +1384,9 @@
       <c r="F32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="G32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1314,6 +1413,9 @@
       <c r="F33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="G33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1340,6 +1442,9 @@
       <c r="F34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="G34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1366,6 +1471,9 @@
       <c r="F35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="G35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1392,6 +1500,9 @@
       <c r="F36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="G36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1418,6 +1529,9 @@
       <c r="F37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="G37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1444,6 +1558,9 @@
       <c r="F38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="G38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1470,6 +1587,9 @@
       <c r="F39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="G39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1496,6 +1616,9 @@
       <c r="F40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1522,6 +1645,9 @@
       <c r="F41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1548,6 +1674,9 @@
       <c r="F42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1574,6 +1703,9 @@
       <c r="F43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1600,6 +1732,9 @@
       <c r="F44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1626,6 +1761,9 @@
       <c r="F45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="G45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1652,6 +1790,9 @@
       <c r="F46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="G46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1678,6 +1819,9 @@
       <c r="F47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="G47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1704,6 +1848,9 @@
       <c r="F48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="G48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1730,6 +1877,9 @@
       <c r="F49" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="G49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1756,6 +1906,9 @@
       <c r="F50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="G50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1782,6 +1935,9 @@
       <c r="F51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="G51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1808,6 +1964,9 @@
       <c r="F52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="G52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1834,6 +1993,9 @@
       <c r="F53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="G53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1860,6 +2022,9 @@
       <c r="F54" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="G54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1886,6 +2051,9 @@
       <c r="F55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="G55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1912,6 +2080,9 @@
       <c r="F56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="G56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1938,6 +2109,9 @@
       <c r="F57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1964,6 +2138,9 @@
       <c r="F58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="G58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1990,6 +2167,9 @@
       <c r="F59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="G59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2016,6 +2196,9 @@
       <c r="F60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="G60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2042,6 +2225,9 @@
       <c r="F61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="G61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2068,6 +2254,9 @@
       <c r="F62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="G62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2094,6 +2283,9 @@
       <c r="F63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="G63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2120,6 +2312,9 @@
       <c r="F64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="G64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2146,6 +2341,9 @@
       <c r="F65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2172,6 +2370,9 @@
       <c r="F66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2198,6 +2399,9 @@
       <c r="F67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2224,6 +2428,9 @@
       <c r="F68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2250,6 +2457,9 @@
       <c r="F69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2276,6 +2486,9 @@
       <c r="F70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2302,6 +2515,9 @@
       <c r="F71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2328,6 +2544,9 @@
       <c r="F72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2354,6 +2573,9 @@
       <c r="F73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2380,6 +2602,9 @@
       <c r="F74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2406,6 +2631,9 @@
       <c r="F75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2432,6 +2660,9 @@
       <c r="F76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2458,6 +2689,9 @@
       <c r="F77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2484,6 +2718,9 @@
       <c r="F78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2510,6 +2747,9 @@
       <c r="F79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2536,6 +2776,9 @@
       <c r="F80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2562,6 +2805,9 @@
       <c r="F81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2588,6 +2834,9 @@
       <c r="F82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2614,6 +2863,9 @@
       <c r="F83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2640,6 +2892,9 @@
       <c r="F84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2666,6 +2921,9 @@
       <c r="F85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2692,6 +2950,9 @@
       <c r="F86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2718,6 +2979,9 @@
       <c r="F87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2744,6 +3008,9 @@
       <c r="F88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2770,6 +3037,9 @@
       <c r="F89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2796,6 +3066,9 @@
       <c r="F90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2822,6 +3095,9 @@
       <c r="F91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2848,6 +3124,9 @@
       <c r="F92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2874,6 +3153,9 @@
       <c r="F93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2900,6 +3182,9 @@
       <c r="F94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2926,6 +3211,9 @@
       <c r="F95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="G95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2952,6 +3240,9 @@
       <c r="F96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="G96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2978,6 +3269,9 @@
       <c r="F97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="G97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3004,6 +3298,9 @@
       <c r="F98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="G98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3030,6 +3327,9 @@
       <c r="F99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="G99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3056,6 +3356,9 @@
       <c r="F100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="G100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3082,6 +3385,9 @@
       <c r="F101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="G101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3108,6 +3414,9 @@
       <c r="F102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="G102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3134,6 +3443,9 @@
       <c r="F103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="G103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3160,6 +3472,9 @@
       <c r="F104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="G104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3186,6 +3501,9 @@
       <c r="F105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="G105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3212,6 +3530,9 @@
       <c r="F106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="G106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3238,6 +3559,9 @@
       <c r="F107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="G107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3264,6 +3588,9 @@
       <c r="F108" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="G108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3290,6 +3617,9 @@
       <c r="F109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="G109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3316,6 +3646,9 @@
       <c r="F110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="G110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -3342,6 +3675,9 @@
       <c r="F111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="G111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3368,6 +3704,9 @@
       <c r="F112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="G112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3394,6 +3733,9 @@
       <c r="F113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="G113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3420,6 +3762,9 @@
       <c r="F114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="G114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -3446,6 +3791,9 @@
       <c r="F115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="G115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3472,6 +3820,9 @@
       <c r="F116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3498,6 +3849,9 @@
       <c r="F117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3524,6 +3878,9 @@
       <c r="F118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3550,6 +3907,9 @@
       <c r="F119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3576,6 +3936,9 @@
       <c r="F120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3602,6 +3965,9 @@
       <c r="F121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="G121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3628,6 +3994,9 @@
       <c r="F122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="G122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3654,6 +4023,9 @@
       <c r="F123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="G123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3680,6 +4052,9 @@
       <c r="F124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="G124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3706,6 +4081,9 @@
       <c r="F125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="G125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3732,6 +4110,9 @@
       <c r="F126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="G126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3758,6 +4139,9 @@
       <c r="F127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="G127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3784,6 +4168,9 @@
       <c r="F128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="G128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3810,6 +4197,9 @@
       <c r="F129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="G129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3836,6 +4226,9 @@
       <c r="F130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="G130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3862,6 +4255,9 @@
       <c r="F131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="G131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3888,6 +4284,9 @@
       <c r="F132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="G132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -3914,6 +4313,9 @@
       <c r="F133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="G133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3940,6 +4342,9 @@
       <c r="F134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="G134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3966,6 +4371,9 @@
       <c r="F135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="G135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3992,6 +4400,9 @@
       <c r="F136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="G136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -4018,6 +4429,9 @@
       <c r="F137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="G137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4044,6 +4458,9 @@
       <c r="F138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="G138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -4070,6 +4487,9 @@
       <c r="F139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -4096,6 +4516,9 @@
       <c r="F140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -4122,6 +4545,9 @@
       <c r="F141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4148,6 +4574,9 @@
       <c r="F142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -4174,6 +4603,9 @@
       <c r="F143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -4200,6 +4632,9 @@
       <c r="F144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="G144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -4226,6 +4661,9 @@
       <c r="F145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="G145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -4252,6 +4690,9 @@
       <c r="F146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="G146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -4278,6 +4719,9 @@
       <c r="F147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="G147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -4304,6 +4748,9 @@
       <c r="F148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="G148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -4330,6 +4777,9 @@
       <c r="F149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="G149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4356,6 +4806,9 @@
       <c r="F150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="G150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -4382,6 +4835,9 @@
       <c r="F151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="G151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -4408,6 +4864,9 @@
       <c r="F152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="G152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -4434,6 +4893,9 @@
       <c r="F153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="G153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -4460,6 +4922,9 @@
       <c r="F154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="G154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -4486,6 +4951,9 @@
       <c r="F155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="G155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -4512,6 +4980,9 @@
       <c r="F156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="G156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -4538,6 +5009,9 @@
       <c r="F157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="G157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -4564,6 +5038,9 @@
       <c r="F158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="G158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -4590,6 +5067,9 @@
       <c r="F159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="G159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -4616,6 +5096,9 @@
       <c r="F160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="G160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -4642,6 +5125,9 @@
       <c r="F161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="G161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -4668,6 +5154,9 @@
       <c r="F162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="G162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -4694,6 +5183,9 @@
       <c r="F163" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="G163" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -4720,9 +5212,12 @@
       <c r="F164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="G164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F164"/>
+  <autoFilter ref="A1:G164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$G$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$H$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:H164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,6 +489,11 @@
           <t>2026-09-04 19:14</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -517,6 +523,9 @@
       <c r="G2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="H2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -546,6 +555,9 @@
       <c r="G3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="H3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -575,6 +587,9 @@
       <c r="G4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="H4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -604,6 +619,9 @@
       <c r="G5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="H5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -633,6 +651,9 @@
       <c r="G6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="H6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -662,6 +683,9 @@
       <c r="G7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="H7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -691,6 +715,9 @@
       <c r="G8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="H8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -720,6 +747,9 @@
       <c r="G9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="H9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -749,6 +779,9 @@
       <c r="G10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="H10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -778,6 +811,9 @@
       <c r="G11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="H11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -807,6 +843,9 @@
       <c r="G12" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="H12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -836,6 +875,9 @@
       <c r="G13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="H13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -865,6 +907,9 @@
       <c r="G14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="H14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -894,6 +939,9 @@
       <c r="G15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="H15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -923,6 +971,9 @@
       <c r="G16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="H16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -952,6 +1003,9 @@
       <c r="G17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="H17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -981,6 +1035,9 @@
       <c r="G18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="H18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1010,6 +1067,9 @@
       <c r="G19" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="H19" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1039,6 +1099,9 @@
       <c r="G20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="H20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1068,6 +1131,9 @@
       <c r="G21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="H21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1097,6 +1163,9 @@
       <c r="G22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="H22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1126,6 +1195,9 @@
       <c r="G23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="H23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1155,6 +1227,9 @@
       <c r="G24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1184,6 +1259,9 @@
       <c r="G25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="H25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1213,6 +1291,9 @@
       <c r="G26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="H26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1242,6 +1323,9 @@
       <c r="G27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1271,6 +1355,9 @@
       <c r="G28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="H28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1300,6 +1387,9 @@
       <c r="G29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="H29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1329,6 +1419,9 @@
       <c r="G30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="H30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1358,6 +1451,9 @@
       <c r="G31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="H31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1387,6 +1483,9 @@
       <c r="G32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="H32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1416,6 +1515,9 @@
       <c r="G33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="H33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1445,6 +1547,9 @@
       <c r="G34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="H34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1474,6 +1579,9 @@
       <c r="G35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="H35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1503,6 +1611,9 @@
       <c r="G36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="H36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1532,6 +1643,9 @@
       <c r="G37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="H37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1561,6 +1675,9 @@
       <c r="G38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="H38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1590,6 +1707,9 @@
       <c r="G39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="H39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1619,6 +1739,9 @@
       <c r="G40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1648,6 +1771,9 @@
       <c r="G41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1677,6 +1803,9 @@
       <c r="G42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1706,6 +1835,9 @@
       <c r="G43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1735,6 +1867,9 @@
       <c r="G44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1764,6 +1899,9 @@
       <c r="G45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="H45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1793,6 +1931,9 @@
       <c r="G46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="H46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1822,6 +1963,9 @@
       <c r="G47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="H47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1851,6 +1995,9 @@
       <c r="G48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="H48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1880,6 +2027,9 @@
       <c r="G49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1909,6 +2059,9 @@
       <c r="G50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="H50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1938,6 +2091,9 @@
       <c r="G51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="H51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1967,6 +2123,9 @@
       <c r="G52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="H52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1996,6 +2155,9 @@
       <c r="G53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="H53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2025,6 +2187,9 @@
       <c r="G54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="H54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2054,6 +2219,9 @@
       <c r="G55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="H55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2083,6 +2251,9 @@
       <c r="G56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="H56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2112,6 +2283,9 @@
       <c r="G57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2141,6 +2315,9 @@
       <c r="G58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="H58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2170,6 +2347,9 @@
       <c r="G59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="H59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2199,6 +2379,9 @@
       <c r="G60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="H60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2228,6 +2411,9 @@
       <c r="G61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="H61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2257,6 +2443,9 @@
       <c r="G62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="H62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2286,6 +2475,9 @@
       <c r="G63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="H63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2315,6 +2507,9 @@
       <c r="G64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="H64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2344,6 +2539,9 @@
       <c r="G65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2373,6 +2571,9 @@
       <c r="G66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2402,6 +2603,9 @@
       <c r="G67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2431,6 +2635,9 @@
       <c r="G68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2460,6 +2667,9 @@
       <c r="G69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2489,6 +2699,9 @@
       <c r="G70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2518,6 +2731,9 @@
       <c r="G71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2547,6 +2763,9 @@
       <c r="G72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2576,6 +2795,9 @@
       <c r="G73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2605,6 +2827,9 @@
       <c r="G74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2634,6 +2859,9 @@
       <c r="G75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2663,6 +2891,9 @@
       <c r="G76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2692,6 +2923,9 @@
       <c r="G77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2721,6 +2955,9 @@
       <c r="G78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2750,6 +2987,9 @@
       <c r="G79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2779,6 +3019,9 @@
       <c r="G80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2808,6 +3051,9 @@
       <c r="G81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2837,6 +3083,9 @@
       <c r="G82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2866,6 +3115,9 @@
       <c r="G83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2895,6 +3147,9 @@
       <c r="G84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2924,6 +3179,9 @@
       <c r="G85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2953,6 +3211,9 @@
       <c r="G86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2982,6 +3243,9 @@
       <c r="G87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3011,6 +3275,9 @@
       <c r="G88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3040,6 +3307,9 @@
       <c r="G89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3069,6 +3339,9 @@
       <c r="G90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3098,6 +3371,9 @@
       <c r="G91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3127,6 +3403,9 @@
       <c r="G92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3156,6 +3435,9 @@
       <c r="G93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3185,6 +3467,9 @@
       <c r="G94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3214,6 +3499,9 @@
       <c r="G95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="H95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3243,6 +3531,9 @@
       <c r="G96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="H96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3272,6 +3563,9 @@
       <c r="G97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="H97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3301,6 +3595,9 @@
       <c r="G98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3330,6 +3627,9 @@
       <c r="G99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3359,6 +3659,9 @@
       <c r="G100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="H100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3388,6 +3691,9 @@
       <c r="G101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="H101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3417,6 +3723,9 @@
       <c r="G102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="H102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3446,6 +3755,9 @@
       <c r="G103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="H103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3475,6 +3787,9 @@
       <c r="G104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="H104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3504,6 +3819,9 @@
       <c r="G105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="H105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3533,6 +3851,9 @@
       <c r="G106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="H106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3562,6 +3883,9 @@
       <c r="G107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="H107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3591,6 +3915,9 @@
       <c r="G108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3620,6 +3947,9 @@
       <c r="G109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="H109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3649,6 +3979,9 @@
       <c r="G110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="H110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -3678,6 +4011,9 @@
       <c r="G111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="H111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3707,6 +4043,9 @@
       <c r="G112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="H112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3736,6 +4075,9 @@
       <c r="G113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="H113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3765,6 +4107,9 @@
       <c r="G114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="H114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -3794,6 +4139,9 @@
       <c r="G115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="H115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3823,6 +4171,9 @@
       <c r="G116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3852,6 +4203,9 @@
       <c r="G117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3881,6 +4235,9 @@
       <c r="G118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3910,6 +4267,9 @@
       <c r="G119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3939,6 +4299,9 @@
       <c r="G120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3968,6 +4331,9 @@
       <c r="G121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="H121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3997,6 +4363,9 @@
       <c r="G122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="H122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4026,6 +4395,9 @@
       <c r="G123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="H123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4055,6 +4427,9 @@
       <c r="G124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="H124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4084,6 +4459,9 @@
       <c r="G125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="H125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4113,6 +4491,9 @@
       <c r="G126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="H126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -4142,6 +4523,9 @@
       <c r="G127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="H127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4171,6 +4555,9 @@
       <c r="G128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="H128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -4200,6 +4587,9 @@
       <c r="G129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="H129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -4229,6 +4619,9 @@
       <c r="G130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="H130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -4258,6 +4651,9 @@
       <c r="G131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="H131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -4287,6 +4683,9 @@
       <c r="G132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="H132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -4316,6 +4715,9 @@
       <c r="G133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="H133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4345,6 +4747,9 @@
       <c r="G134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="H134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -4374,6 +4779,9 @@
       <c r="G135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="H135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -4403,6 +4811,9 @@
       <c r="G136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="H136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -4432,6 +4843,9 @@
       <c r="G137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="H137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4461,6 +4875,9 @@
       <c r="G138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="H138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -4490,6 +4907,9 @@
       <c r="G139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -4519,6 +4939,9 @@
       <c r="G140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -4548,6 +4971,9 @@
       <c r="G141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4577,6 +5003,9 @@
       <c r="G142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -4606,6 +5035,9 @@
       <c r="G143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -4635,6 +5067,9 @@
       <c r="G144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="H144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -4664,6 +5099,9 @@
       <c r="G145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="H145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -4693,6 +5131,9 @@
       <c r="G146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="H146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -4722,6 +5163,9 @@
       <c r="G147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="H147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -4751,6 +5195,9 @@
       <c r="G148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="H148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -4780,6 +5227,9 @@
       <c r="G149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="H149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4809,6 +5259,9 @@
       <c r="G150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="H150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -4838,6 +5291,9 @@
       <c r="G151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="H151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -4867,6 +5323,9 @@
       <c r="G152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="H152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -4896,6 +5355,9 @@
       <c r="G153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="H153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -4925,6 +5387,9 @@
       <c r="G154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="H154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -4954,6 +5419,9 @@
       <c r="G155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="H155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -4983,6 +5451,9 @@
       <c r="G156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="H156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -5012,6 +5483,9 @@
       <c r="G157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="H157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -5041,6 +5515,9 @@
       <c r="G158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="H158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -5070,6 +5547,9 @@
       <c r="G159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="H159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -5099,6 +5579,9 @@
       <c r="G160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="H160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -5128,6 +5611,9 @@
       <c r="G161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="H161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -5157,6 +5643,9 @@
       <c r="G162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="H162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -5186,6 +5675,9 @@
       <c r="G163" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="H163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -5215,9 +5707,12 @@
       <c r="G164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="H164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G164"/>
+  <autoFilter ref="A1:H164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 06:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$H$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$I$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H164"/>
+  <dimension ref="A1:I164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -451,6 +451,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,6 +495,11 @@
           <t>2026-09-04 22:09</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 01:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -526,6 +532,9 @@
       <c r="H2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -558,6 +567,9 @@
       <c r="H3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="I3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -590,6 +602,9 @@
       <c r="H4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="I4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -622,6 +637,9 @@
       <c r="H5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="I5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -654,6 +672,9 @@
       <c r="H6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -686,6 +707,9 @@
       <c r="H7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="I7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -718,6 +742,9 @@
       <c r="H8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="I8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -750,6 +777,9 @@
       <c r="H9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="I9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -782,6 +812,9 @@
       <c r="H10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="I10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -814,6 +847,9 @@
       <c r="H11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="I11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -846,6 +882,9 @@
       <c r="H12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -878,6 +917,9 @@
       <c r="H13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="I13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -910,6 +952,9 @@
       <c r="H14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="I14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -942,6 +987,9 @@
       <c r="H15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="I15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -974,6 +1022,9 @@
       <c r="H16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="I16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1006,6 +1057,9 @@
       <c r="H17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="I17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1038,6 +1092,9 @@
       <c r="H18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="I18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1070,6 +1127,9 @@
       <c r="H19" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="I19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1102,6 +1162,9 @@
       <c r="H20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="I20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1134,6 +1197,9 @@
       <c r="H21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="I21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1166,6 +1232,9 @@
       <c r="H22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="I22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1198,6 +1267,9 @@
       <c r="H23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="I23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1230,6 +1302,9 @@
       <c r="H24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1262,6 +1337,9 @@
       <c r="H25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="I25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1294,6 +1372,9 @@
       <c r="H26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="I26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1326,6 +1407,9 @@
       <c r="H27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1358,6 +1442,9 @@
       <c r="H28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="I28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1390,6 +1477,9 @@
       <c r="H29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="I29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1422,6 +1512,9 @@
       <c r="H30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="I30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1454,6 +1547,9 @@
       <c r="H31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="I31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1486,6 +1582,9 @@
       <c r="H32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="I32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1518,6 +1617,9 @@
       <c r="H33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="I33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1550,6 +1652,9 @@
       <c r="H34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="I34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1582,6 +1687,9 @@
       <c r="H35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="I35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1614,6 +1722,9 @@
       <c r="H36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="I36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1646,6 +1757,9 @@
       <c r="H37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="I37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1678,6 +1792,9 @@
       <c r="H38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="I38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1710,6 +1827,9 @@
       <c r="H39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="I39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1742,6 +1862,9 @@
       <c r="H40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1774,6 +1897,9 @@
       <c r="H41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1806,6 +1932,9 @@
       <c r="H42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1838,6 +1967,9 @@
       <c r="H43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1870,6 +2002,9 @@
       <c r="H44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1902,6 +2037,9 @@
       <c r="H45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="I45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1934,6 +2072,9 @@
       <c r="H46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="I46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1966,6 +2107,9 @@
       <c r="H47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="I47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1998,6 +2142,9 @@
       <c r="H48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="I48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2030,6 +2177,9 @@
       <c r="H49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2062,6 +2212,9 @@
       <c r="H50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="I50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2094,6 +2247,9 @@
       <c r="H51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="I51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2126,6 +2282,9 @@
       <c r="H52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="I52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2158,6 +2317,9 @@
       <c r="H53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="I53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2190,6 +2352,9 @@
       <c r="H54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="I54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2222,6 +2387,9 @@
       <c r="H55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="I55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2254,6 +2422,9 @@
       <c r="H56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="I56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2286,6 +2457,9 @@
       <c r="H57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2318,6 +2492,9 @@
       <c r="H58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="I58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2350,6 +2527,9 @@
       <c r="H59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="I59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2382,6 +2562,9 @@
       <c r="H60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="I60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2414,6 +2597,9 @@
       <c r="H61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="I61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2446,6 +2632,9 @@
       <c r="H62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="I62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2478,6 +2667,9 @@
       <c r="H63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="I63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2510,6 +2702,9 @@
       <c r="H64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="I64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2542,6 +2737,9 @@
       <c r="H65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2574,6 +2772,9 @@
       <c r="H66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2606,6 +2807,9 @@
       <c r="H67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2638,6 +2842,9 @@
       <c r="H68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2670,6 +2877,9 @@
       <c r="H69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2702,6 +2912,9 @@
       <c r="H70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2734,6 +2947,9 @@
       <c r="H71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2766,6 +2982,9 @@
       <c r="H72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2798,6 +3017,9 @@
       <c r="H73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2830,6 +3052,9 @@
       <c r="H74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2862,6 +3087,9 @@
       <c r="H75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2894,6 +3122,9 @@
       <c r="H76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2926,6 +3157,9 @@
       <c r="H77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2958,6 +3192,9 @@
       <c r="H78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2990,6 +3227,9 @@
       <c r="H79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3022,6 +3262,9 @@
       <c r="H80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3054,6 +3297,9 @@
       <c r="H81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3086,6 +3332,9 @@
       <c r="H82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3118,6 +3367,9 @@
       <c r="H83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3150,6 +3402,9 @@
       <c r="H84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3182,6 +3437,9 @@
       <c r="H85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3214,6 +3472,9 @@
       <c r="H86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3246,6 +3507,9 @@
       <c r="H87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3278,6 +3542,9 @@
       <c r="H88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3310,6 +3577,9 @@
       <c r="H89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3342,6 +3612,9 @@
       <c r="H90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3374,6 +3647,9 @@
       <c r="H91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3406,6 +3682,9 @@
       <c r="H92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3438,6 +3717,9 @@
       <c r="H93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3470,6 +3752,9 @@
       <c r="H94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3502,6 +3787,9 @@
       <c r="H95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="I95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3534,6 +3822,9 @@
       <c r="H96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="I96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3566,6 +3857,9 @@
       <c r="H97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="I97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3598,6 +3892,9 @@
       <c r="H98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3630,6 +3927,9 @@
       <c r="H99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3662,6 +3962,9 @@
       <c r="H100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="I100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3694,6 +3997,9 @@
       <c r="H101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="I101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3726,6 +4032,9 @@
       <c r="H102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="I102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3758,6 +4067,9 @@
       <c r="H103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="I103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3790,6 +4102,9 @@
       <c r="H104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="I104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3822,6 +4137,9 @@
       <c r="H105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="I105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3854,6 +4172,9 @@
       <c r="H106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="I106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3886,6 +4207,9 @@
       <c r="H107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="I107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3918,6 +4242,9 @@
       <c r="H108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3950,6 +4277,9 @@
       <c r="H109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="I109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3982,6 +4312,9 @@
       <c r="H110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="I110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4014,6 +4347,9 @@
       <c r="H111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="I111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4046,6 +4382,9 @@
       <c r="H112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="I112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4078,6 +4417,9 @@
       <c r="H113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="I113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4110,6 +4452,9 @@
       <c r="H114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="I114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4142,6 +4487,9 @@
       <c r="H115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="I115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4174,6 +4522,9 @@
       <c r="H116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4206,6 +4557,9 @@
       <c r="H117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4238,6 +4592,9 @@
       <c r="H118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4270,6 +4627,9 @@
       <c r="H119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4302,6 +4662,9 @@
       <c r="H120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4334,6 +4697,9 @@
       <c r="H121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="I121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4366,6 +4732,9 @@
       <c r="H122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="I122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4398,6 +4767,9 @@
       <c r="H123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="I123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4430,6 +4802,9 @@
       <c r="H124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="I124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4462,6 +4837,9 @@
       <c r="H125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="I125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4494,6 +4872,9 @@
       <c r="H126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="I126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -4526,6 +4907,9 @@
       <c r="H127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="I127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4558,6 +4942,9 @@
       <c r="H128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="I128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -4590,6 +4977,9 @@
       <c r="H129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="I129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -4622,6 +5012,9 @@
       <c r="H130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="I130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -4654,6 +5047,9 @@
       <c r="H131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="I131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -4686,6 +5082,9 @@
       <c r="H132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="I132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -4718,6 +5117,9 @@
       <c r="H133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="I133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4750,6 +5152,9 @@
       <c r="H134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="I134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -4782,6 +5187,9 @@
       <c r="H135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="I135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -4814,6 +5222,9 @@
       <c r="H136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="I136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -4846,6 +5257,9 @@
       <c r="H137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="I137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4878,6 +5292,9 @@
       <c r="H138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="I138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -4910,6 +5327,9 @@
       <c r="H139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -4942,6 +5362,9 @@
       <c r="H140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -4974,6 +5397,9 @@
       <c r="H141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5006,6 +5432,9 @@
       <c r="H142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5038,6 +5467,9 @@
       <c r="H143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5070,6 +5502,9 @@
       <c r="H144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="I144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5102,6 +5537,9 @@
       <c r="H145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="I145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5134,6 +5572,9 @@
       <c r="H146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="I146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5166,6 +5607,9 @@
       <c r="H147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="I147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5198,6 +5642,9 @@
       <c r="H148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="I148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -5230,6 +5677,9 @@
       <c r="H149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="I149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -5262,6 +5712,9 @@
       <c r="H150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="I150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -5294,6 +5747,9 @@
       <c r="H151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="I151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5326,6 +5782,9 @@
       <c r="H152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="I152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5358,6 +5817,9 @@
       <c r="H153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="I153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -5390,6 +5852,9 @@
       <c r="H154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="I154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -5422,6 +5887,9 @@
       <c r="H155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="I155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -5454,6 +5922,9 @@
       <c r="H156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="I156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -5486,6 +5957,9 @@
       <c r="H157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="I157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -5518,6 +5992,9 @@
       <c r="H158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="I158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -5550,6 +6027,9 @@
       <c r="H159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="I159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -5582,6 +6062,9 @@
       <c r="H160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="I160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -5614,6 +6097,9 @@
       <c r="H161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="I161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -5646,6 +6132,9 @@
       <c r="H162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="I162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -5678,6 +6167,9 @@
       <c r="H163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="I163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -5710,9 +6202,12 @@
       <c r="H164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="I164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H164"/>
+  <autoFilter ref="A1:I164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 09:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$I$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$J$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I164"/>
+  <dimension ref="A1:J164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -452,6 +452,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,6 +501,11 @@
           <t>2026-09-05 01:11</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 04:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -535,6 +541,9 @@
       <c r="I2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="J2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -570,6 +579,9 @@
       <c r="I3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="J3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -605,6 +617,9 @@
       <c r="I4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="J4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -640,6 +655,9 @@
       <c r="I5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="J5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -675,6 +693,9 @@
       <c r="I6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="J6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -710,6 +731,9 @@
       <c r="I7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="J7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -745,6 +769,9 @@
       <c r="I8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="J8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -780,6 +807,9 @@
       <c r="I9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="J9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -815,6 +845,9 @@
       <c r="I10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="J10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -850,6 +883,9 @@
       <c r="I11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="J11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -885,6 +921,9 @@
       <c r="I12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -920,6 +959,9 @@
       <c r="I13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="J13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -955,6 +997,9 @@
       <c r="I14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="J14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -990,6 +1035,9 @@
       <c r="I15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="J15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1025,6 +1073,9 @@
       <c r="I16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="J16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1060,6 +1111,9 @@
       <c r="I17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="J17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1095,6 +1149,9 @@
       <c r="I18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="J18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1130,6 +1187,9 @@
       <c r="I19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="J19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1165,6 +1225,9 @@
       <c r="I20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="J20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1200,6 +1263,9 @@
       <c r="I21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="J21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1235,6 +1301,9 @@
       <c r="I22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="J22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1270,6 +1339,9 @@
       <c r="I23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="J23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1305,6 +1377,9 @@
       <c r="I24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1340,6 +1415,9 @@
       <c r="I25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="J25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1375,6 +1453,9 @@
       <c r="I26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="J26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1410,6 +1491,9 @@
       <c r="I27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1445,6 +1529,9 @@
       <c r="I28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="J28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1480,6 +1567,9 @@
       <c r="I29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="J29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1515,6 +1605,9 @@
       <c r="I30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="J30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1550,6 +1643,9 @@
       <c r="I31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="J31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1585,6 +1681,9 @@
       <c r="I32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="J32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1620,6 +1719,9 @@
       <c r="I33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="J33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1655,6 +1757,9 @@
       <c r="I34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="J34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1690,6 +1795,9 @@
       <c r="I35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="J35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1725,6 +1833,9 @@
       <c r="I36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="J36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1760,6 +1871,9 @@
       <c r="I37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="J37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1795,6 +1909,9 @@
       <c r="I38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="J38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1830,6 +1947,9 @@
       <c r="I39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="J39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1865,6 +1985,9 @@
       <c r="I40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1900,6 +2023,9 @@
       <c r="I41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1935,6 +2061,9 @@
       <c r="I42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1970,6 +2099,9 @@
       <c r="I43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2005,6 +2137,9 @@
       <c r="I44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2040,6 +2175,9 @@
       <c r="I45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="J45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2075,6 +2213,9 @@
       <c r="I46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="J46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2110,6 +2251,9 @@
       <c r="I47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="J47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2145,6 +2289,9 @@
       <c r="I48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="J48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2180,6 +2327,9 @@
       <c r="I49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2215,6 +2365,9 @@
       <c r="I50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="J50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2250,6 +2403,9 @@
       <c r="I51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="J51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2285,6 +2441,9 @@
       <c r="I52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="J52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2320,6 +2479,9 @@
       <c r="I53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="J53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2355,6 +2517,9 @@
       <c r="I54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="J54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2390,6 +2555,9 @@
       <c r="I55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="J55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2425,6 +2593,9 @@
       <c r="I56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="J56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2460,6 +2631,9 @@
       <c r="I57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2495,6 +2669,9 @@
       <c r="I58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="J58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2530,6 +2707,9 @@
       <c r="I59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="J59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2565,6 +2745,9 @@
       <c r="I60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="J60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2600,6 +2783,9 @@
       <c r="I61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="J61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2635,6 +2821,9 @@
       <c r="I62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="J62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2670,6 +2859,9 @@
       <c r="I63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="J63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2705,6 +2897,9 @@
       <c r="I64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="J64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2740,6 +2935,9 @@
       <c r="I65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2775,6 +2973,9 @@
       <c r="I66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2810,6 +3011,9 @@
       <c r="I67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2845,6 +3049,9 @@
       <c r="I68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2880,6 +3087,9 @@
       <c r="I69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2915,6 +3125,9 @@
       <c r="I70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2950,6 +3163,9 @@
       <c r="I71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2985,6 +3201,9 @@
       <c r="I72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3020,6 +3239,9 @@
       <c r="I73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3055,6 +3277,9 @@
       <c r="I74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3090,6 +3315,9 @@
       <c r="I75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3125,6 +3353,9 @@
       <c r="I76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3160,6 +3391,9 @@
       <c r="I77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3195,6 +3429,9 @@
       <c r="I78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3230,6 +3467,9 @@
       <c r="I79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3265,6 +3505,9 @@
       <c r="I80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3300,6 +3543,9 @@
       <c r="I81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3335,6 +3581,9 @@
       <c r="I82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3370,6 +3619,9 @@
       <c r="I83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3405,6 +3657,9 @@
       <c r="I84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3440,6 +3695,9 @@
       <c r="I85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J85" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3475,6 +3733,9 @@
       <c r="I86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3510,6 +3771,9 @@
       <c r="I87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3545,6 +3809,9 @@
       <c r="I88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3580,6 +3847,9 @@
       <c r="I89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3615,6 +3885,9 @@
       <c r="I90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3650,6 +3923,9 @@
       <c r="I91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3685,6 +3961,9 @@
       <c r="I92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3720,6 +3999,9 @@
       <c r="I93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3755,6 +4037,9 @@
       <c r="I94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3790,6 +4075,9 @@
       <c r="I95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="J95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3825,6 +4113,9 @@
       <c r="I96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="J96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3860,6 +4151,9 @@
       <c r="I97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="J97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3895,6 +4189,9 @@
       <c r="I98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3930,6 +4227,9 @@
       <c r="I99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3965,6 +4265,9 @@
       <c r="I100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="J100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4000,6 +4303,9 @@
       <c r="I101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="J101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4035,6 +4341,9 @@
       <c r="I102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="J102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4070,6 +4379,9 @@
       <c r="I103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="J103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4105,6 +4417,9 @@
       <c r="I104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="J104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4140,6 +4455,9 @@
       <c r="I105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="J105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4175,6 +4493,9 @@
       <c r="I106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="J106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4210,6 +4531,9 @@
       <c r="I107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="J107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4245,6 +4569,9 @@
       <c r="I108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4280,6 +4607,9 @@
       <c r="I109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="J109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4315,6 +4645,9 @@
       <c r="I110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="J110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4350,6 +4683,9 @@
       <c r="I111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="J111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4385,6 +4721,9 @@
       <c r="I112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="J112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4420,6 +4759,9 @@
       <c r="I113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="J113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4455,6 +4797,9 @@
       <c r="I114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="J114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4490,6 +4835,9 @@
       <c r="I115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="J115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4525,6 +4873,9 @@
       <c r="I116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4560,6 +4911,9 @@
       <c r="I117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4595,6 +4949,9 @@
       <c r="I118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4630,6 +4987,9 @@
       <c r="I119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4665,6 +5025,9 @@
       <c r="I120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4700,6 +5063,9 @@
       <c r="I121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="J121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4735,6 +5101,9 @@
       <c r="I122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="J122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4770,6 +5139,9 @@
       <c r="I123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="J123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4805,6 +5177,9 @@
       <c r="I124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="J124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4840,6 +5215,9 @@
       <c r="I125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="J125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4875,6 +5253,9 @@
       <c r="I126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="J126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -4910,6 +5291,9 @@
       <c r="I127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="J127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4945,6 +5329,9 @@
       <c r="I128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="J128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -4980,6 +5367,9 @@
       <c r="I129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="J129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5015,6 +5405,9 @@
       <c r="I130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="J130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5050,6 +5443,9 @@
       <c r="I131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="J131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5085,6 +5481,9 @@
       <c r="I132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="J132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5120,6 +5519,9 @@
       <c r="I133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="J133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5155,6 +5557,9 @@
       <c r="I134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="J134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5190,6 +5595,9 @@
       <c r="I135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="J135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5225,6 +5633,9 @@
       <c r="I136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="J136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5260,6 +5671,9 @@
       <c r="I137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="J137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5295,6 +5709,9 @@
       <c r="I138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="J138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5330,6 +5747,9 @@
       <c r="I139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -5365,6 +5785,9 @@
       <c r="I140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5400,6 +5823,9 @@
       <c r="I141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5435,6 +5861,9 @@
       <c r="I142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5470,6 +5899,9 @@
       <c r="I143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5505,6 +5937,9 @@
       <c r="I144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="J144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5540,6 +5975,9 @@
       <c r="I145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="J145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5575,6 +6013,9 @@
       <c r="I146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="J146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5610,6 +6051,9 @@
       <c r="I147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="J147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5645,6 +6089,9 @@
       <c r="I148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="J148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -5680,6 +6127,9 @@
       <c r="I149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="J149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -5715,6 +6165,9 @@
       <c r="I150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="J150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -5750,6 +6203,9 @@
       <c r="I151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="J151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5785,6 +6241,9 @@
       <c r="I152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="J152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5820,6 +6279,9 @@
       <c r="I153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="J153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -5855,6 +6317,9 @@
       <c r="I154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="J154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -5890,6 +6355,9 @@
       <c r="I155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="J155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -5925,6 +6393,9 @@
       <c r="I156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="J156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -5960,6 +6431,9 @@
       <c r="I157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="J157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -5995,6 +6469,9 @@
       <c r="I158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="J158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6030,6 +6507,9 @@
       <c r="I159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="J159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6065,6 +6545,9 @@
       <c r="I160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="J160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6100,6 +6583,9 @@
       <c r="I161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="J161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6135,6 +6621,9 @@
       <c r="I162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="J162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -6170,6 +6659,9 @@
       <c r="I163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="J163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6205,9 +6697,12 @@
       <c r="I164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="J164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I164"/>
+  <autoFilter ref="A1:J164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 12:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$J$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$K$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J164"/>
+  <dimension ref="A1:K164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -453,6 +453,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,6 +507,11 @@
           <t>2026-09-05 04:08</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 07:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -544,6 +550,9 @@
       <c r="J2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="K2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -582,6 +591,9 @@
       <c r="J3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="K3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -620,6 +632,9 @@
       <c r="J4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="K4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -658,6 +673,9 @@
       <c r="J5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="K5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -696,6 +714,9 @@
       <c r="J6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="K6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -734,6 +755,9 @@
       <c r="J7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="K7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -772,6 +796,9 @@
       <c r="J8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="K8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -810,6 +837,9 @@
       <c r="J9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="K9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -848,6 +878,9 @@
       <c r="J10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="K10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -886,6 +919,9 @@
       <c r="J11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="K11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -924,6 +960,9 @@
       <c r="J12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -962,6 +1001,9 @@
       <c r="J13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="K13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1000,6 +1042,9 @@
       <c r="J14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="K14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1038,6 +1083,9 @@
       <c r="J15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="K15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1076,6 +1124,9 @@
       <c r="J16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="K16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1114,6 +1165,9 @@
       <c r="J17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="K17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1152,6 +1206,9 @@
       <c r="J18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="K18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1190,6 +1247,9 @@
       <c r="J19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="K19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1228,6 +1288,9 @@
       <c r="J20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="K20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1266,6 +1329,9 @@
       <c r="J21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="K21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1304,6 +1370,9 @@
       <c r="J22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="K22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1342,6 +1411,9 @@
       <c r="J23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="K23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1380,6 +1452,9 @@
       <c r="J24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1418,6 +1493,9 @@
       <c r="J25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="K25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1456,6 +1534,9 @@
       <c r="J26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="K26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1494,6 +1575,9 @@
       <c r="J27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1532,6 +1616,9 @@
       <c r="J28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="K28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1570,6 +1657,9 @@
       <c r="J29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="K29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1608,6 +1698,9 @@
       <c r="J30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="K30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1646,6 +1739,9 @@
       <c r="J31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="K31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1684,6 +1780,9 @@
       <c r="J32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="K32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1722,6 +1821,9 @@
       <c r="J33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="K33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1760,6 +1862,9 @@
       <c r="J34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="K34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1798,6 +1903,9 @@
       <c r="J35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="K35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1836,6 +1944,9 @@
       <c r="J36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="K36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1874,6 +1985,9 @@
       <c r="J37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="K37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1912,6 +2026,9 @@
       <c r="J38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="K38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1950,6 +2067,9 @@
       <c r="J39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="K39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1988,6 +2108,9 @@
       <c r="J40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2026,6 +2149,9 @@
       <c r="J41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2064,6 +2190,9 @@
       <c r="J42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2102,6 +2231,9 @@
       <c r="J43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2140,6 +2272,9 @@
       <c r="J44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2178,6 +2313,9 @@
       <c r="J45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="K45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2216,6 +2354,9 @@
       <c r="J46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="K46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2254,6 +2395,9 @@
       <c r="J47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="K47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2292,6 +2436,9 @@
       <c r="J48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="K48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2330,6 +2477,9 @@
       <c r="J49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2368,6 +2518,9 @@
       <c r="J50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="K50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2406,6 +2559,9 @@
       <c r="J51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="K51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2444,6 +2600,9 @@
       <c r="J52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="K52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2482,6 +2641,9 @@
       <c r="J53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="K53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2520,6 +2682,9 @@
       <c r="J54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="K54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2558,6 +2723,9 @@
       <c r="J55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="K55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2596,6 +2764,9 @@
       <c r="J56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="K56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2634,6 +2805,9 @@
       <c r="J57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2672,6 +2846,9 @@
       <c r="J58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="K58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2710,6 +2887,9 @@
       <c r="J59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="K59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2748,6 +2928,9 @@
       <c r="J60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="K60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2786,6 +2969,9 @@
       <c r="J61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="K61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2824,6 +3010,9 @@
       <c r="J62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="K62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2862,6 +3051,9 @@
       <c r="J63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="K63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2900,6 +3092,9 @@
       <c r="J64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="K64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2938,6 +3133,9 @@
       <c r="J65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2976,6 +3174,9 @@
       <c r="J66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3014,6 +3215,9 @@
       <c r="J67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3052,6 +3256,9 @@
       <c r="J68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3090,6 +3297,9 @@
       <c r="J69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3128,6 +3338,9 @@
       <c r="J70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3166,6 +3379,9 @@
       <c r="J71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3204,6 +3420,9 @@
       <c r="J72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3242,6 +3461,9 @@
       <c r="J73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3280,6 +3502,9 @@
       <c r="J74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3318,6 +3543,9 @@
       <c r="J75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3356,6 +3584,9 @@
       <c r="J76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3394,6 +3625,9 @@
       <c r="J77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3432,6 +3666,9 @@
       <c r="J78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3470,6 +3707,9 @@
       <c r="J79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3508,6 +3748,9 @@
       <c r="J80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3546,6 +3789,9 @@
       <c r="J81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3584,6 +3830,9 @@
       <c r="J82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3622,6 +3871,9 @@
       <c r="J83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3660,6 +3912,9 @@
       <c r="J84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3698,6 +3953,9 @@
       <c r="J85" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3736,6 +3994,9 @@
       <c r="J86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3774,6 +4035,9 @@
       <c r="J87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3812,6 +4076,9 @@
       <c r="J88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3850,6 +4117,9 @@
       <c r="J89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3888,6 +4158,9 @@
       <c r="J90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3926,6 +4199,9 @@
       <c r="J91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3964,6 +4240,9 @@
       <c r="J92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4002,6 +4281,9 @@
       <c r="J93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4040,6 +4322,9 @@
       <c r="J94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4078,6 +4363,9 @@
       <c r="J95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="K95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4116,6 +4404,9 @@
       <c r="J96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="K96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4154,6 +4445,9 @@
       <c r="J97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="K97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4192,6 +4486,9 @@
       <c r="J98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4230,6 +4527,9 @@
       <c r="J99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4268,6 +4568,9 @@
       <c r="J100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="K100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4306,6 +4609,9 @@
       <c r="J101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="K101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4344,6 +4650,9 @@
       <c r="J102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="K102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4382,6 +4691,9 @@
       <c r="J103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="K103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4420,6 +4732,9 @@
       <c r="J104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="K104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4458,6 +4773,9 @@
       <c r="J105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="K105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4496,6 +4814,9 @@
       <c r="J106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="K106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4534,6 +4855,9 @@
       <c r="J107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="K107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4572,6 +4896,9 @@
       <c r="J108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4610,6 +4937,9 @@
       <c r="J109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="K109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4648,6 +4978,9 @@
       <c r="J110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="K110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4686,6 +5019,9 @@
       <c r="J111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="K111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4724,6 +5060,9 @@
       <c r="J112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="K112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4762,6 +5101,9 @@
       <c r="J113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="K113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4800,6 +5142,9 @@
       <c r="J114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="K114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4838,6 +5183,9 @@
       <c r="J115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="K115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4876,6 +5224,9 @@
       <c r="J116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4914,6 +5265,9 @@
       <c r="J117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4952,6 +5306,9 @@
       <c r="J118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4990,6 +5347,9 @@
       <c r="J119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5028,6 +5388,9 @@
       <c r="J120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5066,6 +5429,9 @@
       <c r="J121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="K121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5104,6 +5470,9 @@
       <c r="J122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="K122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5142,6 +5511,9 @@
       <c r="J123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="K123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5180,6 +5552,9 @@
       <c r="J124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="K124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5218,6 +5593,9 @@
       <c r="J125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="K125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5256,6 +5634,9 @@
       <c r="J126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="K126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5294,6 +5675,9 @@
       <c r="J127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="K127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -5332,6 +5716,9 @@
       <c r="J128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="K128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5370,6 +5757,9 @@
       <c r="J129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="K129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5408,6 +5798,9 @@
       <c r="J130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="K130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5446,6 +5839,9 @@
       <c r="J131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="K131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5484,6 +5880,9 @@
       <c r="J132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="K132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5522,6 +5921,9 @@
       <c r="J133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="K133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5560,6 +5962,9 @@
       <c r="J134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="K134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5598,6 +6003,9 @@
       <c r="J135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="K135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5636,6 +6044,9 @@
       <c r="J136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="K136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5674,6 +6085,9 @@
       <c r="J137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="K137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5712,6 +6126,9 @@
       <c r="J138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="K138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5750,6 +6167,9 @@
       <c r="J139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -5788,6 +6208,9 @@
       <c r="J140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5826,6 +6249,9 @@
       <c r="J141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5864,6 +6290,9 @@
       <c r="J142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5902,6 +6331,9 @@
       <c r="J143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5940,6 +6372,9 @@
       <c r="J144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="K144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5978,6 +6413,9 @@
       <c r="J145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="K145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6016,6 +6454,9 @@
       <c r="J146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="K146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6054,6 +6495,9 @@
       <c r="J147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="K147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6092,6 +6536,9 @@
       <c r="J148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="K148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -6130,6 +6577,9 @@
       <c r="J149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="K149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -6168,6 +6618,9 @@
       <c r="J150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="K150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -6206,6 +6659,9 @@
       <c r="J151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="K151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -6244,6 +6700,9 @@
       <c r="J152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="K152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -6282,6 +6741,9 @@
       <c r="J153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="K153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6320,6 +6782,9 @@
       <c r="J154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="K154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6358,6 +6823,9 @@
       <c r="J155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="K155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6396,6 +6864,9 @@
       <c r="J156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="K156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6434,6 +6905,9 @@
       <c r="J157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="K157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6472,6 +6946,9 @@
       <c r="J158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="K158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6510,6 +6987,9 @@
       <c r="J159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="K159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6548,6 +7028,9 @@
       <c r="J160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="K160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6586,6 +7069,9 @@
       <c r="J161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="K161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6624,6 +7110,9 @@
       <c r="J162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="K162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -6662,6 +7151,9 @@
       <c r="J163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="K163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6700,9 +7192,12 @@
       <c r="J164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="K164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J164"/>
+  <autoFilter ref="A1:K164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 15:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$K$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$L$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K164"/>
+  <dimension ref="A1:L164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -454,6 +454,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>2026-09-05 07:10</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 10:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -553,6 +559,9 @@
       <c r="K2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="L2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -594,6 +603,9 @@
       <c r="K3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="L3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -635,6 +647,9 @@
       <c r="K4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="L4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -676,6 +691,9 @@
       <c r="K5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="L5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -717,6 +735,9 @@
       <c r="K6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="L6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -758,6 +779,9 @@
       <c r="K7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="L7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -799,6 +823,9 @@
       <c r="K8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="L8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -840,6 +867,9 @@
       <c r="K9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="L9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -881,6 +911,9 @@
       <c r="K10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="L10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -922,6 +955,9 @@
       <c r="K11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="L11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -963,6 +999,9 @@
       <c r="K12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1004,6 +1043,9 @@
       <c r="K13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="L13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1045,6 +1087,9 @@
       <c r="K14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="L14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1086,6 +1131,9 @@
       <c r="K15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="L15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1127,6 +1175,9 @@
       <c r="K16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="L16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1168,6 +1219,9 @@
       <c r="K17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="L17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1209,6 +1263,9 @@
       <c r="K18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="L18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1250,6 +1307,9 @@
       <c r="K19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="L19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1291,6 +1351,9 @@
       <c r="K20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="L20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1332,6 +1395,9 @@
       <c r="K21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="L21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1373,6 +1439,9 @@
       <c r="K22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="L22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1414,6 +1483,9 @@
       <c r="K23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="L23" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1455,6 +1527,9 @@
       <c r="K24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1496,6 +1571,9 @@
       <c r="K25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="L25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1537,6 +1615,9 @@
       <c r="K26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="L26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1578,6 +1659,9 @@
       <c r="K27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1619,6 +1703,9 @@
       <c r="K28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="L28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1660,6 +1747,9 @@
       <c r="K29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="L29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1701,6 +1791,9 @@
       <c r="K30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="L30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1742,6 +1835,9 @@
       <c r="K31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="L31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1783,6 +1879,9 @@
       <c r="K32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="L32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1824,6 +1923,9 @@
       <c r="K33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="L33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1865,6 +1967,9 @@
       <c r="K34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="L34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1906,6 +2011,9 @@
       <c r="K35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="L35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1947,6 +2055,9 @@
       <c r="K36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="L36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1988,6 +2099,9 @@
       <c r="K37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="L37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2029,6 +2143,9 @@
       <c r="K38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="L38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2070,6 +2187,9 @@
       <c r="K39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="L39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2111,6 +2231,9 @@
       <c r="K40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2152,6 +2275,9 @@
       <c r="K41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2193,6 +2319,9 @@
       <c r="K42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2234,6 +2363,9 @@
       <c r="K43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2275,6 +2407,9 @@
       <c r="K44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2316,6 +2451,9 @@
       <c r="K45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="L45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2357,6 +2495,9 @@
       <c r="K46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="L46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2398,6 +2539,9 @@
       <c r="K47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="L47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2439,6 +2583,9 @@
       <c r="K48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="L48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2480,6 +2627,9 @@
       <c r="K49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2521,6 +2671,9 @@
       <c r="K50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="L50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2562,6 +2715,9 @@
       <c r="K51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="L51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2603,6 +2759,9 @@
       <c r="K52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="L52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2644,6 +2803,9 @@
       <c r="K53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="L53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2685,6 +2847,9 @@
       <c r="K54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="L54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2726,6 +2891,9 @@
       <c r="K55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="L55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2767,6 +2935,9 @@
       <c r="K56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="L56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2808,6 +2979,9 @@
       <c r="K57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2849,6 +3023,9 @@
       <c r="K58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="L58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2890,6 +3067,9 @@
       <c r="K59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="L59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2931,6 +3111,9 @@
       <c r="K60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="L60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2972,6 +3155,9 @@
       <c r="K61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="L61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3013,6 +3199,9 @@
       <c r="K62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="L62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3054,6 +3243,9 @@
       <c r="K63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="L63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3095,6 +3287,9 @@
       <c r="K64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="L64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3136,6 +3331,9 @@
       <c r="K65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3177,6 +3375,9 @@
       <c r="K66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3218,6 +3419,9 @@
       <c r="K67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3259,6 +3463,9 @@
       <c r="K68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3300,6 +3507,9 @@
       <c r="K69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3341,6 +3551,9 @@
       <c r="K70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3382,6 +3595,9 @@
       <c r="K71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3423,6 +3639,9 @@
       <c r="K72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3464,6 +3683,9 @@
       <c r="K73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3505,6 +3727,9 @@
       <c r="K74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3546,6 +3771,9 @@
       <c r="K75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3587,6 +3815,9 @@
       <c r="K76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3628,6 +3859,9 @@
       <c r="K77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3669,6 +3903,9 @@
       <c r="K78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3710,6 +3947,9 @@
       <c r="K79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3751,6 +3991,9 @@
       <c r="K80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3792,6 +4035,9 @@
       <c r="K81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3833,6 +4079,9 @@
       <c r="K82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3874,6 +4123,9 @@
       <c r="K83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3915,6 +4167,9 @@
       <c r="K84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3956,6 +4211,9 @@
       <c r="K85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="L85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3997,6 +4255,9 @@
       <c r="K86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4038,6 +4299,9 @@
       <c r="K87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4079,6 +4343,9 @@
       <c r="K88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4120,6 +4387,9 @@
       <c r="K89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4161,6 +4431,9 @@
       <c r="K90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4202,6 +4475,9 @@
       <c r="K91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4243,6 +4519,9 @@
       <c r="K92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4284,6 +4563,9 @@
       <c r="K93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4325,6 +4607,9 @@
       <c r="K94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4366,6 +4651,9 @@
       <c r="K95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="L95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4407,6 +4695,9 @@
       <c r="K96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="L96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4448,6 +4739,9 @@
       <c r="K97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="L97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4489,6 +4783,9 @@
       <c r="K98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4530,6 +4827,9 @@
       <c r="K99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L99" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4571,6 +4871,9 @@
       <c r="K100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="L100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4612,6 +4915,9 @@
       <c r="K101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="L101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4653,6 +4959,9 @@
       <c r="K102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="L102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4694,6 +5003,9 @@
       <c r="K103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="L103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4735,6 +5047,9 @@
       <c r="K104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="L104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4776,6 +5091,9 @@
       <c r="K105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="L105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4817,6 +5135,9 @@
       <c r="K106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="L106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4858,6 +5179,9 @@
       <c r="K107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="L107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4899,6 +5223,9 @@
       <c r="K108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4940,6 +5267,9 @@
       <c r="K109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="L109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4981,6 +5311,9 @@
       <c r="K110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="L110" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5022,6 +5355,9 @@
       <c r="K111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="L111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5063,6 +5399,9 @@
       <c r="K112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="L112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5104,6 +5443,9 @@
       <c r="K113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="L113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5145,6 +5487,9 @@
       <c r="K114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="L114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5186,6 +5531,9 @@
       <c r="K115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="L115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5227,6 +5575,9 @@
       <c r="K116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5268,6 +5619,9 @@
       <c r="K117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5309,6 +5663,9 @@
       <c r="K118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5350,6 +5707,9 @@
       <c r="K119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5391,6 +5751,9 @@
       <c r="K120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5432,6 +5795,9 @@
       <c r="K121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="L121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5473,6 +5839,9 @@
       <c r="K122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="L122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5514,6 +5883,9 @@
       <c r="K123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="L123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5555,6 +5927,9 @@
       <c r="K124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="L124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5596,6 +5971,9 @@
       <c r="K125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="L125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5637,6 +6015,9 @@
       <c r="K126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="L126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5678,6 +6059,9 @@
       <c r="K127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="L127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -5719,6 +6103,9 @@
       <c r="K128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="L128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5760,6 +6147,9 @@
       <c r="K129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="L129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5801,6 +6191,9 @@
       <c r="K130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="L130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5842,6 +6235,9 @@
       <c r="K131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="L131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5883,6 +6279,9 @@
       <c r="K132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="L132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5924,6 +6323,9 @@
       <c r="K133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="L133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5965,6 +6367,9 @@
       <c r="K134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="L134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -6006,6 +6411,9 @@
       <c r="K135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="L135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6047,6 +6455,9 @@
       <c r="K136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="L136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6088,6 +6499,9 @@
       <c r="K137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="L137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6129,6 +6543,9 @@
       <c r="K138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="L138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6170,6 +6587,9 @@
       <c r="K139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6211,6 +6631,9 @@
       <c r="K140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -6252,6 +6675,9 @@
       <c r="K141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -6293,6 +6719,9 @@
       <c r="K142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -6334,6 +6763,9 @@
       <c r="K143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6375,6 +6807,9 @@
       <c r="K144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="L144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -6416,6 +6851,9 @@
       <c r="K145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="L145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6457,6 +6895,9 @@
       <c r="K146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="L146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6498,6 +6939,9 @@
       <c r="K147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="L147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6539,6 +6983,9 @@
       <c r="K148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="L148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -6580,6 +7027,9 @@
       <c r="K149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="L149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -6621,6 +7071,9 @@
       <c r="K150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="L150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -6662,6 +7115,9 @@
       <c r="K151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="L151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -6703,6 +7159,9 @@
       <c r="K152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="L152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -6744,6 +7203,9 @@
       <c r="K153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="L153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6785,6 +7247,9 @@
       <c r="K154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="L154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6826,6 +7291,9 @@
       <c r="K155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="L155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6867,6 +7335,9 @@
       <c r="K156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="L156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6908,6 +7379,9 @@
       <c r="K157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="L157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6949,6 +7423,9 @@
       <c r="K158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="L158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6990,6 +7467,9 @@
       <c r="K159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="L159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -7031,6 +7511,9 @@
       <c r="K160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="L160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -7072,6 +7555,9 @@
       <c r="K161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="L161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -7113,6 +7599,9 @@
       <c r="K162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="L162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -7154,6 +7643,9 @@
       <c r="K163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="L163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -7195,9 +7687,12 @@
       <c r="K164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="L164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K164"/>
+  <autoFilter ref="A1:L164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 18:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$L$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$M$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:M164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,6 +519,11 @@
           <t>2026-09-05 10:08</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -562,6 +568,9 @@
       <c r="L2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="M2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -606,6 +615,9 @@
       <c r="L3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="M3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -650,6 +662,9 @@
       <c r="L4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="M4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -694,6 +709,9 @@
       <c r="L5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="M5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -738,6 +756,9 @@
       <c r="L6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="M6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -782,6 +803,9 @@
       <c r="L7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="M7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -826,6 +850,9 @@
       <c r="L8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="M8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -870,6 +897,9 @@
       <c r="L9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="M9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -914,6 +944,9 @@
       <c r="L10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="M10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -958,6 +991,9 @@
       <c r="L11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="M11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1002,6 +1038,9 @@
       <c r="L12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1046,6 +1085,9 @@
       <c r="L13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="M13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1090,6 +1132,9 @@
       <c r="L14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="M14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1134,6 +1179,9 @@
       <c r="L15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="M15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1178,6 +1226,9 @@
       <c r="L16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="M16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1222,6 +1273,9 @@
       <c r="L17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="M17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1266,6 +1320,9 @@
       <c r="L18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="M18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1310,6 +1367,9 @@
       <c r="L19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="M19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1354,6 +1414,9 @@
       <c r="L20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="M20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1398,6 +1461,9 @@
       <c r="L21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="M21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1442,6 +1508,9 @@
       <c r="L22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="M22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1486,6 +1555,9 @@
       <c r="L23" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="M23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1530,6 +1602,9 @@
       <c r="L24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1574,6 +1649,9 @@
       <c r="L25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="M25" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1618,6 +1696,9 @@
       <c r="L26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="M26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1662,6 +1743,9 @@
       <c r="L27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1706,6 +1790,9 @@
       <c r="L28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="M28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1750,6 +1837,9 @@
       <c r="L29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="M29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1794,6 +1884,9 @@
       <c r="L30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="M30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1838,6 +1931,9 @@
       <c r="L31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="M31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1882,6 +1978,9 @@
       <c r="L32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="M32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1926,6 +2025,9 @@
       <c r="L33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="M33" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1970,6 +2072,9 @@
       <c r="L34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="M34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2014,6 +2119,9 @@
       <c r="L35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="M35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2058,6 +2166,9 @@
       <c r="L36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="M36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2102,6 +2213,9 @@
       <c r="L37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="M37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2146,6 +2260,9 @@
       <c r="L38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="M38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2190,6 +2307,9 @@
       <c r="L39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="M39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2234,6 +2354,9 @@
       <c r="L40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2278,6 +2401,9 @@
       <c r="L41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2322,6 +2448,9 @@
       <c r="L42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2366,6 +2495,9 @@
       <c r="L43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2410,6 +2542,9 @@
       <c r="L44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2454,6 +2589,9 @@
       <c r="L45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="M45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2498,6 +2636,9 @@
       <c r="L46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="M46" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2542,6 +2683,9 @@
       <c r="L47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="M47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2586,6 +2730,9 @@
       <c r="L48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="M48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2630,6 +2777,9 @@
       <c r="L49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2674,6 +2824,9 @@
       <c r="L50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="M50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2718,6 +2871,9 @@
       <c r="L51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="M51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2762,6 +2918,9 @@
       <c r="L52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="M52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2806,6 +2965,9 @@
       <c r="L53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="M53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2850,6 +3012,9 @@
       <c r="L54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="M54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2894,6 +3059,9 @@
       <c r="L55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="M55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2938,6 +3106,9 @@
       <c r="L56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="M56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2982,6 +3153,9 @@
       <c r="L57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3026,6 +3200,9 @@
       <c r="L58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="M58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3070,6 +3247,9 @@
       <c r="L59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="M59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3114,6 +3294,9 @@
       <c r="L60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="M60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3158,6 +3341,9 @@
       <c r="L61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="M61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3202,6 +3388,9 @@
       <c r="L62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="M62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3246,6 +3435,9 @@
       <c r="L63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="M63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3290,6 +3482,9 @@
       <c r="L64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="M64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3334,6 +3529,9 @@
       <c r="L65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3378,6 +3576,9 @@
       <c r="L66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3422,6 +3623,9 @@
       <c r="L67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3466,6 +3670,9 @@
       <c r="L68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3510,6 +3717,9 @@
       <c r="L69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3554,6 +3764,9 @@
       <c r="L70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3598,6 +3811,9 @@
       <c r="L71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3642,6 +3858,9 @@
       <c r="L72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3686,6 +3905,9 @@
       <c r="L73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3730,6 +3952,9 @@
       <c r="L74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3774,6 +3999,9 @@
       <c r="L75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3818,6 +4046,9 @@
       <c r="L76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3862,6 +4093,9 @@
       <c r="L77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3906,6 +4140,9 @@
       <c r="L78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3950,6 +4187,9 @@
       <c r="L79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3994,6 +4234,9 @@
       <c r="L80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4038,6 +4281,9 @@
       <c r="L81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4082,6 +4328,9 @@
       <c r="L82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4126,6 +4375,9 @@
       <c r="L83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4170,6 +4422,9 @@
       <c r="L84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4214,6 +4469,9 @@
       <c r="L85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="M85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4258,6 +4516,9 @@
       <c r="L86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4302,6 +4563,9 @@
       <c r="L87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4346,6 +4610,9 @@
       <c r="L88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4390,6 +4657,9 @@
       <c r="L89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4434,6 +4704,9 @@
       <c r="L90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4478,6 +4751,9 @@
       <c r="L91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4522,6 +4798,9 @@
       <c r="L92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4566,6 +4845,9 @@
       <c r="L93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4610,6 +4892,9 @@
       <c r="L94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4654,6 +4939,9 @@
       <c r="L95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="M95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4698,6 +4986,9 @@
       <c r="L96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="M96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4742,6 +5033,9 @@
       <c r="L97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="M97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4786,6 +5080,9 @@
       <c r="L98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4830,6 +5127,9 @@
       <c r="L99" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4874,6 +5174,9 @@
       <c r="L100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="M100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4918,6 +5221,9 @@
       <c r="L101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="M101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4962,6 +5268,9 @@
       <c r="L102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="M102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5006,6 +5315,9 @@
       <c r="L103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="M103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5050,6 +5362,9 @@
       <c r="L104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="M104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5094,6 +5409,9 @@
       <c r="L105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="M105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5138,6 +5456,9 @@
       <c r="L106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="M106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5182,6 +5503,9 @@
       <c r="L107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="M107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5226,6 +5550,9 @@
       <c r="L108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5270,6 +5597,9 @@
       <c r="L109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="M109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5314,6 +5644,9 @@
       <c r="L110" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="M110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5358,6 +5691,9 @@
       <c r="L111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="M111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5402,6 +5738,9 @@
       <c r="L112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="M112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5446,6 +5785,9 @@
       <c r="L113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="M113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5490,6 +5832,9 @@
       <c r="L114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="M114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5534,6 +5879,9 @@
       <c r="L115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="M115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5578,6 +5926,9 @@
       <c r="L116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5622,6 +5973,9 @@
       <c r="L117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5666,6 +6020,9 @@
       <c r="L118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5710,6 +6067,9 @@
       <c r="L119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5754,6 +6114,9 @@
       <c r="L120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5798,6 +6161,9 @@
       <c r="L121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="M121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5842,6 +6208,9 @@
       <c r="L122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="M122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5886,6 +6255,9 @@
       <c r="L123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="M123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5930,6 +6302,9 @@
       <c r="L124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="M124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5974,6 +6349,9 @@
       <c r="L125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="M125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6018,6 +6396,9 @@
       <c r="L126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="M126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6062,6 +6443,9 @@
       <c r="L127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="M127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6106,6 +6490,9 @@
       <c r="L128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="M128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6150,6 +6537,9 @@
       <c r="L129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="M129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6194,6 +6584,9 @@
       <c r="L130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="M130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -6238,6 +6631,9 @@
       <c r="L131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="M131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6282,6 +6678,9 @@
       <c r="L132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="M132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -6326,6 +6725,9 @@
       <c r="L133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="M133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -6370,6 +6772,9 @@
       <c r="L134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="M134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -6414,6 +6819,9 @@
       <c r="L135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="M135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6458,6 +6866,9 @@
       <c r="L136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="M136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6502,6 +6913,9 @@
       <c r="L137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="M137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6546,6 +6960,9 @@
       <c r="L138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="M138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6590,6 +7007,9 @@
       <c r="L139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6634,6 +7054,9 @@
       <c r="L140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -6678,6 +7101,9 @@
       <c r="L141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -6722,6 +7148,9 @@
       <c r="L142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -6766,6 +7195,9 @@
       <c r="L143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6810,6 +7242,9 @@
       <c r="L144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="M144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -6854,6 +7289,9 @@
       <c r="L145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="M145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6898,6 +7336,9 @@
       <c r="L146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="M146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6942,6 +7383,9 @@
       <c r="L147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="M147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6986,6 +7430,9 @@
       <c r="L148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="M148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -7030,6 +7477,9 @@
       <c r="L149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="M149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -7074,6 +7524,9 @@
       <c r="L150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="M150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -7118,6 +7571,9 @@
       <c r="L151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="M151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -7162,6 +7618,9 @@
       <c r="L152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="M152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -7206,6 +7665,9 @@
       <c r="L153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="M153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -7250,6 +7712,9 @@
       <c r="L154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="M154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -7294,6 +7759,9 @@
       <c r="L155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="M155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -7338,6 +7806,9 @@
       <c r="L156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="M156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -7382,6 +7853,9 @@
       <c r="L157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="M157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -7426,6 +7900,9 @@
       <c r="L158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="M158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -7470,6 +7947,9 @@
       <c r="L159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="M159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -7514,6 +7994,9 @@
       <c r="L160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="M160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -7558,6 +8041,9 @@
       <c r="L161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="M161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -7602,6 +8088,9 @@
       <c r="L162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="M162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -7646,6 +8135,9 @@
       <c r="L163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="M163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -7690,9 +8182,12 @@
       <c r="L164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="M164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L164"/>
+  <autoFilter ref="A1:M164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-05 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$M$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$N$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M164"/>
+  <dimension ref="A1:N164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,7 @@
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,6 +525,11 @@
           <t>2026-09-05 13:10</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -571,6 +577,9 @@
       <c r="M2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="N2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -618,6 +627,9 @@
       <c r="M3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="N3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -665,6 +677,9 @@
       <c r="M4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -712,6 +727,9 @@
       <c r="M5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -759,6 +777,9 @@
       <c r="M6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -806,6 +827,9 @@
       <c r="M7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -853,6 +877,9 @@
       <c r="M8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="N8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -900,6 +927,9 @@
       <c r="M9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -947,6 +977,9 @@
       <c r="M10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -994,6 +1027,9 @@
       <c r="M11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1041,6 +1077,9 @@
       <c r="M12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1088,6 +1127,9 @@
       <c r="M13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="N13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1135,6 +1177,9 @@
       <c r="M14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="N14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1182,6 +1227,9 @@
       <c r="M15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="N15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1229,6 +1277,9 @@
       <c r="M16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="N16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1276,6 +1327,9 @@
       <c r="M17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="N17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1323,6 +1377,9 @@
       <c r="M18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="N18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1370,6 +1427,9 @@
       <c r="M19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="N19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1417,6 +1477,9 @@
       <c r="M20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="N20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1464,6 +1527,9 @@
       <c r="M21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="N21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1511,6 +1577,9 @@
       <c r="M22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="N22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1558,6 +1627,9 @@
       <c r="M23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="N23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1605,6 +1677,9 @@
       <c r="M24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="N24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1652,6 +1727,9 @@
       <c r="M25" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="N25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1699,6 +1777,9 @@
       <c r="M26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="N26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1746,6 +1827,9 @@
       <c r="M27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="N27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1793,6 +1877,9 @@
       <c r="M28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="N28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1840,6 +1927,9 @@
       <c r="M29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="N29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1887,6 +1977,9 @@
       <c r="M30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="N30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1934,6 +2027,9 @@
       <c r="M31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="N31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1981,6 +2077,9 @@
       <c r="M32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="N32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2028,6 +2127,9 @@
       <c r="M33" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="N33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2075,6 +2177,9 @@
       <c r="M34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="N34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2122,6 +2227,9 @@
       <c r="M35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="N35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2169,6 +2277,9 @@
       <c r="M36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="N36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2216,6 +2327,9 @@
       <c r="M37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="N37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2263,6 +2377,9 @@
       <c r="M38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="N38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2310,6 +2427,9 @@
       <c r="M39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="N39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2357,6 +2477,9 @@
       <c r="M40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2404,6 +2527,9 @@
       <c r="M41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2451,6 +2577,9 @@
       <c r="M42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2498,6 +2627,9 @@
       <c r="M43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2545,6 +2677,9 @@
       <c r="M44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2592,6 +2727,9 @@
       <c r="M45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="N45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2639,6 +2777,9 @@
       <c r="M46" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="N46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2686,6 +2827,9 @@
       <c r="M47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="N47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2733,6 +2877,9 @@
       <c r="M48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="N48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2780,6 +2927,9 @@
       <c r="M49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="N49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2827,6 +2977,9 @@
       <c r="M50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="N50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2874,6 +3027,9 @@
       <c r="M51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="N51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2921,6 +3077,9 @@
       <c r="M52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="N52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2968,6 +3127,9 @@
       <c r="M53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="N53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3015,6 +3177,9 @@
       <c r="M54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="N54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3062,6 +3227,9 @@
       <c r="M55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="N55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3109,6 +3277,9 @@
       <c r="M56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="N56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3156,6 +3327,9 @@
       <c r="M57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3203,6 +3377,9 @@
       <c r="M58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="N58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3250,6 +3427,9 @@
       <c r="M59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="N59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3297,6 +3477,9 @@
       <c r="M60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="N60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3344,6 +3527,9 @@
       <c r="M61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="N61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3391,6 +3577,9 @@
       <c r="M62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="N62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3438,6 +3627,9 @@
       <c r="M63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="N63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3485,6 +3677,9 @@
       <c r="M64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="N64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3532,6 +3727,9 @@
       <c r="M65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3579,6 +3777,9 @@
       <c r="M66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3626,6 +3827,9 @@
       <c r="M67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3673,6 +3877,9 @@
       <c r="M68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3720,6 +3927,9 @@
       <c r="M69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3767,6 +3977,9 @@
       <c r="M70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3814,6 +4027,9 @@
       <c r="M71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3861,6 +4077,9 @@
       <c r="M72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3908,6 +4127,9 @@
       <c r="M73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3955,6 +4177,9 @@
       <c r="M74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4002,6 +4227,9 @@
       <c r="M75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4049,6 +4277,9 @@
       <c r="M76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4096,6 +4327,9 @@
       <c r="M77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4143,6 +4377,9 @@
       <c r="M78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4190,6 +4427,9 @@
       <c r="M79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4237,6 +4477,9 @@
       <c r="M80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4284,6 +4527,9 @@
       <c r="M81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4331,6 +4577,9 @@
       <c r="M82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4378,6 +4627,9 @@
       <c r="M83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4425,6 +4677,9 @@
       <c r="M84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4472,6 +4727,9 @@
       <c r="M85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="N85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4519,6 +4777,9 @@
       <c r="M86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4566,6 +4827,9 @@
       <c r="M87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4613,6 +4877,9 @@
       <c r="M88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4660,6 +4927,9 @@
       <c r="M89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4707,6 +4977,9 @@
       <c r="M90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4754,6 +5027,9 @@
       <c r="M91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4801,6 +5077,9 @@
       <c r="M92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4848,6 +5127,9 @@
       <c r="M93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4895,6 +5177,9 @@
       <c r="M94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4942,6 +5227,9 @@
       <c r="M95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="N95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4989,6 +5277,9 @@
       <c r="M96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="N96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5036,6 +5327,9 @@
       <c r="M97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="N97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5083,6 +5377,9 @@
       <c r="M98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="N98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5130,6 +5427,9 @@
       <c r="M99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5177,6 +5477,9 @@
       <c r="M100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="N100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5224,6 +5527,9 @@
       <c r="M101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="N101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5271,6 +5577,9 @@
       <c r="M102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="N102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5318,6 +5627,9 @@
       <c r="M103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="N103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5365,6 +5677,9 @@
       <c r="M104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="N104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5412,6 +5727,9 @@
       <c r="M105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="N105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5459,6 +5777,9 @@
       <c r="M106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="N106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5506,6 +5827,9 @@
       <c r="M107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="N107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5553,6 +5877,9 @@
       <c r="M108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5600,6 +5927,9 @@
       <c r="M109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="N109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5647,6 +5977,9 @@
       <c r="M110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="N110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5694,6 +6027,9 @@
       <c r="M111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="N111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5741,6 +6077,9 @@
       <c r="M112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="N112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5788,6 +6127,9 @@
       <c r="M113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="N113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5835,6 +6177,9 @@
       <c r="M114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="N114" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5882,6 +6227,9 @@
       <c r="M115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="N115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5929,6 +6277,9 @@
       <c r="M116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5976,6 +6327,9 @@
       <c r="M117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6023,6 +6377,9 @@
       <c r="M118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6070,6 +6427,9 @@
       <c r="M119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6117,6 +6477,9 @@
       <c r="M120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6164,6 +6527,9 @@
       <c r="M121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="N121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6211,6 +6577,9 @@
       <c r="M122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="N122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6258,6 +6627,9 @@
       <c r="M123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="N123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6305,6 +6677,9 @@
       <c r="M124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="N124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6352,6 +6727,9 @@
       <c r="M125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="N125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6399,6 +6777,9 @@
       <c r="M126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="N126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6446,6 +6827,9 @@
       <c r="M127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="N127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6493,6 +6877,9 @@
       <c r="M128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="N128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6540,6 +6927,9 @@
       <c r="M129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="N129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6587,6 +6977,9 @@
       <c r="M130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="N130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -6634,6 +7027,9 @@
       <c r="M131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="N131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6681,6 +7077,9 @@
       <c r="M132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="N132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -6728,6 +7127,9 @@
       <c r="M133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="N133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -6775,6 +7177,9 @@
       <c r="M134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="N134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -6822,6 +7227,9 @@
       <c r="M135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="N135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6869,6 +7277,9 @@
       <c r="M136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="N136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6916,6 +7327,9 @@
       <c r="M137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="N137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6963,6 +7377,9 @@
       <c r="M138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="N138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -7010,6 +7427,9 @@
       <c r="M139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -7057,6 +7477,9 @@
       <c r="M140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7104,6 +7527,9 @@
       <c r="M141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7151,6 +7577,9 @@
       <c r="M142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -7198,6 +7627,9 @@
       <c r="M143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -7245,6 +7677,9 @@
       <c r="M144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="N144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -7292,6 +7727,9 @@
       <c r="M145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="N145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -7339,6 +7777,9 @@
       <c r="M146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="N146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -7386,6 +7827,9 @@
       <c r="M147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="N147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -7433,6 +7877,9 @@
       <c r="M148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="N148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -7480,6 +7927,9 @@
       <c r="M149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="N149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -7527,6 +7977,9 @@
       <c r="M150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="N150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -7574,6 +8027,9 @@
       <c r="M151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="N151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -7621,6 +8077,9 @@
       <c r="M152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="N152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -7668,6 +8127,9 @@
       <c r="M153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="N153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -7715,6 +8177,9 @@
       <c r="M154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="N154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -7762,6 +8227,9 @@
       <c r="M155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="N155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -7809,6 +8277,9 @@
       <c r="M156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="N156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -7856,6 +8327,9 @@
       <c r="M157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="N157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -7903,6 +8377,9 @@
       <c r="M158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="N158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -7950,6 +8427,9 @@
       <c r="M159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="N159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -7997,6 +8477,9 @@
       <c r="M160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="N160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -8044,6 +8527,9 @@
       <c r="M161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="N161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -8091,6 +8577,9 @@
       <c r="M162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="N162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -8138,6 +8627,9 @@
       <c r="M163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="N163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -8185,9 +8677,12 @@
       <c r="M164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="N164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M164"/>
+  <autoFilter ref="A1:N164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 00:16 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$N$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$O$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N164"/>
+  <dimension ref="A1:O164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -457,6 +457,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,6 +531,11 @@
           <t>2026-09-05 16:08</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 19:15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -580,6 +586,9 @@
       <c r="N2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,6 +639,9 @@
       <c r="N3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="O3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -680,6 +692,9 @@
       <c r="N4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="O4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -730,6 +745,9 @@
       <c r="N5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="O5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -780,6 +798,9 @@
       <c r="N6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="O6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -830,6 +851,9 @@
       <c r="N7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="O7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -880,6 +904,9 @@
       <c r="N8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="O8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -930,6 +957,9 @@
       <c r="N9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="O9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -980,6 +1010,9 @@
       <c r="N10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1030,6 +1063,9 @@
       <c r="N11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="O11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1080,6 +1116,9 @@
       <c r="N12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1130,6 +1169,9 @@
       <c r="N13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="O13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1180,6 +1222,9 @@
       <c r="N14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="O14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1230,6 +1275,9 @@
       <c r="N15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="O15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1280,6 +1328,9 @@
       <c r="N16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="O16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1330,6 +1381,9 @@
       <c r="N17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="O17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1380,6 +1434,9 @@
       <c r="N18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="O18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1430,6 +1487,9 @@
       <c r="N19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="O19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1480,6 +1540,9 @@
       <c r="N20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="O20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1530,6 +1593,9 @@
       <c r="N21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="O21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1580,6 +1646,9 @@
       <c r="N22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="O22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1630,6 +1699,9 @@
       <c r="N23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="O23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1680,6 +1752,9 @@
       <c r="N24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="O24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1730,6 +1805,9 @@
       <c r="N25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1780,6 +1858,9 @@
       <c r="N26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="O26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1830,6 +1911,9 @@
       <c r="N27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="O27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1880,6 +1964,9 @@
       <c r="N28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="O28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1930,6 +2017,9 @@
       <c r="N29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="O29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1980,6 +2070,9 @@
       <c r="N30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="O30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2030,6 +2123,9 @@
       <c r="N31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="O31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2080,6 +2176,9 @@
       <c r="N32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="O32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2130,6 +2229,9 @@
       <c r="N33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="O33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2180,6 +2282,9 @@
       <c r="N34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="O34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2230,6 +2335,9 @@
       <c r="N35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="O35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2280,6 +2388,9 @@
       <c r="N36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="O36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2330,6 +2441,9 @@
       <c r="N37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="O37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2380,6 +2494,9 @@
       <c r="N38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="O38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2430,6 +2547,9 @@
       <c r="N39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="O39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2480,6 +2600,9 @@
       <c r="N40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2530,6 +2653,9 @@
       <c r="N41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2580,6 +2706,9 @@
       <c r="N42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2630,6 +2759,9 @@
       <c r="N43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2680,6 +2812,9 @@
       <c r="N44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2730,6 +2865,9 @@
       <c r="N45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="O45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2780,6 +2918,9 @@
       <c r="N46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="O46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2830,6 +2971,9 @@
       <c r="N47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="O47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2880,6 +3024,9 @@
       <c r="N48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="O48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2930,6 +3077,9 @@
       <c r="N49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="O49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2980,6 +3130,9 @@
       <c r="N50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="O50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3030,6 +3183,9 @@
       <c r="N51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="O51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3080,6 +3236,9 @@
       <c r="N52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="O52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3130,6 +3289,9 @@
       <c r="N53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="O53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3180,6 +3342,9 @@
       <c r="N54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="O54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3230,6 +3395,9 @@
       <c r="N55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="O55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3280,6 +3448,9 @@
       <c r="N56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="O56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3330,6 +3501,9 @@
       <c r="N57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3380,6 +3554,9 @@
       <c r="N58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="O58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3430,6 +3607,9 @@
       <c r="N59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="O59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3480,6 +3660,9 @@
       <c r="N60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="O60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3530,6 +3713,9 @@
       <c r="N61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="O61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3580,6 +3766,9 @@
       <c r="N62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="O62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3630,6 +3819,9 @@
       <c r="N63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="O63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3680,6 +3872,9 @@
       <c r="N64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="O64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3730,6 +3925,9 @@
       <c r="N65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3780,6 +3978,9 @@
       <c r="N66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3830,6 +4031,9 @@
       <c r="N67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3880,6 +4084,9 @@
       <c r="N68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3930,6 +4137,9 @@
       <c r="N69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3980,6 +4190,9 @@
       <c r="N70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4030,6 +4243,9 @@
       <c r="N71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4080,6 +4296,9 @@
       <c r="N72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4130,6 +4349,9 @@
       <c r="N73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4180,6 +4402,9 @@
       <c r="N74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4230,6 +4455,9 @@
       <c r="N75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4280,6 +4508,9 @@
       <c r="N76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4330,6 +4561,9 @@
       <c r="N77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4380,6 +4614,9 @@
       <c r="N78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4430,6 +4667,9 @@
       <c r="N79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4480,6 +4720,9 @@
       <c r="N80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4530,6 +4773,9 @@
       <c r="N81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4580,6 +4826,9 @@
       <c r="N82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4630,6 +4879,9 @@
       <c r="N83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4680,6 +4932,9 @@
       <c r="N84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4730,6 +4985,9 @@
       <c r="N85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="O85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4780,6 +5038,9 @@
       <c r="N86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4830,6 +5091,9 @@
       <c r="N87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4880,6 +5144,9 @@
       <c r="N88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4930,6 +5197,9 @@
       <c r="N89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4980,6 +5250,9 @@
       <c r="N90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5030,6 +5303,9 @@
       <c r="N91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5080,6 +5356,9 @@
       <c r="N92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5130,6 +5409,9 @@
       <c r="N93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5180,6 +5462,9 @@
       <c r="N94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5230,6 +5515,9 @@
       <c r="N95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="O95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5280,6 +5568,9 @@
       <c r="N96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="O96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5330,6 +5621,9 @@
       <c r="N97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="O97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5380,6 +5674,9 @@
       <c r="N98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="O98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5430,6 +5727,9 @@
       <c r="N99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5480,6 +5780,9 @@
       <c r="N100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="O100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5530,6 +5833,9 @@
       <c r="N101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="O101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5580,6 +5886,9 @@
       <c r="N102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="O102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5630,6 +5939,9 @@
       <c r="N103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="O103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5680,6 +5992,9 @@
       <c r="N104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="O104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5730,6 +6045,9 @@
       <c r="N105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="O105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5780,6 +6098,9 @@
       <c r="N106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="O106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5830,6 +6151,9 @@
       <c r="N107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="O107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5880,6 +6204,9 @@
       <c r="N108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5930,6 +6257,9 @@
       <c r="N109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="O109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5980,6 +6310,9 @@
       <c r="N110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="O110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6030,6 +6363,9 @@
       <c r="N111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="O111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6080,6 +6416,9 @@
       <c r="N112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="O112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6130,6 +6469,9 @@
       <c r="N113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="O113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6180,6 +6522,9 @@
       <c r="N114" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="O114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6230,6 +6575,9 @@
       <c r="N115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="O115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6280,6 +6628,9 @@
       <c r="N116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6330,6 +6681,9 @@
       <c r="N117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6380,6 +6734,9 @@
       <c r="N118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6430,6 +6787,9 @@
       <c r="N119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6480,6 +6840,9 @@
       <c r="N120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6530,6 +6893,9 @@
       <c r="N121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="O121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6580,6 +6946,9 @@
       <c r="N122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="O122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6630,6 +6999,9 @@
       <c r="N123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="O123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6680,6 +7052,9 @@
       <c r="N124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="O124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6730,6 +7105,9 @@
       <c r="N125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="O125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6780,6 +7158,9 @@
       <c r="N126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="O126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6830,6 +7211,9 @@
       <c r="N127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="O127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6880,6 +7264,9 @@
       <c r="N128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="O128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6930,6 +7317,9 @@
       <c r="N129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="O129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6980,6 +7370,9 @@
       <c r="N130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="O130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7030,6 +7423,9 @@
       <c r="N131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="O131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7080,6 +7476,9 @@
       <c r="N132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="O132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7130,6 +7529,9 @@
       <c r="N133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="O133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -7180,6 +7582,9 @@
       <c r="N134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="O134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -7230,6 +7635,9 @@
       <c r="N135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="O135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -7280,6 +7688,9 @@
       <c r="N136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="O136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -7330,6 +7741,9 @@
       <c r="N137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="O137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -7380,6 +7794,9 @@
       <c r="N138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="O138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -7430,6 +7847,9 @@
       <c r="N139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -7480,6 +7900,9 @@
       <c r="N140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7530,6 +7953,9 @@
       <c r="N141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7580,6 +8006,9 @@
       <c r="N142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -7630,6 +8059,9 @@
       <c r="N143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -7680,6 +8112,9 @@
       <c r="N144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="O144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -7730,6 +8165,9 @@
       <c r="N145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="O145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -7780,6 +8218,9 @@
       <c r="N146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="O146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -7830,6 +8271,9 @@
       <c r="N147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="O147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -7880,6 +8324,9 @@
       <c r="N148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="O148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -7930,6 +8377,9 @@
       <c r="N149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="O149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -7980,6 +8430,9 @@
       <c r="N150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="O150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -8030,6 +8483,9 @@
       <c r="N151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="O151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -8080,6 +8536,9 @@
       <c r="N152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="O152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -8130,6 +8589,9 @@
       <c r="N153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="O153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -8180,6 +8642,9 @@
       <c r="N154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="O154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -8230,6 +8695,9 @@
       <c r="N155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="O155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -8280,6 +8748,9 @@
       <c r="N156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="O156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -8330,6 +8801,9 @@
       <c r="N157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="O157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -8380,6 +8854,9 @@
       <c r="N158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="O158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -8430,6 +8907,9 @@
       <c r="N159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="O159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -8480,6 +8960,9 @@
       <c r="N160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="O160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -8530,6 +9013,9 @@
       <c r="N161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="O161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -8580,6 +9066,9 @@
       <c r="N162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="O162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -8630,6 +9119,9 @@
       <c r="N163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="O163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -8680,9 +9172,12 @@
       <c r="N164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="O164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N164"/>
+  <autoFilter ref="A1:O164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$O$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$P$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O164"/>
+  <dimension ref="A1:P164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,7 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,6 +537,11 @@
           <t>2026-09-05 19:15</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-05 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -589,6 +595,9 @@
       <c r="O2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="P2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -642,6 +651,9 @@
       <c r="O3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="P3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -695,6 +707,9 @@
       <c r="O4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -748,6 +763,9 @@
       <c r="O5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -801,6 +819,9 @@
       <c r="O6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -854,6 +875,9 @@
       <c r="O7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -907,6 +931,9 @@
       <c r="O8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="P8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -960,6 +987,9 @@
       <c r="O9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="P9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1013,6 +1043,9 @@
       <c r="O10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="P10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1066,6 +1099,9 @@
       <c r="O11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="P11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1119,6 +1155,9 @@
       <c r="O12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1172,6 +1211,9 @@
       <c r="O13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="P13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1225,6 +1267,9 @@
       <c r="O14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1278,6 +1323,9 @@
       <c r="O15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="P15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1331,6 +1379,9 @@
       <c r="O16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1384,6 +1435,9 @@
       <c r="O17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="P17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1437,6 +1491,9 @@
       <c r="O18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1490,6 +1547,9 @@
       <c r="O19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="P19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1543,6 +1603,9 @@
       <c r="O20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1596,6 +1659,9 @@
       <c r="O21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="P21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1649,6 +1715,9 @@
       <c r="O22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="P22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1702,6 +1771,9 @@
       <c r="O23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="P23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1755,6 +1827,9 @@
       <c r="O24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="P24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1808,6 +1883,9 @@
       <c r="O25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1861,6 +1939,9 @@
       <c r="O26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="P26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1914,6 +1995,9 @@
       <c r="O27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="P27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1967,6 +2051,9 @@
       <c r="O28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="P28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2020,6 +2107,9 @@
       <c r="O29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="P29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2073,6 +2163,9 @@
       <c r="O30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="P30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2126,6 +2219,9 @@
       <c r="O31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="P31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2179,6 +2275,9 @@
       <c r="O32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="P32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2232,6 +2331,9 @@
       <c r="O33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="P33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2285,6 +2387,9 @@
       <c r="O34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="P34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2338,6 +2443,9 @@
       <c r="O35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="P35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2391,6 +2499,9 @@
       <c r="O36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="P36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2444,6 +2555,9 @@
       <c r="O37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="P37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2497,6 +2611,9 @@
       <c r="O38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="P38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2550,6 +2667,9 @@
       <c r="O39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="P39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2603,6 +2723,9 @@
       <c r="O40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2656,6 +2779,9 @@
       <c r="O41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2709,6 +2835,9 @@
       <c r="O42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2762,6 +2891,9 @@
       <c r="O43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2815,6 +2947,9 @@
       <c r="O44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2868,6 +3003,9 @@
       <c r="O45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="P45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2921,6 +3059,9 @@
       <c r="O46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="P46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2974,6 +3115,9 @@
       <c r="O47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="P47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3027,6 +3171,9 @@
       <c r="O48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="P48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3080,6 +3227,9 @@
       <c r="O49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="P49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3133,6 +3283,9 @@
       <c r="O50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="P50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3186,6 +3339,9 @@
       <c r="O51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="P51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3239,6 +3395,9 @@
       <c r="O52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="P52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3292,6 +3451,9 @@
       <c r="O53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="P53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3345,6 +3507,9 @@
       <c r="O54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="P54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3398,6 +3563,9 @@
       <c r="O55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="P55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3451,6 +3619,9 @@
       <c r="O56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="P56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3504,6 +3675,9 @@
       <c r="O57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3557,6 +3731,9 @@
       <c r="O58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="P58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3610,6 +3787,9 @@
       <c r="O59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="P59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3663,6 +3843,9 @@
       <c r="O60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="P60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3716,6 +3899,9 @@
       <c r="O61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="P61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3769,6 +3955,9 @@
       <c r="O62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="P62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3822,6 +4011,9 @@
       <c r="O63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="P63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3875,6 +4067,9 @@
       <c r="O64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="P64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3928,6 +4123,9 @@
       <c r="O65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3981,6 +4179,9 @@
       <c r="O66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4034,6 +4235,9 @@
       <c r="O67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4087,6 +4291,9 @@
       <c r="O68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4140,6 +4347,9 @@
       <c r="O69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4193,6 +4403,9 @@
       <c r="O70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4246,6 +4459,9 @@
       <c r="O71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4299,6 +4515,9 @@
       <c r="O72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4352,6 +4571,9 @@
       <c r="O73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4405,6 +4627,9 @@
       <c r="O74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4458,6 +4683,9 @@
       <c r="O75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4511,6 +4739,9 @@
       <c r="O76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4564,6 +4795,9 @@
       <c r="O77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4617,6 +4851,9 @@
       <c r="O78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4670,6 +4907,9 @@
       <c r="O79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4723,6 +4963,9 @@
       <c r="O80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4776,6 +5019,9 @@
       <c r="O81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4829,6 +5075,9 @@
       <c r="O82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4882,6 +5131,9 @@
       <c r="O83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4935,6 +5187,9 @@
       <c r="O84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4988,6 +5243,9 @@
       <c r="O85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="P85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5041,6 +5299,9 @@
       <c r="O86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5094,6 +5355,9 @@
       <c r="O87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5147,6 +5411,9 @@
       <c r="O88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5200,6 +5467,9 @@
       <c r="O89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5253,6 +5523,9 @@
       <c r="O90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5306,6 +5579,9 @@
       <c r="O91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5359,6 +5635,9 @@
       <c r="O92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5412,6 +5691,9 @@
       <c r="O93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5465,6 +5747,9 @@
       <c r="O94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5518,6 +5803,9 @@
       <c r="O95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="P95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5571,6 +5859,9 @@
       <c r="O96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="P96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5624,6 +5915,9 @@
       <c r="O97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="P97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5677,6 +5971,9 @@
       <c r="O98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="P98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5730,6 +6027,9 @@
       <c r="O99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5783,6 +6083,9 @@
       <c r="O100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="P100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5836,6 +6139,9 @@
       <c r="O101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="P101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5889,6 +6195,9 @@
       <c r="O102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="P102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5942,6 +6251,9 @@
       <c r="O103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="P103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5995,6 +6307,9 @@
       <c r="O104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="P104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6048,6 +6363,9 @@
       <c r="O105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="P105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6101,6 +6419,9 @@
       <c r="O106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="P106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6154,6 +6475,9 @@
       <c r="O107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="P107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6207,6 +6531,9 @@
       <c r="O108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -6260,6 +6587,9 @@
       <c r="O109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="P109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6313,6 +6643,9 @@
       <c r="O110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="P110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6366,6 +6699,9 @@
       <c r="O111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="P111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6419,6 +6755,9 @@
       <c r="O112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="P112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6472,6 +6811,9 @@
       <c r="O113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="P113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6525,6 +6867,9 @@
       <c r="O114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="P114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6578,6 +6923,9 @@
       <c r="O115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="P115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6631,6 +6979,9 @@
       <c r="O116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6684,6 +7035,9 @@
       <c r="O117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6737,6 +7091,9 @@
       <c r="O118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6790,6 +7147,9 @@
       <c r="O119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6843,6 +7203,9 @@
       <c r="O120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6896,6 +7259,9 @@
       <c r="O121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="P121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6949,6 +7315,9 @@
       <c r="O122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="P122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7002,6 +7371,9 @@
       <c r="O123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="P123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7055,6 +7427,9 @@
       <c r="O124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="P124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7108,6 +7483,9 @@
       <c r="O125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="P125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -7161,6 +7539,9 @@
       <c r="O126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="P126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7214,6 +7595,9 @@
       <c r="O127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="P127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -7267,6 +7651,9 @@
       <c r="O128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="P128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -7320,6 +7707,9 @@
       <c r="O129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="P129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -7373,6 +7763,9 @@
       <c r="O130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="P130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7426,6 +7819,9 @@
       <c r="O131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="P131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7479,6 +7875,9 @@
       <c r="O132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="P132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7532,6 +7931,9 @@
       <c r="O133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="P133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -7585,6 +7987,9 @@
       <c r="O134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="P134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -7638,6 +8043,9 @@
       <c r="O135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="P135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -7691,6 +8099,9 @@
       <c r="O136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="P136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -7744,6 +8155,9 @@
       <c r="O137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="P137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -7797,6 +8211,9 @@
       <c r="O138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="P138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -7850,6 +8267,9 @@
       <c r="O139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -7903,6 +8323,9 @@
       <c r="O140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7956,6 +8379,9 @@
       <c r="O141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8009,6 +8435,9 @@
       <c r="O142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -8062,6 +8491,9 @@
       <c r="O143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -8115,6 +8547,9 @@
       <c r="O144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="P144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -8168,6 +8603,9 @@
       <c r="O145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="P145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -8221,6 +8659,9 @@
       <c r="O146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="P146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -8274,6 +8715,9 @@
       <c r="O147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="P147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -8327,6 +8771,9 @@
       <c r="O148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="P148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -8380,6 +8827,9 @@
       <c r="O149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="P149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -8433,6 +8883,9 @@
       <c r="O150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="P150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -8486,6 +8939,9 @@
       <c r="O151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="P151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -8539,6 +8995,9 @@
       <c r="O152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="P152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -8592,6 +9051,9 @@
       <c r="O153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="P153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -8645,6 +9107,9 @@
       <c r="O154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="P154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -8698,6 +9163,9 @@
       <c r="O155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="P155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -8751,6 +9219,9 @@
       <c r="O156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="P156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -8804,6 +9275,9 @@
       <c r="O157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="P157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -8857,6 +9331,9 @@
       <c r="O158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="P158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -8910,6 +9387,9 @@
       <c r="O159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="P159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -8963,6 +9443,9 @@
       <c r="O160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="P160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -9016,6 +9499,9 @@
       <c r="O161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="P161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -9069,6 +9555,9 @@
       <c r="O162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="P162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -9122,6 +9611,9 @@
       <c r="O163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="P163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -9175,9 +9667,12 @@
       <c r="O164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="P164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O164"/>
+  <autoFilter ref="A1:P164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 06:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$P$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Q$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P164"/>
+  <dimension ref="A1:Q164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -459,6 +459,7 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,6 +543,11 @@
           <t>2026-09-05 22:09</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 01:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -598,6 +604,9 @@
       <c r="P2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="Q2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,6 +663,9 @@
       <c r="P3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="Q3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -710,6 +722,9 @@
       <c r="P4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="Q4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -766,6 +781,9 @@
       <c r="P5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Q5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -822,6 +840,9 @@
       <c r="P6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Q6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -878,6 +899,9 @@
       <c r="P7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="Q7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -934,6 +958,9 @@
       <c r="P8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="Q8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -990,6 +1017,9 @@
       <c r="P9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="Q9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1046,6 +1076,9 @@
       <c r="P10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="Q10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1102,6 +1135,9 @@
       <c r="P11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="Q11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1158,6 +1194,9 @@
       <c r="P12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1214,6 +1253,9 @@
       <c r="P13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="Q13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1270,6 +1312,9 @@
       <c r="P14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Q14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1326,6 +1371,9 @@
       <c r="P15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Q15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1382,6 +1430,9 @@
       <c r="P16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Q16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1438,6 +1489,9 @@
       <c r="P17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Q17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1494,6 +1548,9 @@
       <c r="P18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Q18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1550,6 +1607,9 @@
       <c r="P19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="Q19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1606,6 +1666,9 @@
       <c r="P20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="Q20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1662,6 +1725,9 @@
       <c r="P21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="Q21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1718,6 +1784,9 @@
       <c r="P22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Q22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1774,6 +1843,9 @@
       <c r="P23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Q23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1830,6 +1902,9 @@
       <c r="P24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Q24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1886,6 +1961,9 @@
       <c r="P25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1942,6 +2020,9 @@
       <c r="P26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="Q26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1998,6 +2079,9 @@
       <c r="P27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Q27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2054,6 +2138,9 @@
       <c r="P28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="Q28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2110,6 +2197,9 @@
       <c r="P29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="Q29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2166,6 +2256,9 @@
       <c r="P30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Q30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2222,6 +2315,9 @@
       <c r="P31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Q31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2278,6 +2374,9 @@
       <c r="P32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Q32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2334,6 +2433,9 @@
       <c r="P33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Q33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2390,6 +2492,9 @@
       <c r="P34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="Q34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2446,6 +2551,9 @@
       <c r="P35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Q35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2502,6 +2610,9 @@
       <c r="P36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Q36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2558,6 +2669,9 @@
       <c r="P37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Q37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2614,6 +2728,9 @@
       <c r="P38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Q38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2670,6 +2787,9 @@
       <c r="P39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Q39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2726,6 +2846,9 @@
       <c r="P40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2782,6 +2905,9 @@
       <c r="P41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2838,6 +2964,9 @@
       <c r="P42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2894,6 +3023,9 @@
       <c r="P43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2950,6 +3082,9 @@
       <c r="P44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3006,6 +3141,9 @@
       <c r="P45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Q45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3062,6 +3200,9 @@
       <c r="P46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="Q46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3118,6 +3259,9 @@
       <c r="P47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Q47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3174,6 +3318,9 @@
       <c r="P48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Q48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3230,6 +3377,9 @@
       <c r="P49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Q49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3286,6 +3436,9 @@
       <c r="P50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="Q50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3342,6 +3495,9 @@
       <c r="P51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Q51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3398,6 +3554,9 @@
       <c r="P52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Q52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3454,6 +3613,9 @@
       <c r="P53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Q53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3510,6 +3672,9 @@
       <c r="P54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="Q54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3566,6 +3731,9 @@
       <c r="P55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Q55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3622,6 +3790,9 @@
       <c r="P56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Q56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3678,6 +3849,9 @@
       <c r="P57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3734,6 +3908,9 @@
       <c r="P58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Q58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3790,6 +3967,9 @@
       <c r="P59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Q59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3846,6 +4026,9 @@
       <c r="P60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Q60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3902,6 +4085,9 @@
       <c r="P61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Q61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3958,6 +4144,9 @@
       <c r="P62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Q62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4014,6 +4203,9 @@
       <c r="P63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Q63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4070,6 +4262,9 @@
       <c r="P64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Q64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4126,6 +4321,9 @@
       <c r="P65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4182,6 +4380,9 @@
       <c r="P66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4238,6 +4439,9 @@
       <c r="P67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4294,6 +4498,9 @@
       <c r="P68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4350,6 +4557,9 @@
       <c r="P69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4406,6 +4616,9 @@
       <c r="P70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4462,6 +4675,9 @@
       <c r="P71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4518,6 +4734,9 @@
       <c r="P72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4574,6 +4793,9 @@
       <c r="P73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4630,6 +4852,9 @@
       <c r="P74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4686,6 +4911,9 @@
       <c r="P75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4742,6 +4970,9 @@
       <c r="P76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4798,6 +5029,9 @@
       <c r="P77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4854,6 +5088,9 @@
       <c r="P78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4910,6 +5147,9 @@
       <c r="P79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4966,6 +5206,9 @@
       <c r="P80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5022,6 +5265,9 @@
       <c r="P81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5078,6 +5324,9 @@
       <c r="P82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5134,6 +5383,9 @@
       <c r="P83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5190,6 +5442,9 @@
       <c r="P84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5246,6 +5501,9 @@
       <c r="P85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Q85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5302,6 +5560,9 @@
       <c r="P86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5358,6 +5619,9 @@
       <c r="P87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5414,6 +5678,9 @@
       <c r="P88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5470,6 +5737,9 @@
       <c r="P89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5526,6 +5796,9 @@
       <c r="P90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5582,6 +5855,9 @@
       <c r="P91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5638,6 +5914,9 @@
       <c r="P92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5694,6 +5973,9 @@
       <c r="P93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5750,6 +6032,9 @@
       <c r="P94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5806,6 +6091,9 @@
       <c r="P95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Q95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5862,6 +6150,9 @@
       <c r="P96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Q96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5918,6 +6209,9 @@
       <c r="P97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Q97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5974,6 +6268,9 @@
       <c r="P98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Q98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6030,6 +6327,9 @@
       <c r="P99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6086,6 +6386,9 @@
       <c r="P100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Q100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6142,6 +6445,9 @@
       <c r="P101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Q101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6198,6 +6504,9 @@
       <c r="P102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Q102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6254,6 +6563,9 @@
       <c r="P103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Q103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6310,6 +6622,9 @@
       <c r="P104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Q104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6366,6 +6681,9 @@
       <c r="P105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Q105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6422,6 +6740,9 @@
       <c r="P106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Q106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6478,6 +6799,9 @@
       <c r="P107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="Q107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6534,6 +6858,9 @@
       <c r="P108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -6590,6 +6917,9 @@
       <c r="P109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Q109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6646,6 +6976,9 @@
       <c r="P110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Q110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6702,6 +7035,9 @@
       <c r="P111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Q111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6758,6 +7094,9 @@
       <c r="P112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Q112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6814,6 +7153,9 @@
       <c r="P113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Q113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6870,6 +7212,9 @@
       <c r="P114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Q114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6926,6 +7271,9 @@
       <c r="P115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Q115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6982,6 +7330,9 @@
       <c r="P116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7038,6 +7389,9 @@
       <c r="P117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7094,6 +7448,9 @@
       <c r="P118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7150,6 +7507,9 @@
       <c r="P119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7206,6 +7566,9 @@
       <c r="P120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7262,6 +7625,9 @@
       <c r="P121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Q121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7318,6 +7684,9 @@
       <c r="P122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Q122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7374,6 +7743,9 @@
       <c r="P123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Q123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7430,6 +7802,9 @@
       <c r="P124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Q124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7486,6 +7861,9 @@
       <c r="P125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Q125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -7542,6 +7920,9 @@
       <c r="P126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Q126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7598,6 +7979,9 @@
       <c r="P127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Q127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -7654,6 +8038,9 @@
       <c r="P128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Q128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -7710,6 +8097,9 @@
       <c r="P129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Q129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -7766,6 +8156,9 @@
       <c r="P130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Q130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7822,6 +8215,9 @@
       <c r="P131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Q131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7878,6 +8274,9 @@
       <c r="P132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="Q132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7934,6 +8333,9 @@
       <c r="P133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Q133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -7990,6 +8392,9 @@
       <c r="P134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Q134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8046,6 +8451,9 @@
       <c r="P135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Q135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8102,6 +8510,9 @@
       <c r="P136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Q136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8158,6 +8569,9 @@
       <c r="P137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Q137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -8214,6 +8628,9 @@
       <c r="P138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="Q138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -8270,6 +8687,9 @@
       <c r="P139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8326,6 +8746,9 @@
       <c r="P140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -8382,6 +8805,9 @@
       <c r="P141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8438,6 +8864,9 @@
       <c r="P142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -8494,6 +8923,9 @@
       <c r="P143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -8550,6 +8982,9 @@
       <c r="P144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Q144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -8606,6 +9041,9 @@
       <c r="P145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="Q145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -8662,6 +9100,9 @@
       <c r="P146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Q146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -8718,6 +9159,9 @@
       <c r="P147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Q147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -8774,6 +9218,9 @@
       <c r="P148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="Q148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -8830,6 +9277,9 @@
       <c r="P149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="Q149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -8886,6 +9336,9 @@
       <c r="P150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="Q150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -8942,6 +9395,9 @@
       <c r="P151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="Q151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -8998,6 +9454,9 @@
       <c r="P152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Q152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9054,6 +9513,9 @@
       <c r="P153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Q153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -9110,6 +9572,9 @@
       <c r="P154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="Q154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -9166,6 +9631,9 @@
       <c r="P155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="Q155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -9222,6 +9690,9 @@
       <c r="P156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Q156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -9278,6 +9749,9 @@
       <c r="P157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Q157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -9334,6 +9808,9 @@
       <c r="P158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Q158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -9390,6 +9867,9 @@
       <c r="P159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Q159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -9446,6 +9926,9 @@
       <c r="P160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Q160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -9502,6 +9985,9 @@
       <c r="P161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Q161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -9558,6 +10044,9 @@
       <c r="P162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="Q162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -9614,6 +10103,9 @@
       <c r="P163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="Q163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -9670,9 +10162,12 @@
       <c r="P164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="Q164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P164"/>
+  <autoFilter ref="A1:Q164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Q$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$R$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q164"/>
+  <dimension ref="A1:R164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -460,6 +460,7 @@
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +549,11 @@
           <t>2026-09-06 01:11</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -607,6 +613,9 @@
       <c r="Q2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="R2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -666,6 +675,9 @@
       <c r="Q3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="R3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -725,6 +737,9 @@
       <c r="Q4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="R4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -784,6 +799,9 @@
       <c r="Q5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="R5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -843,6 +861,9 @@
       <c r="Q6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="R6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -902,6 +923,9 @@
       <c r="Q7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="R7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -961,6 +985,9 @@
       <c r="Q8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="R8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1020,6 +1047,9 @@
       <c r="Q9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="R9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1079,6 +1109,9 @@
       <c r="Q10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="R10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1138,6 +1171,9 @@
       <c r="Q11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="R11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1197,6 +1233,9 @@
       <c r="Q12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1256,6 +1295,9 @@
       <c r="Q13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="R13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1315,6 +1357,9 @@
       <c r="Q14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="R14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1374,6 +1419,9 @@
       <c r="Q15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="R15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1433,6 +1481,9 @@
       <c r="Q16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="R16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1492,6 +1543,9 @@
       <c r="Q17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="R17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1551,6 +1605,9 @@
       <c r="Q18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="R18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1610,6 +1667,9 @@
       <c r="Q19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="R19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1669,6 +1729,9 @@
       <c r="Q20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="R20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1728,6 +1791,9 @@
       <c r="Q21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="R21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1787,6 +1853,9 @@
       <c r="Q22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="R22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1846,6 +1915,9 @@
       <c r="Q23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="R23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1905,6 +1977,9 @@
       <c r="Q24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="R24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1964,6 +2039,9 @@
       <c r="Q25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2023,6 +2101,9 @@
       <c r="Q26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="R26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2082,6 +2163,9 @@
       <c r="Q27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="R27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2141,6 +2225,9 @@
       <c r="Q28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="R28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2200,6 +2287,9 @@
       <c r="Q29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="R29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2259,6 +2349,9 @@
       <c r="Q30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="R30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2318,6 +2411,9 @@
       <c r="Q31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="R31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2377,6 +2473,9 @@
       <c r="Q32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="R32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2436,6 +2535,9 @@
       <c r="Q33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="R33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2495,6 +2597,9 @@
       <c r="Q34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="R34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2554,6 +2659,9 @@
       <c r="Q35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="R35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2613,6 +2721,9 @@
       <c r="Q36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="R36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2672,6 +2783,9 @@
       <c r="Q37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="R37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2731,6 +2845,9 @@
       <c r="Q38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="R38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2790,6 +2907,9 @@
       <c r="Q39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="R39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2849,6 +2969,9 @@
       <c r="Q40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2908,6 +3031,9 @@
       <c r="Q41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2967,6 +3093,9 @@
       <c r="Q42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3026,6 +3155,9 @@
       <c r="Q43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3085,6 +3217,9 @@
       <c r="Q44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3144,6 +3279,9 @@
       <c r="Q45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="R45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3203,6 +3341,9 @@
       <c r="Q46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="R46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3262,6 +3403,9 @@
       <c r="Q47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="R47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3321,6 +3465,9 @@
       <c r="Q48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="R48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3380,6 +3527,9 @@
       <c r="Q49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="R49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3439,6 +3589,9 @@
       <c r="Q50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="R50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3498,6 +3651,9 @@
       <c r="Q51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="R51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3557,6 +3713,9 @@
       <c r="Q52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="R52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3616,6 +3775,9 @@
       <c r="Q53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="R53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3675,6 +3837,9 @@
       <c r="Q54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="R54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3734,6 +3899,9 @@
       <c r="Q55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="R55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3793,6 +3961,9 @@
       <c r="Q56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="R56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3852,6 +4023,9 @@
       <c r="Q57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3911,6 +4085,9 @@
       <c r="Q58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="R58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3970,6 +4147,9 @@
       <c r="Q59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="R59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4029,6 +4209,9 @@
       <c r="Q60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="R60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4088,6 +4271,9 @@
       <c r="Q61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="R61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4147,6 +4333,9 @@
       <c r="Q62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="R62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4206,6 +4395,9 @@
       <c r="Q63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="R63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4265,6 +4457,9 @@
       <c r="Q64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="R64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4324,6 +4519,9 @@
       <c r="Q65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4383,6 +4581,9 @@
       <c r="Q66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4442,6 +4643,9 @@
       <c r="Q67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4501,6 +4705,9 @@
       <c r="Q68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4560,6 +4767,9 @@
       <c r="Q69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4619,6 +4829,9 @@
       <c r="Q70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4678,6 +4891,9 @@
       <c r="Q71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4737,6 +4953,9 @@
       <c r="Q72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4796,6 +5015,9 @@
       <c r="Q73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4855,6 +5077,9 @@
       <c r="Q74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4914,6 +5139,9 @@
       <c r="Q75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4973,6 +5201,9 @@
       <c r="Q76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5032,6 +5263,9 @@
       <c r="Q77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5091,6 +5325,9 @@
       <c r="Q78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5150,6 +5387,9 @@
       <c r="Q79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5209,6 +5449,9 @@
       <c r="Q80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5268,6 +5511,9 @@
       <c r="Q81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5327,6 +5573,9 @@
       <c r="Q82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5386,6 +5635,9 @@
       <c r="Q83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5445,6 +5697,9 @@
       <c r="Q84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5504,6 +5759,9 @@
       <c r="Q85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="R85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5563,6 +5821,9 @@
       <c r="Q86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5622,6 +5883,9 @@
       <c r="Q87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5681,6 +5945,9 @@
       <c r="Q88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5740,6 +6007,9 @@
       <c r="Q89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5799,6 +6069,9 @@
       <c r="Q90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5858,6 +6131,9 @@
       <c r="Q91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5917,6 +6193,9 @@
       <c r="Q92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5976,6 +6255,9 @@
       <c r="Q93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6035,6 +6317,9 @@
       <c r="Q94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6094,6 +6379,9 @@
       <c r="Q95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="R95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6153,6 +6441,9 @@
       <c r="Q96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="R96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6212,6 +6503,9 @@
       <c r="Q97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="R97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6271,6 +6565,9 @@
       <c r="Q98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="R98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6330,6 +6627,9 @@
       <c r="Q99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6389,6 +6689,9 @@
       <c r="Q100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="R100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6448,6 +6751,9 @@
       <c r="Q101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="R101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6507,6 +6813,9 @@
       <c r="Q102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="R102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6566,6 +6875,9 @@
       <c r="Q103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="R103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6625,6 +6937,9 @@
       <c r="Q104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="R104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6684,6 +6999,9 @@
       <c r="Q105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="R105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6743,6 +7061,9 @@
       <c r="Q106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="R106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6802,6 +7123,9 @@
       <c r="Q107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="R107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6861,6 +7185,9 @@
       <c r="Q108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -6920,6 +7247,9 @@
       <c r="Q109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="R109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6979,6 +7309,9 @@
       <c r="Q110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="R110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7038,6 +7371,9 @@
       <c r="Q111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="R111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7097,6 +7433,9 @@
       <c r="Q112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="R112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7156,6 +7495,9 @@
       <c r="Q113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="R113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7215,6 +7557,9 @@
       <c r="Q114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="R114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7274,6 +7619,9 @@
       <c r="Q115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="R115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7333,6 +7681,9 @@
       <c r="Q116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7392,6 +7743,9 @@
       <c r="Q117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7451,6 +7805,9 @@
       <c r="Q118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7510,6 +7867,9 @@
       <c r="Q119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7569,6 +7929,9 @@
       <c r="Q120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7628,6 +7991,9 @@
       <c r="Q121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="R121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7687,6 +8053,9 @@
       <c r="Q122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="R122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7746,6 +8115,9 @@
       <c r="Q123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="R123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7805,6 +8177,9 @@
       <c r="Q124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="R124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7864,6 +8239,9 @@
       <c r="Q125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="R125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -7923,6 +8301,9 @@
       <c r="Q126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="R126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7982,6 +8363,9 @@
       <c r="Q127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="R127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8041,6 +8425,9 @@
       <c r="Q128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="R128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8100,6 +8487,9 @@
       <c r="Q129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="R129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8159,6 +8549,9 @@
       <c r="Q130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="R130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8218,6 +8611,9 @@
       <c r="Q131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="R131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8277,6 +8673,9 @@
       <c r="Q132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="R132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8336,6 +8735,9 @@
       <c r="Q133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="R133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8395,6 +8797,9 @@
       <c r="Q134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="R134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8454,6 +8859,9 @@
       <c r="Q135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="R135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8513,6 +8921,9 @@
       <c r="Q136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="R136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8572,6 +8983,9 @@
       <c r="Q137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="R137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -8631,6 +9045,9 @@
       <c r="Q138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="R138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -8690,6 +9107,9 @@
       <c r="Q139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8749,6 +9169,9 @@
       <c r="Q140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -8808,6 +9231,9 @@
       <c r="Q141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8867,6 +9293,9 @@
       <c r="Q142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -8926,6 +9355,9 @@
       <c r="Q143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -8985,6 +9417,9 @@
       <c r="Q144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="R144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9044,6 +9479,9 @@
       <c r="Q145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="R145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9103,6 +9541,9 @@
       <c r="Q146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="R146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -9162,6 +9603,9 @@
       <c r="Q147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="R147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9221,6 +9665,9 @@
       <c r="Q148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="R148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9280,6 +9727,9 @@
       <c r="Q149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="R149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9339,6 +9789,9 @@
       <c r="Q150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="R150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9398,6 +9851,9 @@
       <c r="Q151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="R151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9457,6 +9913,9 @@
       <c r="Q152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="R152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9516,6 +9975,9 @@
       <c r="Q153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="R153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -9575,6 +10037,9 @@
       <c r="Q154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="R154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -9634,6 +10099,9 @@
       <c r="Q155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="R155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -9693,6 +10161,9 @@
       <c r="Q156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="R156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -9752,6 +10223,9 @@
       <c r="Q157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="R157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -9811,6 +10285,9 @@
       <c r="Q158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="R158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -9870,6 +10347,9 @@
       <c r="Q159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="R159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -9929,6 +10409,9 @@
       <c r="Q160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="R160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -9988,6 +10471,9 @@
       <c r="Q161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="R161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -10047,6 +10533,9 @@
       <c r="Q162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="R162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -10106,6 +10595,9 @@
       <c r="Q163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="R163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -10165,9 +10657,12 @@
       <c r="Q164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="R164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q164"/>
+  <autoFilter ref="A1:R164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 12:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$R$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$S$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R164"/>
+  <dimension ref="A1:S164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,7 @@
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,6 +555,11 @@
           <t>2026-09-06 04:09</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 07:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -616,6 +622,9 @@
       <c r="R2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -678,6 +687,9 @@
       <c r="R3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="S3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -740,6 +752,9 @@
       <c r="R4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="S4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -802,6 +817,9 @@
       <c r="R5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="S5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -864,6 +882,9 @@
       <c r="R6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="S6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -926,6 +947,9 @@
       <c r="R7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="S7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -988,6 +1012,9 @@
       <c r="R8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="S8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1050,6 +1077,9 @@
       <c r="R9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="S9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1112,6 +1142,9 @@
       <c r="R10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="S10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1174,6 +1207,9 @@
       <c r="R11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="S11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1236,6 +1272,9 @@
       <c r="R12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1298,6 +1337,9 @@
       <c r="R13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="S13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1360,6 +1402,9 @@
       <c r="R14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="S14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1422,6 +1467,9 @@
       <c r="R15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="S15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1484,6 +1532,9 @@
       <c r="R16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="S16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1546,6 +1597,9 @@
       <c r="R17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="S17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1608,6 +1662,9 @@
       <c r="R18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="S18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1670,6 +1727,9 @@
       <c r="R19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="S19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1732,6 +1792,9 @@
       <c r="R20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="S20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1794,6 +1857,9 @@
       <c r="R21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="S21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1856,6 +1922,9 @@
       <c r="R22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="S22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1918,6 +1987,9 @@
       <c r="R23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="S23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1980,6 +2052,9 @@
       <c r="R24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="S24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2042,6 +2117,9 @@
       <c r="R25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2104,6 +2182,9 @@
       <c r="R26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="S26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2166,6 +2247,9 @@
       <c r="R27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="S27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2228,6 +2312,9 @@
       <c r="R28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="S28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2290,6 +2377,9 @@
       <c r="R29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="S29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2352,6 +2442,9 @@
       <c r="R30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="S30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2414,6 +2507,9 @@
       <c r="R31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="S31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2476,6 +2572,9 @@
       <c r="R32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="S32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2538,6 +2637,9 @@
       <c r="R33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="S33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2600,6 +2702,9 @@
       <c r="R34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="S34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2662,6 +2767,9 @@
       <c r="R35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="S35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2724,6 +2832,9 @@
       <c r="R36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="S36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2786,6 +2897,9 @@
       <c r="R37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="S37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2848,6 +2962,9 @@
       <c r="R38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="S38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2910,6 +3027,9 @@
       <c r="R39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="S39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2972,6 +3092,9 @@
       <c r="R40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3034,6 +3157,9 @@
       <c r="R41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3096,6 +3222,9 @@
       <c r="R42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3158,6 +3287,9 @@
       <c r="R43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3220,6 +3352,9 @@
       <c r="R44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3282,6 +3417,9 @@
       <c r="R45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="S45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3344,6 +3482,9 @@
       <c r="R46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="S46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3406,6 +3547,9 @@
       <c r="R47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="S47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3468,6 +3612,9 @@
       <c r="R48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="S48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3530,6 +3677,9 @@
       <c r="R49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="S49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3592,6 +3742,9 @@
       <c r="R50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="S50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3654,6 +3807,9 @@
       <c r="R51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="S51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3716,6 +3872,9 @@
       <c r="R52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="S52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3778,6 +3937,9 @@
       <c r="R53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="S53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3840,6 +4002,9 @@
       <c r="R54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="S54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3902,6 +4067,9 @@
       <c r="R55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="S55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3964,6 +4132,9 @@
       <c r="R56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="S56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4026,6 +4197,9 @@
       <c r="R57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4088,6 +4262,9 @@
       <c r="R58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="S58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4150,6 +4327,9 @@
       <c r="R59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="S59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4212,6 +4392,9 @@
       <c r="R60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="S60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4274,6 +4457,9 @@
       <c r="R61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="S61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4336,6 +4522,9 @@
       <c r="R62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="S62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4398,6 +4587,9 @@
       <c r="R63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="S63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4460,6 +4652,9 @@
       <c r="R64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="S64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4522,6 +4717,9 @@
       <c r="R65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4584,6 +4782,9 @@
       <c r="R66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4646,6 +4847,9 @@
       <c r="R67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4708,6 +4912,9 @@
       <c r="R68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4770,6 +4977,9 @@
       <c r="R69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4832,6 +5042,9 @@
       <c r="R70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4894,6 +5107,9 @@
       <c r="R71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4956,6 +5172,9 @@
       <c r="R72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5018,6 +5237,9 @@
       <c r="R73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5080,6 +5302,9 @@
       <c r="R74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5142,6 +5367,9 @@
       <c r="R75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5204,6 +5432,9 @@
       <c r="R76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5266,6 +5497,9 @@
       <c r="R77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5328,6 +5562,9 @@
       <c r="R78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5390,6 +5627,9 @@
       <c r="R79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5452,6 +5692,9 @@
       <c r="R80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5514,6 +5757,9 @@
       <c r="R81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5576,6 +5822,9 @@
       <c r="R82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5638,6 +5887,9 @@
       <c r="R83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5700,6 +5952,9 @@
       <c r="R84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5762,6 +6017,9 @@
       <c r="R85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="S85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5824,6 +6082,9 @@
       <c r="R86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5886,6 +6147,9 @@
       <c r="R87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5948,6 +6212,9 @@
       <c r="R88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6010,6 +6277,9 @@
       <c r="R89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6072,6 +6342,9 @@
       <c r="R90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6134,6 +6407,9 @@
       <c r="R91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6196,6 +6472,9 @@
       <c r="R92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6258,6 +6537,9 @@
       <c r="R93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6320,6 +6602,9 @@
       <c r="R94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6382,6 +6667,9 @@
       <c r="R95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="S95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6444,6 +6732,9 @@
       <c r="R96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="S96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6506,6 +6797,9 @@
       <c r="R97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="S97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6568,6 +6862,9 @@
       <c r="R98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="S98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6630,6 +6927,9 @@
       <c r="R99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6692,6 +6992,9 @@
       <c r="R100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="S100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6754,6 +7057,9 @@
       <c r="R101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="S101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6816,6 +7122,9 @@
       <c r="R102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="S102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6878,6 +7187,9 @@
       <c r="R103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="S103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6940,6 +7252,9 @@
       <c r="R104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="S104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7002,6 +7317,9 @@
       <c r="R105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="S105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7064,6 +7382,9 @@
       <c r="R106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="S106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7126,6 +7447,9 @@
       <c r="R107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="S107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7188,6 +7512,9 @@
       <c r="R108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7250,6 +7577,9 @@
       <c r="R109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="S109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7312,6 +7642,9 @@
       <c r="R110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="S110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7374,6 +7707,9 @@
       <c r="R111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="S111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7436,6 +7772,9 @@
       <c r="R112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="S112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7498,6 +7837,9 @@
       <c r="R113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="S113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7560,6 +7902,9 @@
       <c r="R114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="S114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7622,6 +7967,9 @@
       <c r="R115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="S115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7684,6 +8032,9 @@
       <c r="R116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7746,6 +8097,9 @@
       <c r="R117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7808,6 +8162,9 @@
       <c r="R118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7870,6 +8227,9 @@
       <c r="R119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7932,6 +8292,9 @@
       <c r="R120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7994,6 +8357,9 @@
       <c r="R121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="S121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8056,6 +8422,9 @@
       <c r="R122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="S122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8118,6 +8487,9 @@
       <c r="R123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="S123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8180,6 +8552,9 @@
       <c r="R124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="S124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8242,6 +8617,9 @@
       <c r="R125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="S125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8304,6 +8682,9 @@
       <c r="R126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="S126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8366,6 +8747,9 @@
       <c r="R127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="S127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8428,6 +8812,9 @@
       <c r="R128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="S128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8490,6 +8877,9 @@
       <c r="R129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="S129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8552,6 +8942,9 @@
       <c r="R130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="S130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8614,6 +9007,9 @@
       <c r="R131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="S131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8676,6 +9072,9 @@
       <c r="R132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="S132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8738,6 +9137,9 @@
       <c r="R133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="S133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8800,6 +9202,9 @@
       <c r="R134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="S134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8862,6 +9267,9 @@
       <c r="R135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="S135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8924,6 +9332,9 @@
       <c r="R136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="S136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8986,6 +9397,9 @@
       <c r="R137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="S137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9048,6 +9462,9 @@
       <c r="R138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="S138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9110,6 +9527,9 @@
       <c r="R139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -9172,6 +9592,9 @@
       <c r="R140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -9234,6 +9657,9 @@
       <c r="R141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9296,6 +9722,9 @@
       <c r="R142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -9358,6 +9787,9 @@
       <c r="R143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -9420,6 +9852,9 @@
       <c r="R144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="S144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9482,6 +9917,9 @@
       <c r="R145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="S145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9544,6 +9982,9 @@
       <c r="R146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="S146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -9606,6 +10047,9 @@
       <c r="R147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="S147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9668,6 +10112,9 @@
       <c r="R148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="S148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9730,6 +10177,9 @@
       <c r="R149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="S149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9792,6 +10242,9 @@
       <c r="R150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="S150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9854,6 +10307,9 @@
       <c r="R151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="S151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9916,6 +10372,9 @@
       <c r="R152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="S152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9978,6 +10437,9 @@
       <c r="R153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="S153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -10040,6 +10502,9 @@
       <c r="R154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="S154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -10102,6 +10567,9 @@
       <c r="R155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="S155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -10164,6 +10632,9 @@
       <c r="R156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="S156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -10226,6 +10697,9 @@
       <c r="R157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="S157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -10288,6 +10762,9 @@
       <c r="R158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="S158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -10350,6 +10827,9 @@
       <c r="R159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="S159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -10412,6 +10892,9 @@
       <c r="R160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="S160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -10474,6 +10957,9 @@
       <c r="R161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="S161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -10536,6 +11022,9 @@
       <c r="R162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="S162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -10598,6 +11087,9 @@
       <c r="R163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="S163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -10660,9 +11152,12 @@
       <c r="R164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="S164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R164"/>
+  <autoFilter ref="A1:S164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$S$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$T$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S164"/>
+  <dimension ref="A1:T164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -462,6 +462,7 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -560,6 +561,11 @@
           <t>2026-09-06 07:11</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -625,6 +631,9 @@
       <c r="S2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -690,6 +699,9 @@
       <c r="S3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -755,6 +767,9 @@
       <c r="S4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -820,6 +835,9 @@
       <c r="S5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -885,6 +903,9 @@
       <c r="S6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -950,6 +971,9 @@
       <c r="S7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1015,6 +1039,9 @@
       <c r="S8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1080,6 +1107,9 @@
       <c r="S9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1145,6 +1175,9 @@
       <c r="S10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1210,6 +1243,9 @@
       <c r="S11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1275,6 +1311,9 @@
       <c r="S12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1340,6 +1379,9 @@
       <c r="S13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="T13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1405,6 +1447,9 @@
       <c r="S14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="T14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1470,6 +1515,9 @@
       <c r="S15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="T15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1535,6 +1583,9 @@
       <c r="S16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="T16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1600,6 +1651,9 @@
       <c r="S17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="T17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1665,6 +1719,9 @@
       <c r="S18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="T18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1730,6 +1787,9 @@
       <c r="S19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="T19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1795,6 +1855,9 @@
       <c r="S20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="T20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1860,6 +1923,9 @@
       <c r="S21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="T21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1925,6 +1991,9 @@
       <c r="S22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="T22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1990,6 +2059,9 @@
       <c r="S23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2055,6 +2127,9 @@
       <c r="S24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="T24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2120,6 +2195,9 @@
       <c r="S25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2185,6 +2263,9 @@
       <c r="S26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="T26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2250,6 +2331,9 @@
       <c r="S27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="T27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2315,6 +2399,9 @@
       <c r="S28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="T28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2380,6 +2467,9 @@
       <c r="S29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="T29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2445,6 +2535,9 @@
       <c r="S30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2510,6 +2603,9 @@
       <c r="S31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="T31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2575,6 +2671,9 @@
       <c r="S32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2640,6 +2739,9 @@
       <c r="S33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="T33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2705,6 +2807,9 @@
       <c r="S34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="T34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2770,6 +2875,9 @@
       <c r="S35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="T35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2835,6 +2943,9 @@
       <c r="S36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="T36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2900,6 +3011,9 @@
       <c r="S37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="T37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2965,6 +3079,9 @@
       <c r="S38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="T38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3030,6 +3147,9 @@
       <c r="S39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="T39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3095,6 +3215,9 @@
       <c r="S40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3160,6 +3283,9 @@
       <c r="S41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3225,6 +3351,9 @@
       <c r="S42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3290,6 +3419,9 @@
       <c r="S43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3355,6 +3487,9 @@
       <c r="S44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3420,6 +3555,9 @@
       <c r="S45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="T45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3485,6 +3623,9 @@
       <c r="S46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="T46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3550,6 +3691,9 @@
       <c r="S47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3615,6 +3759,9 @@
       <c r="S48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="T48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3680,6 +3827,9 @@
       <c r="S49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="T49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3745,6 +3895,9 @@
       <c r="S50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="T50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3810,6 +3963,9 @@
       <c r="S51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="T51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3875,6 +4031,9 @@
       <c r="S52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="T52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3940,6 +4099,9 @@
       <c r="S53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="T53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4005,6 +4167,9 @@
       <c r="S54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="T54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4070,6 +4235,9 @@
       <c r="S55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="T55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4135,6 +4303,9 @@
       <c r="S56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="T56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4200,6 +4371,9 @@
       <c r="S57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4265,6 +4439,9 @@
       <c r="S58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="T58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4330,6 +4507,9 @@
       <c r="S59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="T59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4395,6 +4575,9 @@
       <c r="S60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="T60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4460,6 +4643,9 @@
       <c r="S61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="T61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4525,6 +4711,9 @@
       <c r="S62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="T62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4590,6 +4779,9 @@
       <c r="S63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="T63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4655,6 +4847,9 @@
       <c r="S64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="T64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4720,6 +4915,9 @@
       <c r="S65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4785,6 +4983,9 @@
       <c r="S66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4850,6 +5051,9 @@
       <c r="S67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4915,6 +5119,9 @@
       <c r="S68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4980,6 +5187,9 @@
       <c r="S69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5045,6 +5255,9 @@
       <c r="S70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5110,6 +5323,9 @@
       <c r="S71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5175,6 +5391,9 @@
       <c r="S72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5240,6 +5459,9 @@
       <c r="S73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5305,6 +5527,9 @@
       <c r="S74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5370,6 +5595,9 @@
       <c r="S75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5435,6 +5663,9 @@
       <c r="S76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5500,6 +5731,9 @@
       <c r="S77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5565,6 +5799,9 @@
       <c r="S78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5630,6 +5867,9 @@
       <c r="S79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5695,6 +5935,9 @@
       <c r="S80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5760,6 +6003,9 @@
       <c r="S81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5825,6 +6071,9 @@
       <c r="S82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5890,6 +6139,9 @@
       <c r="S83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5955,6 +6207,9 @@
       <c r="S84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6020,6 +6275,9 @@
       <c r="S85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="T85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6085,6 +6343,9 @@
       <c r="S86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6150,6 +6411,9 @@
       <c r="S87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6215,6 +6479,9 @@
       <c r="S88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6280,6 +6547,9 @@
       <c r="S89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6345,6 +6615,9 @@
       <c r="S90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6410,6 +6683,9 @@
       <c r="S91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6475,6 +6751,9 @@
       <c r="S92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6540,6 +6819,9 @@
       <c r="S93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6605,6 +6887,9 @@
       <c r="S94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6670,6 +6955,9 @@
       <c r="S95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="T95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6735,6 +7023,9 @@
       <c r="S96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="T96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6800,6 +7091,9 @@
       <c r="S97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="T97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6865,6 +7159,9 @@
       <c r="S98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="T98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6930,6 +7227,9 @@
       <c r="S99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6995,6 +7295,9 @@
       <c r="S100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="T100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7060,6 +7363,9 @@
       <c r="S101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="T101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7125,6 +7431,9 @@
       <c r="S102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="T102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7190,6 +7499,9 @@
       <c r="S103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="T103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7255,6 +7567,9 @@
       <c r="S104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="T104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7320,6 +7635,9 @@
       <c r="S105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="T105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7385,6 +7703,9 @@
       <c r="S106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="T106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7450,6 +7771,9 @@
       <c r="S107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="T107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7515,6 +7839,9 @@
       <c r="S108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7580,6 +7907,9 @@
       <c r="S109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="T109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7645,6 +7975,9 @@
       <c r="S110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="T110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7710,6 +8043,9 @@
       <c r="S111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="T111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7775,6 +8111,9 @@
       <c r="S112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="T112" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7840,6 +8179,9 @@
       <c r="S113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="T113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7905,6 +8247,9 @@
       <c r="S114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="T114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7970,6 +8315,9 @@
       <c r="S115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="T115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8035,6 +8383,9 @@
       <c r="S116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8100,6 +8451,9 @@
       <c r="S117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8165,6 +8519,9 @@
       <c r="S118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8230,6 +8587,9 @@
       <c r="S119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8295,6 +8655,9 @@
       <c r="S120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -8360,6 +8723,9 @@
       <c r="S121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="T121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8425,6 +8791,9 @@
       <c r="S122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="T122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8490,6 +8859,9 @@
       <c r="S123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="T123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8555,6 +8927,9 @@
       <c r="S124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="T124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8620,6 +8995,9 @@
       <c r="S125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="T125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8685,6 +9063,9 @@
       <c r="S126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="T126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8750,6 +9131,9 @@
       <c r="S127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="T127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8815,6 +9199,9 @@
       <c r="S128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="T128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8880,6 +9267,9 @@
       <c r="S129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="T129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8945,6 +9335,9 @@
       <c r="S130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="T130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9010,6 +9403,9 @@
       <c r="S131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="T131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9075,6 +9471,9 @@
       <c r="S132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="T132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9140,6 +9539,9 @@
       <c r="S133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="T133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9205,6 +9607,9 @@
       <c r="S134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="T134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -9270,6 +9675,9 @@
       <c r="S135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="T135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -9335,6 +9743,9 @@
       <c r="S136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="T136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -9400,6 +9811,9 @@
       <c r="S137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="T137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9465,6 +9879,9 @@
       <c r="S138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="T138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9530,6 +9947,9 @@
       <c r="S139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -9595,6 +10015,9 @@
       <c r="S140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -9660,6 +10083,9 @@
       <c r="S141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9725,6 +10151,9 @@
       <c r="S142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -9790,6 +10219,9 @@
       <c r="S143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -9855,6 +10287,9 @@
       <c r="S144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="T144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9920,6 +10355,9 @@
       <c r="S145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="T145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9985,6 +10423,9 @@
       <c r="S146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="T146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -10050,6 +10491,9 @@
       <c r="S147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="T147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -10115,6 +10559,9 @@
       <c r="S148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="T148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -10180,6 +10627,9 @@
       <c r="S149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="T149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -10245,6 +10695,9 @@
       <c r="S150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="T150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -10310,6 +10763,9 @@
       <c r="S151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="T151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -10375,6 +10831,9 @@
       <c r="S152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="T152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -10440,6 +10899,9 @@
       <c r="S153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="T153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -10505,6 +10967,9 @@
       <c r="S154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="T154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -10570,6 +11035,9 @@
       <c r="S155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="T155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -10635,6 +11103,9 @@
       <c r="S156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="T156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -10700,6 +11171,9 @@
       <c r="S157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="T157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -10765,6 +11239,9 @@
       <c r="S158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="T158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -10830,6 +11307,9 @@
       <c r="S159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="T159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -10895,6 +11375,9 @@
       <c r="S160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="T160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -10960,6 +11443,9 @@
       <c r="S161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="T161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -11025,6 +11511,9 @@
       <c r="S162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="T162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -11090,6 +11579,9 @@
       <c r="S163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="T163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -11155,9 +11647,12 @@
       <c r="S164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="T164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S164"/>
+  <autoFilter ref="A1:T164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 18:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$T$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$U$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T164"/>
+  <dimension ref="A1:U164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -463,6 +463,7 @@
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,6 +567,11 @@
           <t>2026-09-06 10:09</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -634,6 +640,9 @@
       <c r="T2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -702,6 +711,9 @@
       <c r="T3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -770,6 +782,9 @@
       <c r="T4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -838,6 +853,9 @@
       <c r="T5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -906,6 +924,9 @@
       <c r="T6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -974,6 +995,9 @@
       <c r="T7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1042,6 +1066,9 @@
       <c r="T8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1110,6 +1137,9 @@
       <c r="T9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1178,6 +1208,9 @@
       <c r="T10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1246,6 +1279,9 @@
       <c r="T11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1314,6 +1350,9 @@
       <c r="T12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1382,6 +1421,9 @@
       <c r="T13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="U13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1450,6 +1492,9 @@
       <c r="T14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="U14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1518,6 +1563,9 @@
       <c r="T15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="U15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1586,6 +1634,9 @@
       <c r="T16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="U16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1654,6 +1705,9 @@
       <c r="T17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="U17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1722,6 +1776,9 @@
       <c r="T18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="U18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1790,6 +1847,9 @@
       <c r="T19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="U19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1858,6 +1918,9 @@
       <c r="T20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="U20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1926,6 +1989,9 @@
       <c r="T21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="U21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1994,6 +2060,9 @@
       <c r="T22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="U22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2062,6 +2131,9 @@
       <c r="T23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="U23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2130,6 +2202,9 @@
       <c r="T24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="U24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2198,6 +2273,9 @@
       <c r="T25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2266,6 +2344,9 @@
       <c r="T26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="U26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2334,6 +2415,9 @@
       <c r="T27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="U27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2402,6 +2486,9 @@
       <c r="T28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="U28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2470,6 +2557,9 @@
       <c r="T29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="U29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2538,6 +2628,9 @@
       <c r="T30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="U30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2606,6 +2699,9 @@
       <c r="T31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="U31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2674,6 +2770,9 @@
       <c r="T32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="U32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2742,6 +2841,9 @@
       <c r="T33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="U33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2810,6 +2912,9 @@
       <c r="T34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="U34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2878,6 +2983,9 @@
       <c r="T35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="U35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2946,6 +3054,9 @@
       <c r="T36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="U36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3014,6 +3125,9 @@
       <c r="T37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="U37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3082,6 +3196,9 @@
       <c r="T38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="U38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3150,6 +3267,9 @@
       <c r="T39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="U39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3218,6 +3338,9 @@
       <c r="T40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3286,6 +3409,9 @@
       <c r="T41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3354,6 +3480,9 @@
       <c r="T42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3422,6 +3551,9 @@
       <c r="T43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3490,6 +3622,9 @@
       <c r="T44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3558,6 +3693,9 @@
       <c r="T45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="U45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3626,6 +3764,9 @@
       <c r="T46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="U46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3694,6 +3835,9 @@
       <c r="T47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="U47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3762,6 +3906,9 @@
       <c r="T48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="U48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3830,6 +3977,9 @@
       <c r="T49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="U49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3898,6 +4048,9 @@
       <c r="T50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="U50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3966,6 +4119,9 @@
       <c r="T51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="U51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4034,6 +4190,9 @@
       <c r="T52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="U52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4102,6 +4261,9 @@
       <c r="T53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="U53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4170,6 +4332,9 @@
       <c r="T54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="U54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4238,6 +4403,9 @@
       <c r="T55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="U55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4306,6 +4474,9 @@
       <c r="T56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="U56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4374,6 +4545,9 @@
       <c r="T57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4442,6 +4616,9 @@
       <c r="T58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="U58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4510,6 +4687,9 @@
       <c r="T59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="U59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4578,6 +4758,9 @@
       <c r="T60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="U60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4646,6 +4829,9 @@
       <c r="T61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="U61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4714,6 +4900,9 @@
       <c r="T62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="U62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4782,6 +4971,9 @@
       <c r="T63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="U63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4850,6 +5042,9 @@
       <c r="T64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="U64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4918,6 +5113,9 @@
       <c r="T65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4986,6 +5184,9 @@
       <c r="T66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5054,6 +5255,9 @@
       <c r="T67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5122,6 +5326,9 @@
       <c r="T68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5190,6 +5397,9 @@
       <c r="T69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5258,6 +5468,9 @@
       <c r="T70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5326,6 +5539,9 @@
       <c r="T71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5394,6 +5610,9 @@
       <c r="T72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5462,6 +5681,9 @@
       <c r="T73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5530,6 +5752,9 @@
       <c r="T74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5598,6 +5823,9 @@
       <c r="T75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5666,6 +5894,9 @@
       <c r="T76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5734,6 +5965,9 @@
       <c r="T77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5802,6 +6036,9 @@
       <c r="T78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5870,6 +6107,9 @@
       <c r="T79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5938,6 +6178,9 @@
       <c r="T80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6006,6 +6249,9 @@
       <c r="T81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6074,6 +6320,9 @@
       <c r="T82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6142,6 +6391,9 @@
       <c r="T83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6210,6 +6462,9 @@
       <c r="T84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6278,6 +6533,9 @@
       <c r="T85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="U85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6346,6 +6604,9 @@
       <c r="T86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6414,6 +6675,9 @@
       <c r="T87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6482,6 +6746,9 @@
       <c r="T88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6550,6 +6817,9 @@
       <c r="T89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6618,6 +6888,9 @@
       <c r="T90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6686,6 +6959,9 @@
       <c r="T91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6754,6 +7030,9 @@
       <c r="T92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6822,6 +7101,9 @@
       <c r="T93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6890,6 +7172,9 @@
       <c r="T94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6958,6 +7243,9 @@
       <c r="T95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="U95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7026,6 +7314,9 @@
       <c r="T96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="U96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7094,6 +7385,9 @@
       <c r="T97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="U97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7162,6 +7456,9 @@
       <c r="T98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="U98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7230,6 +7527,9 @@
       <c r="T99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7298,6 +7598,9 @@
       <c r="T100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="U100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7366,6 +7669,9 @@
       <c r="T101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="U101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7434,6 +7740,9 @@
       <c r="T102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="U102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7502,6 +7811,9 @@
       <c r="T103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="U103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7570,6 +7882,9 @@
       <c r="T104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="U104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7638,6 +7953,9 @@
       <c r="T105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="U105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7706,6 +8024,9 @@
       <c r="T106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="U106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7774,6 +8095,9 @@
       <c r="T107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="U107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7842,6 +8166,9 @@
       <c r="T108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7910,6 +8237,9 @@
       <c r="T109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="U109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7978,6 +8308,9 @@
       <c r="T110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="U110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8046,6 +8379,9 @@
       <c r="T111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="U111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8114,6 +8450,9 @@
       <c r="T112" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="U112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8182,6 +8521,9 @@
       <c r="T113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="U113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8250,6 +8592,9 @@
       <c r="T114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="U114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8318,6 +8663,9 @@
       <c r="T115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="U115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8386,6 +8734,9 @@
       <c r="T116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8454,6 +8805,9 @@
       <c r="T117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8522,6 +8876,9 @@
       <c r="T118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8590,6 +8947,9 @@
       <c r="T119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8658,6 +9018,9 @@
       <c r="T120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -8726,6 +9089,9 @@
       <c r="T121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="U121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8794,6 +9160,9 @@
       <c r="T122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="U122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8862,6 +9231,9 @@
       <c r="T123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="U123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8930,6 +9302,9 @@
       <c r="T124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="U124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8998,6 +9373,9 @@
       <c r="T125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="U125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9066,6 +9444,9 @@
       <c r="T126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="U126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9134,6 +9515,9 @@
       <c r="T127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="U127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9202,6 +9586,9 @@
       <c r="T128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="U128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9270,6 +9657,9 @@
       <c r="T129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="U129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9338,6 +9728,9 @@
       <c r="T130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="U130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9406,6 +9799,9 @@
       <c r="T131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="U131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9474,6 +9870,9 @@
       <c r="T132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="U132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9542,6 +9941,9 @@
       <c r="T133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="U133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9610,6 +10012,9 @@
       <c r="T134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="U134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -9678,6 +10083,9 @@
       <c r="T135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="U135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -9746,6 +10154,9 @@
       <c r="T136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="U136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -9814,6 +10225,9 @@
       <c r="T137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="U137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9882,6 +10296,9 @@
       <c r="T138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="U138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9950,6 +10367,9 @@
       <c r="T139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10018,6 +10438,9 @@
       <c r="T140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10086,6 +10509,9 @@
       <c r="T141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10154,6 +10580,9 @@
       <c r="T142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10222,6 +10651,9 @@
       <c r="T143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10290,6 +10722,9 @@
       <c r="T144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="U144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -10358,6 +10793,9 @@
       <c r="T145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="U145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -10426,6 +10864,9 @@
       <c r="T146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="U146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -10494,6 +10935,9 @@
       <c r="T147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="U147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -10562,6 +11006,9 @@
       <c r="T148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="U148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -10630,6 +11077,9 @@
       <c r="T149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="U149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -10698,6 +11148,9 @@
       <c r="T150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="U150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -10766,6 +11219,9 @@
       <c r="T151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="U151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -10834,6 +11290,9 @@
       <c r="T152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="U152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -10902,6 +11361,9 @@
       <c r="T153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="U153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -10970,6 +11432,9 @@
       <c r="T154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="U154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11038,6 +11503,9 @@
       <c r="T155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="U155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -11106,6 +11574,9 @@
       <c r="T156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="U156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -11174,6 +11645,9 @@
       <c r="T157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="U157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11242,6 +11716,9 @@
       <c r="T158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="U158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -11310,6 +11787,9 @@
       <c r="T159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="U159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11378,6 +11858,9 @@
       <c r="T160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="U160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -11446,6 +11929,9 @@
       <c r="T161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="U161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -11514,6 +12000,9 @@
       <c r="T162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="U162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -11582,6 +12071,9 @@
       <c r="T163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="U163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -11650,9 +12142,12 @@
       <c r="T164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="U164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T164"/>
+  <autoFilter ref="A1:U164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-06 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$U$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$V$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U164"/>
+  <dimension ref="A1:V164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -464,6 +464,7 @@
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +573,11 @@
           <t>2026-09-06 13:10</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -643,6 +649,9 @@
       <c r="U2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="V2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -714,6 +723,9 @@
       <c r="U3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="V3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -785,6 +797,9 @@
       <c r="U4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="V4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -856,6 +871,9 @@
       <c r="U5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="V5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -927,6 +945,9 @@
       <c r="U6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="V6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -998,6 +1019,9 @@
       <c r="U7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="V7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1069,6 +1093,9 @@
       <c r="U8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="V8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1140,6 +1167,9 @@
       <c r="U9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="V9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1211,6 +1241,9 @@
       <c r="U10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="V10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1282,6 +1315,9 @@
       <c r="U11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="V11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1353,6 +1389,9 @@
       <c r="U12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1424,6 +1463,9 @@
       <c r="U13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="V13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1495,6 +1537,9 @@
       <c r="U14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="V14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1566,6 +1611,9 @@
       <c r="U15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="V15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1637,6 +1685,9 @@
       <c r="U16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="V16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1708,6 +1759,9 @@
       <c r="U17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="V17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1779,6 +1833,9 @@
       <c r="U18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="V18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1850,6 +1907,9 @@
       <c r="U19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="V19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1921,6 +1981,9 @@
       <c r="U20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="V20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1992,6 +2055,9 @@
       <c r="U21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="V21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2063,6 +2129,9 @@
       <c r="U22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="V22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2134,6 +2203,9 @@
       <c r="U23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="V23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2205,6 +2277,9 @@
       <c r="U24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="V24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2276,6 +2351,9 @@
       <c r="U25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2347,6 +2425,9 @@
       <c r="U26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="V26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2418,6 +2499,9 @@
       <c r="U27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="V27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2489,6 +2573,9 @@
       <c r="U28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="V28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2560,6 +2647,9 @@
       <c r="U29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="V29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2631,6 +2721,9 @@
       <c r="U30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="V30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2702,6 +2795,9 @@
       <c r="U31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="V31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2773,6 +2869,9 @@
       <c r="U32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="V32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2844,6 +2943,9 @@
       <c r="U33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="V33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2915,6 +3017,9 @@
       <c r="U34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="V34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2986,6 +3091,9 @@
       <c r="U35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="V35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3057,6 +3165,9 @@
       <c r="U36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="V36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3128,6 +3239,9 @@
       <c r="U37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="V37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3199,6 +3313,9 @@
       <c r="U38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="V38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3270,6 +3387,9 @@
       <c r="U39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="V39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3341,6 +3461,9 @@
       <c r="U40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3412,6 +3535,9 @@
       <c r="U41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3483,6 +3609,9 @@
       <c r="U42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3554,6 +3683,9 @@
       <c r="U43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3625,6 +3757,9 @@
       <c r="U44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3696,6 +3831,9 @@
       <c r="U45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="V45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3767,6 +3905,9 @@
       <c r="U46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="V46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3838,6 +3979,9 @@
       <c r="U47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="V47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3909,6 +4053,9 @@
       <c r="U48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="V48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3980,6 +4127,9 @@
       <c r="U49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="V49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4051,6 +4201,9 @@
       <c r="U50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="V50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4122,6 +4275,9 @@
       <c r="U51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="V51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4193,6 +4349,9 @@
       <c r="U52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="V52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4264,6 +4423,9 @@
       <c r="U53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="V53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4335,6 +4497,9 @@
       <c r="U54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="V54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4406,6 +4571,9 @@
       <c r="U55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="V55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4477,6 +4645,9 @@
       <c r="U56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="V56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4548,6 +4719,9 @@
       <c r="U57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4619,6 +4793,9 @@
       <c r="U58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="V58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4690,6 +4867,9 @@
       <c r="U59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="V59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4761,6 +4941,9 @@
       <c r="U60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="V60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4832,6 +5015,9 @@
       <c r="U61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="V61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4903,6 +5089,9 @@
       <c r="U62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="V62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4974,6 +5163,9 @@
       <c r="U63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="V63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5045,6 +5237,9 @@
       <c r="U64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="V64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5116,6 +5311,9 @@
       <c r="U65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5187,6 +5385,9 @@
       <c r="U66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5258,6 +5459,9 @@
       <c r="U67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5329,6 +5533,9 @@
       <c r="U68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5400,6 +5607,9 @@
       <c r="U69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5471,6 +5681,9 @@
       <c r="U70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5542,6 +5755,9 @@
       <c r="U71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5613,6 +5829,9 @@
       <c r="U72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5684,6 +5903,9 @@
       <c r="U73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5755,6 +5977,9 @@
       <c r="U74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5826,6 +6051,9 @@
       <c r="U75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5897,6 +6125,9 @@
       <c r="U76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5968,6 +6199,9 @@
       <c r="U77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6039,6 +6273,9 @@
       <c r="U78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6110,6 +6347,9 @@
       <c r="U79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6181,6 +6421,9 @@
       <c r="U80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6252,6 +6495,9 @@
       <c r="U81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6323,6 +6569,9 @@
       <c r="U82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6394,6 +6643,9 @@
       <c r="U83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6465,6 +6717,9 @@
       <c r="U84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6536,6 +6791,9 @@
       <c r="U85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="V85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6607,6 +6865,9 @@
       <c r="U86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6678,6 +6939,9 @@
       <c r="U87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6749,6 +7013,9 @@
       <c r="U88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6820,6 +7087,9 @@
       <c r="U89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6891,6 +7161,9 @@
       <c r="U90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6962,6 +7235,9 @@
       <c r="U91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7033,6 +7309,9 @@
       <c r="U92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7104,6 +7383,9 @@
       <c r="U93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7175,6 +7457,9 @@
       <c r="U94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7246,6 +7531,9 @@
       <c r="U95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="V95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7317,6 +7605,9 @@
       <c r="U96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="V96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7388,6 +7679,9 @@
       <c r="U97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="V97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7459,6 +7753,9 @@
       <c r="U98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="V98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7530,6 +7827,9 @@
       <c r="U99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7601,6 +7901,9 @@
       <c r="U100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="V100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7672,6 +7975,9 @@
       <c r="U101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="V101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7743,6 +8049,9 @@
       <c r="U102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="V102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7814,6 +8123,9 @@
       <c r="U103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="V103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7885,6 +8197,9 @@
       <c r="U104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="V104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7956,6 +8271,9 @@
       <c r="U105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="V105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8027,6 +8345,9 @@
       <c r="U106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="V106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8098,6 +8419,9 @@
       <c r="U107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="V107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8169,6 +8493,9 @@
       <c r="U108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8240,6 +8567,9 @@
       <c r="U109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="V109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8311,6 +8641,9 @@
       <c r="U110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="V110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8382,6 +8715,9 @@
       <c r="U111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="V111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8453,6 +8789,9 @@
       <c r="U112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="V112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8524,6 +8863,9 @@
       <c r="U113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="V113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8595,6 +8937,9 @@
       <c r="U114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="V114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8666,6 +9011,9 @@
       <c r="U115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="V115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8737,6 +9085,9 @@
       <c r="U116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8808,6 +9159,9 @@
       <c r="U117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8879,6 +9233,9 @@
       <c r="U118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8950,6 +9307,9 @@
       <c r="U119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9021,6 +9381,9 @@
       <c r="U120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9092,6 +9455,9 @@
       <c r="U121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="V121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9163,6 +9529,9 @@
       <c r="U122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="V122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9234,6 +9603,9 @@
       <c r="U123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="V123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9305,6 +9677,9 @@
       <c r="U124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="V124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9376,6 +9751,9 @@
       <c r="U125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="V125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9447,6 +9825,9 @@
       <c r="U126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="V126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9518,6 +9899,9 @@
       <c r="U127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="V127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9589,6 +9973,9 @@
       <c r="U128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="V128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9660,6 +10047,9 @@
       <c r="U129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="V129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9731,6 +10121,9 @@
       <c r="U130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="V130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9802,6 +10195,9 @@
       <c r="U131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="V131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9873,6 +10269,9 @@
       <c r="U132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="V132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9944,6 +10343,9 @@
       <c r="U133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="V133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10015,6 +10417,9 @@
       <c r="U134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="V134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10086,6 +10491,9 @@
       <c r="U135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="V135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10157,6 +10565,9 @@
       <c r="U136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="V136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10228,6 +10639,9 @@
       <c r="U137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="V137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10299,6 +10713,9 @@
       <c r="U138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="V138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10370,6 +10787,9 @@
       <c r="U139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10441,6 +10861,9 @@
       <c r="U140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10512,6 +10935,9 @@
       <c r="U141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10583,6 +11009,9 @@
       <c r="U142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10654,6 +11083,9 @@
       <c r="U143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10725,6 +11157,9 @@
       <c r="U144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="V144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -10796,6 +11231,9 @@
       <c r="U145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="V145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -10867,6 +11305,9 @@
       <c r="U146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="V146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -10938,6 +11379,9 @@
       <c r="U147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="V147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -11009,6 +11453,9 @@
       <c r="U148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="V148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11080,6 +11527,9 @@
       <c r="U149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="V149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11151,6 +11601,9 @@
       <c r="U150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="V150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11222,6 +11675,9 @@
       <c r="U151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="V151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11293,6 +11749,9 @@
       <c r="U152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="V152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11364,6 +11823,9 @@
       <c r="U153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="V153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11435,6 +11897,9 @@
       <c r="U154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="V154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11506,6 +11971,9 @@
       <c r="U155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="V155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -11577,6 +12045,9 @@
       <c r="U156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="V156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -11648,6 +12119,9 @@
       <c r="U157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="V157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11719,6 +12193,9 @@
       <c r="U158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="V158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -11790,6 +12267,9 @@
       <c r="U159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="V159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11861,6 +12341,9 @@
       <c r="U160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="V160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -11932,6 +12415,9 @@
       <c r="U161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="V161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12003,6 +12489,9 @@
       <c r="U162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="V162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -12074,6 +12563,9 @@
       <c r="U163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="V163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -12145,9 +12637,12 @@
       <c r="U164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="V164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U164"/>
+  <autoFilter ref="A1:V164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 00:16 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$V$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$W$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V164"/>
+  <dimension ref="A1:W164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -465,6 +465,7 @@
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,6 +579,11 @@
           <t>2026-09-06 16:08</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -652,6 +658,9 @@
       <c r="V2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="W2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -726,6 +735,9 @@
       <c r="V3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="W3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -800,6 +812,9 @@
       <c r="V4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="W4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -874,6 +889,9 @@
       <c r="V5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="W5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -948,6 +966,9 @@
       <c r="V6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="W6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1022,6 +1043,9 @@
       <c r="V7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="W7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1096,6 +1120,9 @@
       <c r="V8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="W8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1170,6 +1197,9 @@
       <c r="V9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="W9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1244,6 +1274,9 @@
       <c r="V10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="W10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1318,6 +1351,9 @@
       <c r="V11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="W11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1392,6 +1428,9 @@
       <c r="V12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1466,6 +1505,9 @@
       <c r="V13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="W13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1540,6 +1582,9 @@
       <c r="V14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="W14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1614,6 +1659,9 @@
       <c r="V15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="W15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1688,6 +1736,9 @@
       <c r="V16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="W16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1762,6 +1813,9 @@
       <c r="V17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="W17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1836,6 +1890,9 @@
       <c r="V18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="W18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1910,6 +1967,9 @@
       <c r="V19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="W19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1984,6 +2044,9 @@
       <c r="V20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="W20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2058,6 +2121,9 @@
       <c r="V21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="W21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2132,6 +2198,9 @@
       <c r="V22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="W22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2206,6 +2275,9 @@
       <c r="V23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="W23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2280,6 +2352,9 @@
       <c r="V24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="W24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2354,6 +2429,9 @@
       <c r="V25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2428,6 +2506,9 @@
       <c r="V26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="W26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2502,6 +2583,9 @@
       <c r="V27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="W27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2576,6 +2660,9 @@
       <c r="V28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="W28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2650,6 +2737,9 @@
       <c r="V29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="W29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2724,6 +2814,9 @@
       <c r="V30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="W30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2798,6 +2891,9 @@
       <c r="V31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="W31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2872,6 +2968,9 @@
       <c r="V32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="W32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2946,6 +3045,9 @@
       <c r="V33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="W33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3020,6 +3122,9 @@
       <c r="V34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="W34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3094,6 +3199,9 @@
       <c r="V35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="W35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3168,6 +3276,9 @@
       <c r="V36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="W36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3242,6 +3353,9 @@
       <c r="V37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="W37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3316,6 +3430,9 @@
       <c r="V38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="W38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3390,6 +3507,9 @@
       <c r="V39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="W39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3464,6 +3584,9 @@
       <c r="V40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3538,6 +3661,9 @@
       <c r="V41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3612,6 +3738,9 @@
       <c r="V42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3686,6 +3815,9 @@
       <c r="V43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3760,6 +3892,9 @@
       <c r="V44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3834,6 +3969,9 @@
       <c r="V45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="W45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3908,6 +4046,9 @@
       <c r="V46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="W46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3982,6 +4123,9 @@
       <c r="V47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="W47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4056,6 +4200,9 @@
       <c r="V48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="W48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4130,6 +4277,9 @@
       <c r="V49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="W49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4204,6 +4354,9 @@
       <c r="V50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="W50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4278,6 +4431,9 @@
       <c r="V51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="W51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4352,6 +4508,9 @@
       <c r="V52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="W52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4426,6 +4585,9 @@
       <c r="V53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="W53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4500,6 +4662,9 @@
       <c r="V54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="W54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4574,6 +4739,9 @@
       <c r="V55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="W55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4648,6 +4816,9 @@
       <c r="V56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="W56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4722,6 +4893,9 @@
       <c r="V57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4796,6 +4970,9 @@
       <c r="V58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="W58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4870,6 +5047,9 @@
       <c r="V59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="W59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4944,6 +5124,9 @@
       <c r="V60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="W60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5018,6 +5201,9 @@
       <c r="V61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="W61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5092,6 +5278,9 @@
       <c r="V62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="W62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5166,6 +5355,9 @@
       <c r="V63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="W63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5240,6 +5432,9 @@
       <c r="V64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="W64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5314,6 +5509,9 @@
       <c r="V65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5388,6 +5586,9 @@
       <c r="V66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5462,6 +5663,9 @@
       <c r="V67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5536,6 +5740,9 @@
       <c r="V68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5610,6 +5817,9 @@
       <c r="V69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5684,6 +5894,9 @@
       <c r="V70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5758,6 +5971,9 @@
       <c r="V71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5832,6 +6048,9 @@
       <c r="V72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5906,6 +6125,9 @@
       <c r="V73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5980,6 +6202,9 @@
       <c r="V74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6054,6 +6279,9 @@
       <c r="V75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6128,6 +6356,9 @@
       <c r="V76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6202,6 +6433,9 @@
       <c r="V77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6276,6 +6510,9 @@
       <c r="V78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6350,6 +6587,9 @@
       <c r="V79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6424,6 +6664,9 @@
       <c r="V80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6498,6 +6741,9 @@
       <c r="V81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6572,6 +6818,9 @@
       <c r="V82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6646,6 +6895,9 @@
       <c r="V83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6720,6 +6972,9 @@
       <c r="V84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6794,6 +7049,9 @@
       <c r="V85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="W85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6868,6 +7126,9 @@
       <c r="V86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6942,6 +7203,9 @@
       <c r="V87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7016,6 +7280,9 @@
       <c r="V88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7090,6 +7357,9 @@
       <c r="V89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7164,6 +7434,9 @@
       <c r="V90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7238,6 +7511,9 @@
       <c r="V91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7312,6 +7588,9 @@
       <c r="V92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7386,6 +7665,9 @@
       <c r="V93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W93" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7460,6 +7742,9 @@
       <c r="V94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7534,6 +7819,9 @@
       <c r="V95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="W95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7608,6 +7896,9 @@
       <c r="V96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="W96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7682,6 +7973,9 @@
       <c r="V97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="W97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7756,6 +8050,9 @@
       <c r="V98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="W98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7830,6 +8127,9 @@
       <c r="V99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7904,6 +8204,9 @@
       <c r="V100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="W100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7978,6 +8281,9 @@
       <c r="V101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="W101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8052,6 +8358,9 @@
       <c r="V102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="W102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8126,6 +8435,9 @@
       <c r="V103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="W103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8200,6 +8512,9 @@
       <c r="V104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="W104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8274,6 +8589,9 @@
       <c r="V105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="W105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8348,6 +8666,9 @@
       <c r="V106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="W106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8422,6 +8743,9 @@
       <c r="V107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="W107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8496,6 +8820,9 @@
       <c r="V108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8570,6 +8897,9 @@
       <c r="V109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="W109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8644,6 +8974,9 @@
       <c r="V110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="W110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8718,6 +9051,9 @@
       <c r="V111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="W111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8792,6 +9128,9 @@
       <c r="V112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="W112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8866,6 +9205,9 @@
       <c r="V113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="W113" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8940,6 +9282,9 @@
       <c r="V114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="W114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9014,6 +9359,9 @@
       <c r="V115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="W115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9088,6 +9436,9 @@
       <c r="V116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9162,6 +9513,9 @@
       <c r="V117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9236,6 +9590,9 @@
       <c r="V118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9310,6 +9667,9 @@
       <c r="V119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9384,6 +9744,9 @@
       <c r="V120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9458,6 +9821,9 @@
       <c r="V121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="W121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9532,6 +9898,9 @@
       <c r="V122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="W122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9606,6 +9975,9 @@
       <c r="V123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="W123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9680,6 +10052,9 @@
       <c r="V124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="W124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9754,6 +10129,9 @@
       <c r="V125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="W125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9828,6 +10206,9 @@
       <c r="V126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="W126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9902,6 +10283,9 @@
       <c r="V127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="W127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9976,6 +10360,9 @@
       <c r="V128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="W128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -10050,6 +10437,9 @@
       <c r="V129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="W129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10124,6 +10514,9 @@
       <c r="V130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="W130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10198,6 +10591,9 @@
       <c r="V131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="W131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10272,6 +10668,9 @@
       <c r="V132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="W132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -10346,6 +10745,9 @@
       <c r="V133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="W133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10420,6 +10822,9 @@
       <c r="V134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="W134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10494,6 +10899,9 @@
       <c r="V135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="W135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10568,6 +10976,9 @@
       <c r="V136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="W136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10642,6 +11053,9 @@
       <c r="V137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="W137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10716,6 +11130,9 @@
       <c r="V138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="W138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10790,6 +11207,9 @@
       <c r="V139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10864,6 +11284,9 @@
       <c r="V140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10938,6 +11361,9 @@
       <c r="V141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -11012,6 +11438,9 @@
       <c r="V142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -11086,6 +11515,9 @@
       <c r="V143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -11160,6 +11592,9 @@
       <c r="V144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="W144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -11234,6 +11669,9 @@
       <c r="V145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="W145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -11308,6 +11746,9 @@
       <c r="V146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="W146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11382,6 +11823,9 @@
       <c r="V147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="W147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -11456,6 +11900,9 @@
       <c r="V148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="W148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11530,6 +11977,9 @@
       <c r="V149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="W149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11604,6 +12054,9 @@
       <c r="V150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="W150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11678,6 +12131,9 @@
       <c r="V151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="W151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11752,6 +12208,9 @@
       <c r="V152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="W152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11826,6 +12285,9 @@
       <c r="V153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="W153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11900,6 +12362,9 @@
       <c r="V154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="W154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11974,6 +12439,9 @@
       <c r="V155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="W155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12048,6 +12516,9 @@
       <c r="V156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="W156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -12122,6 +12593,9 @@
       <c r="V157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="W157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -12196,6 +12670,9 @@
       <c r="V158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="W158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -12270,6 +12747,9 @@
       <c r="V159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="W159" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -12344,6 +12824,9 @@
       <c r="V160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="W160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -12418,6 +12901,9 @@
       <c r="V161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="W161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12492,6 +12978,9 @@
       <c r="V162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="W162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -12566,6 +13055,9 @@
       <c r="V163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="W163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -12640,9 +13132,12 @@
       <c r="V164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="W164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V164"/>
+  <autoFilter ref="A1:W164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 03:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$W$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$X$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W164"/>
+  <dimension ref="A1:X164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,7 @@
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,6 +585,11 @@
           <t>2026-09-06 19:15</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -661,6 +667,9 @@
       <c r="W2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="X2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -738,6 +747,9 @@
       <c r="W3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="X3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -815,6 +827,9 @@
       <c r="W4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="X4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -892,6 +907,9 @@
       <c r="W5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="X5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -969,6 +987,9 @@
       <c r="W6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="X6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1046,6 +1067,9 @@
       <c r="W7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="X7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1123,6 +1147,9 @@
       <c r="W8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="X8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1200,6 +1227,9 @@
       <c r="W9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="X9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1277,6 +1307,9 @@
       <c r="W10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="X10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1354,6 +1387,9 @@
       <c r="W11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="X11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1431,6 +1467,9 @@
       <c r="W12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1508,6 +1547,9 @@
       <c r="W13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="X13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1585,6 +1627,9 @@
       <c r="W14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="X14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1662,6 +1707,9 @@
       <c r="W15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="X15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1739,6 +1787,9 @@
       <c r="W16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="X16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1816,6 +1867,9 @@
       <c r="W17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="X17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1893,6 +1947,9 @@
       <c r="W18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="X18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1970,6 +2027,9 @@
       <c r="W19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="X19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2047,6 +2107,9 @@
       <c r="W20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="X20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2124,6 +2187,9 @@
       <c r="W21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="X21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2201,6 +2267,9 @@
       <c r="W22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="X22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2278,6 +2347,9 @@
       <c r="W23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="X23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2355,6 +2427,9 @@
       <c r="W24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="X24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2432,6 +2507,9 @@
       <c r="W25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2509,6 +2587,9 @@
       <c r="W26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="X26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2586,6 +2667,9 @@
       <c r="W27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="X27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2663,6 +2747,9 @@
       <c r="W28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="X28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2740,6 +2827,9 @@
       <c r="W29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="X29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2817,6 +2907,9 @@
       <c r="W30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="X30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2894,6 +2987,9 @@
       <c r="W31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="X31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2971,6 +3067,9 @@
       <c r="W32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="X32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3048,6 +3147,9 @@
       <c r="W33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="X33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3125,6 +3227,9 @@
       <c r="W34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="X34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3202,6 +3307,9 @@
       <c r="W35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="X35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3279,6 +3387,9 @@
       <c r="W36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="X36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3356,6 +3467,9 @@
       <c r="W37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="X37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3433,6 +3547,9 @@
       <c r="W38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="X38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3510,6 +3627,9 @@
       <c r="W39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="X39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3587,6 +3707,9 @@
       <c r="W40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3664,6 +3787,9 @@
       <c r="W41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3741,6 +3867,9 @@
       <c r="W42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3818,6 +3947,9 @@
       <c r="W43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3895,6 +4027,9 @@
       <c r="W44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3972,6 +4107,9 @@
       <c r="W45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="X45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4049,6 +4187,9 @@
       <c r="W46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="X46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4126,6 +4267,9 @@
       <c r="W47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="X47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4203,6 +4347,9 @@
       <c r="W48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="X48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4280,6 +4427,9 @@
       <c r="W49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="X49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4357,6 +4507,9 @@
       <c r="W50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="X50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4434,6 +4587,9 @@
       <c r="W51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="X51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4511,6 +4667,9 @@
       <c r="W52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="X52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4588,6 +4747,9 @@
       <c r="W53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="X53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4665,6 +4827,9 @@
       <c r="W54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="X54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4742,6 +4907,9 @@
       <c r="W55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="X55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4819,6 +4987,9 @@
       <c r="W56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="X56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4896,6 +5067,9 @@
       <c r="W57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4973,6 +5147,9 @@
       <c r="W58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="X58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5050,6 +5227,9 @@
       <c r="W59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="X59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5127,6 +5307,9 @@
       <c r="W60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="X60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5204,6 +5387,9 @@
       <c r="W61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="X61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5281,6 +5467,9 @@
       <c r="W62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="X62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5358,6 +5547,9 @@
       <c r="W63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="X63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5435,6 +5627,9 @@
       <c r="W64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="X64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5512,6 +5707,9 @@
       <c r="W65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5589,6 +5787,9 @@
       <c r="W66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5666,6 +5867,9 @@
       <c r="W67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5743,6 +5947,9 @@
       <c r="W68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5820,6 +6027,9 @@
       <c r="W69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5897,6 +6107,9 @@
       <c r="W70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5974,6 +6187,9 @@
       <c r="W71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6051,6 +6267,9 @@
       <c r="W72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6128,6 +6347,9 @@
       <c r="W73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6205,6 +6427,9 @@
       <c r="W74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6282,6 +6507,9 @@
       <c r="W75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6359,6 +6587,9 @@
       <c r="W76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6436,6 +6667,9 @@
       <c r="W77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6513,6 +6747,9 @@
       <c r="W78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6590,6 +6827,9 @@
       <c r="W79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6667,6 +6907,9 @@
       <c r="W80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6744,6 +6987,9 @@
       <c r="W81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6821,6 +7067,9 @@
       <c r="W82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6898,6 +7147,9 @@
       <c r="W83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6975,6 +7227,9 @@
       <c r="W84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7052,6 +7307,9 @@
       <c r="W85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="X85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7129,6 +7387,9 @@
       <c r="W86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7206,6 +7467,9 @@
       <c r="W87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7283,6 +7547,9 @@
       <c r="W88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7360,6 +7627,9 @@
       <c r="W89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7437,6 +7707,9 @@
       <c r="W90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7514,6 +7787,9 @@
       <c r="W91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7591,6 +7867,9 @@
       <c r="W92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7668,6 +7947,9 @@
       <c r="W93" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7745,6 +8027,9 @@
       <c r="W94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7822,6 +8107,9 @@
       <c r="W95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="X95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7899,6 +8187,9 @@
       <c r="W96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="X96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7976,6 +8267,9 @@
       <c r="W97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="X97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8053,6 +8347,9 @@
       <c r="W98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="X98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8130,6 +8427,9 @@
       <c r="W99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -8207,6 +8507,9 @@
       <c r="W100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="X100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -8284,6 +8587,9 @@
       <c r="W101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="X101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8361,6 +8667,9 @@
       <c r="W102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="X102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8438,6 +8747,9 @@
       <c r="W103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="X103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8515,6 +8827,9 @@
       <c r="W104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="X104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8592,6 +8907,9 @@
       <c r="W105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="X105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8669,6 +8987,9 @@
       <c r="W106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="X106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8746,6 +9067,9 @@
       <c r="W107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="X107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8823,6 +9147,9 @@
       <c r="W108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8900,6 +9227,9 @@
       <c r="W109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="X109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8977,6 +9307,9 @@
       <c r="W110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="X110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -9054,6 +9387,9 @@
       <c r="W111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="X111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -9131,6 +9467,9 @@
       <c r="W112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="X112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -9208,6 +9547,9 @@
       <c r="W113" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="X113" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -9285,6 +9627,9 @@
       <c r="W114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="X114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9362,6 +9707,9 @@
       <c r="W115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="X115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9439,6 +9787,9 @@
       <c r="W116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9516,6 +9867,9 @@
       <c r="W117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9593,6 +9947,9 @@
       <c r="W118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9670,6 +10027,9 @@
       <c r="W119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9747,6 +10107,9 @@
       <c r="W120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9824,6 +10187,9 @@
       <c r="W121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="X121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9901,6 +10267,9 @@
       <c r="W122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="X122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9978,6 +10347,9 @@
       <c r="W123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="X123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -10055,6 +10427,9 @@
       <c r="W124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="X124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -10132,6 +10507,9 @@
       <c r="W125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="X125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10209,6 +10587,9 @@
       <c r="W126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="X126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -10286,6 +10667,9 @@
       <c r="W127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="X127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -10363,6 +10747,9 @@
       <c r="W128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="X128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -10440,6 +10827,9 @@
       <c r="W129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="X129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10517,6 +10907,9 @@
       <c r="W130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="X130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10594,6 +10987,9 @@
       <c r="W131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="X131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10671,6 +11067,9 @@
       <c r="W132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="X132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -10748,6 +11147,9 @@
       <c r="W133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="X133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10825,6 +11227,9 @@
       <c r="W134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="X134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10902,6 +11307,9 @@
       <c r="W135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="X135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10979,6 +11387,9 @@
       <c r="W136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="X136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -11056,6 +11467,9 @@
       <c r="W137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="X137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -11133,6 +11547,9 @@
       <c r="W138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="X138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -11210,6 +11627,9 @@
       <c r="W139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -11287,6 +11707,9 @@
       <c r="W140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -11364,6 +11787,9 @@
       <c r="W141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -11441,6 +11867,9 @@
       <c r="W142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -11518,6 +11947,9 @@
       <c r="W143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -11595,6 +12027,9 @@
       <c r="W144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="X144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -11672,6 +12107,9 @@
       <c r="W145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="X145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -11749,6 +12187,9 @@
       <c r="W146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="X146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11826,6 +12267,9 @@
       <c r="W147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="X147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -11903,6 +12347,9 @@
       <c r="W148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="X148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11980,6 +12427,9 @@
       <c r="W149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="X149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12057,6 +12507,9 @@
       <c r="W150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="X150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12134,6 +12587,9 @@
       <c r="W151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="X151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -12211,6 +12667,9 @@
       <c r="W152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="X152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -12288,6 +12747,9 @@
       <c r="W153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="X153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -12365,6 +12827,9 @@
       <c r="W154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="X154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -12442,6 +12907,9 @@
       <c r="W155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="X155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12519,6 +12987,9 @@
       <c r="W156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="X156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -12596,6 +13067,9 @@
       <c r="W157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="X157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -12673,6 +13147,9 @@
       <c r="W158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="X158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -12750,6 +13227,9 @@
       <c r="W159" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="X159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -12827,6 +13307,9 @@
       <c r="W160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="X160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -12904,6 +13387,9 @@
       <c r="W161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="X161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12981,6 +13467,9 @@
       <c r="W162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="X162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13058,6 +13547,9 @@
       <c r="W163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="X163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -13135,9 +13627,12 @@
       <c r="W164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="X164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W164"/>
+  <autoFilter ref="A1:X164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 06:13 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$X$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Y$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X164"/>
+  <dimension ref="A1:Y164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -590,6 +591,11 @@
           <t>2026-09-06 22:10</t>
         </is>
       </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 01:13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -670,6 +676,9 @@
       <c r="X2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="Y2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -750,6 +759,9 @@
       <c r="X3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="Y3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -830,6 +842,9 @@
       <c r="X4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="Y4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -910,6 +925,9 @@
       <c r="X5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Y5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -990,6 +1008,9 @@
       <c r="X6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Y6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1070,6 +1091,9 @@
       <c r="X7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="Y7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1150,6 +1174,9 @@
       <c r="X8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="Y8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1230,6 +1257,9 @@
       <c r="X9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="Y9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1310,6 +1340,9 @@
       <c r="X10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="Y10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1390,6 +1423,9 @@
       <c r="X11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="Y11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1470,6 +1506,9 @@
       <c r="X12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1550,6 +1589,9 @@
       <c r="X13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="Y13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1630,6 +1672,9 @@
       <c r="X14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Y14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1710,6 +1755,9 @@
       <c r="X15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Y15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1790,6 +1838,9 @@
       <c r="X16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Y16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1870,6 +1921,9 @@
       <c r="X17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Y17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1950,6 +2004,9 @@
       <c r="X18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Y18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2030,6 +2087,9 @@
       <c r="X19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="Y19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2110,6 +2170,9 @@
       <c r="X20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="Y20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2190,6 +2253,9 @@
       <c r="X21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="Y21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2270,6 +2336,9 @@
       <c r="X22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Y22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2350,6 +2419,9 @@
       <c r="X23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Y23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2430,6 +2502,9 @@
       <c r="X24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Y24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2510,6 +2585,9 @@
       <c r="X25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2590,6 +2668,9 @@
       <c r="X26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="Y26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2670,6 +2751,9 @@
       <c r="X27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Y27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2750,6 +2834,9 @@
       <c r="X28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="Y28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2830,6 +2917,9 @@
       <c r="X29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="Y29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2910,6 +3000,9 @@
       <c r="X30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Y30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2990,6 +3083,9 @@
       <c r="X31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Y31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3070,6 +3166,9 @@
       <c r="X32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Y32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3150,6 +3249,9 @@
       <c r="X33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Y33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3230,6 +3332,9 @@
       <c r="X34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="Y34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3310,6 +3415,9 @@
       <c r="X35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Y35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3390,6 +3498,9 @@
       <c r="X36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Y36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3470,6 +3581,9 @@
       <c r="X37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Y37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3550,6 +3664,9 @@
       <c r="X38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Y38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3630,6 +3747,9 @@
       <c r="X39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Y39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3710,6 +3830,9 @@
       <c r="X40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3790,6 +3913,9 @@
       <c r="X41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3870,6 +3996,9 @@
       <c r="X42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3950,6 +4079,9 @@
       <c r="X43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4030,6 +4162,9 @@
       <c r="X44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4110,6 +4245,9 @@
       <c r="X45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Y45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4190,6 +4328,9 @@
       <c r="X46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="Y46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4270,6 +4411,9 @@
       <c r="X47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Y47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4350,6 +4494,9 @@
       <c r="X48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Y48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4430,6 +4577,9 @@
       <c r="X49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Y49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4510,6 +4660,9 @@
       <c r="X50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="Y50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4590,6 +4743,9 @@
       <c r="X51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Y51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4670,6 +4826,9 @@
       <c r="X52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Y52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4750,6 +4909,9 @@
       <c r="X53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Y53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4830,6 +4992,9 @@
       <c r="X54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="Y54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4910,6 +5075,9 @@
       <c r="X55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Y55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4990,6 +5158,9 @@
       <c r="X56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Y56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5070,6 +5241,9 @@
       <c r="X57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5150,6 +5324,9 @@
       <c r="X58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Y58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5230,6 +5407,9 @@
       <c r="X59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Y59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5310,6 +5490,9 @@
       <c r="X60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Y60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5390,6 +5573,9 @@
       <c r="X61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Y61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5470,6 +5656,9 @@
       <c r="X62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Y62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5550,6 +5739,9 @@
       <c r="X63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Y63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5630,6 +5822,9 @@
       <c r="X64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Y64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5710,6 +5905,9 @@
       <c r="X65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5790,6 +5988,9 @@
       <c r="X66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5870,6 +6071,9 @@
       <c r="X67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5950,6 +6154,9 @@
       <c r="X68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6030,6 +6237,9 @@
       <c r="X69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6110,6 +6320,9 @@
       <c r="X70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6190,6 +6403,9 @@
       <c r="X71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6270,6 +6486,9 @@
       <c r="X72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6350,6 +6569,9 @@
       <c r="X73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6430,6 +6652,9 @@
       <c r="X74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6510,6 +6735,9 @@
       <c r="X75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6590,6 +6818,9 @@
       <c r="X76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6670,6 +6901,9 @@
       <c r="X77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6750,6 +6984,9 @@
       <c r="X78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6830,6 +7067,9 @@
       <c r="X79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6910,6 +7150,9 @@
       <c r="X80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6990,6 +7233,9 @@
       <c r="X81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7070,6 +7316,9 @@
       <c r="X82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7150,6 +7399,9 @@
       <c r="X83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7230,6 +7482,9 @@
       <c r="X84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7310,6 +7565,9 @@
       <c r="X85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Y85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7390,6 +7648,9 @@
       <c r="X86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7470,6 +7731,9 @@
       <c r="X87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7550,6 +7814,9 @@
       <c r="X88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7630,6 +7897,9 @@
       <c r="X89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7710,6 +7980,9 @@
       <c r="X90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7790,6 +8063,9 @@
       <c r="X91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7870,6 +8146,9 @@
       <c r="X92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7950,6 +8229,9 @@
       <c r="X93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="Y93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8030,6 +8312,9 @@
       <c r="X94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8110,6 +8395,9 @@
       <c r="X95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Y95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8190,6 +8478,9 @@
       <c r="X96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Y96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8270,6 +8561,9 @@
       <c r="X97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Y97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8350,6 +8644,9 @@
       <c r="X98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Y98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8430,6 +8727,9 @@
       <c r="X99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -8510,6 +8810,9 @@
       <c r="X100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Y100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -8590,6 +8893,9 @@
       <c r="X101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Y101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8670,6 +8976,9 @@
       <c r="X102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Y102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8750,6 +9059,9 @@
       <c r="X103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Y103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8830,6 +9142,9 @@
       <c r="X104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Y104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8910,6 +9225,9 @@
       <c r="X105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Y105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8990,6 +9308,9 @@
       <c r="X106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Y106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9070,6 +9391,9 @@
       <c r="X107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="Y107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9150,6 +9474,9 @@
       <c r="X108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -9230,6 +9557,9 @@
       <c r="X109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Y109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -9310,6 +9640,9 @@
       <c r="X110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Y110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -9390,6 +9723,9 @@
       <c r="X111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Y111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -9470,6 +9806,9 @@
       <c r="X112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Y112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -9550,6 +9889,9 @@
       <c r="X113" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="Y113" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -9630,6 +9972,9 @@
       <c r="X114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Y114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9710,6 +10055,9 @@
       <c r="X115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Y115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9790,6 +10138,9 @@
       <c r="X116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9870,6 +10221,9 @@
       <c r="X117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9950,6 +10304,9 @@
       <c r="X118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10030,6 +10387,9 @@
       <c r="X119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10110,6 +10470,9 @@
       <c r="X120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -10190,6 +10553,9 @@
       <c r="X121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Y121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -10270,6 +10636,9 @@
       <c r="X122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Y122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10350,6 +10719,9 @@
       <c r="X123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Y123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -10430,6 +10802,9 @@
       <c r="X124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Y124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -10510,6 +10885,9 @@
       <c r="X125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Y125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10590,6 +10968,9 @@
       <c r="X126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Y126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -10670,6 +11051,9 @@
       <c r="X127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Y127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -10750,6 +11134,9 @@
       <c r="X128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Y128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -10830,6 +11217,9 @@
       <c r="X129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Y129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10910,6 +11300,9 @@
       <c r="X130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Y130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10990,6 +11383,9 @@
       <c r="X131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Y131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11070,6 +11466,9 @@
       <c r="X132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="Y132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11150,6 +11549,9 @@
       <c r="X133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Y133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -11230,6 +11632,9 @@
       <c r="X134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Y134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -11310,6 +11715,9 @@
       <c r="X135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Y135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -11390,6 +11798,9 @@
       <c r="X136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Y136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -11470,6 +11881,9 @@
       <c r="X137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Y137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -11550,6 +11964,9 @@
       <c r="X138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="Y138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -11630,6 +12047,9 @@
       <c r="X139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -11710,6 +12130,9 @@
       <c r="X140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -11790,6 +12213,9 @@
       <c r="X141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -11870,6 +12296,9 @@
       <c r="X142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -11950,6 +12379,9 @@
       <c r="X143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12030,6 +12462,9 @@
       <c r="X144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Y144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12110,6 +12545,9 @@
       <c r="X145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="Y145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -12190,6 +12628,9 @@
       <c r="X146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Y146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -12270,6 +12711,9 @@
       <c r="X147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Y147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -12350,6 +12794,9 @@
       <c r="X148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="Y148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -12430,6 +12877,9 @@
       <c r="X149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="Y149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12510,6 +12960,9 @@
       <c r="X150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="Y150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12590,6 +13043,9 @@
       <c r="X151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="Y151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -12670,6 +13126,9 @@
       <c r="X152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Y152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -12750,6 +13209,9 @@
       <c r="X153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Y153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -12830,6 +13292,9 @@
       <c r="X154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="Y154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -12910,6 +13375,9 @@
       <c r="X155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="Y155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12990,6 +13458,9 @@
       <c r="X156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Y156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -13070,6 +13541,9 @@
       <c r="X157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Y157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -13150,6 +13624,9 @@
       <c r="X158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Y158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -13230,6 +13707,9 @@
       <c r="X159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="Y159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -13310,6 +13790,9 @@
       <c r="X160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Y160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -13390,6 +13873,9 @@
       <c r="X161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Y161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -13470,6 +13956,9 @@
       <c r="X162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="Y162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13550,6 +14039,9 @@
       <c r="X163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="Y163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -13630,9 +14122,12 @@
       <c r="X164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="Y164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X164"/>
+  <autoFilter ref="A1:Y164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 09:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Y$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Z$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y164"/>
+  <dimension ref="A1:Z164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,7 @@
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -596,6 +597,11 @@
           <t>2026-09-07 01:13</t>
         </is>
       </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 04:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -679,6 +685,9 @@
       <c r="Y2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="Z2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -762,6 +771,9 @@
       <c r="Y3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="Z3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -845,6 +857,9 @@
       <c r="Y4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="Z4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -928,6 +943,9 @@
       <c r="Y5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Z5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1011,6 +1029,9 @@
       <c r="Y6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="Z6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1094,6 +1115,9 @@
       <c r="Y7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="Z7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1177,6 +1201,9 @@
       <c r="Y8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="Z8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1260,6 +1287,9 @@
       <c r="Y9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="Z9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1343,6 +1373,9 @@
       <c r="Y10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="Z10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1426,6 +1459,9 @@
       <c r="Y11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="Z11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1509,6 +1545,9 @@
       <c r="Y12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1592,6 +1631,9 @@
       <c r="Y13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="Z13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1675,6 +1717,9 @@
       <c r="Y14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Z14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1758,6 +1803,9 @@
       <c r="Y15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="Z15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1841,6 +1889,9 @@
       <c r="Y16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Z16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1924,6 +1975,9 @@
       <c r="Y17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Z17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2007,6 +2061,9 @@
       <c r="Y18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Z18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2090,6 +2147,9 @@
       <c r="Y19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="Z19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2173,6 +2233,9 @@
       <c r="Y20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="Z20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2256,6 +2319,9 @@
       <c r="Y21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="Z21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2339,6 +2405,9 @@
       <c r="Y22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="Z22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2422,6 +2491,9 @@
       <c r="Y23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Z23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2505,6 +2577,9 @@
       <c r="Y24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Z24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2588,6 +2663,9 @@
       <c r="Y25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2671,6 +2749,9 @@
       <c r="Y26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="Z26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2754,6 +2835,9 @@
       <c r="Y27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Z27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2837,6 +2921,9 @@
       <c r="Y28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="Z28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2920,6 +3007,9 @@
       <c r="Y29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="Z29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3003,6 +3093,9 @@
       <c r="Y30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Z30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3086,6 +3179,9 @@
       <c r="Y31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Z31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3169,6 +3265,9 @@
       <c r="Y32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Z32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3252,6 +3351,9 @@
       <c r="Y33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Z33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3335,6 +3437,9 @@
       <c r="Y34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="Z34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3418,6 +3523,9 @@
       <c r="Y35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Z35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3501,6 +3609,9 @@
       <c r="Y36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Z36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3584,6 +3695,9 @@
       <c r="Y37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Z37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3667,6 +3781,9 @@
       <c r="Y38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Z38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3750,6 +3867,9 @@
       <c r="Y39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="Z39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3833,6 +3953,9 @@
       <c r="Y40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3916,6 +4039,9 @@
       <c r="Y41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3999,6 +4125,9 @@
       <c r="Y42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4082,6 +4211,9 @@
       <c r="Y43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4165,6 +4297,9 @@
       <c r="Y44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4248,6 +4383,9 @@
       <c r="Y45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="Z45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4331,6 +4469,9 @@
       <c r="Y46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="Z46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4414,6 +4555,9 @@
       <c r="Y47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Z47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4497,6 +4641,9 @@
       <c r="Y48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="Z48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4580,6 +4727,9 @@
       <c r="Y49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Z49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4663,6 +4813,9 @@
       <c r="Y50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="Z50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4746,6 +4899,9 @@
       <c r="Y51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Z51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4829,6 +4985,9 @@
       <c r="Y52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="Z52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4912,6 +5071,9 @@
       <c r="Y53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Z53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4995,6 +5157,9 @@
       <c r="Y54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="Z54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5078,6 +5243,9 @@
       <c r="Y55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Z55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5161,6 +5329,9 @@
       <c r="Y56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="Z56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5244,6 +5415,9 @@
       <c r="Y57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5327,6 +5501,9 @@
       <c r="Y58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Z58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5410,6 +5587,9 @@
       <c r="Y59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Z59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5493,6 +5673,9 @@
       <c r="Y60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="Z60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5576,6 +5759,9 @@
       <c r="Y61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Z61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5659,6 +5845,9 @@
       <c r="Y62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Z62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5742,6 +5931,9 @@
       <c r="Y63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Z63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5825,6 +6017,9 @@
       <c r="Y64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="Z64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5908,6 +6103,9 @@
       <c r="Y65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5991,6 +6189,9 @@
       <c r="Y66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6074,6 +6275,9 @@
       <c r="Y67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6157,6 +6361,9 @@
       <c r="Y68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6240,6 +6447,9 @@
       <c r="Y69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6323,6 +6533,9 @@
       <c r="Y70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6406,6 +6619,9 @@
       <c r="Y71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6489,6 +6705,9 @@
       <c r="Y72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6572,6 +6791,9 @@
       <c r="Y73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6655,6 +6877,9 @@
       <c r="Y74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6738,6 +6963,9 @@
       <c r="Y75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6821,6 +7049,9 @@
       <c r="Y76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6904,6 +7135,9 @@
       <c r="Y77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6987,6 +7221,9 @@
       <c r="Y78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7070,6 +7307,9 @@
       <c r="Y79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7153,6 +7393,9 @@
       <c r="Y80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7236,6 +7479,9 @@
       <c r="Y81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7319,6 +7565,9 @@
       <c r="Y82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7402,6 +7651,9 @@
       <c r="Y83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7485,6 +7737,9 @@
       <c r="Y84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7568,6 +7823,9 @@
       <c r="Y85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Z85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7651,6 +7909,9 @@
       <c r="Y86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7734,6 +7995,9 @@
       <c r="Y87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7817,6 +8081,9 @@
       <c r="Y88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7900,6 +8167,9 @@
       <c r="Y89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7983,6 +8253,9 @@
       <c r="Y90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8066,6 +8339,9 @@
       <c r="Y91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8149,6 +8425,9 @@
       <c r="Y92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8232,6 +8511,9 @@
       <c r="Y93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="Z93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8315,6 +8597,9 @@
       <c r="Y94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8398,6 +8683,9 @@
       <c r="Y95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Z95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8481,6 +8769,9 @@
       <c r="Y96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Z96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8564,6 +8855,9 @@
       <c r="Y97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="Z97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8647,6 +8941,9 @@
       <c r="Y98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Z98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8730,6 +9027,9 @@
       <c r="Y99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -8813,6 +9113,9 @@
       <c r="Y100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Z100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -8896,6 +9199,9 @@
       <c r="Y101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Z101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8979,6 +9285,9 @@
       <c r="Y102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Z102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9062,6 +9371,9 @@
       <c r="Y103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="Z103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9145,6 +9457,9 @@
       <c r="Y104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Z104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9228,6 +9543,9 @@
       <c r="Y105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Z105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9311,6 +9629,9 @@
       <c r="Y106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="Z106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9394,6 +9715,9 @@
       <c r="Y107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="Z107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9477,6 +9801,9 @@
       <c r="Y108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -9560,6 +9887,9 @@
       <c r="Y109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="Z109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -9643,6 +9973,9 @@
       <c r="Y110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="Z110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -9726,6 +10059,9 @@
       <c r="Y111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Z111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -9809,6 +10145,9 @@
       <c r="Y112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Z112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -9892,6 +10231,9 @@
       <c r="Y113" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="Z113" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -9975,6 +10317,9 @@
       <c r="Y114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Z114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10058,6 +10403,9 @@
       <c r="Y115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="Z115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10141,6 +10489,9 @@
       <c r="Y116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10224,6 +10575,9 @@
       <c r="Y117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10307,6 +10661,9 @@
       <c r="Y118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10390,6 +10747,9 @@
       <c r="Y119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10473,6 +10833,9 @@
       <c r="Y120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -10556,6 +10919,9 @@
       <c r="Y121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="Z121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -10639,6 +11005,9 @@
       <c r="Y122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="Z122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10722,6 +11091,9 @@
       <c r="Y123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="Z123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -10805,6 +11177,9 @@
       <c r="Y124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Z124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -10888,6 +11263,9 @@
       <c r="Y125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Z125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10971,6 +11349,9 @@
       <c r="Y126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Z126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11054,6 +11435,9 @@
       <c r="Y127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="Z127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11137,6 +11521,9 @@
       <c r="Y128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Z128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11220,6 +11607,9 @@
       <c r="Y129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Z129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11303,6 +11693,9 @@
       <c r="Y130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Z130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11386,6 +11779,9 @@
       <c r="Y131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="Z131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11469,6 +11865,9 @@
       <c r="Y132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="Z132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11552,6 +11951,9 @@
       <c r="Y133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Z133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -11635,6 +12037,9 @@
       <c r="Y134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="Z134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -11718,6 +12123,9 @@
       <c r="Y135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Z135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -11801,6 +12209,9 @@
       <c r="Y136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Z136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -11884,6 +12295,9 @@
       <c r="Y137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="Z137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -11967,6 +12381,9 @@
       <c r="Y138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="Z138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12050,6 +12467,9 @@
       <c r="Y139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12133,6 +12553,9 @@
       <c r="Y140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12216,6 +12639,9 @@
       <c r="Y141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12299,6 +12725,9 @@
       <c r="Y142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -12382,6 +12811,9 @@
       <c r="Y143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12465,6 +12897,9 @@
       <c r="Y144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="Z144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12548,6 +12983,9 @@
       <c r="Y145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="Z145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -12631,6 +13069,9 @@
       <c r="Y146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Z146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -12714,6 +13155,9 @@
       <c r="Y147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="Z147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -12797,6 +13241,9 @@
       <c r="Y148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="Z148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -12880,6 +13327,9 @@
       <c r="Y149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="Z149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12963,6 +13413,9 @@
       <c r="Y150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="Z150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -13046,6 +13499,9 @@
       <c r="Y151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="Z151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -13129,6 +13585,9 @@
       <c r="Y152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Z152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -13212,6 +13671,9 @@
       <c r="Y153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="Z153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -13295,6 +13757,9 @@
       <c r="Y154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="Z154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -13378,6 +13843,9 @@
       <c r="Y155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="Z155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -13461,6 +13929,9 @@
       <c r="Y156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Z156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -13544,6 +14015,9 @@
       <c r="Y157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="Z157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -13627,6 +14101,9 @@
       <c r="Y158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Z158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -13710,6 +14187,9 @@
       <c r="Y159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="Z159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -13793,6 +14273,9 @@
       <c r="Y160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Z160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -13876,6 +14359,9 @@
       <c r="Y161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="Z161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -13959,6 +14445,9 @@
       <c r="Y162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="Z162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -14042,6 +14531,9 @@
       <c r="Y163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="Z163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -14125,9 +14617,12 @@
       <c r="Y164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="Z164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y164"/>
+  <autoFilter ref="A1:Z164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 09:49 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$Z$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AA$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z164"/>
+  <dimension ref="A1:AA164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -469,6 +469,7 @@
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,6 +603,11 @@
           <t>2026-09-07 04:10</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 04:49</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -688,6 +694,9 @@
       <c r="Z2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AA2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -774,6 +783,9 @@
       <c r="Z3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AA3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -860,6 +872,9 @@
       <c r="Z4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AA4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -946,6 +961,9 @@
       <c r="Z5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AA5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1032,6 +1050,9 @@
       <c r="Z6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AA6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1118,6 +1139,9 @@
       <c r="Z7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AA7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1204,6 +1228,9 @@
       <c r="Z8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="AA8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1290,6 +1317,9 @@
       <c r="Z9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AA9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1376,6 +1406,9 @@
       <c r="Z10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AA10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1462,6 +1495,9 @@
       <c r="Z11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AA11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1548,6 +1584,9 @@
       <c r="Z12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1634,6 +1673,9 @@
       <c r="Z13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AA13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1720,6 +1762,9 @@
       <c r="Z14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AA14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1806,6 +1851,9 @@
       <c r="Z15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AA15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1892,6 +1940,9 @@
       <c r="Z16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AA16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1978,6 +2029,9 @@
       <c r="Z17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AA17" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2064,6 +2118,9 @@
       <c r="Z18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AA18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2150,6 +2207,9 @@
       <c r="Z19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AA19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2236,6 +2296,9 @@
       <c r="Z20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="AA20" s="3" t="n">
+        <v>20.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2322,6 +2385,9 @@
       <c r="Z21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AA21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2408,6 +2474,9 @@
       <c r="Z22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AA22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2494,6 +2563,9 @@
       <c r="Z23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AA23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2580,6 +2652,9 @@
       <c r="Z24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AA24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2666,6 +2741,9 @@
       <c r="Z25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2752,6 +2830,9 @@
       <c r="Z26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AA26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2838,6 +2919,9 @@
       <c r="Z27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AA27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2924,6 +3008,9 @@
       <c r="Z28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AA28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3010,6 +3097,9 @@
       <c r="Z29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="AA29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3096,6 +3186,9 @@
       <c r="Z30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AA30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3182,6 +3275,9 @@
       <c r="Z31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AA31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3268,6 +3364,9 @@
       <c r="Z32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AA32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3354,6 +3453,9 @@
       <c r="Z33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AA33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3440,6 +3542,9 @@
       <c r="Z34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="AA34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3526,6 +3631,9 @@
       <c r="Z35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AA35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3612,6 +3720,9 @@
       <c r="Z36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AA36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3698,6 +3809,9 @@
       <c r="Z37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AA37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3784,6 +3898,9 @@
       <c r="Z38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AA38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3870,6 +3987,9 @@
       <c r="Z39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AA39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3956,6 +4076,9 @@
       <c r="Z40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4042,6 +4165,9 @@
       <c r="Z41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4128,6 +4254,9 @@
       <c r="Z42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4214,6 +4343,9 @@
       <c r="Z43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4300,6 +4432,9 @@
       <c r="Z44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4386,6 +4521,9 @@
       <c r="Z45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AA45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4472,6 +4610,9 @@
       <c r="Z46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AA46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4558,6 +4699,9 @@
       <c r="Z47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AA47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4644,6 +4788,9 @@
       <c r="Z48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AA48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4730,6 +4877,9 @@
       <c r="Z49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AA49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4816,6 +4966,9 @@
       <c r="Z50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AA50" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4902,6 +5055,9 @@
       <c r="Z51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AA51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4988,6 +5144,9 @@
       <c r="Z52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AA52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5074,6 +5233,9 @@
       <c r="Z53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AA53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5160,6 +5322,9 @@
       <c r="Z54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AA54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5246,6 +5411,9 @@
       <c r="Z55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AA55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5332,6 +5500,9 @@
       <c r="Z56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AA56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5418,6 +5589,9 @@
       <c r="Z57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5504,6 +5678,9 @@
       <c r="Z58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AA58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5590,6 +5767,9 @@
       <c r="Z59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AA59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5676,6 +5856,9 @@
       <c r="Z60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AA60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5762,6 +5945,9 @@
       <c r="Z61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AA61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5848,6 +6034,9 @@
       <c r="Z62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AA62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5934,6 +6123,9 @@
       <c r="Z63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AA63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6020,6 +6212,9 @@
       <c r="Z64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AA64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6106,6 +6301,9 @@
       <c r="Z65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6192,6 +6390,9 @@
       <c r="Z66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6278,6 +6479,9 @@
       <c r="Z67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6364,6 +6568,9 @@
       <c r="Z68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6450,6 +6657,9 @@
       <c r="Z69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6536,6 +6746,9 @@
       <c r="Z70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6622,6 +6835,9 @@
       <c r="Z71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6708,6 +6924,9 @@
       <c r="Z72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6794,6 +7013,9 @@
       <c r="Z73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6880,6 +7102,9 @@
       <c r="Z74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6966,6 +7191,9 @@
       <c r="Z75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7052,6 +7280,9 @@
       <c r="Z76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7138,6 +7369,9 @@
       <c r="Z77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7224,6 +7458,9 @@
       <c r="Z78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7310,6 +7547,9 @@
       <c r="Z79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7396,6 +7636,9 @@
       <c r="Z80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7482,6 +7725,9 @@
       <c r="Z81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7568,6 +7814,9 @@
       <c r="Z82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7654,6 +7903,9 @@
       <c r="Z83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7740,6 +7992,9 @@
       <c r="Z84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7826,6 +8081,9 @@
       <c r="Z85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AA85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7912,6 +8170,9 @@
       <c r="Z86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7998,6 +8259,9 @@
       <c r="Z87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8084,6 +8348,9 @@
       <c r="Z88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8170,6 +8437,9 @@
       <c r="Z89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8256,6 +8526,9 @@
       <c r="Z90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8342,6 +8615,9 @@
       <c r="Z91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8428,6 +8704,9 @@
       <c r="Z92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8514,6 +8793,9 @@
       <c r="Z93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AA93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8600,6 +8882,9 @@
       <c r="Z94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8686,6 +8971,9 @@
       <c r="Z95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AA95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8772,6 +9060,9 @@
       <c r="Z96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AA96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8858,6 +9149,9 @@
       <c r="Z97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AA97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8944,6 +9238,9 @@
       <c r="Z98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AA98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9030,6 +9327,9 @@
       <c r="Z99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9116,6 +9416,9 @@
       <c r="Z100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AA100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9202,6 +9505,9 @@
       <c r="Z101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AA101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9288,6 +9594,9 @@
       <c r="Z102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AA102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9374,6 +9683,9 @@
       <c r="Z103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AA103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9460,6 +9772,9 @@
       <c r="Z104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AA104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9546,6 +9861,9 @@
       <c r="Z105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AA105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9632,6 +9950,9 @@
       <c r="Z106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AA106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9718,6 +10039,9 @@
       <c r="Z107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AA107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9804,6 +10128,9 @@
       <c r="Z108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -9890,6 +10217,9 @@
       <c r="Z109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AA109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -9976,6 +10306,9 @@
       <c r="Z110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AA110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10062,6 +10395,9 @@
       <c r="Z111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AA111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10148,6 +10484,9 @@
       <c r="Z112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AA112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10234,6 +10573,9 @@
       <c r="Z113" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="AA113" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10320,6 +10662,9 @@
       <c r="Z114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AA114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10406,6 +10751,9 @@
       <c r="Z115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AA115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10492,6 +10840,9 @@
       <c r="Z116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10578,6 +10929,9 @@
       <c r="Z117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10664,6 +11018,9 @@
       <c r="Z118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10750,6 +11107,9 @@
       <c r="Z119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10836,6 +11196,9 @@
       <c r="Z120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -10922,6 +11285,9 @@
       <c r="Z121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AA121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11008,6 +11374,9 @@
       <c r="Z122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AA122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11094,6 +11463,9 @@
       <c r="Z123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AA123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11180,6 +11552,9 @@
       <c r="Z124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AA124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11266,6 +11641,9 @@
       <c r="Z125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AA125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11352,6 +11730,9 @@
       <c r="Z126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AA126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11438,6 +11819,9 @@
       <c r="Z127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AA127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11524,6 +11908,9 @@
       <c r="Z128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AA128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11610,6 +11997,9 @@
       <c r="Z129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AA129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11696,6 +12086,9 @@
       <c r="Z130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AA130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11782,6 +12175,9 @@
       <c r="Z131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AA131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11868,6 +12264,9 @@
       <c r="Z132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AA132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11954,6 +12353,9 @@
       <c r="Z133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AA133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -12040,6 +12442,9 @@
       <c r="Z134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AA134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12126,6 +12531,9 @@
       <c r="Z135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AA135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -12212,6 +12620,9 @@
       <c r="Z136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AA136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12298,6 +12709,9 @@
       <c r="Z137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AA137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -12384,6 +12798,9 @@
       <c r="Z138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AA138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12470,6 +12887,9 @@
       <c r="Z139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12556,6 +12976,9 @@
       <c r="Z140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12642,6 +13065,9 @@
       <c r="Z141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12728,6 +13154,9 @@
       <c r="Z142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -12814,6 +13243,9 @@
       <c r="Z143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12900,6 +13332,9 @@
       <c r="Z144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AA144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12986,6 +13421,9 @@
       <c r="Z145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AA145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -13072,6 +13510,9 @@
       <c r="Z146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AA146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -13158,6 +13599,9 @@
       <c r="Z147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AA147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -13244,6 +13688,9 @@
       <c r="Z148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AA148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -13330,6 +13777,9 @@
       <c r="Z149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AA149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -13416,6 +13866,9 @@
       <c r="Z150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AA150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -13502,6 +13955,9 @@
       <c r="Z151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AA151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -13588,6 +14044,9 @@
       <c r="Z152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AA152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -13674,6 +14133,9 @@
       <c r="Z153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AA153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -13760,6 +14222,9 @@
       <c r="Z154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AA154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -13846,6 +14311,9 @@
       <c r="Z155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AA155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -13932,6 +14400,9 @@
       <c r="Z156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AA156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -14018,6 +14489,9 @@
       <c r="Z157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AA157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -14104,6 +14578,9 @@
       <c r="Z158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AA158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -14190,6 +14667,9 @@
       <c r="Z159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AA159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -14276,6 +14756,9 @@
       <c r="Z160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AA160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -14362,6 +14845,9 @@
       <c r="Z161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AA161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -14448,6 +14934,9 @@
       <c r="Z162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AA162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -14534,6 +15023,9 @@
       <c r="Z163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AA163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -14620,9 +15112,12 @@
       <c r="Z164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AA164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z164"/>
+  <autoFilter ref="A1:AA164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AA$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AB$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA164"/>
+  <dimension ref="A1:AB164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -470,6 +470,7 @@
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -608,6 +609,11 @@
           <t>2026-09-07 04:49</t>
         </is>
       </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -697,6 +703,9 @@
       <c r="AA2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AB2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -786,6 +795,9 @@
       <c r="AA3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AB3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -875,6 +887,9 @@
       <c r="AA4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AB4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -964,6 +979,9 @@
       <c r="AA5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AB5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1053,6 +1071,9 @@
       <c r="AA6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AB6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1142,6 +1163,9 @@
       <c r="AA7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AB7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1231,6 +1255,9 @@
       <c r="AA8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="AB8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1320,6 +1347,9 @@
       <c r="AA9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AB9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1409,6 +1439,9 @@
       <c r="AA10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AB10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1498,6 +1531,9 @@
       <c r="AA11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AB11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1587,6 +1623,9 @@
       <c r="AA12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1676,6 +1715,9 @@
       <c r="AA13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AB13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1765,6 +1807,9 @@
       <c r="AA14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AB14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1854,6 +1899,9 @@
       <c r="AA15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AB15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1943,6 +1991,9 @@
       <c r="AA16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AB16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2032,6 +2083,9 @@
       <c r="AA17" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AB17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2121,6 +2175,9 @@
       <c r="AA18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AB18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2210,6 +2267,9 @@
       <c r="AA19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AB19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2299,6 +2359,9 @@
       <c r="AA20" s="3" t="n">
         <v>20.45</v>
       </c>
+      <c r="AB20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2388,6 +2451,9 @@
       <c r="AA21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AB21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2477,6 +2543,9 @@
       <c r="AA22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AB22" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2566,6 +2635,9 @@
       <c r="AA23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AB23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2655,6 +2727,9 @@
       <c r="AA24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AB24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2744,6 +2819,9 @@
       <c r="AA25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2833,6 +2911,9 @@
       <c r="AA26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AB26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2922,6 +3003,9 @@
       <c r="AA27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AB27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3011,6 +3095,9 @@
       <c r="AA28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AB28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3100,6 +3187,9 @@
       <c r="AA29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="AB29" s="3" t="n">
+        <v>20.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3189,6 +3279,9 @@
       <c r="AA30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AB30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3278,6 +3371,9 @@
       <c r="AA31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AB31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3367,6 +3463,9 @@
       <c r="AA32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AB32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3456,6 +3555,9 @@
       <c r="AA33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AB33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3545,6 +3647,9 @@
       <c r="AA34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="AB34" s="3" t="n">
+        <v>20.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3634,6 +3739,9 @@
       <c r="AA35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AB35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3723,6 +3831,9 @@
       <c r="AA36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AB36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3812,6 +3923,9 @@
       <c r="AA37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AB37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3901,6 +4015,9 @@
       <c r="AA38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AB38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3990,6 +4107,9 @@
       <c r="AA39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AB39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4079,6 +4199,9 @@
       <c r="AA40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4168,6 +4291,9 @@
       <c r="AA41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4257,6 +4383,9 @@
       <c r="AA42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4346,6 +4475,9 @@
       <c r="AA43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4435,6 +4567,9 @@
       <c r="AA44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4524,6 +4659,9 @@
       <c r="AA45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AB45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4613,6 +4751,9 @@
       <c r="AA46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AB46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4702,6 +4843,9 @@
       <c r="AA47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AB47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4791,6 +4935,9 @@
       <c r="AA48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AB48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4880,6 +5027,9 @@
       <c r="AA49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AB49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4969,6 +5119,9 @@
       <c r="AA50" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AB50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5058,6 +5211,9 @@
       <c r="AA51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AB51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5147,6 +5303,9 @@
       <c r="AA52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AB52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5236,6 +5395,9 @@
       <c r="AA53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AB53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5325,6 +5487,9 @@
       <c r="AA54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AB54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5414,6 +5579,9 @@
       <c r="AA55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AB55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5503,6 +5671,9 @@
       <c r="AA56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AB56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5592,6 +5763,9 @@
       <c r="AA57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5681,6 +5855,9 @@
       <c r="AA58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AB58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5770,6 +5947,9 @@
       <c r="AA59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AB59" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5859,6 +6039,9 @@
       <c r="AA60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AB60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5948,6 +6131,9 @@
       <c r="AA61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AB61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6037,6 +6223,9 @@
       <c r="AA62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AB62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -6126,6 +6315,9 @@
       <c r="AA63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AB63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6215,6 +6407,9 @@
       <c r="AA64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AB64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6304,6 +6499,9 @@
       <c r="AA65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6393,6 +6591,9 @@
       <c r="AA66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6482,6 +6683,9 @@
       <c r="AA67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6571,6 +6775,9 @@
       <c r="AA68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6660,6 +6867,9 @@
       <c r="AA69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6749,6 +6959,9 @@
       <c r="AA70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6838,6 +7051,9 @@
       <c r="AA71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6927,6 +7143,9 @@
       <c r="AA72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -7016,6 +7235,9 @@
       <c r="AA73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -7105,6 +7327,9 @@
       <c r="AA74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7194,6 +7419,9 @@
       <c r="AA75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7283,6 +7511,9 @@
       <c r="AA76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7372,6 +7603,9 @@
       <c r="AA77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7461,6 +7695,9 @@
       <c r="AA78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7550,6 +7787,9 @@
       <c r="AA79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7639,6 +7879,9 @@
       <c r="AA80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7728,6 +7971,9 @@
       <c r="AA81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7817,6 +8063,9 @@
       <c r="AA82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7906,6 +8155,9 @@
       <c r="AA83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7995,6 +8247,9 @@
       <c r="AA84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -8084,6 +8339,9 @@
       <c r="AA85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AB85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8173,6 +8431,9 @@
       <c r="AA86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8262,6 +8523,9 @@
       <c r="AA87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8351,6 +8615,9 @@
       <c r="AA88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8440,6 +8707,9 @@
       <c r="AA89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8529,6 +8799,9 @@
       <c r="AA90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8618,6 +8891,9 @@
       <c r="AA91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8707,6 +8983,9 @@
       <c r="AA92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8796,6 +9075,9 @@
       <c r="AA93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AB93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8885,6 +9167,9 @@
       <c r="AA94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB94" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8974,6 +9259,9 @@
       <c r="AA95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AB95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -9063,6 +9351,9 @@
       <c r="AA96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AB96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -9152,6 +9443,9 @@
       <c r="AA97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AB97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -9241,6 +9535,9 @@
       <c r="AA98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AB98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9330,6 +9627,9 @@
       <c r="AA99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9419,6 +9719,9 @@
       <c r="AA100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AB100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9508,6 +9811,9 @@
       <c r="AA101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AB101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9597,6 +9903,9 @@
       <c r="AA102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AB102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9686,6 +9995,9 @@
       <c r="AA103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AB103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9775,6 +10087,9 @@
       <c r="AA104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AB104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9864,6 +10179,9 @@
       <c r="AA105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AB105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9953,6 +10271,9 @@
       <c r="AA106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AB106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -10042,6 +10363,9 @@
       <c r="AA107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AB107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -10131,6 +10455,9 @@
       <c r="AA108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10220,6 +10547,9 @@
       <c r="AA109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AB109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -10309,6 +10639,9 @@
       <c r="AA110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AB110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10398,6 +10731,9 @@
       <c r="AA111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AB111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10487,6 +10823,9 @@
       <c r="AA112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AB112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10576,6 +10915,9 @@
       <c r="AA113" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="AB113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10665,6 +11007,9 @@
       <c r="AA114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AB114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10754,6 +11099,9 @@
       <c r="AA115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AB115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10843,6 +11191,9 @@
       <c r="AA116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10932,6 +11283,9 @@
       <c r="AA117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -11021,6 +11375,9 @@
       <c r="AA118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -11110,6 +11467,9 @@
       <c r="AA119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -11199,6 +11559,9 @@
       <c r="AA120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -11288,6 +11651,9 @@
       <c r="AA121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AB121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11377,6 +11743,9 @@
       <c r="AA122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AB122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11466,6 +11835,9 @@
       <c r="AA123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AB123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11555,6 +11927,9 @@
       <c r="AA124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AB124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11644,6 +12019,9 @@
       <c r="AA125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AB125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11733,6 +12111,9 @@
       <c r="AA126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AB126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11822,6 +12203,9 @@
       <c r="AA127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AB127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11911,6 +12295,9 @@
       <c r="AA128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AB128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -12000,6 +12387,9 @@
       <c r="AA129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AB129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -12089,6 +12479,9 @@
       <c r="AA130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AB130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -12178,6 +12571,9 @@
       <c r="AA131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AB131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -12267,6 +12663,9 @@
       <c r="AA132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AB132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -12356,6 +12755,9 @@
       <c r="AA133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AB133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -12445,6 +12847,9 @@
       <c r="AA134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AB134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12534,6 +12939,9 @@
       <c r="AA135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AB135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -12623,6 +13031,9 @@
       <c r="AA136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AB136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12712,6 +13123,9 @@
       <c r="AA137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AB137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -12801,6 +13215,9 @@
       <c r="AA138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AB138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12890,6 +13307,9 @@
       <c r="AA139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12979,6 +13399,9 @@
       <c r="AA140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -13068,6 +13491,9 @@
       <c r="AA141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -13157,6 +13583,9 @@
       <c r="AA142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -13246,6 +13675,9 @@
       <c r="AA143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -13335,6 +13767,9 @@
       <c r="AA144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AB144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -13424,6 +13859,9 @@
       <c r="AA145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AB145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -13513,6 +13951,9 @@
       <c r="AA146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AB146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -13602,6 +14043,9 @@
       <c r="AA147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AB147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -13691,6 +14135,9 @@
       <c r="AA148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AB148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -13780,6 +14227,9 @@
       <c r="AA149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AB149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -13869,6 +14319,9 @@
       <c r="AA150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AB150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -13958,6 +14411,9 @@
       <c r="AA151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AB151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -14047,6 +14503,9 @@
       <c r="AA152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AB152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -14136,6 +14595,9 @@
       <c r="AA153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AB153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -14225,6 +14687,9 @@
       <c r="AA154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AB154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -14314,6 +14779,9 @@
       <c r="AA155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AB155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -14403,6 +14871,9 @@
       <c r="AA156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AB156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -14492,6 +14963,9 @@
       <c r="AA157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AB157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -14581,6 +15055,9 @@
       <c r="AA158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AB158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -14670,6 +15147,9 @@
       <c r="AA159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AB159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -14759,6 +15239,9 @@
       <c r="AA160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AB160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -14848,6 +15331,9 @@
       <c r="AA161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AB161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -14937,6 +15423,9 @@
       <c r="AA162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AB162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -15026,6 +15515,9 @@
       <c r="AA163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AB163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -15115,9 +15607,12 @@
       <c r="AA164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AB164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA164"/>
+  <autoFilter ref="A1:AB164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AB$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AC$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB164"/>
+  <dimension ref="A1:AC164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,7 @@
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,6 +615,11 @@
           <t>2026-09-07 10:09</t>
         </is>
       </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -706,6 +712,9 @@
       <c r="AB2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AC2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -798,6 +807,9 @@
       <c r="AB3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AC3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -890,6 +902,9 @@
       <c r="AB4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AC4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -982,6 +997,9 @@
       <c r="AB5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AC5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1074,6 +1092,9 @@
       <c r="AB6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AC6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1166,6 +1187,9 @@
       <c r="AB7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AC7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1258,6 +1282,9 @@
       <c r="AB8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="AC8" s="3" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1350,6 +1377,9 @@
       <c r="AB9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AC9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1442,6 +1472,9 @@
       <c r="AB10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AC10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1534,6 +1567,9 @@
       <c r="AB11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AC11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1626,6 +1662,9 @@
       <c r="AB12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1718,6 +1757,9 @@
       <c r="AB13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AC13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1810,6 +1852,9 @@
       <c r="AB14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AC14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1902,6 +1947,9 @@
       <c r="AB15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AC15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1994,6 +2042,9 @@
       <c r="AB16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AC16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2086,6 +2137,9 @@
       <c r="AB17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AC17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2178,6 +2232,9 @@
       <c r="AB18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AC18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2270,6 +2327,9 @@
       <c r="AB19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AC19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2362,6 +2422,9 @@
       <c r="AB20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AC20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2454,6 +2517,9 @@
       <c r="AB21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AC21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2546,6 +2612,9 @@
       <c r="AB22" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AC22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2638,6 +2707,9 @@
       <c r="AB23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AC23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2730,6 +2802,9 @@
       <c r="AB24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AC24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2822,6 +2897,9 @@
       <c r="AB25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2914,6 +2992,9 @@
       <c r="AB26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AC26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3006,6 +3087,9 @@
       <c r="AB27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AC27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3098,6 +3182,9 @@
       <c r="AB28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AC28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3190,6 +3277,9 @@
       <c r="AB29" s="3" t="n">
         <v>20.55</v>
       </c>
+      <c r="AC29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3282,6 +3372,9 @@
       <c r="AB30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AC30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3374,6 +3467,9 @@
       <c r="AB31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AC31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3466,6 +3562,9 @@
       <c r="AB32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AC32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3558,6 +3657,9 @@
       <c r="AB33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AC33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3650,6 +3752,9 @@
       <c r="AB34" s="3" t="n">
         <v>20.66</v>
       </c>
+      <c r="AC34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3742,6 +3847,9 @@
       <c r="AB35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AC35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3834,6 +3942,9 @@
       <c r="AB36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AC36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3926,6 +4037,9 @@
       <c r="AB37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AC37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4018,6 +4132,9 @@
       <c r="AB38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AC38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4110,6 +4227,9 @@
       <c r="AB39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AC39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4202,6 +4322,9 @@
       <c r="AB40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4294,6 +4417,9 @@
       <c r="AB41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4386,6 +4512,9 @@
       <c r="AB42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4478,6 +4607,9 @@
       <c r="AB43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4570,6 +4702,9 @@
       <c r="AB44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4662,6 +4797,9 @@
       <c r="AB45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AC45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4754,6 +4892,9 @@
       <c r="AB46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AC46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4846,6 +4987,9 @@
       <c r="AB47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AC47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4938,6 +5082,9 @@
       <c r="AB48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AC48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5030,6 +5177,9 @@
       <c r="AB49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AC49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5122,6 +5272,9 @@
       <c r="AB50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AC50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5214,6 +5367,9 @@
       <c r="AB51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AC51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5306,6 +5462,9 @@
       <c r="AB52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AC52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5398,6 +5557,9 @@
       <c r="AB53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AC53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5490,6 +5652,9 @@
       <c r="AB54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AC54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5582,6 +5747,9 @@
       <c r="AB55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AC55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5674,6 +5842,9 @@
       <c r="AB56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AC56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5766,6 +5937,9 @@
       <c r="AB57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5858,6 +6032,9 @@
       <c r="AB58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AC58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5950,6 +6127,9 @@
       <c r="AB59" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AC59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6042,6 +6222,9 @@
       <c r="AB60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AC60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -6134,6 +6317,9 @@
       <c r="AB61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AC61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6226,6 +6412,9 @@
       <c r="AB62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AC62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -6318,6 +6507,9 @@
       <c r="AB63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AC63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6410,6 +6602,9 @@
       <c r="AB64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AC64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6502,6 +6697,9 @@
       <c r="AB65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6594,6 +6792,9 @@
       <c r="AB66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6686,6 +6887,9 @@
       <c r="AB67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6778,6 +6982,9 @@
       <c r="AB68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6870,6 +7077,9 @@
       <c r="AB69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6962,6 +7172,9 @@
       <c r="AB70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -7054,6 +7267,9 @@
       <c r="AB71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -7146,6 +7362,9 @@
       <c r="AB72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -7238,6 +7457,9 @@
       <c r="AB73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -7330,6 +7552,9 @@
       <c r="AB74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7422,6 +7647,9 @@
       <c r="AB75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7514,6 +7742,9 @@
       <c r="AB76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7606,6 +7837,9 @@
       <c r="AB77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7698,6 +7932,9 @@
       <c r="AB78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7790,6 +8027,9 @@
       <c r="AB79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7882,6 +8122,9 @@
       <c r="AB80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7974,6 +8217,9 @@
       <c r="AB81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -8066,6 +8312,9 @@
       <c r="AB82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8158,6 +8407,9 @@
       <c r="AB83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -8250,6 +8502,9 @@
       <c r="AB84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -8342,6 +8597,9 @@
       <c r="AB85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AC85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8434,6 +8692,9 @@
       <c r="AB86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8526,6 +8787,9 @@
       <c r="AB87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8618,6 +8882,9 @@
       <c r="AB88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8710,6 +8977,9 @@
       <c r="AB89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8802,6 +9072,9 @@
       <c r="AB90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8894,6 +9167,9 @@
       <c r="AB91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8986,6 +9262,9 @@
       <c r="AB92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -9078,6 +9357,9 @@
       <c r="AB93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AC93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -9170,6 +9452,9 @@
       <c r="AB94" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -9262,6 +9547,9 @@
       <c r="AB95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AC95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -9354,6 +9642,9 @@
       <c r="AB96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AC96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -9446,6 +9737,9 @@
       <c r="AB97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AC97" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -9538,6 +9832,9 @@
       <c r="AB98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AC98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9630,6 +9927,9 @@
       <c r="AB99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9722,6 +10022,9 @@
       <c r="AB100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AC100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9814,6 +10117,9 @@
       <c r="AB101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AC101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9906,6 +10212,9 @@
       <c r="AB102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AC102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9998,6 +10307,9 @@
       <c r="AB103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AC103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -10090,6 +10402,9 @@
       <c r="AB104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AC104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -10182,6 +10497,9 @@
       <c r="AB105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AC105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -10274,6 +10592,9 @@
       <c r="AB106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AC106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -10366,6 +10687,9 @@
       <c r="AB107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AC107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -10458,6 +10782,9 @@
       <c r="AB108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10550,6 +10877,9 @@
       <c r="AB109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AC109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -10642,6 +10972,9 @@
       <c r="AB110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AC110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10734,6 +11067,9 @@
       <c r="AB111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AC111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10826,6 +11162,9 @@
       <c r="AB112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AC112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10918,6 +11257,9 @@
       <c r="AB113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AC113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -11010,6 +11352,9 @@
       <c r="AB114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AC114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -11102,6 +11447,9 @@
       <c r="AB115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AC115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -11194,6 +11542,9 @@
       <c r="AB116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -11286,6 +11637,9 @@
       <c r="AB117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -11378,6 +11732,9 @@
       <c r="AB118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -11470,6 +11827,9 @@
       <c r="AB119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -11562,6 +11922,9 @@
       <c r="AB120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -11654,6 +12017,9 @@
       <c r="AB121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AC121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11746,6 +12112,9 @@
       <c r="AB122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AC122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11838,6 +12207,9 @@
       <c r="AB123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AC123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11930,6 +12302,9 @@
       <c r="AB124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AC124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -12022,6 +12397,9 @@
       <c r="AB125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AC125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -12114,6 +12492,9 @@
       <c r="AB126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AC126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -12206,6 +12587,9 @@
       <c r="AB127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AC127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -12298,6 +12682,9 @@
       <c r="AB128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AC128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -12390,6 +12777,9 @@
       <c r="AB129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AC129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -12482,6 +12872,9 @@
       <c r="AB130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AC130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -12574,6 +12967,9 @@
       <c r="AB131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AC131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -12666,6 +13062,9 @@
       <c r="AB132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AC132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -12758,6 +13157,9 @@
       <c r="AB133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AC133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -12850,6 +13252,9 @@
       <c r="AB134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AC134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12942,6 +13347,9 @@
       <c r="AB135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AC135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -13034,6 +13442,9 @@
       <c r="AB136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AC136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -13126,6 +13537,9 @@
       <c r="AB137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AC137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -13218,6 +13632,9 @@
       <c r="AB138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AC138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -13310,6 +13727,9 @@
       <c r="AB139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -13402,6 +13822,9 @@
       <c r="AB140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -13494,6 +13917,9 @@
       <c r="AB141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -13586,6 +14012,9 @@
       <c r="AB142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -13678,6 +14107,9 @@
       <c r="AB143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -13770,6 +14202,9 @@
       <c r="AB144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AC144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -13862,6 +14297,9 @@
       <c r="AB145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AC145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -13954,6 +14392,9 @@
       <c r="AB146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AC146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -14046,6 +14487,9 @@
       <c r="AB147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AC147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -14138,6 +14582,9 @@
       <c r="AB148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AC148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -14230,6 +14677,9 @@
       <c r="AB149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AC149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -14322,6 +14772,9 @@
       <c r="AB150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AC150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -14414,6 +14867,9 @@
       <c r="AB151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AC151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -14506,6 +14962,9 @@
       <c r="AB152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AC152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -14598,6 +15057,9 @@
       <c r="AB153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AC153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -14690,6 +15152,9 @@
       <c r="AB154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AC154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -14782,6 +15247,9 @@
       <c r="AB155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AC155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -14874,6 +15342,9 @@
       <c r="AB156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AC156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -14966,6 +15437,9 @@
       <c r="AB157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AC157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -15058,6 +15532,9 @@
       <c r="AB158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AC158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -15150,6 +15627,9 @@
       <c r="AB159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AC159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -15242,6 +15722,9 @@
       <c r="AB160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AC160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -15334,6 +15817,9 @@
       <c r="AB161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AC161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -15426,6 +15912,9 @@
       <c r="AB162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AC162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -15518,6 +16007,9 @@
       <c r="AB163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AC163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -15610,9 +16102,12 @@
       <c r="AB164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AC164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB164"/>
+  <autoFilter ref="A1:AC164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-07 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AC$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AD$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC164"/>
+  <dimension ref="A1:AD164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -472,6 +472,7 @@
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="16" customWidth="1" min="28" max="28"/>
     <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -620,6 +621,11 @@
           <t>2026-09-07 13:11</t>
         </is>
       </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 16:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -715,6 +721,9 @@
       <c r="AC2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AD2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -810,6 +819,9 @@
       <c r="AC3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AD3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -905,6 +917,9 @@
       <c r="AC4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AD4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1000,6 +1015,9 @@
       <c r="AC5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AD5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1095,6 +1113,9 @@
       <c r="AC6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AD6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1190,6 +1211,9 @@
       <c r="AC7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AD7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1285,6 +1309,9 @@
       <c r="AC8" s="3" t="n">
         <v>19.99</v>
       </c>
+      <c r="AD8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1380,6 +1407,9 @@
       <c r="AC9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AD9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1475,6 +1505,9 @@
       <c r="AC10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AD10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1570,6 +1603,9 @@
       <c r="AC11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AD11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1665,6 +1701,9 @@
       <c r="AC12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1760,6 +1799,9 @@
       <c r="AC13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AD13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1855,6 +1897,9 @@
       <c r="AC14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AD14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1950,6 +1995,9 @@
       <c r="AC15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AD15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2045,6 +2093,9 @@
       <c r="AC16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AD16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2140,6 +2191,9 @@
       <c r="AC17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AD17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2235,6 +2289,9 @@
       <c r="AC18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AD18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2330,6 +2387,9 @@
       <c r="AC19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AD19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2425,6 +2485,9 @@
       <c r="AC20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AD20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2520,6 +2583,9 @@
       <c r="AC21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AD21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2615,6 +2681,9 @@
       <c r="AC22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AD22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2710,6 +2779,9 @@
       <c r="AC23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AD23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2805,6 +2877,9 @@
       <c r="AC24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AD24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2900,6 +2975,9 @@
       <c r="AC25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2995,6 +3073,9 @@
       <c r="AC26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AD26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3090,6 +3171,9 @@
       <c r="AC27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AD27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3185,6 +3269,9 @@
       <c r="AC28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AD28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3280,6 +3367,9 @@
       <c r="AC29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AD29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3375,6 +3465,9 @@
       <c r="AC30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AD30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3470,6 +3563,9 @@
       <c r="AC31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AD31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3565,6 +3661,9 @@
       <c r="AC32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AD32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3660,6 +3759,9 @@
       <c r="AC33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AD33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3755,6 +3857,9 @@
       <c r="AC34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AD34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3850,6 +3955,9 @@
       <c r="AC35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AD35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3945,6 +4053,9 @@
       <c r="AC36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AD36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4040,6 +4151,9 @@
       <c r="AC37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AD37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4135,6 +4249,9 @@
       <c r="AC38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AD38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4230,6 +4347,9 @@
       <c r="AC39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AD39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4325,6 +4445,9 @@
       <c r="AC40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4420,6 +4543,9 @@
       <c r="AC41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4515,6 +4641,9 @@
       <c r="AC42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4610,6 +4739,9 @@
       <c r="AC43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4705,6 +4837,9 @@
       <c r="AC44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4800,6 +4935,9 @@
       <c r="AC45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AD45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4895,6 +5033,9 @@
       <c r="AC46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AD46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4990,6 +5131,9 @@
       <c r="AC47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AD47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5085,6 +5229,9 @@
       <c r="AC48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AD48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5180,6 +5327,9 @@
       <c r="AC49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AD49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5275,6 +5425,9 @@
       <c r="AC50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AD50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5370,6 +5523,9 @@
       <c r="AC51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AD51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5465,6 +5621,9 @@
       <c r="AC52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AD52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5560,6 +5719,9 @@
       <c r="AC53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AD53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5655,6 +5817,9 @@
       <c r="AC54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AD54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5750,6 +5915,9 @@
       <c r="AC55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AD55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5845,6 +6013,9 @@
       <c r="AC56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AD56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5940,6 +6111,9 @@
       <c r="AC57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6035,6 +6209,9 @@
       <c r="AC58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AD58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6130,6 +6307,9 @@
       <c r="AC59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AD59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6225,6 +6405,9 @@
       <c r="AC60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AD60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -6320,6 +6503,9 @@
       <c r="AC61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AD61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6415,6 +6601,9 @@
       <c r="AC62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AD62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -6510,6 +6699,9 @@
       <c r="AC63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AD63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6605,6 +6797,9 @@
       <c r="AC64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AD64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6700,6 +6895,9 @@
       <c r="AC65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6795,6 +6993,9 @@
       <c r="AC66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6890,6 +7091,9 @@
       <c r="AC67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6985,6 +7189,9 @@
       <c r="AC68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -7080,6 +7287,9 @@
       <c r="AC69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -7175,6 +7385,9 @@
       <c r="AC70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -7270,6 +7483,9 @@
       <c r="AC71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -7365,6 +7581,9 @@
       <c r="AC72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -7460,6 +7679,9 @@
       <c r="AC73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -7555,6 +7777,9 @@
       <c r="AC74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7650,6 +7875,9 @@
       <c r="AC75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7745,6 +7973,9 @@
       <c r="AC76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7840,6 +8071,9 @@
       <c r="AC77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7935,6 +8169,9 @@
       <c r="AC78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8030,6 +8267,9 @@
       <c r="AC79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -8125,6 +8365,9 @@
       <c r="AC80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -8220,6 +8463,9 @@
       <c r="AC81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -8315,6 +8561,9 @@
       <c r="AC82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8410,6 +8659,9 @@
       <c r="AC83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -8505,6 +8757,9 @@
       <c r="AC84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -8600,6 +8855,9 @@
       <c r="AC85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AD85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8695,6 +8953,9 @@
       <c r="AC86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8790,6 +9051,9 @@
       <c r="AC87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8885,6 +9149,9 @@
       <c r="AC88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8980,6 +9247,9 @@
       <c r="AC89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -9075,6 +9345,9 @@
       <c r="AC90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -9170,6 +9443,9 @@
       <c r="AC91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -9265,6 +9541,9 @@
       <c r="AC92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -9360,6 +9639,9 @@
       <c r="AC93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AD93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -9455,6 +9737,9 @@
       <c r="AC94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AD94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -9550,6 +9835,9 @@
       <c r="AC95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AD95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -9645,6 +9933,9 @@
       <c r="AC96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AD96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -9740,6 +10031,9 @@
       <c r="AC97" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AD97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -9835,6 +10129,9 @@
       <c r="AC98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AD98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9930,6 +10227,9 @@
       <c r="AC99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -10025,6 +10325,9 @@
       <c r="AC100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AD100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -10120,6 +10423,9 @@
       <c r="AC101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AD101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -10215,6 +10521,9 @@
       <c r="AC102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AD102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -10310,6 +10619,9 @@
       <c r="AC103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AD103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -10405,6 +10717,9 @@
       <c r="AC104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AD104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -10500,6 +10815,9 @@
       <c r="AC105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AD105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -10595,6 +10913,9 @@
       <c r="AC106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AD106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -10690,6 +11011,9 @@
       <c r="AC107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AD107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -10785,6 +11109,9 @@
       <c r="AC108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10880,6 +11207,9 @@
       <c r="AC109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AD109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -10975,6 +11305,9 @@
       <c r="AC110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AD110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -11070,6 +11403,9 @@
       <c r="AC111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AD111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -11165,6 +11501,9 @@
       <c r="AC112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AD112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -11260,6 +11599,9 @@
       <c r="AC113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AD113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -11355,6 +11697,9 @@
       <c r="AC114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AD114" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -11450,6 +11795,9 @@
       <c r="AC115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AD115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -11545,6 +11893,9 @@
       <c r="AC116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -11640,6 +11991,9 @@
       <c r="AC117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -11735,6 +12089,9 @@
       <c r="AC118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -11830,6 +12187,9 @@
       <c r="AC119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -11925,6 +12285,9 @@
       <c r="AC120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -12020,6 +12383,9 @@
       <c r="AC121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AD121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -12115,6 +12481,9 @@
       <c r="AC122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AD122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -12210,6 +12579,9 @@
       <c r="AC123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AD123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -12305,6 +12677,9 @@
       <c r="AC124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AD124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -12400,6 +12775,9 @@
       <c r="AC125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AD125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -12495,6 +12873,9 @@
       <c r="AC126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AD126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -12590,6 +12971,9 @@
       <c r="AC127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AD127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -12685,6 +13069,9 @@
       <c r="AC128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AD128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -12780,6 +13167,9 @@
       <c r="AC129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AD129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -12875,6 +13265,9 @@
       <c r="AC130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AD130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -12970,6 +13363,9 @@
       <c r="AC131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AD131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -13065,6 +13461,9 @@
       <c r="AC132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AD132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -13160,6 +13559,9 @@
       <c r="AC133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AD133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -13255,6 +13657,9 @@
       <c r="AC134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AD134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -13350,6 +13755,9 @@
       <c r="AC135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AD135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -13445,6 +13853,9 @@
       <c r="AC136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AD136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -13540,6 +13951,9 @@
       <c r="AC137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AD137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -13635,6 +14049,9 @@
       <c r="AC138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AD138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -13730,6 +14147,9 @@
       <c r="AC139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -13825,6 +14245,9 @@
       <c r="AC140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -13920,6 +14343,9 @@
       <c r="AC141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -14015,6 +14441,9 @@
       <c r="AC142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -14110,6 +14539,9 @@
       <c r="AC143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -14205,6 +14637,9 @@
       <c r="AC144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AD144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -14300,6 +14735,9 @@
       <c r="AC145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AD145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -14395,6 +14833,9 @@
       <c r="AC146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AD146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -14490,6 +14931,9 @@
       <c r="AC147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AD147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -14585,6 +15029,9 @@
       <c r="AC148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AD148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -14680,6 +15127,9 @@
       <c r="AC149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AD149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -14775,6 +15225,9 @@
       <c r="AC150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AD150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -14870,6 +15323,9 @@
       <c r="AC151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AD151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -14965,6 +15421,9 @@
       <c r="AC152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AD152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -15060,6 +15519,9 @@
       <c r="AC153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AD153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -15155,6 +15617,9 @@
       <c r="AC154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AD154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -15250,6 +15715,9 @@
       <c r="AC155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AD155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -15345,6 +15813,9 @@
       <c r="AC156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AD156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -15440,6 +15911,9 @@
       <c r="AC157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AD157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -15535,6 +16009,9 @@
       <c r="AC158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AD158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -15630,6 +16107,9 @@
       <c r="AC159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AD159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -15725,6 +16205,9 @@
       <c r="AC160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AD160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -15820,6 +16303,9 @@
       <c r="AC161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AD161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -15915,6 +16401,9 @@
       <c r="AC162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AD162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -16010,6 +16499,9 @@
       <c r="AC163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AD163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -16105,9 +16597,12 @@
       <c r="AC164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AD164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC164"/>
+  <autoFilter ref="A1:AD164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 00:15 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AD$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AE$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD164"/>
+  <dimension ref="A1:AE164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,7 @@
     <col width="16" customWidth="1" min="28" max="28"/>
     <col width="16" customWidth="1" min="29" max="29"/>
     <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -626,6 +627,11 @@
           <t>2026-09-07 16:09</t>
         </is>
       </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 19:15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -724,6 +730,9 @@
       <c r="AD2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AE2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -822,6 +831,9 @@
       <c r="AD3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AE3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -920,6 +932,9 @@
       <c r="AD4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AE4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1018,6 +1033,9 @@
       <c r="AD5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AE5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1116,6 +1134,9 @@
       <c r="AD6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AE6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1214,6 +1235,9 @@
       <c r="AD7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AE7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1312,6 +1336,9 @@
       <c r="AD8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AE8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1410,6 +1437,9 @@
       <c r="AD9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AE9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1508,6 +1538,9 @@
       <c r="AD10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AE10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1606,6 +1639,9 @@
       <c r="AD11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AE11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1704,6 +1740,9 @@
       <c r="AD12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1802,6 +1841,9 @@
       <c r="AD13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AE13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1900,6 +1942,9 @@
       <c r="AD14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AE14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1998,6 +2043,9 @@
       <c r="AD15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AE15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2096,6 +2144,9 @@
       <c r="AD16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AE16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2194,6 +2245,9 @@
       <c r="AD17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AE17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2292,6 +2346,9 @@
       <c r="AD18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AE18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2390,6 +2447,9 @@
       <c r="AD19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AE19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2488,6 +2548,9 @@
       <c r="AD20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AE20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2586,6 +2649,9 @@
       <c r="AD21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AE21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2684,6 +2750,9 @@
       <c r="AD22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AE22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2782,6 +2851,9 @@
       <c r="AD23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AE23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2880,6 +2952,9 @@
       <c r="AD24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AE24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2978,6 +3053,9 @@
       <c r="AD25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3076,6 +3154,9 @@
       <c r="AD26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AE26" s="3" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3174,6 +3255,9 @@
       <c r="AD27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AE27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3272,6 +3356,9 @@
       <c r="AD28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AE28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3370,6 +3457,9 @@
       <c r="AD29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AE29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3468,6 +3558,9 @@
       <c r="AD30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AE30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3566,6 +3659,9 @@
       <c r="AD31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AE31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3664,6 +3760,9 @@
       <c r="AD32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AE32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3762,6 +3861,9 @@
       <c r="AD33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AE33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3860,6 +3962,9 @@
       <c r="AD34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AE34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3958,6 +4063,9 @@
       <c r="AD35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AE35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4056,6 +4164,9 @@
       <c r="AD36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AE36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4154,6 +4265,9 @@
       <c r="AD37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AE37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4252,6 +4366,9 @@
       <c r="AD38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AE38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4350,6 +4467,9 @@
       <c r="AD39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AE39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4448,6 +4568,9 @@
       <c r="AD40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4546,6 +4669,9 @@
       <c r="AD41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4644,6 +4770,9 @@
       <c r="AD42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4742,6 +4871,9 @@
       <c r="AD43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4840,6 +4972,9 @@
       <c r="AD44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4938,6 +5073,9 @@
       <c r="AD45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AE45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5036,6 +5174,9 @@
       <c r="AD46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AE46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5134,6 +5275,9 @@
       <c r="AD47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AE47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5232,6 +5376,9 @@
       <c r="AD48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AE48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5330,6 +5477,9 @@
       <c r="AD49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AE49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5428,6 +5578,9 @@
       <c r="AD50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AE50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5526,6 +5679,9 @@
       <c r="AD51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AE51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5624,6 +5780,9 @@
       <c r="AD52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AE52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5722,6 +5881,9 @@
       <c r="AD53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AE53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5820,6 +5982,9 @@
       <c r="AD54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AE54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5918,6 +6083,9 @@
       <c r="AD55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AE55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6016,6 +6184,9 @@
       <c r="AD56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AE56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6114,6 +6285,9 @@
       <c r="AD57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6212,6 +6386,9 @@
       <c r="AD58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AE58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6310,6 +6487,9 @@
       <c r="AD59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AE59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6408,6 +6588,9 @@
       <c r="AD60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AE60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -6506,6 +6689,9 @@
       <c r="AD61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AE61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6604,6 +6790,9 @@
       <c r="AD62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AE62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -6702,6 +6891,9 @@
       <c r="AD63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AE63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6800,6 +6992,9 @@
       <c r="AD64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AE64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6898,6 +7093,9 @@
       <c r="AD65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6996,6 +7194,9 @@
       <c r="AD66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7094,6 +7295,9 @@
       <c r="AD67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7192,6 +7396,9 @@
       <c r="AD68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -7290,6 +7497,9 @@
       <c r="AD69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -7388,6 +7598,9 @@
       <c r="AD70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -7486,6 +7699,9 @@
       <c r="AD71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -7584,6 +7800,9 @@
       <c r="AD72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -7682,6 +7901,9 @@
       <c r="AD73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -7780,6 +8002,9 @@
       <c r="AD74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7878,6 +8103,9 @@
       <c r="AD75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7976,6 +8204,9 @@
       <c r="AD76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -8074,6 +8305,9 @@
       <c r="AD77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -8172,6 +8406,9 @@
       <c r="AD78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8270,6 +8507,9 @@
       <c r="AD79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -8368,6 +8608,9 @@
       <c r="AD80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -8466,6 +8709,9 @@
       <c r="AD81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -8564,6 +8810,9 @@
       <c r="AD82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8662,6 +8911,9 @@
       <c r="AD83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -8760,6 +9012,9 @@
       <c r="AD84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -8858,6 +9113,9 @@
       <c r="AD85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AE85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8956,6 +9214,9 @@
       <c r="AD86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9054,6 +9315,9 @@
       <c r="AD87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9152,6 +9416,9 @@
       <c r="AD88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -9250,6 +9517,9 @@
       <c r="AD89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -9348,6 +9618,9 @@
       <c r="AD90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -9446,6 +9719,9 @@
       <c r="AD91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -9544,6 +9820,9 @@
       <c r="AD92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -9642,6 +9921,9 @@
       <c r="AD93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AE93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -9740,6 +10022,9 @@
       <c r="AD94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AE94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -9838,6 +10123,9 @@
       <c r="AD95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AE95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -9936,6 +10224,9 @@
       <c r="AD96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AE96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -10034,6 +10325,9 @@
       <c r="AD97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AE97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -10132,6 +10426,9 @@
       <c r="AD98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AE98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -10230,6 +10527,9 @@
       <c r="AD99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -10328,6 +10628,9 @@
       <c r="AD100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AE100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -10426,6 +10729,9 @@
       <c r="AD101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AE101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -10524,6 +10830,9 @@
       <c r="AD102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AE102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -10622,6 +10931,9 @@
       <c r="AD103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AE103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -10720,6 +11032,9 @@
       <c r="AD104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AE104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -10818,6 +11133,9 @@
       <c r="AD105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AE105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -10916,6 +11234,9 @@
       <c r="AD106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AE106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -11014,6 +11335,9 @@
       <c r="AD107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AE107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -11112,6 +11436,9 @@
       <c r="AD108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -11210,6 +11537,9 @@
       <c r="AD109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AE109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -11308,6 +11638,9 @@
       <c r="AD110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AE110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -11406,6 +11739,9 @@
       <c r="AD111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AE111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -11504,6 +11840,9 @@
       <c r="AD112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AE112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -11602,6 +11941,9 @@
       <c r="AD113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AE113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -11700,6 +12042,9 @@
       <c r="AD114" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AE114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -11798,6 +12143,9 @@
       <c r="AD115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AE115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -11896,6 +12244,9 @@
       <c r="AD116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -11994,6 +12345,9 @@
       <c r="AD117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -12092,6 +12446,9 @@
       <c r="AD118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -12190,6 +12547,9 @@
       <c r="AD119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -12288,6 +12648,9 @@
       <c r="AD120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -12386,6 +12749,9 @@
       <c r="AD121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AE121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -12484,6 +12850,9 @@
       <c r="AD122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AE122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -12582,6 +12951,9 @@
       <c r="AD123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AE123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -12680,6 +13052,9 @@
       <c r="AD124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AE124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -12778,6 +13153,9 @@
       <c r="AD125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AE125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -12876,6 +13254,9 @@
       <c r="AD126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AE126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -12974,6 +13355,9 @@
       <c r="AD127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AE127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -13072,6 +13456,9 @@
       <c r="AD128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AE128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -13170,6 +13557,9 @@
       <c r="AD129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AE129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -13268,6 +13658,9 @@
       <c r="AD130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AE130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -13366,6 +13759,9 @@
       <c r="AD131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AE131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -13464,6 +13860,9 @@
       <c r="AD132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AE132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -13562,6 +13961,9 @@
       <c r="AD133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AE133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -13660,6 +14062,9 @@
       <c r="AD134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AE134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -13758,6 +14163,9 @@
       <c r="AD135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AE135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -13856,6 +14264,9 @@
       <c r="AD136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AE136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -13954,6 +14365,9 @@
       <c r="AD137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AE137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -14052,6 +14466,9 @@
       <c r="AD138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AE138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -14150,6 +14567,9 @@
       <c r="AD139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -14248,6 +14668,9 @@
       <c r="AD140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -14346,6 +14769,9 @@
       <c r="AD141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -14444,6 +14870,9 @@
       <c r="AD142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -14542,6 +14971,9 @@
       <c r="AD143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -14640,6 +15072,9 @@
       <c r="AD144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AE144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -14738,6 +15173,9 @@
       <c r="AD145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AE145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -14836,6 +15274,9 @@
       <c r="AD146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AE146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -14934,6 +15375,9 @@
       <c r="AD147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AE147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -15032,6 +15476,9 @@
       <c r="AD148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AE148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -15130,6 +15577,9 @@
       <c r="AD149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AE149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -15228,6 +15678,9 @@
       <c r="AD150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AE150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -15326,6 +15779,9 @@
       <c r="AD151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AE151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -15424,6 +15880,9 @@
       <c r="AD152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AE152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -15522,6 +15981,9 @@
       <c r="AD153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AE153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -15620,6 +16082,9 @@
       <c r="AD154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AE154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -15718,6 +16183,9 @@
       <c r="AD155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AE155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -15816,6 +16284,9 @@
       <c r="AD156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AE156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -15914,6 +16385,9 @@
       <c r="AD157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AE157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -16012,6 +16486,9 @@
       <c r="AD158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AE158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -16110,6 +16587,9 @@
       <c r="AD159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AE159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -16208,6 +16688,9 @@
       <c r="AD160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AE160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -16306,6 +16789,9 @@
       <c r="AD161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AE161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -16404,6 +16890,9 @@
       <c r="AD162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AE162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -16502,6 +16991,9 @@
       <c r="AD163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AE163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -16600,9 +17092,12 @@
       <c r="AD164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AE164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD164"/>
+  <autoFilter ref="A1:AE164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AE$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AF$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE164"/>
+  <dimension ref="A1:AF164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,7 @@
     <col width="16" customWidth="1" min="29" max="29"/>
     <col width="16" customWidth="1" min="30" max="30"/>
     <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,6 +633,11 @@
           <t>2026-09-07 19:15</t>
         </is>
       </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -733,6 +739,9 @@
       <c r="AE2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AF2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -834,6 +843,9 @@
       <c r="AE3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AF3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -935,6 +947,9 @@
       <c r="AE4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AF4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1036,6 +1051,9 @@
       <c r="AE5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AF5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1137,6 +1155,9 @@
       <c r="AE6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AF6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1238,6 +1259,9 @@
       <c r="AE7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AF7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1339,6 +1363,9 @@
       <c r="AE8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AF8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1440,6 +1467,9 @@
       <c r="AE9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AF9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1541,6 +1571,9 @@
       <c r="AE10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AF10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1642,6 +1675,9 @@
       <c r="AE11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AF11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1743,6 +1779,9 @@
       <c r="AE12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1844,6 +1883,9 @@
       <c r="AE13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AF13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1945,6 +1987,9 @@
       <c r="AE14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AF14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2046,6 +2091,9 @@
       <c r="AE15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AF15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2147,6 +2195,9 @@
       <c r="AE16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AF16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2248,6 +2299,9 @@
       <c r="AE17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AF17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2349,6 +2403,9 @@
       <c r="AE18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AF18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2450,6 +2507,9 @@
       <c r="AE19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AF19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2551,6 +2611,9 @@
       <c r="AE20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AF20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2652,6 +2715,9 @@
       <c r="AE21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AF21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2753,6 +2819,9 @@
       <c r="AE22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AF22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2854,6 +2923,9 @@
       <c r="AE23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AF23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2955,6 +3027,9 @@
       <c r="AE24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AF24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3056,6 +3131,9 @@
       <c r="AE25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3157,6 +3235,9 @@
       <c r="AE26" s="3" t="n">
         <v>20.5</v>
       </c>
+      <c r="AF26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3258,6 +3339,9 @@
       <c r="AE27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AF27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3359,6 +3443,9 @@
       <c r="AE28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AF28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3460,6 +3547,9 @@
       <c r="AE29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AF29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3561,6 +3651,9 @@
       <c r="AE30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AF30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3662,6 +3755,9 @@
       <c r="AE31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AF31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3763,6 +3859,9 @@
       <c r="AE32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AF32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3864,6 +3963,9 @@
       <c r="AE33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AF33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3965,6 +4067,9 @@
       <c r="AE34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AF34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4066,6 +4171,9 @@
       <c r="AE35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AF35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4167,6 +4275,9 @@
       <c r="AE36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AF36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4268,6 +4379,9 @@
       <c r="AE37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AF37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4369,6 +4483,9 @@
       <c r="AE38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AF38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4470,6 +4587,9 @@
       <c r="AE39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AF39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4571,6 +4691,9 @@
       <c r="AE40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4672,6 +4795,9 @@
       <c r="AE41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4773,6 +4899,9 @@
       <c r="AE42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4874,6 +5003,9 @@
       <c r="AE43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4975,6 +5107,9 @@
       <c r="AE44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5076,6 +5211,9 @@
       <c r="AE45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AF45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5177,6 +5315,9 @@
       <c r="AE46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AF46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5278,6 +5419,9 @@
       <c r="AE47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AF47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5379,6 +5523,9 @@
       <c r="AE48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AF48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5480,6 +5627,9 @@
       <c r="AE49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AF49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5581,6 +5731,9 @@
       <c r="AE50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AF50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5682,6 +5835,9 @@
       <c r="AE51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AF51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5783,6 +5939,9 @@
       <c r="AE52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AF52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5884,6 +6043,9 @@
       <c r="AE53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AF53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5985,6 +6147,9 @@
       <c r="AE54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AF54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6086,6 +6251,9 @@
       <c r="AE55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AF55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6187,6 +6355,9 @@
       <c r="AE56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AF56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6288,6 +6459,9 @@
       <c r="AE57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6389,6 +6563,9 @@
       <c r="AE58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AF58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6490,6 +6667,9 @@
       <c r="AE59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AF59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6591,6 +6771,9 @@
       <c r="AE60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AF60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -6692,6 +6875,9 @@
       <c r="AE61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AF61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6793,6 +6979,9 @@
       <c r="AE62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AF62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -6894,6 +7083,9 @@
       <c r="AE63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AF63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6995,6 +7187,9 @@
       <c r="AE64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AF64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7096,6 +7291,9 @@
       <c r="AE65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7197,6 +7395,9 @@
       <c r="AE66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7298,6 +7499,9 @@
       <c r="AE67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7399,6 +7603,9 @@
       <c r="AE68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -7500,6 +7707,9 @@
       <c r="AE69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -7601,6 +7811,9 @@
       <c r="AE70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -7702,6 +7915,9 @@
       <c r="AE71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -7803,6 +8019,9 @@
       <c r="AE72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -7904,6 +8123,9 @@
       <c r="AE73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8005,6 +8227,9 @@
       <c r="AE74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8106,6 +8331,9 @@
       <c r="AE75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8207,6 +8435,9 @@
       <c r="AE76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -8308,6 +8539,9 @@
       <c r="AE77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -8409,6 +8643,9 @@
       <c r="AE78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8510,6 +8747,9 @@
       <c r="AE79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -8611,6 +8851,9 @@
       <c r="AE80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -8712,6 +8955,9 @@
       <c r="AE81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -8813,6 +9059,9 @@
       <c r="AE82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8914,6 +9163,9 @@
       <c r="AE83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9015,6 +9267,9 @@
       <c r="AE84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -9116,6 +9371,9 @@
       <c r="AE85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AF85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -9217,6 +9475,9 @@
       <c r="AE86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9318,6 +9579,9 @@
       <c r="AE87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9419,6 +9683,9 @@
       <c r="AE88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -9520,6 +9787,9 @@
       <c r="AE89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -9621,6 +9891,9 @@
       <c r="AE90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -9722,6 +9995,9 @@
       <c r="AE91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -9823,6 +10099,9 @@
       <c r="AE92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -9924,6 +10203,9 @@
       <c r="AE93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AF93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -10025,6 +10307,9 @@
       <c r="AE94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AF94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -10126,6 +10411,9 @@
       <c r="AE95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AF95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -10227,6 +10515,9 @@
       <c r="AE96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AF96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -10328,6 +10619,9 @@
       <c r="AE97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AF97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -10429,6 +10723,9 @@
       <c r="AE98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AF98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -10530,6 +10827,9 @@
       <c r="AE99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -10631,6 +10931,9 @@
       <c r="AE100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AF100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -10732,6 +11035,9 @@
       <c r="AE101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AF101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -10833,6 +11139,9 @@
       <c r="AE102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AF102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -10934,6 +11243,9 @@
       <c r="AE103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AF103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -11035,6 +11347,9 @@
       <c r="AE104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AF104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -11136,6 +11451,9 @@
       <c r="AE105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AF105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -11237,6 +11555,9 @@
       <c r="AE106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AF106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -11338,6 +11659,9 @@
       <c r="AE107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AF107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -11439,6 +11763,9 @@
       <c r="AE108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -11540,6 +11867,9 @@
       <c r="AE109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AF109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -11641,6 +11971,9 @@
       <c r="AE110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AF110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -11742,6 +12075,9 @@
       <c r="AE111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AF111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -11843,6 +12179,9 @@
       <c r="AE112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AF112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -11944,6 +12283,9 @@
       <c r="AE113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AF113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -12045,6 +12387,9 @@
       <c r="AE114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AF114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -12146,6 +12491,9 @@
       <c r="AE115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AF115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -12247,6 +12595,9 @@
       <c r="AE116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -12348,6 +12699,9 @@
       <c r="AE117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -12449,6 +12803,9 @@
       <c r="AE118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -12550,6 +12907,9 @@
       <c r="AE119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -12651,6 +13011,9 @@
       <c r="AE120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -12752,6 +13115,9 @@
       <c r="AE121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AF121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -12853,6 +13219,9 @@
       <c r="AE122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AF122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -12954,6 +13323,9 @@
       <c r="AE123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AF123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -13055,6 +13427,9 @@
       <c r="AE124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AF124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -13156,6 +13531,9 @@
       <c r="AE125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AF125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -13257,6 +13635,9 @@
       <c r="AE126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AF126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -13358,6 +13739,9 @@
       <c r="AE127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AF127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -13459,6 +13843,9 @@
       <c r="AE128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AF128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -13560,6 +13947,9 @@
       <c r="AE129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AF129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -13661,6 +14051,9 @@
       <c r="AE130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AF130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -13762,6 +14155,9 @@
       <c r="AE131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AF131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -13863,6 +14259,9 @@
       <c r="AE132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AF132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -13964,6 +14363,9 @@
       <c r="AE133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AF133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -14065,6 +14467,9 @@
       <c r="AE134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AF134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -14166,6 +14571,9 @@
       <c r="AE135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AF135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -14267,6 +14675,9 @@
       <c r="AE136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AF136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -14368,6 +14779,9 @@
       <c r="AE137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AF137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -14469,6 +14883,9 @@
       <c r="AE138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AF138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -14570,6 +14987,9 @@
       <c r="AE139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -14671,6 +15091,9 @@
       <c r="AE140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -14772,6 +15195,9 @@
       <c r="AE141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -14873,6 +15299,9 @@
       <c r="AE142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -14974,6 +15403,9 @@
       <c r="AE143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -15075,6 +15507,9 @@
       <c r="AE144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AF144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -15176,6 +15611,9 @@
       <c r="AE145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AF145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -15277,6 +15715,9 @@
       <c r="AE146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AF146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -15378,6 +15819,9 @@
       <c r="AE147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AF147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -15479,6 +15923,9 @@
       <c r="AE148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AF148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -15580,6 +16027,9 @@
       <c r="AE149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AF149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -15681,6 +16131,9 @@
       <c r="AE150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AF150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -15782,6 +16235,9 @@
       <c r="AE151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AF151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -15883,6 +16339,9 @@
       <c r="AE152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AF152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -15984,6 +16443,9 @@
       <c r="AE153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AF153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -16085,6 +16547,9 @@
       <c r="AE154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AF154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -16186,6 +16651,9 @@
       <c r="AE155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AF155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -16287,6 +16755,9 @@
       <c r="AE156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AF156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -16388,6 +16859,9 @@
       <c r="AE157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AF157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -16489,6 +16963,9 @@
       <c r="AE158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AF158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -16590,6 +17067,9 @@
       <c r="AE159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AF159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -16691,6 +17171,9 @@
       <c r="AE160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AF160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -16792,6 +17275,9 @@
       <c r="AE161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AF161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -16893,6 +17379,9 @@
       <c r="AE162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AF162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -16994,6 +17483,9 @@
       <c r="AE163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AF163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -17095,9 +17587,12 @@
       <c r="AE164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AF164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE164"/>
+  <autoFilter ref="A1:AF164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AF$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AG$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF164"/>
+  <dimension ref="A1:AG164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,7 @@
     <col width="16" customWidth="1" min="30" max="30"/>
     <col width="16" customWidth="1" min="31" max="31"/>
     <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -638,6 +639,11 @@
           <t>2026-09-07 22:09</t>
         </is>
       </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -742,6 +748,9 @@
       <c r="AF2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AG2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -846,6 +855,9 @@
       <c r="AF3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AG3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -950,6 +962,9 @@
       <c r="AF4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AG4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1054,6 +1069,9 @@
       <c r="AF5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AG5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1158,6 +1176,9 @@
       <c r="AF6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AG6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1262,6 +1283,9 @@
       <c r="AF7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AG7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1366,6 +1390,9 @@
       <c r="AF8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AG8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1470,6 +1497,9 @@
       <c r="AF9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AG9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1574,6 +1604,9 @@
       <c r="AF10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AG10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1678,6 +1711,9 @@
       <c r="AF11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AG11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1782,6 +1818,9 @@
       <c r="AF12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1886,6 +1925,9 @@
       <c r="AF13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AG13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1990,6 +2032,9 @@
       <c r="AF14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AG14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2094,6 +2139,9 @@
       <c r="AF15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AG15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2198,6 +2246,9 @@
       <c r="AF16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AG16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2302,6 +2353,9 @@
       <c r="AF17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AG17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2406,6 +2460,9 @@
       <c r="AF18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AG18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2510,6 +2567,9 @@
       <c r="AF19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AG19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2614,6 +2674,9 @@
       <c r="AF20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AG20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2718,6 +2781,9 @@
       <c r="AF21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AG21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2822,6 +2888,9 @@
       <c r="AF22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AG22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2926,6 +2995,9 @@
       <c r="AF23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AG23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3030,6 +3102,9 @@
       <c r="AF24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AG24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3134,6 +3209,9 @@
       <c r="AF25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3238,6 +3316,9 @@
       <c r="AF26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AG26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3342,6 +3423,9 @@
       <c r="AF27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AG27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3446,6 +3530,9 @@
       <c r="AF28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AG28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3550,6 +3637,9 @@
       <c r="AF29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AG29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3654,6 +3744,9 @@
       <c r="AF30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AG30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3758,6 +3851,9 @@
       <c r="AF31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AG31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3862,6 +3958,9 @@
       <c r="AF32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AG32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3966,6 +4065,9 @@
       <c r="AF33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AG33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4070,6 +4172,9 @@
       <c r="AF34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AG34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4174,6 +4279,9 @@
       <c r="AF35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AG35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4278,6 +4386,9 @@
       <c r="AF36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AG36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4382,6 +4493,9 @@
       <c r="AF37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AG37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4486,6 +4600,9 @@
       <c r="AF38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AG38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4590,6 +4707,9 @@
       <c r="AF39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AG39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4694,6 +4814,9 @@
       <c r="AF40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4798,6 +4921,9 @@
       <c r="AF41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4902,6 +5028,9 @@
       <c r="AF42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5006,6 +5135,9 @@
       <c r="AF43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5110,6 +5242,9 @@
       <c r="AF44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5214,6 +5349,9 @@
       <c r="AF45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AG45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5318,6 +5456,9 @@
       <c r="AF46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AG46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5422,6 +5563,9 @@
       <c r="AF47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AG47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5526,6 +5670,9 @@
       <c r="AF48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AG48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5630,6 +5777,9 @@
       <c r="AF49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AG49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5734,6 +5884,9 @@
       <c r="AF50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AG50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5838,6 +5991,9 @@
       <c r="AF51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AG51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5942,6 +6098,9 @@
       <c r="AF52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AG52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6046,6 +6205,9 @@
       <c r="AF53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AG53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6150,6 +6312,9 @@
       <c r="AF54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AG54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6254,6 +6419,9 @@
       <c r="AF55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AG55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6358,6 +6526,9 @@
       <c r="AF56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AG56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6462,6 +6633,9 @@
       <c r="AF57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6566,6 +6740,9 @@
       <c r="AF58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AG58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6670,6 +6847,9 @@
       <c r="AF59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AG59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6774,6 +6954,9 @@
       <c r="AF60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AG60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -6878,6 +7061,9 @@
       <c r="AF61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AG61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6982,6 +7168,9 @@
       <c r="AF62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AG62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7086,6 +7275,9 @@
       <c r="AF63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AG63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7190,6 +7382,9 @@
       <c r="AF64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AG64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7294,6 +7489,9 @@
       <c r="AF65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7398,6 +7596,9 @@
       <c r="AF66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7502,6 +7703,9 @@
       <c r="AF67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7606,6 +7810,9 @@
       <c r="AF68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -7710,6 +7917,9 @@
       <c r="AF69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -7814,6 +8024,9 @@
       <c r="AF70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -7918,6 +8131,9 @@
       <c r="AF71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8022,6 +8238,9 @@
       <c r="AF72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8126,6 +8345,9 @@
       <c r="AF73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8230,6 +8452,9 @@
       <c r="AF74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8334,6 +8559,9 @@
       <c r="AF75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8438,6 +8666,9 @@
       <c r="AF76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -8542,6 +8773,9 @@
       <c r="AF77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -8646,6 +8880,9 @@
       <c r="AF78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8750,6 +8987,9 @@
       <c r="AF79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -8854,6 +9094,9 @@
       <c r="AF80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -8958,6 +9201,9 @@
       <c r="AF81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9062,6 +9308,9 @@
       <c r="AF82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9166,6 +9415,9 @@
       <c r="AF83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9270,6 +9522,9 @@
       <c r="AF84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -9374,6 +9629,9 @@
       <c r="AF85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AG85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -9478,6 +9736,9 @@
       <c r="AF86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9582,6 +9843,9 @@
       <c r="AF87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9686,6 +9950,9 @@
       <c r="AF88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -9790,6 +10057,9 @@
       <c r="AF89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -9894,6 +10164,9 @@
       <c r="AF90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -9998,6 +10271,9 @@
       <c r="AF91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10102,6 +10378,9 @@
       <c r="AF92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -10206,6 +10485,9 @@
       <c r="AF93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AG93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -10310,6 +10592,9 @@
       <c r="AF94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AG94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -10414,6 +10699,9 @@
       <c r="AF95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AG95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -10518,6 +10806,9 @@
       <c r="AF96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AG96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -10622,6 +10913,9 @@
       <c r="AF97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AG97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -10726,6 +11020,9 @@
       <c r="AF98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AG98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -10830,6 +11127,9 @@
       <c r="AF99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -10934,6 +11234,9 @@
       <c r="AF100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AG100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -11038,6 +11341,9 @@
       <c r="AF101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AG101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -11142,6 +11448,9 @@
       <c r="AF102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AG102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -11246,6 +11555,9 @@
       <c r="AF103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AG103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -11350,6 +11662,9 @@
       <c r="AF104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AG104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -11454,6 +11769,9 @@
       <c r="AF105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AG105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -11558,6 +11876,9 @@
       <c r="AF106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AG106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -11662,6 +11983,9 @@
       <c r="AF107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AG107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -11766,6 +12090,9 @@
       <c r="AF108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -11870,6 +12197,9 @@
       <c r="AF109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AG109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -11974,6 +12304,9 @@
       <c r="AF110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AG110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -12078,6 +12411,9 @@
       <c r="AF111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AG111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -12182,6 +12518,9 @@
       <c r="AF112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AG112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -12286,6 +12625,9 @@
       <c r="AF113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AG113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -12390,6 +12732,9 @@
       <c r="AF114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AG114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -12494,6 +12839,9 @@
       <c r="AF115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AG115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -12598,6 +12946,9 @@
       <c r="AF116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -12702,6 +13053,9 @@
       <c r="AF117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -12806,6 +13160,9 @@
       <c r="AF118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -12910,6 +13267,9 @@
       <c r="AF119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -13014,6 +13374,9 @@
       <c r="AF120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -13118,6 +13481,9 @@
       <c r="AF121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AG121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -13222,6 +13588,9 @@
       <c r="AF122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AG122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -13326,6 +13695,9 @@
       <c r="AF123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AG123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -13430,6 +13802,9 @@
       <c r="AF124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AG124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -13534,6 +13909,9 @@
       <c r="AF125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AG125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -13638,6 +14016,9 @@
       <c r="AF126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AG126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -13742,6 +14123,9 @@
       <c r="AF127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AG127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -13846,6 +14230,9 @@
       <c r="AF128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AG128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -13950,6 +14337,9 @@
       <c r="AF129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AG129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -14054,6 +14444,9 @@
       <c r="AF130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AG130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -14158,6 +14551,9 @@
       <c r="AF131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AG131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -14262,6 +14658,9 @@
       <c r="AF132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AG132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -14366,6 +14765,9 @@
       <c r="AF133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AG133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -14470,6 +14872,9 @@
       <c r="AF134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AG134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -14574,6 +14979,9 @@
       <c r="AF135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AG135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -14678,6 +15086,9 @@
       <c r="AF136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AG136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -14782,6 +15193,9 @@
       <c r="AF137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AG137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -14886,6 +15300,9 @@
       <c r="AF138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AG138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -14990,6 +15407,9 @@
       <c r="AF139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -15094,6 +15514,9 @@
       <c r="AF140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -15198,6 +15621,9 @@
       <c r="AF141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -15302,6 +15728,9 @@
       <c r="AF142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -15406,6 +15835,9 @@
       <c r="AF143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -15510,6 +15942,9 @@
       <c r="AF144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AG144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -15614,6 +16049,9 @@
       <c r="AF145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AG145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -15718,6 +16156,9 @@
       <c r="AF146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AG146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -15822,6 +16263,9 @@
       <c r="AF147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AG147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -15926,6 +16370,9 @@
       <c r="AF148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AG148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -16030,6 +16477,9 @@
       <c r="AF149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AG149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -16134,6 +16584,9 @@
       <c r="AF150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AG150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -16238,6 +16691,9 @@
       <c r="AF151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AG151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -16342,6 +16798,9 @@
       <c r="AF152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AG152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -16446,6 +16905,9 @@
       <c r="AF153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AG153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -16550,6 +17012,9 @@
       <c r="AF154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AG154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -16654,6 +17119,9 @@
       <c r="AF155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AG155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -16758,6 +17226,9 @@
       <c r="AF156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AG156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -16862,6 +17333,9 @@
       <c r="AF157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AG157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -16966,6 +17440,9 @@
       <c r="AF158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AG158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -17070,6 +17547,9 @@
       <c r="AF159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AG159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -17174,6 +17654,9 @@
       <c r="AF160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AG160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -17278,6 +17761,9 @@
       <c r="AF161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AG161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -17382,6 +17868,9 @@
       <c r="AF162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AG162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -17486,6 +17975,9 @@
       <c r="AF163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AG163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -17590,9 +18082,12 @@
       <c r="AF164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AG164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF164"/>
+  <autoFilter ref="A1:AG164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 09:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AG$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AH$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG164"/>
+  <dimension ref="A1:AH164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -476,6 +476,7 @@
     <col width="16" customWidth="1" min="31" max="31"/>
     <col width="16" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,6 +645,11 @@
           <t>2026-09-08 01:12</t>
         </is>
       </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 04:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -751,6 +757,9 @@
       <c r="AG2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AH2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -858,6 +867,9 @@
       <c r="AG3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AH3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -965,6 +977,9 @@
       <c r="AG4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AH4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1072,6 +1087,9 @@
       <c r="AG5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AH5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1179,6 +1197,9 @@
       <c r="AG6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AH6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1286,6 +1307,9 @@
       <c r="AG7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AH7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1393,6 +1417,9 @@
       <c r="AG8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AH8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1500,6 +1527,9 @@
       <c r="AG9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AH9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1607,6 +1637,9 @@
       <c r="AG10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AH10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1714,6 +1747,9 @@
       <c r="AG11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AH11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1821,6 +1857,9 @@
       <c r="AG12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1928,6 +1967,9 @@
       <c r="AG13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AH13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2035,6 +2077,9 @@
       <c r="AG14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AH14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2142,6 +2187,9 @@
       <c r="AG15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AH15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2249,6 +2297,9 @@
       <c r="AG16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AH16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2356,6 +2407,9 @@
       <c r="AG17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AH17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2463,6 +2517,9 @@
       <c r="AG18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AH18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2570,6 +2627,9 @@
       <c r="AG19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AH19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2677,6 +2737,9 @@
       <c r="AG20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AH20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2784,6 +2847,9 @@
       <c r="AG21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AH21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2891,6 +2957,9 @@
       <c r="AG22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AH22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2998,6 +3067,9 @@
       <c r="AG23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AH23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3105,6 +3177,9 @@
       <c r="AG24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AH24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3212,6 +3287,9 @@
       <c r="AG25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3319,6 +3397,9 @@
       <c r="AG26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AH26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3426,6 +3507,9 @@
       <c r="AG27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AH27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3533,6 +3617,9 @@
       <c r="AG28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AH28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3640,6 +3727,9 @@
       <c r="AG29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AH29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3747,6 +3837,9 @@
       <c r="AG30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AH30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3854,6 +3947,9 @@
       <c r="AG31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AH31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3961,6 +4057,9 @@
       <c r="AG32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AH32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4068,6 +4167,9 @@
       <c r="AG33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AH33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4175,6 +4277,9 @@
       <c r="AG34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AH34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4282,6 +4387,9 @@
       <c r="AG35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AH35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4389,6 +4497,9 @@
       <c r="AG36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AH36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4496,6 +4607,9 @@
       <c r="AG37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AH37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4603,6 +4717,9 @@
       <c r="AG38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AH38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4710,6 +4827,9 @@
       <c r="AG39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AH39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4817,6 +4937,9 @@
       <c r="AG40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4924,6 +5047,9 @@
       <c r="AG41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5031,6 +5157,9 @@
       <c r="AG42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5138,6 +5267,9 @@
       <c r="AG43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5245,6 +5377,9 @@
       <c r="AG44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5352,6 +5487,9 @@
       <c r="AG45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AH45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5459,6 +5597,9 @@
       <c r="AG46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AH46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5566,6 +5707,9 @@
       <c r="AG47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AH47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5673,6 +5817,9 @@
       <c r="AG48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AH48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5780,6 +5927,9 @@
       <c r="AG49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AH49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5887,6 +6037,9 @@
       <c r="AG50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AH50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5994,6 +6147,9 @@
       <c r="AG51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AH51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6101,6 +6257,9 @@
       <c r="AG52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AH52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6208,6 +6367,9 @@
       <c r="AG53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AH53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6315,6 +6477,9 @@
       <c r="AG54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AH54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6422,6 +6587,9 @@
       <c r="AG55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AH55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6529,6 +6697,9 @@
       <c r="AG56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AH56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6636,6 +6807,9 @@
       <c r="AG57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6743,6 +6917,9 @@
       <c r="AG58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AH58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -6850,6 +7027,9 @@
       <c r="AG59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AH59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -6957,6 +7137,9 @@
       <c r="AG60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AH60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7064,6 +7247,9 @@
       <c r="AG61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AH61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7171,6 +7357,9 @@
       <c r="AG62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AH62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7278,6 +7467,9 @@
       <c r="AG63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AH63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7385,6 +7577,9 @@
       <c r="AG64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AH64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7492,6 +7687,9 @@
       <c r="AG65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7599,6 +7797,9 @@
       <c r="AG66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7706,6 +7907,9 @@
       <c r="AG67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -7813,6 +8017,9 @@
       <c r="AG68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -7920,6 +8127,9 @@
       <c r="AG69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8027,6 +8237,9 @@
       <c r="AG70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8134,6 +8347,9 @@
       <c r="AG71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8241,6 +8457,9 @@
       <c r="AG72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8348,6 +8567,9 @@
       <c r="AG73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8455,6 +8677,9 @@
       <c r="AG74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8562,6 +8787,9 @@
       <c r="AG75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8669,6 +8897,9 @@
       <c r="AG76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -8776,6 +9007,9 @@
       <c r="AG77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -8883,6 +9117,9 @@
       <c r="AG78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8990,6 +9227,9 @@
       <c r="AG79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9097,6 +9337,9 @@
       <c r="AG80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9204,6 +9447,9 @@
       <c r="AG81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9311,6 +9557,9 @@
       <c r="AG82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9418,6 +9667,9 @@
       <c r="AG83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9525,6 +9777,9 @@
       <c r="AG84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -9632,6 +9887,9 @@
       <c r="AG85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AH85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -9739,6 +9997,9 @@
       <c r="AG86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9846,6 +10107,9 @@
       <c r="AG87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9953,6 +10217,9 @@
       <c r="AG88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -10060,6 +10327,9 @@
       <c r="AG89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -10167,6 +10437,9 @@
       <c r="AG90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -10274,6 +10547,9 @@
       <c r="AG91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10381,6 +10657,9 @@
       <c r="AG92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -10488,6 +10767,9 @@
       <c r="AG93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AH93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -10595,6 +10877,9 @@
       <c r="AG94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AH94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -10702,6 +10987,9 @@
       <c r="AG95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AH95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -10809,6 +11097,9 @@
       <c r="AG96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AH96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -10916,6 +11207,9 @@
       <c r="AG97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AH97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11023,6 +11317,9 @@
       <c r="AG98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AH98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -11130,6 +11427,9 @@
       <c r="AG99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -11237,6 +11537,9 @@
       <c r="AG100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AH100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -11344,6 +11647,9 @@
       <c r="AG101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AH101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -11451,6 +11757,9 @@
       <c r="AG102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AH102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -11558,6 +11867,9 @@
       <c r="AG103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AH103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -11665,6 +11977,9 @@
       <c r="AG104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AH104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -11772,6 +12087,9 @@
       <c r="AG105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AH105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -11879,6 +12197,9 @@
       <c r="AG106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AH106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -11986,6 +12307,9 @@
       <c r="AG107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AH107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -12093,6 +12417,9 @@
       <c r="AG108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -12200,6 +12527,9 @@
       <c r="AG109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AH109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -12307,6 +12637,9 @@
       <c r="AG110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AH110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -12414,6 +12747,9 @@
       <c r="AG111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AH111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -12521,6 +12857,9 @@
       <c r="AG112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AH112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -12628,6 +12967,9 @@
       <c r="AG113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AH113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -12735,6 +13077,9 @@
       <c r="AG114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AH114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -12842,6 +13187,9 @@
       <c r="AG115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AH115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -12949,6 +13297,9 @@
       <c r="AG116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -13056,6 +13407,9 @@
       <c r="AG117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -13163,6 +13517,9 @@
       <c r="AG118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -13270,6 +13627,9 @@
       <c r="AG119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -13377,6 +13737,9 @@
       <c r="AG120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -13484,6 +13847,9 @@
       <c r="AG121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AH121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -13591,6 +13957,9 @@
       <c r="AG122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AH122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -13698,6 +14067,9 @@
       <c r="AG123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AH123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -13805,6 +14177,9 @@
       <c r="AG124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AH124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -13912,6 +14287,9 @@
       <c r="AG125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AH125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -14019,6 +14397,9 @@
       <c r="AG126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AH126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -14126,6 +14507,9 @@
       <c r="AG127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AH127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -14233,6 +14617,9 @@
       <c r="AG128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AH128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -14340,6 +14727,9 @@
       <c r="AG129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AH129" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -14447,6 +14837,9 @@
       <c r="AG130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AH130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -14554,6 +14947,9 @@
       <c r="AG131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AH131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -14661,6 +15057,9 @@
       <c r="AG132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AH132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -14768,6 +15167,9 @@
       <c r="AG133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AH133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -14875,6 +15277,9 @@
       <c r="AG134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AH134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -14982,6 +15387,9 @@
       <c r="AG135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AH135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -15089,6 +15497,9 @@
       <c r="AG136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AH136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -15196,6 +15607,9 @@
       <c r="AG137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AH137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -15303,6 +15717,9 @@
       <c r="AG138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AH138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -15410,6 +15827,9 @@
       <c r="AG139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -15517,6 +15937,9 @@
       <c r="AG140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -15624,6 +16047,9 @@
       <c r="AG141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -15731,6 +16157,9 @@
       <c r="AG142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -15838,6 +16267,9 @@
       <c r="AG143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -15945,6 +16377,9 @@
       <c r="AG144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AH144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -16052,6 +16487,9 @@
       <c r="AG145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AH145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -16159,6 +16597,9 @@
       <c r="AG146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AH146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -16266,6 +16707,9 @@
       <c r="AG147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AH147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -16373,6 +16817,9 @@
       <c r="AG148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AH148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -16480,6 +16927,9 @@
       <c r="AG149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AH149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -16587,6 +17037,9 @@
       <c r="AG150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AH150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -16694,6 +17147,9 @@
       <c r="AG151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AH151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -16801,6 +17257,9 @@
       <c r="AG152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AH152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -16908,6 +17367,9 @@
       <c r="AG153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AH153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17015,6 +17477,9 @@
       <c r="AG154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AH154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -17122,6 +17587,9 @@
       <c r="AG155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AH155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -17229,6 +17697,9 @@
       <c r="AG156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AH156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -17336,6 +17807,9 @@
       <c r="AG157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AH157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -17443,6 +17917,9 @@
       <c r="AG158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AH158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -17550,6 +18027,9 @@
       <c r="AG159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AH159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -17657,6 +18137,9 @@
       <c r="AG160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AH160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -17764,6 +18247,9 @@
       <c r="AG161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AH161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -17871,6 +18357,9 @@
       <c r="AG162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AH162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -17978,6 +18467,9 @@
       <c r="AG163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AH163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -18085,9 +18577,12 @@
       <c r="AG164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AH164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG164"/>
+  <autoFilter ref="A1:AH164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 12:13 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AH$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AI$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH164"/>
+  <dimension ref="A1:AI164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -477,6 +477,7 @@
     <col width="16" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -650,6 +651,11 @@
           <t>2026-09-08 04:10</t>
         </is>
       </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 07:13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -760,6 +766,9 @@
       <c r="AH2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AI2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -870,6 +879,9 @@
       <c r="AH3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AI3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -980,6 +992,9 @@
       <c r="AH4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AI4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1090,6 +1105,9 @@
       <c r="AH5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AI5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1200,6 +1218,9 @@
       <c r="AH6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AI6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1310,6 +1331,9 @@
       <c r="AH7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AI7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1420,6 +1444,9 @@
       <c r="AH8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AI8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1530,6 +1557,9 @@
       <c r="AH9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AI9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1640,6 +1670,9 @@
       <c r="AH10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AI10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1750,6 +1783,9 @@
       <c r="AH11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AI11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1860,6 +1896,9 @@
       <c r="AH12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1970,6 +2009,9 @@
       <c r="AH13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AI13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2080,6 +2122,9 @@
       <c r="AH14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AI14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2190,6 +2235,9 @@
       <c r="AH15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AI15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2300,6 +2348,9 @@
       <c r="AH16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AI16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2410,6 +2461,9 @@
       <c r="AH17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AI17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2520,6 +2574,9 @@
       <c r="AH18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AI18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2630,6 +2687,9 @@
       <c r="AH19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AI19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2740,6 +2800,9 @@
       <c r="AH20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AI20" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2850,6 +2913,9 @@
       <c r="AH21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AI21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2960,6 +3026,9 @@
       <c r="AH22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AI22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3070,6 +3139,9 @@
       <c r="AH23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AI23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3180,6 +3252,9 @@
       <c r="AH24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AI24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3290,6 +3365,9 @@
       <c r="AH25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3400,6 +3478,9 @@
       <c r="AH26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AI26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3510,6 +3591,9 @@
       <c r="AH27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AI27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3620,6 +3704,9 @@
       <c r="AH28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AI28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3730,6 +3817,9 @@
       <c r="AH29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AI29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3840,6 +3930,9 @@
       <c r="AH30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AI30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3950,6 +4043,9 @@
       <c r="AH31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AI31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4060,6 +4156,9 @@
       <c r="AH32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AI32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4170,6 +4269,9 @@
       <c r="AH33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AI33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4280,6 +4382,9 @@
       <c r="AH34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AI34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4390,6 +4495,9 @@
       <c r="AH35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AI35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4500,6 +4608,9 @@
       <c r="AH36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AI36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4610,6 +4721,9 @@
       <c r="AH37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AI37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4720,6 +4834,9 @@
       <c r="AH38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AI38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4830,6 +4947,9 @@
       <c r="AH39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AI39" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4940,6 +5060,9 @@
       <c r="AH40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5050,6 +5173,9 @@
       <c r="AH41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5160,6 +5286,9 @@
       <c r="AH42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5270,6 +5399,9 @@
       <c r="AH43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5380,6 +5512,9 @@
       <c r="AH44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5490,6 +5625,9 @@
       <c r="AH45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AI45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5600,6 +5738,9 @@
       <c r="AH46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AI46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5710,6 +5851,9 @@
       <c r="AH47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AI47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5820,6 +5964,9 @@
       <c r="AH48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AI48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5930,6 +6077,9 @@
       <c r="AH49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AI49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6040,6 +6190,9 @@
       <c r="AH50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AI50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6150,6 +6303,9 @@
       <c r="AH51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AI51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6260,6 +6416,9 @@
       <c r="AH52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AI52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6370,6 +6529,9 @@
       <c r="AH53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AI53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6480,6 +6642,9 @@
       <c r="AH54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AI54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6590,6 +6755,9 @@
       <c r="AH55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AI55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6700,6 +6868,9 @@
       <c r="AH56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AI56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6810,6 +6981,9 @@
       <c r="AH57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -6920,6 +7094,9 @@
       <c r="AH58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AI58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7030,6 +7207,9 @@
       <c r="AH59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AI59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7140,6 +7320,9 @@
       <c r="AH60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AI60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7250,6 +7433,9 @@
       <c r="AH61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AI61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7360,6 +7546,9 @@
       <c r="AH62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AI62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7470,6 +7659,9 @@
       <c r="AH63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AI63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7580,6 +7772,9 @@
       <c r="AH64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AI64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7690,6 +7885,9 @@
       <c r="AH65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -7800,6 +7998,9 @@
       <c r="AH66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -7910,6 +8111,9 @@
       <c r="AH67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8020,6 +8224,9 @@
       <c r="AH68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8130,6 +8337,9 @@
       <c r="AH69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8240,6 +8450,9 @@
       <c r="AH70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8350,6 +8563,9 @@
       <c r="AH71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8460,6 +8676,9 @@
       <c r="AH72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8570,6 +8789,9 @@
       <c r="AH73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8680,6 +8902,9 @@
       <c r="AH74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8790,6 +9015,9 @@
       <c r="AH75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -8900,6 +9128,9 @@
       <c r="AH76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9010,6 +9241,9 @@
       <c r="AH77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9120,6 +9354,9 @@
       <c r="AH78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9230,6 +9467,9 @@
       <c r="AH79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9340,6 +9580,9 @@
       <c r="AH80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9450,6 +9693,9 @@
       <c r="AH81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9560,6 +9806,9 @@
       <c r="AH82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9670,6 +9919,9 @@
       <c r="AH83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9780,6 +10032,9 @@
       <c r="AH84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -9890,6 +10145,9 @@
       <c r="AH85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AI85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -10000,6 +10258,9 @@
       <c r="AH86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -10110,6 +10371,9 @@
       <c r="AH87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -10220,6 +10484,9 @@
       <c r="AH88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -10330,6 +10597,9 @@
       <c r="AH89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -10440,6 +10710,9 @@
       <c r="AH90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -10550,6 +10823,9 @@
       <c r="AH91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10660,6 +10936,9 @@
       <c r="AH92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -10770,6 +11049,9 @@
       <c r="AH93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AI93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -10880,6 +11162,9 @@
       <c r="AH94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AI94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -10990,6 +11275,9 @@
       <c r="AH95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AI95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11100,6 +11388,9 @@
       <c r="AH96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AI96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -11210,6 +11501,9 @@
       <c r="AH97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AI97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11320,6 +11614,9 @@
       <c r="AH98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AI98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -11430,6 +11727,9 @@
       <c r="AH99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -11540,6 +11840,9 @@
       <c r="AH100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AI100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -11650,6 +11953,9 @@
       <c r="AH101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AI101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -11760,6 +12066,9 @@
       <c r="AH102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AI102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -11870,6 +12179,9 @@
       <c r="AH103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AI103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -11980,6 +12292,9 @@
       <c r="AH104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AI104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -12090,6 +12405,9 @@
       <c r="AH105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AI105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -12200,6 +12518,9 @@
       <c r="AH106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AI106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -12310,6 +12631,9 @@
       <c r="AH107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AI107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -12420,6 +12744,9 @@
       <c r="AH108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -12530,6 +12857,9 @@
       <c r="AH109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AI109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -12640,6 +12970,9 @@
       <c r="AH110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AI110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -12750,6 +13083,9 @@
       <c r="AH111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AI111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -12860,6 +13196,9 @@
       <c r="AH112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AI112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -12970,6 +13309,9 @@
       <c r="AH113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AI113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -13080,6 +13422,9 @@
       <c r="AH114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AI114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -13190,6 +13535,9 @@
       <c r="AH115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AI115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -13300,6 +13648,9 @@
       <c r="AH116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -13410,6 +13761,9 @@
       <c r="AH117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -13520,6 +13874,9 @@
       <c r="AH118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -13630,6 +13987,9 @@
       <c r="AH119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -13740,6 +14100,9 @@
       <c r="AH120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -13850,6 +14213,9 @@
       <c r="AH121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AI121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -13960,6 +14326,9 @@
       <c r="AH122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AI122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -14070,6 +14439,9 @@
       <c r="AH123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AI123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -14180,6 +14552,9 @@
       <c r="AH124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AI124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -14290,6 +14665,9 @@
       <c r="AH125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AI125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -14400,6 +14778,9 @@
       <c r="AH126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AI126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -14510,6 +14891,9 @@
       <c r="AH127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AI127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -14620,6 +15004,9 @@
       <c r="AH128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AI128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -14730,6 +15117,9 @@
       <c r="AH129" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AI129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -14840,6 +15230,9 @@
       <c r="AH130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AI130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -14950,6 +15343,9 @@
       <c r="AH131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AI131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -15060,6 +15456,9 @@
       <c r="AH132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AI132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -15170,6 +15569,9 @@
       <c r="AH133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AI133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -15280,6 +15682,9 @@
       <c r="AH134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AI134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -15390,6 +15795,9 @@
       <c r="AH135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AI135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -15500,6 +15908,9 @@
       <c r="AH136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AI136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -15610,6 +16021,9 @@
       <c r="AH137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AI137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -15720,6 +16134,9 @@
       <c r="AH138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AI138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -15830,6 +16247,9 @@
       <c r="AH139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -15940,6 +16360,9 @@
       <c r="AH140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -16050,6 +16473,9 @@
       <c r="AH141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -16160,6 +16586,9 @@
       <c r="AH142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -16270,6 +16699,9 @@
       <c r="AH143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -16380,6 +16812,9 @@
       <c r="AH144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AI144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -16490,6 +16925,9 @@
       <c r="AH145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AI145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -16600,6 +17038,9 @@
       <c r="AH146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AI146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -16710,6 +17151,9 @@
       <c r="AH147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AI147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -16820,6 +17264,9 @@
       <c r="AH148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AI148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -16930,6 +17377,9 @@
       <c r="AH149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AI149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -17040,6 +17490,9 @@
       <c r="AH150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AI150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -17150,6 +17603,9 @@
       <c r="AH151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AI151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -17260,6 +17716,9 @@
       <c r="AH152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AI152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -17370,6 +17829,9 @@
       <c r="AH153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AI153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17480,6 +17942,9 @@
       <c r="AH154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AI154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -17590,6 +18055,9 @@
       <c r="AH155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AI155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -17700,6 +18168,9 @@
       <c r="AH156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AI156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -17810,6 +18281,9 @@
       <c r="AH157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AI157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -17920,6 +18394,9 @@
       <c r="AH158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AI158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -18030,6 +18507,9 @@
       <c r="AH159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AI159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -18140,6 +18620,9 @@
       <c r="AH160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AI160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -18250,6 +18733,9 @@
       <c r="AH161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AI161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -18360,6 +18846,9 @@
       <c r="AH162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AI162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -18470,6 +18959,9 @@
       <c r="AH163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AI163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -18580,9 +19072,12 @@
       <c r="AH164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AI164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH164"/>
+  <autoFilter ref="A1:AI164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 15:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AI$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AJ$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI164"/>
+  <dimension ref="A1:AJ164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,7 @@
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="16" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="16" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -656,6 +657,11 @@
           <t>2026-09-08 07:13</t>
         </is>
       </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 10:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -769,6 +775,9 @@
       <c r="AI2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AJ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -882,6 +891,9 @@
       <c r="AI3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AJ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -995,6 +1007,9 @@
       <c r="AI4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AJ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1108,6 +1123,9 @@
       <c r="AI5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AJ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1221,6 +1239,9 @@
       <c r="AI6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AJ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1334,6 +1355,9 @@
       <c r="AI7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AJ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1447,6 +1471,9 @@
       <c r="AI8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AJ8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1560,6 +1587,9 @@
       <c r="AI9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AJ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1673,6 +1703,9 @@
       <c r="AI10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AJ10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1786,6 +1819,9 @@
       <c r="AI11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AJ11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1899,6 +1935,9 @@
       <c r="AI12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2012,6 +2051,9 @@
       <c r="AI13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AJ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2125,6 +2167,9 @@
       <c r="AI14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AJ14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2238,6 +2283,9 @@
       <c r="AI15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AJ15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2351,6 +2399,9 @@
       <c r="AI16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AJ16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2464,6 +2515,9 @@
       <c r="AI17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AJ17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2577,6 +2631,9 @@
       <c r="AI18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AJ18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2690,6 +2747,9 @@
       <c r="AI19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AJ19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2803,6 +2863,9 @@
       <c r="AI20" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AJ20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2916,6 +2979,9 @@
       <c r="AI21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AJ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3029,6 +3095,9 @@
       <c r="AI22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AJ22" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3142,6 +3211,9 @@
       <c r="AI23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AJ23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3255,6 +3327,9 @@
       <c r="AI24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AJ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3368,6 +3443,9 @@
       <c r="AI25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3481,6 +3559,9 @@
       <c r="AI26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AJ26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3594,6 +3675,9 @@
       <c r="AI27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AJ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3707,6 +3791,9 @@
       <c r="AI28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AJ28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3820,6 +3907,9 @@
       <c r="AI29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AJ29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3933,6 +4023,9 @@
       <c r="AI30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AJ30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4046,6 +4139,9 @@
       <c r="AI31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AJ31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4159,6 +4255,9 @@
       <c r="AI32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AJ32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4272,6 +4371,9 @@
       <c r="AI33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AJ33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4385,6 +4487,9 @@
       <c r="AI34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AJ34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4498,6 +4603,9 @@
       <c r="AI35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AJ35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4611,6 +4719,9 @@
       <c r="AI36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AJ36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4724,6 +4835,9 @@
       <c r="AI37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AJ37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4837,6 +4951,9 @@
       <c r="AI38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AJ38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4950,6 +5067,9 @@
       <c r="AI39" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AJ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5063,6 +5183,9 @@
       <c r="AI40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5176,6 +5299,9 @@
       <c r="AI41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5289,6 +5415,9 @@
       <c r="AI42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5402,6 +5531,9 @@
       <c r="AI43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5515,6 +5647,9 @@
       <c r="AI44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5628,6 +5763,9 @@
       <c r="AI45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AJ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5741,6 +5879,9 @@
       <c r="AI46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AJ46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5854,6 +5995,9 @@
       <c r="AI47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AJ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5967,6 +6111,9 @@
       <c r="AI48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AJ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6080,6 +6227,9 @@
       <c r="AI49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AJ49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6193,6 +6343,9 @@
       <c r="AI50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AJ50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6306,6 +6459,9 @@
       <c r="AI51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AJ51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6419,6 +6575,9 @@
       <c r="AI52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AJ52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6532,6 +6691,9 @@
       <c r="AI53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AJ53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6645,6 +6807,9 @@
       <c r="AI54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AJ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6758,6 +6923,9 @@
       <c r="AI55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AJ55" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6871,6 +7039,9 @@
       <c r="AI56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AJ56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -6984,6 +7155,9 @@
       <c r="AI57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7097,6 +7271,9 @@
       <c r="AI58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AJ58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7210,6 +7387,9 @@
       <c r="AI59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AJ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7323,6 +7503,9 @@
       <c r="AI60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AJ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7436,6 +7619,9 @@
       <c r="AI61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AJ61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7549,6 +7735,9 @@
       <c r="AI62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AJ62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7662,6 +7851,9 @@
       <c r="AI63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AJ63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7775,6 +7967,9 @@
       <c r="AI64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AJ64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -7888,6 +8083,9 @@
       <c r="AI65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8001,6 +8199,9 @@
       <c r="AI66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8114,6 +8315,9 @@
       <c r="AI67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8227,6 +8431,9 @@
       <c r="AI68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8340,6 +8547,9 @@
       <c r="AI69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8453,6 +8663,9 @@
       <c r="AI70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8566,6 +8779,9 @@
       <c r="AI71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8679,6 +8895,9 @@
       <c r="AI72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -8792,6 +9011,9 @@
       <c r="AI73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -8905,6 +9127,9 @@
       <c r="AI74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9018,6 +9243,9 @@
       <c r="AI75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9131,6 +9359,9 @@
       <c r="AI76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9244,6 +9475,9 @@
       <c r="AI77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9357,6 +9591,9 @@
       <c r="AI78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9470,6 +9707,9 @@
       <c r="AI79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9583,6 +9823,9 @@
       <c r="AI80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9696,6 +9939,9 @@
       <c r="AI81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9809,6 +10055,9 @@
       <c r="AI82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9922,6 +10171,9 @@
       <c r="AI83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -10035,6 +10287,9 @@
       <c r="AI84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -10148,6 +10403,9 @@
       <c r="AI85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AJ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -10261,6 +10519,9 @@
       <c r="AI86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -10374,6 +10635,9 @@
       <c r="AI87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -10487,6 +10751,9 @@
       <c r="AI88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -10600,6 +10867,9 @@
       <c r="AI89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -10713,6 +10983,9 @@
       <c r="AI90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -10826,6 +11099,9 @@
       <c r="AI91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10939,6 +11215,9 @@
       <c r="AI92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -11052,6 +11331,9 @@
       <c r="AI93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AJ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -11165,6 +11447,9 @@
       <c r="AI94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AJ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -11278,6 +11563,9 @@
       <c r="AI95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AJ95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11391,6 +11679,9 @@
       <c r="AI96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AJ96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -11504,6 +11795,9 @@
       <c r="AI97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AJ97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11617,6 +11911,9 @@
       <c r="AI98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AJ98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -11730,6 +12027,9 @@
       <c r="AI99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -11843,6 +12143,9 @@
       <c r="AI100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AJ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -11956,6 +12259,9 @@
       <c r="AI101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AJ101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -12069,6 +12375,9 @@
       <c r="AI102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AJ102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -12182,6 +12491,9 @@
       <c r="AI103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AJ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -12295,6 +12607,9 @@
       <c r="AI104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AJ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -12408,6 +12723,9 @@
       <c r="AI105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AJ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -12521,6 +12839,9 @@
       <c r="AI106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AJ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -12634,6 +12955,9 @@
       <c r="AI107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AJ107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -12747,6 +13071,9 @@
       <c r="AI108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -12860,6 +13187,9 @@
       <c r="AI109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AJ109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -12973,6 +13303,9 @@
       <c r="AI110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AJ110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -13086,6 +13419,9 @@
       <c r="AI111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AJ111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -13199,6 +13535,9 @@
       <c r="AI112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AJ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -13312,6 +13651,9 @@
       <c r="AI113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AJ113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -13425,6 +13767,9 @@
       <c r="AI114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AJ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -13538,6 +13883,9 @@
       <c r="AI115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AJ115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -13651,6 +13999,9 @@
       <c r="AI116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -13764,6 +14115,9 @@
       <c r="AI117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -13877,6 +14231,9 @@
       <c r="AI118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -13990,6 +14347,9 @@
       <c r="AI119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -14103,6 +14463,9 @@
       <c r="AI120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -14216,6 +14579,9 @@
       <c r="AI121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AJ121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -14329,6 +14695,9 @@
       <c r="AI122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AJ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -14442,6 +14811,9 @@
       <c r="AI123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AJ123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -14555,6 +14927,9 @@
       <c r="AI124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AJ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -14668,6 +15043,9 @@
       <c r="AI125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AJ125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -14781,6 +15159,9 @@
       <c r="AI126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AJ126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -14894,6 +15275,9 @@
       <c r="AI127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AJ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -15007,6 +15391,9 @@
       <c r="AI128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AJ128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -15120,6 +15507,9 @@
       <c r="AI129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AJ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -15233,6 +15623,9 @@
       <c r="AI130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AJ130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -15346,6 +15739,9 @@
       <c r="AI131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AJ131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -15459,6 +15855,9 @@
       <c r="AI132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AJ132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -15572,6 +15971,9 @@
       <c r="AI133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AJ133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -15685,6 +16087,9 @@
       <c r="AI134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AJ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -15798,6 +16203,9 @@
       <c r="AI135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AJ135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -15911,6 +16319,9 @@
       <c r="AI136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AJ136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -16024,6 +16435,9 @@
       <c r="AI137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AJ137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16137,6 +16551,9 @@
       <c r="AI138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AJ138" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -16250,6 +16667,9 @@
       <c r="AI139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -16363,6 +16783,9 @@
       <c r="AI140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -16476,6 +16899,9 @@
       <c r="AI141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -16589,6 +17015,9 @@
       <c r="AI142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -16702,6 +17131,9 @@
       <c r="AI143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -16815,6 +17247,9 @@
       <c r="AI144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AJ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -16928,6 +17363,9 @@
       <c r="AI145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AJ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -17041,6 +17479,9 @@
       <c r="AI146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AJ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -17154,6 +17595,9 @@
       <c r="AI147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AJ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -17267,6 +17711,9 @@
       <c r="AI148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AJ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -17380,6 +17827,9 @@
       <c r="AI149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AJ149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -17493,6 +17943,9 @@
       <c r="AI150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AJ150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -17606,6 +18059,9 @@
       <c r="AI151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AJ151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -17719,6 +18175,9 @@
       <c r="AI152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AJ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -17832,6 +18291,9 @@
       <c r="AI153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AJ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -17945,6 +18407,9 @@
       <c r="AI154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AJ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -18058,6 +18523,9 @@
       <c r="AI155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AJ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -18171,6 +18639,9 @@
       <c r="AI156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AJ156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -18284,6 +18755,9 @@
       <c r="AI157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AJ157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -18397,6 +18871,9 @@
       <c r="AI158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AJ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -18510,6 +18987,9 @@
       <c r="AI159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AJ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -18623,6 +19103,9 @@
       <c r="AI160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AJ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -18736,6 +19219,9 @@
       <c r="AI161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AJ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -18849,6 +19335,9 @@
       <c r="AI162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AJ162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -18962,6 +19451,9 @@
       <c r="AI163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AJ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -19075,9 +19567,12 @@
       <c r="AI164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AJ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI164"/>
+  <autoFilter ref="A1:AJ164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AJ$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AK$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ164"/>
+  <dimension ref="A1:AK165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -479,6 +479,7 @@
     <col width="16" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -662,6 +663,11 @@
           <t>2026-09-08 10:10</t>
         </is>
       </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -778,6 +784,9 @@
       <c r="AJ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AK2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -894,6 +903,9 @@
       <c r="AJ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AK3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1010,6 +1022,9 @@
       <c r="AJ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AK4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1126,6 +1141,9 @@
       <c r="AJ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AK5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1242,6 +1260,9 @@
       <c r="AJ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AK6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1358,6 +1379,9 @@
       <c r="AJ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AK7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1474,6 +1498,9 @@
       <c r="AJ8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AK8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1590,6 +1617,9 @@
       <c r="AJ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AK9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1706,6 +1736,9 @@
       <c r="AJ10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AK10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1822,6 +1855,9 @@
       <c r="AJ11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AK11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1938,6 +1974,9 @@
       <c r="AJ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2054,6 +2093,9 @@
       <c r="AJ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AK13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2170,6 +2212,9 @@
       <c r="AJ14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AK14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2286,6 +2331,9 @@
       <c r="AJ15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AK15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2402,6 +2450,9 @@
       <c r="AJ16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AK16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2518,6 +2569,9 @@
       <c r="AJ17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AK17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2634,6 +2688,9 @@
       <c r="AJ18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AK18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2750,6 +2807,9 @@
       <c r="AJ19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AK19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2866,6 +2926,9 @@
       <c r="AJ20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AK20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2982,6 +3045,9 @@
       <c r="AJ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AK21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3098,6 +3164,9 @@
       <c r="AJ22" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AK22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3214,6 +3283,9 @@
       <c r="AJ23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AK23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3330,6 +3402,9 @@
       <c r="AJ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AK24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3446,6 +3521,9 @@
       <c r="AJ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3562,6 +3640,9 @@
       <c r="AJ26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AK26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3678,6 +3759,9 @@
       <c r="AJ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AK27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3794,6 +3878,9 @@
       <c r="AJ28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AK28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3910,6 +3997,9 @@
       <c r="AJ29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AK29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4026,6 +4116,9 @@
       <c r="AJ30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AK30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4142,6 +4235,9 @@
       <c r="AJ31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AK31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4258,6 +4354,9 @@
       <c r="AJ32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AK32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4374,6 +4473,9 @@
       <c r="AJ33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AK33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4490,6 +4592,9 @@
       <c r="AJ34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AK34" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4606,6 +4711,9 @@
       <c r="AJ35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AK35" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4722,6 +4830,9 @@
       <c r="AJ36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AK36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4838,6 +4949,9 @@
       <c r="AJ37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AK37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4954,6 +5068,9 @@
       <c r="AJ38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AK38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5070,6 +5187,9 @@
       <c r="AJ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AK39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5186,6 +5306,9 @@
       <c r="AJ40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5302,6 +5425,9 @@
       <c r="AJ41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5418,6 +5544,9 @@
       <c r="AJ42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5534,6 +5663,9 @@
       <c r="AJ43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5650,6 +5782,9 @@
       <c r="AJ44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5766,6 +5901,9 @@
       <c r="AJ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AK45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5882,6 +6020,9 @@
       <c r="AJ46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AK46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5998,6 +6139,9 @@
       <c r="AJ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AK47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6114,6 +6258,9 @@
       <c r="AJ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AK48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6230,6 +6377,9 @@
       <c r="AJ49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AK49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6346,6 +6496,9 @@
       <c r="AJ50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AK50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6462,6 +6615,9 @@
       <c r="AJ51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AK51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6578,6 +6734,9 @@
       <c r="AJ52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AK52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6694,6 +6853,9 @@
       <c r="AJ53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AK53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6810,6 +6972,9 @@
       <c r="AJ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AK54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6926,6 +7091,9 @@
       <c r="AJ55" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AK55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7042,6 +7210,9 @@
       <c r="AJ56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AK56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7158,6 +7329,9 @@
       <c r="AJ57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7274,6 +7448,9 @@
       <c r="AJ58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AK58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7390,6 +7567,9 @@
       <c r="AJ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AK59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7506,6 +7686,9 @@
       <c r="AJ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AK60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7622,6 +7805,9 @@
       <c r="AJ61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AK61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7738,6 +7924,9 @@
       <c r="AJ62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AK62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -7854,6 +8043,9 @@
       <c r="AJ63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AK63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -7970,6 +8162,9 @@
       <c r="AJ64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AK64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8086,6 +8281,9 @@
       <c r="AJ65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8202,6 +8400,9 @@
       <c r="AJ66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8318,6 +8519,9 @@
       <c r="AJ67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8434,6 +8638,9 @@
       <c r="AJ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8550,6 +8757,9 @@
       <c r="AJ69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8666,6 +8876,9 @@
       <c r="AJ70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8782,6 +8995,9 @@
       <c r="AJ71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8898,6 +9114,9 @@
       <c r="AJ72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9014,6 +9233,9 @@
       <c r="AJ73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -9130,6 +9352,9 @@
       <c r="AJ74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9246,6 +9471,9 @@
       <c r="AJ75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9362,6 +9590,9 @@
       <c r="AJ76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9478,6 +9709,9 @@
       <c r="AJ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9594,6 +9828,9 @@
       <c r="AJ78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9710,6 +9947,9 @@
       <c r="AJ79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9826,6 +10066,9 @@
       <c r="AJ80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9942,6 +10185,9 @@
       <c r="AJ81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10058,6 +10304,9 @@
       <c r="AJ82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -10174,6 +10423,9 @@
       <c r="AJ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -10290,6 +10542,9 @@
       <c r="AJ84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -10406,6 +10661,9 @@
       <c r="AJ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AK85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -10522,6 +10780,9 @@
       <c r="AJ86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -10638,6 +10899,9 @@
       <c r="AJ87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -10754,6 +11018,9 @@
       <c r="AJ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -10870,6 +11137,9 @@
       <c r="AJ89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -10986,6 +11256,9 @@
       <c r="AJ90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -11102,6 +11375,9 @@
       <c r="AJ91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -11218,6 +11494,9 @@
       <c r="AJ92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -11334,6 +11613,9 @@
       <c r="AJ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AK93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -11450,6 +11732,9 @@
       <c r="AJ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AK94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -11566,6 +11851,9 @@
       <c r="AJ95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AK95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11682,6 +11970,9 @@
       <c r="AJ96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AK96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -11798,6 +12089,9 @@
       <c r="AJ97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AK97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11914,6 +12208,9 @@
       <c r="AJ98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AK98" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -12030,6 +12327,9 @@
       <c r="AJ99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -12146,6 +12446,9 @@
       <c r="AJ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AK100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -12262,6 +12565,9 @@
       <c r="AJ101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AK101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -12378,6 +12684,9 @@
       <c r="AJ102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AK102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -12494,6 +12803,9 @@
       <c r="AJ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AK103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -12610,6 +12922,9 @@
       <c r="AJ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AK104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -12726,6 +13041,9 @@
       <c r="AJ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AK105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -12842,6 +13160,9 @@
       <c r="AJ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AK106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -12958,6 +13279,9 @@
       <c r="AJ107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AK107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -13074,6 +13398,9 @@
       <c r="AJ108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -13190,6 +13517,9 @@
       <c r="AJ109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AK109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -13306,6 +13636,9 @@
       <c r="AJ110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AK110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -13422,6 +13755,9 @@
       <c r="AJ111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AK111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -13538,6 +13874,9 @@
       <c r="AJ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AK112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -13654,6 +13993,9 @@
       <c r="AJ113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AK113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -13770,6 +14112,9 @@
       <c r="AJ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AK114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -13886,6 +14231,9 @@
       <c r="AJ115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AK115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -14002,6 +14350,9 @@
       <c r="AJ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -14118,6 +14469,9 @@
       <c r="AJ117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -14234,6 +14588,9 @@
       <c r="AJ118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -14350,6 +14707,9 @@
       <c r="AJ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -14466,6 +14826,9 @@
       <c r="AJ120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -14582,6 +14945,9 @@
       <c r="AJ121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AK121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -14698,6 +15064,9 @@
       <c r="AJ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AK122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -14814,6 +15183,9 @@
       <c r="AJ123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AK123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -14930,6 +15302,9 @@
       <c r="AJ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AK124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -15046,6 +15421,9 @@
       <c r="AJ125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AK125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -15162,6 +15540,9 @@
       <c r="AJ126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AK126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -15278,6 +15659,9 @@
       <c r="AJ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AK127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -15394,6 +15778,9 @@
       <c r="AJ128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AK128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -15510,6 +15897,9 @@
       <c r="AJ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AK129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -15626,6 +16016,9 @@
       <c r="AJ130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AK130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -15742,6 +16135,9 @@
       <c r="AJ131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AK131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -15858,6 +16254,9 @@
       <c r="AJ132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AK132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -15974,6 +16373,9 @@
       <c r="AJ133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AK133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -16090,6 +16492,9 @@
       <c r="AJ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AK134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -16206,6 +16611,9 @@
       <c r="AJ135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AK135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -16322,6 +16730,9 @@
       <c r="AJ136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AK136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -16438,6 +16849,9 @@
       <c r="AJ137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AK137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16554,6 +16968,9 @@
       <c r="AJ138" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AK138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -16670,6 +17087,9 @@
       <c r="AJ139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -16786,6 +17206,9 @@
       <c r="AJ140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -16902,6 +17325,9 @@
       <c r="AJ141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -17018,6 +17444,9 @@
       <c r="AJ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -17134,6 +17563,9 @@
       <c r="AJ143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -17250,6 +17682,9 @@
       <c r="AJ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AK144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -17366,6 +17801,9 @@
       <c r="AJ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AK145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -17482,6 +17920,9 @@
       <c r="AJ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AK146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -17598,6 +18039,9 @@
       <c r="AJ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AK147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -17714,6 +18158,9 @@
       <c r="AJ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AK148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -17830,6 +18277,9 @@
       <c r="AJ149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AK149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -17946,6 +18396,9 @@
       <c r="AJ150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AK150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -18062,6 +18515,9 @@
       <c r="AJ151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AK151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -18178,6 +18634,9 @@
       <c r="AJ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AK152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -18294,6 +18753,9 @@
       <c r="AJ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AK153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -18410,6 +18872,9 @@
       <c r="AJ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AK154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -18526,6 +18991,9 @@
       <c r="AJ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AK155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -18642,6 +19110,9 @@
       <c r="AJ156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AK156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -18758,6 +19229,9 @@
       <c r="AJ157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AK157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -18874,6 +19348,9 @@
       <c r="AJ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AK158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -18990,6 +19467,9 @@
       <c r="AJ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AK159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -19106,6 +19586,9 @@
       <c r="AJ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AK160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -19222,6 +19705,9 @@
       <c r="AJ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AK161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -19338,6 +19824,9 @@
       <c r="AJ162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AK162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -19454,6 +19943,9 @@
       <c r="AJ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AK163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -19570,9 +20062,32 @@
       <c r="AJ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AK164" s="3" t="n">
+        <v>24.25</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>TUMAN</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>MARIA MELIDA DELGADO OBLITAS</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>SECTOR VILLA EL VALLE S/N</t>
+        </is>
+      </c>
+      <c r="AK165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ164"/>
+  <autoFilter ref="A1:AK165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-08 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AK$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AL$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK165"/>
+  <dimension ref="A1:AL165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,7 @@
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
     <col width="16" customWidth="1" min="37" max="37"/>
+    <col width="16" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -668,6 +669,11 @@
           <t>2026-09-08 13:11</t>
         </is>
       </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -787,6 +793,9 @@
       <c r="AK2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AL2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -906,6 +915,9 @@
       <c r="AK3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AL3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1025,6 +1037,9 @@
       <c r="AK4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AL4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1144,6 +1159,9 @@
       <c r="AK5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AL5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1263,6 +1281,9 @@
       <c r="AK6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AL6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1382,6 +1403,9 @@
       <c r="AK7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AL7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1501,6 +1525,9 @@
       <c r="AK8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AL8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1620,6 +1647,9 @@
       <c r="AK9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AL9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1739,6 +1769,9 @@
       <c r="AK10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AL10" s="3" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1858,6 +1891,9 @@
       <c r="AK11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AL11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1977,6 +2013,9 @@
       <c r="AK12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2096,6 +2135,9 @@
       <c r="AK13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AL13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2215,6 +2257,9 @@
       <c r="AK14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AL14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2334,6 +2379,9 @@
       <c r="AK15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AL15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2453,6 +2501,9 @@
       <c r="AK16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AL16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2572,6 +2623,9 @@
       <c r="AK17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AL17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2691,6 +2745,9 @@
       <c r="AK18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AL18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2810,6 +2867,9 @@
       <c r="AK19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AL19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2929,6 +2989,9 @@
       <c r="AK20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AL20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3048,6 +3111,9 @@
       <c r="AK21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AL21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3167,6 +3233,9 @@
       <c r="AK22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3286,6 +3355,9 @@
       <c r="AK23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AL23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3405,6 +3477,9 @@
       <c r="AK24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AL24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3524,6 +3599,9 @@
       <c r="AK25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3643,6 +3721,9 @@
       <c r="AK26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AL26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3762,6 +3843,9 @@
       <c r="AK27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AL27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3881,6 +3965,9 @@
       <c r="AK28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AL28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4000,6 +4087,9 @@
       <c r="AK29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AL29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4119,6 +4209,9 @@
       <c r="AK30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AL30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4238,6 +4331,9 @@
       <c r="AK31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AL31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4357,6 +4453,9 @@
       <c r="AK32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AL32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4476,6 +4575,9 @@
       <c r="AK33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AL33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4595,6 +4697,9 @@
       <c r="AK34" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AL34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4714,6 +4819,9 @@
       <c r="AK35" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AL35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4833,6 +4941,9 @@
       <c r="AK36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AL36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4952,6 +5063,9 @@
       <c r="AK37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AL37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5071,6 +5185,9 @@
       <c r="AK38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AL38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5190,6 +5307,9 @@
       <c r="AK39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AL39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5309,6 +5429,9 @@
       <c r="AK40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5428,6 +5551,9 @@
       <c r="AK41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5547,6 +5673,9 @@
       <c r="AK42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5666,6 +5795,9 @@
       <c r="AK43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5785,6 +5917,9 @@
       <c r="AK44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5904,6 +6039,9 @@
       <c r="AK45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6023,6 +6161,9 @@
       <c r="AK46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AL46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6142,6 +6283,9 @@
       <c r="AK47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AL47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6261,6 +6405,9 @@
       <c r="AK48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AL48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6380,6 +6527,9 @@
       <c r="AK49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AL49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6499,6 +6649,9 @@
       <c r="AK50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AL50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6618,6 +6771,9 @@
       <c r="AK51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AL51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6737,6 +6893,9 @@
       <c r="AK52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AL52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6856,6 +7015,9 @@
       <c r="AK53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AL53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6975,6 +7137,9 @@
       <c r="AK54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AL54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7094,6 +7259,9 @@
       <c r="AK55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AL55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7213,6 +7381,9 @@
       <c r="AK56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AL56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7332,6 +7503,9 @@
       <c r="AK57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7451,6 +7625,9 @@
       <c r="AK58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AL58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7570,6 +7747,9 @@
       <c r="AK59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AL59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7689,6 +7869,9 @@
       <c r="AK60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AL60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7808,6 +7991,9 @@
       <c r="AK61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AL61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -7927,6 +8113,9 @@
       <c r="AK62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AL62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8046,6 +8235,9 @@
       <c r="AK63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AL63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8165,6 +8357,9 @@
       <c r="AK64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AL64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8284,6 +8479,9 @@
       <c r="AK65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8403,6 +8601,9 @@
       <c r="AK66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8522,6 +8723,9 @@
       <c r="AK67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8641,6 +8845,9 @@
       <c r="AK68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8760,6 +8967,9 @@
       <c r="AK69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -8879,6 +9089,9 @@
       <c r="AK70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8998,6 +9211,9 @@
       <c r="AK71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9117,6 +9333,9 @@
       <c r="AK72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9236,6 +9455,9 @@
       <c r="AK73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -9355,6 +9577,9 @@
       <c r="AK74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9474,6 +9699,9 @@
       <c r="AK75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9593,6 +9821,9 @@
       <c r="AK76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9712,6 +9943,9 @@
       <c r="AK77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9831,6 +10065,9 @@
       <c r="AK78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9950,6 +10187,9 @@
       <c r="AK79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -10069,6 +10309,9 @@
       <c r="AK80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -10188,6 +10431,9 @@
       <c r="AK81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10307,6 +10553,9 @@
       <c r="AK82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -10426,6 +10675,9 @@
       <c r="AK83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -10545,6 +10797,9 @@
       <c r="AK84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -10664,6 +10919,9 @@
       <c r="AK85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AL85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -10783,6 +11041,9 @@
       <c r="AK86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -10902,6 +11163,9 @@
       <c r="AK87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11021,6 +11285,9 @@
       <c r="AK88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11140,6 +11407,9 @@
       <c r="AK89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -11259,6 +11529,9 @@
       <c r="AK90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -11378,6 +11651,9 @@
       <c r="AK91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -11497,6 +11773,9 @@
       <c r="AK92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -11616,6 +11895,9 @@
       <c r="AK93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AL93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -11735,6 +12017,9 @@
       <c r="AK94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AL94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -11854,6 +12139,9 @@
       <c r="AK95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AL95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11973,6 +12261,9 @@
       <c r="AK96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AL96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -12092,6 +12383,9 @@
       <c r="AK97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AL97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -12211,6 +12505,9 @@
       <c r="AK98" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AL98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -12330,6 +12627,9 @@
       <c r="AK99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -12449,6 +12749,9 @@
       <c r="AK100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AL100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -12568,6 +12871,9 @@
       <c r="AK101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AL101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -12687,6 +12993,9 @@
       <c r="AK102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AL102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -12806,6 +13115,9 @@
       <c r="AK103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AL103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -12925,6 +13237,9 @@
       <c r="AK104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AL104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -13044,6 +13359,9 @@
       <c r="AK105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AL105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -13163,6 +13481,9 @@
       <c r="AK106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AL106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -13282,6 +13603,9 @@
       <c r="AK107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AL107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -13401,6 +13725,9 @@
       <c r="AK108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -13520,6 +13847,9 @@
       <c r="AK109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -13639,6 +13969,9 @@
       <c r="AK110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AL110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -13758,6 +14091,9 @@
       <c r="AK111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AL111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -13877,6 +14213,9 @@
       <c r="AK112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AL112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -13996,6 +14335,9 @@
       <c r="AK113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AL113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -14115,6 +14457,9 @@
       <c r="AK114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AL114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -14234,6 +14579,9 @@
       <c r="AK115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AL115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -14353,6 +14701,9 @@
       <c r="AK116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -14472,6 +14823,9 @@
       <c r="AK117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -14591,6 +14945,9 @@
       <c r="AK118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -14710,6 +15067,9 @@
       <c r="AK119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -14829,6 +15189,9 @@
       <c r="AK120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -14948,6 +15311,9 @@
       <c r="AK121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AL121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -15067,6 +15433,9 @@
       <c r="AK122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AL122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -15186,6 +15555,9 @@
       <c r="AK123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AL123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -15305,6 +15677,9 @@
       <c r="AK124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AL124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -15424,6 +15799,9 @@
       <c r="AK125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AL125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -15543,6 +15921,9 @@
       <c r="AK126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AL126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -15662,6 +16043,9 @@
       <c r="AK127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AL127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -15781,6 +16165,9 @@
       <c r="AK128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AL128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -15900,6 +16287,9 @@
       <c r="AK129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AL129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -16019,6 +16409,9 @@
       <c r="AK130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AL130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -16138,6 +16531,9 @@
       <c r="AK131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AL131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -16257,6 +16653,9 @@
       <c r="AK132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AL132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -16376,6 +16775,9 @@
       <c r="AK133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AL133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -16495,6 +16897,9 @@
       <c r="AK134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AL134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -16614,6 +17019,9 @@
       <c r="AK135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AL135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -16733,6 +17141,9 @@
       <c r="AK136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AL136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -16852,6 +17263,9 @@
       <c r="AK137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AL137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16971,6 +17385,9 @@
       <c r="AK138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AL138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -17090,6 +17507,9 @@
       <c r="AK139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -17209,6 +17629,9 @@
       <c r="AK140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -17328,6 +17751,9 @@
       <c r="AK141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -17447,6 +17873,9 @@
       <c r="AK142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -17566,6 +17995,9 @@
       <c r="AK143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -17685,6 +18117,9 @@
       <c r="AK144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AL144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -17804,6 +18239,9 @@
       <c r="AK145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AL145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -17923,6 +18361,9 @@
       <c r="AK146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AL146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -18042,6 +18483,9 @@
       <c r="AK147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AL147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -18161,6 +18605,9 @@
       <c r="AK148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AL148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -18280,6 +18727,9 @@
       <c r="AK149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AL149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -18399,6 +18849,9 @@
       <c r="AK150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AL150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -18518,6 +18971,9 @@
       <c r="AK151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AL151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -18637,6 +19093,9 @@
       <c r="AK152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AL152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -18756,6 +19215,9 @@
       <c r="AK153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AL153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -18875,6 +19337,9 @@
       <c r="AK154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AL154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -18994,6 +19459,9 @@
       <c r="AK155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AL155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -19113,6 +19581,9 @@
       <c r="AK156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AL156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -19232,6 +19703,9 @@
       <c r="AK157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AL157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -19351,6 +19825,9 @@
       <c r="AK158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AL158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -19470,6 +19947,9 @@
       <c r="AK159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AL159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -19589,6 +20069,9 @@
       <c r="AK160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AL160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -19708,6 +20191,9 @@
       <c r="AK161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AL161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -19827,6 +20313,9 @@
       <c r="AK162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AL162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -19946,6 +20435,9 @@
       <c r="AK163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AL163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -20065,6 +20557,9 @@
       <c r="AK164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AL164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -20085,9 +20580,12 @@
       <c r="AK165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AL165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK165"/>
+  <autoFilter ref="A1:AL165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 00:15 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AL$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AM$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL165"/>
+  <dimension ref="A1:AM165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -481,6 +481,7 @@
     <col width="16" customWidth="1" min="36" max="36"/>
     <col width="16" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
+    <col width="16" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -674,6 +675,11 @@
           <t>2026-09-08 16:08</t>
         </is>
       </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 19:15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -796,6 +802,9 @@
       <c r="AL2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AM2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -918,6 +927,9 @@
       <c r="AL3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AM3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1040,6 +1052,9 @@
       <c r="AL4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AM4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1162,6 +1177,9 @@
       <c r="AL5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AM5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1284,6 +1302,9 @@
       <c r="AL6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AM6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1406,6 +1427,9 @@
       <c r="AL7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AM7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1528,6 +1552,9 @@
       <c r="AL8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AM8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1650,6 +1677,9 @@
       <c r="AL9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AM9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1772,6 +1802,9 @@
       <c r="AL10" s="3" t="n">
         <v>20.1</v>
       </c>
+      <c r="AM10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1894,6 +1927,9 @@
       <c r="AL11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AM11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2016,6 +2052,9 @@
       <c r="AL12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2138,6 +2177,9 @@
       <c r="AL13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AM13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2260,6 +2302,9 @@
       <c r="AL14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AM14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2382,6 +2427,9 @@
       <c r="AL15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AM15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2504,6 +2552,9 @@
       <c r="AL16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AM16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2626,6 +2677,9 @@
       <c r="AL17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AM17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2748,6 +2802,9 @@
       <c r="AL18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AM18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2870,6 +2927,9 @@
       <c r="AL19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AM19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2992,6 +3052,9 @@
       <c r="AL20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AM20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3114,6 +3177,9 @@
       <c r="AL21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AM21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3236,6 +3302,9 @@
       <c r="AL22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3358,6 +3427,9 @@
       <c r="AL23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AM23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3480,6 +3552,9 @@
       <c r="AL24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AM24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3602,6 +3677,9 @@
       <c r="AL25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3724,6 +3802,9 @@
       <c r="AL26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AM26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3846,6 +3927,9 @@
       <c r="AL27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AM27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3968,6 +4052,9 @@
       <c r="AL28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AM28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4090,6 +4177,9 @@
       <c r="AL29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AM29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4212,6 +4302,9 @@
       <c r="AL30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AM30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4334,6 +4427,9 @@
       <c r="AL31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AM31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4456,6 +4552,9 @@
       <c r="AL32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AM32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4578,6 +4677,9 @@
       <c r="AL33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AM33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4700,6 +4802,9 @@
       <c r="AL34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4822,6 +4927,9 @@
       <c r="AL35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AM35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4944,6 +5052,9 @@
       <c r="AL36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AM36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5066,6 +5177,9 @@
       <c r="AL37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AM37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5188,6 +5302,9 @@
       <c r="AL38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AM38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5310,6 +5427,9 @@
       <c r="AL39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AM39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5432,6 +5552,9 @@
       <c r="AL40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5554,6 +5677,9 @@
       <c r="AL41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5676,6 +5802,9 @@
       <c r="AL42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5798,6 +5927,9 @@
       <c r="AL43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM43" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5920,6 +6052,9 @@
       <c r="AL44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6042,6 +6177,9 @@
       <c r="AL45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6164,6 +6302,9 @@
       <c r="AL46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AM46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6286,6 +6427,9 @@
       <c r="AL47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AM47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6408,6 +6552,9 @@
       <c r="AL48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AM48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6530,6 +6677,9 @@
       <c r="AL49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AM49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6652,6 +6802,9 @@
       <c r="AL50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AM50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6774,6 +6927,9 @@
       <c r="AL51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AM51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -6896,6 +7052,9 @@
       <c r="AL52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AM52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7018,6 +7177,9 @@
       <c r="AL53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AM53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7140,6 +7302,9 @@
       <c r="AL54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AM54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7262,6 +7427,9 @@
       <c r="AL55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AM55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7384,6 +7552,9 @@
       <c r="AL56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AM56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7506,6 +7677,9 @@
       <c r="AL57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7628,6 +7802,9 @@
       <c r="AL58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AM58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7750,6 +7927,9 @@
       <c r="AL59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AM59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7872,6 +8052,9 @@
       <c r="AL60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AM60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -7994,6 +8177,9 @@
       <c r="AL61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AM61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8116,6 +8302,9 @@
       <c r="AL62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AM62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8238,6 +8427,9 @@
       <c r="AL63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AM63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8360,6 +8552,9 @@
       <c r="AL64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AM64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8482,6 +8677,9 @@
       <c r="AL65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8604,6 +8802,9 @@
       <c r="AL66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8726,6 +8927,9 @@
       <c r="AL67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8848,6 +9052,9 @@
       <c r="AL68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8970,6 +9177,9 @@
       <c r="AL69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM69" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9092,6 +9302,9 @@
       <c r="AL70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9214,6 +9427,9 @@
       <c r="AL71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9336,6 +9552,9 @@
       <c r="AL72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9458,6 +9677,9 @@
       <c r="AL73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM73" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -9580,6 +9802,9 @@
       <c r="AL74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9702,6 +9927,9 @@
       <c r="AL75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9824,6 +10052,9 @@
       <c r="AL76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9946,6 +10177,9 @@
       <c r="AL77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -10068,6 +10302,9 @@
       <c r="AL78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -10190,6 +10427,9 @@
       <c r="AL79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -10312,6 +10552,9 @@
       <c r="AL80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -10434,6 +10677,9 @@
       <c r="AL81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10556,6 +10802,9 @@
       <c r="AL82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -10678,6 +10927,9 @@
       <c r="AL83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -10800,6 +11052,9 @@
       <c r="AL84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -10922,6 +11177,9 @@
       <c r="AL85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AM85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11044,6 +11302,9 @@
       <c r="AL86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM86" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11166,6 +11427,9 @@
       <c r="AL87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11288,6 +11552,9 @@
       <c r="AL88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11410,6 +11677,9 @@
       <c r="AL89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -11532,6 +11802,9 @@
       <c r="AL90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -11654,6 +11927,9 @@
       <c r="AL91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -11776,6 +12052,9 @@
       <c r="AL92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -11898,6 +12177,9 @@
       <c r="AL93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AM93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12020,6 +12302,9 @@
       <c r="AL94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AM94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12142,6 +12427,9 @@
       <c r="AL95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AM95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -12264,6 +12552,9 @@
       <c r="AL96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AM96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -12386,6 +12677,9 @@
       <c r="AL97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AM97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -12508,6 +12802,9 @@
       <c r="AL98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AM98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -12630,6 +12927,9 @@
       <c r="AL99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -12752,6 +13052,9 @@
       <c r="AL100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AM100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -12874,6 +13177,9 @@
       <c r="AL101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AM101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -12996,6 +13302,9 @@
       <c r="AL102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AM102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -13118,6 +13427,9 @@
       <c r="AL103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AM103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -13240,6 +13552,9 @@
       <c r="AL104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AM104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -13362,6 +13677,9 @@
       <c r="AL105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AM105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -13484,6 +13802,9 @@
       <c r="AL106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AM106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -13606,6 +13927,9 @@
       <c r="AL107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AM107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -13728,6 +14052,9 @@
       <c r="AL108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -13850,6 +14177,9 @@
       <c r="AL109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -13972,6 +14302,9 @@
       <c r="AL110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AM110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -14094,6 +14427,9 @@
       <c r="AL111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AM111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -14216,6 +14552,9 @@
       <c r="AL112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AM112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -14338,6 +14677,9 @@
       <c r="AL113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AM113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -14460,6 +14802,9 @@
       <c r="AL114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AM114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -14582,6 +14927,9 @@
       <c r="AL115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AM115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -14704,6 +15052,9 @@
       <c r="AL116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -14826,6 +15177,9 @@
       <c r="AL117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM117" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -14948,6 +15302,9 @@
       <c r="AL118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -15070,6 +15427,9 @@
       <c r="AL119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -15192,6 +15552,9 @@
       <c r="AL120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -15314,6 +15677,9 @@
       <c r="AL121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AM121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -15436,6 +15802,9 @@
       <c r="AL122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AM122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -15558,6 +15927,9 @@
       <c r="AL123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AM123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -15680,6 +16052,9 @@
       <c r="AL124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AM124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -15802,6 +16177,9 @@
       <c r="AL125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AM125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -15924,6 +16302,9 @@
       <c r="AL126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AM126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -16046,6 +16427,9 @@
       <c r="AL127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AM127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -16168,6 +16552,9 @@
       <c r="AL128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AM128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -16290,6 +16677,9 @@
       <c r="AL129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AM129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -16412,6 +16802,9 @@
       <c r="AL130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AM130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -16534,6 +16927,9 @@
       <c r="AL131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AM131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -16656,6 +17052,9 @@
       <c r="AL132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AM132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -16778,6 +17177,9 @@
       <c r="AL133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AM133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -16900,6 +17302,9 @@
       <c r="AL134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AM134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -17022,6 +17427,9 @@
       <c r="AL135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AM135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -17144,6 +17552,9 @@
       <c r="AL136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AM136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -17266,6 +17677,9 @@
       <c r="AL137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AM137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -17388,6 +17802,9 @@
       <c r="AL138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AM138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -17510,6 +17927,9 @@
       <c r="AL139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -17632,6 +18052,9 @@
       <c r="AL140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -17754,6 +18177,9 @@
       <c r="AL141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -17876,6 +18302,9 @@
       <c r="AL142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -17998,6 +18427,9 @@
       <c r="AL143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -18120,6 +18552,9 @@
       <c r="AL144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AM144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -18242,6 +18677,9 @@
       <c r="AL145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AM145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -18364,6 +18802,9 @@
       <c r="AL146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AM146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -18486,6 +18927,9 @@
       <c r="AL147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AM147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -18608,6 +19052,9 @@
       <c r="AL148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AM148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -18730,6 +19177,9 @@
       <c r="AL149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AM149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -18852,6 +19302,9 @@
       <c r="AL150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AM150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -18974,6 +19427,9 @@
       <c r="AL151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AM151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -19096,6 +19552,9 @@
       <c r="AL152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AM152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -19218,6 +19677,9 @@
       <c r="AL153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AM153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -19340,6 +19802,9 @@
       <c r="AL154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AM154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -19462,6 +19927,9 @@
       <c r="AL155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AM155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -19584,6 +20052,9 @@
       <c r="AL156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AM156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -19706,6 +20177,9 @@
       <c r="AL157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AM157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -19828,6 +20302,9 @@
       <c r="AL158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AM158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -19950,6 +20427,9 @@
       <c r="AL159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AM159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -20072,6 +20552,9 @@
       <c r="AL160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AM160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -20194,6 +20677,9 @@
       <c r="AL161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AM161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -20316,6 +20802,9 @@
       <c r="AL162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AM162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -20438,6 +20927,9 @@
       <c r="AL163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AM163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -20560,6 +21052,9 @@
       <c r="AL164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AM164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -20583,9 +21078,12 @@
       <c r="AL165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AM165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AL165"/>
+  <autoFilter ref="A1:AM165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AM$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AN$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM165"/>
+  <dimension ref="A1:AN165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -482,6 +482,7 @@
     <col width="16" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
     <col width="16" customWidth="1" min="39" max="39"/>
+    <col width="16" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -680,6 +681,11 @@
           <t>2026-09-08 19:15</t>
         </is>
       </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -805,6 +811,9 @@
       <c r="AM2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AN2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -930,6 +939,9 @@
       <c r="AM3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AN3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1055,6 +1067,9 @@
       <c r="AM4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AN4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1180,6 +1195,9 @@
       <c r="AM5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AN5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1305,6 +1323,9 @@
       <c r="AM6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AN6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1430,6 +1451,9 @@
       <c r="AM7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AN7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1555,6 +1579,9 @@
       <c r="AM8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AN8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1680,6 +1707,9 @@
       <c r="AM9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AN9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1805,6 +1835,9 @@
       <c r="AM10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AN10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1930,6 +1963,9 @@
       <c r="AM11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AN11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2055,6 +2091,9 @@
       <c r="AM12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2180,6 +2219,9 @@
       <c r="AM13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AN13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2305,6 +2347,9 @@
       <c r="AM14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AN14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2430,6 +2475,9 @@
       <c r="AM15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AN15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2555,6 +2603,9 @@
       <c r="AM16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AN16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2680,6 +2731,9 @@
       <c r="AM17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AN17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2805,6 +2859,9 @@
       <c r="AM18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AN18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2930,6 +2987,9 @@
       <c r="AM19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AN19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3055,6 +3115,9 @@
       <c r="AM20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AN20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3180,6 +3243,9 @@
       <c r="AM21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AN21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3305,6 +3371,9 @@
       <c r="AM22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3430,6 +3499,9 @@
       <c r="AM23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AN23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3555,6 +3627,9 @@
       <c r="AM24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AN24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3680,6 +3755,9 @@
       <c r="AM25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3805,6 +3883,9 @@
       <c r="AM26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AN26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3930,6 +4011,9 @@
       <c r="AM27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AN27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4055,6 +4139,9 @@
       <c r="AM28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AN28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4180,6 +4267,9 @@
       <c r="AM29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AN29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4305,6 +4395,9 @@
       <c r="AM30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AN30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4430,6 +4523,9 @@
       <c r="AM31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AN31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4555,6 +4651,9 @@
       <c r="AM32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AN32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4680,6 +4779,9 @@
       <c r="AM33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AN33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4805,6 +4907,9 @@
       <c r="AM34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4930,6 +5035,9 @@
       <c r="AM35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AN35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5055,6 +5163,9 @@
       <c r="AM36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AN36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5180,6 +5291,9 @@
       <c r="AM37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AN37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5305,6 +5419,9 @@
       <c r="AM38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AN38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5430,6 +5547,9 @@
       <c r="AM39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AN39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5555,6 +5675,9 @@
       <c r="AM40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5680,6 +5803,9 @@
       <c r="AM41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5805,6 +5931,9 @@
       <c r="AM42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5930,6 +6059,9 @@
       <c r="AM43" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6055,6 +6187,9 @@
       <c r="AM44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6180,6 +6315,9 @@
       <c r="AM45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6305,6 +6443,9 @@
       <c r="AM46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AN46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6430,6 +6571,9 @@
       <c r="AM47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AN47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6555,6 +6699,9 @@
       <c r="AM48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AN48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6680,6 +6827,9 @@
       <c r="AM49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AN49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6805,6 +6955,9 @@
       <c r="AM50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AN50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6930,6 +7083,9 @@
       <c r="AM51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AN51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7055,6 +7211,9 @@
       <c r="AM52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AN52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7180,6 +7339,9 @@
       <c r="AM53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AN53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7305,6 +7467,9 @@
       <c r="AM54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AN54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7430,6 +7595,9 @@
       <c r="AM55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AN55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7555,6 +7723,9 @@
       <c r="AM56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AN56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7680,6 +7851,9 @@
       <c r="AM57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7805,6 +7979,9 @@
       <c r="AM58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AN58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7930,6 +8107,9 @@
       <c r="AM59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AN59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8055,6 +8235,9 @@
       <c r="AM60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AN60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8180,6 +8363,9 @@
       <c r="AM61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AN61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8305,6 +8491,9 @@
       <c r="AM62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AN62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8430,6 +8619,9 @@
       <c r="AM63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AN63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8555,6 +8747,9 @@
       <c r="AM64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AN64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8680,6 +8875,9 @@
       <c r="AM65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8805,6 +9003,9 @@
       <c r="AM66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8930,6 +9131,9 @@
       <c r="AM67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9055,6 +9259,9 @@
       <c r="AM68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -9180,6 +9387,9 @@
       <c r="AM69" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN69" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9305,6 +9515,9 @@
       <c r="AM70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9430,6 +9643,9 @@
       <c r="AM71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9555,6 +9771,9 @@
       <c r="AM72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9680,6 +9899,9 @@
       <c r="AM73" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN73" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -9805,6 +10027,9 @@
       <c r="AM74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9930,6 +10155,9 @@
       <c r="AM75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10055,6 +10283,9 @@
       <c r="AM76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -10180,6 +10411,9 @@
       <c r="AM77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -10305,6 +10539,9 @@
       <c r="AM78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -10430,6 +10667,9 @@
       <c r="AM79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -10555,6 +10795,9 @@
       <c r="AM80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -10680,6 +10923,9 @@
       <c r="AM81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10805,6 +11051,9 @@
       <c r="AM82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -10930,6 +11179,9 @@
       <c r="AM83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11055,6 +11307,9 @@
       <c r="AM84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11180,6 +11435,9 @@
       <c r="AM85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AN85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11305,6 +11563,9 @@
       <c r="AM86" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11430,6 +11691,9 @@
       <c r="AM87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11555,6 +11819,9 @@
       <c r="AM88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11680,6 +11947,9 @@
       <c r="AM89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -11805,6 +12075,9 @@
       <c r="AM90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -11930,6 +12203,9 @@
       <c r="AM91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -12055,6 +12331,9 @@
       <c r="AM92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -12180,6 +12459,9 @@
       <c r="AM93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AN93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12305,6 +12587,9 @@
       <c r="AM94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AN94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12430,6 +12715,9 @@
       <c r="AM95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AN95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -12555,6 +12843,9 @@
       <c r="AM96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AN96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -12680,6 +12971,9 @@
       <c r="AM97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AN97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -12805,6 +13099,9 @@
       <c r="AM98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AN98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -12930,6 +13227,9 @@
       <c r="AM99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13055,6 +13355,9 @@
       <c r="AM100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AN100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13180,6 +13483,9 @@
       <c r="AM101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AN101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -13305,6 +13611,9 @@
       <c r="AM102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AN102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -13430,6 +13739,9 @@
       <c r="AM103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AN103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -13555,6 +13867,9 @@
       <c r="AM104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AN104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -13680,6 +13995,9 @@
       <c r="AM105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AN105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -13805,6 +14123,9 @@
       <c r="AM106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AN106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -13930,6 +14251,9 @@
       <c r="AM107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AN107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -14055,6 +14379,9 @@
       <c r="AM108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -14180,6 +14507,9 @@
       <c r="AM109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -14305,6 +14635,9 @@
       <c r="AM110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AN110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -14430,6 +14763,9 @@
       <c r="AM111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AN111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -14555,6 +14891,9 @@
       <c r="AM112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AN112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -14680,6 +15019,9 @@
       <c r="AM113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AN113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -14805,6 +15147,9 @@
       <c r="AM114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AN114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -14930,6 +15275,9 @@
       <c r="AM115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AN115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15055,6 +15403,9 @@
       <c r="AM116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -15180,6 +15531,9 @@
       <c r="AM117" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -15305,6 +15659,9 @@
       <c r="AM118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -15430,6 +15787,9 @@
       <c r="AM119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -15555,6 +15915,9 @@
       <c r="AM120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -15680,6 +16043,9 @@
       <c r="AM121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AN121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -15805,6 +16171,9 @@
       <c r="AM122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AN122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -15930,6 +16299,9 @@
       <c r="AM123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AN123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -16055,6 +16427,9 @@
       <c r="AM124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AN124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -16180,6 +16555,9 @@
       <c r="AM125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AN125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -16305,6 +16683,9 @@
       <c r="AM126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AN126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -16430,6 +16811,9 @@
       <c r="AM127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AN127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -16555,6 +16939,9 @@
       <c r="AM128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AN128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -16680,6 +17067,9 @@
       <c r="AM129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AN129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -16805,6 +17195,9 @@
       <c r="AM130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AN130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -16930,6 +17323,9 @@
       <c r="AM131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AN131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -17055,6 +17451,9 @@
       <c r="AM132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AN132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -17180,6 +17579,9 @@
       <c r="AM133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AN133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -17305,6 +17707,9 @@
       <c r="AM134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AN134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -17430,6 +17835,9 @@
       <c r="AM135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AN135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -17555,6 +17963,9 @@
       <c r="AM136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AN136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -17680,6 +18091,9 @@
       <c r="AM137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AN137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -17805,6 +18219,9 @@
       <c r="AM138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AN138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -17930,6 +18347,9 @@
       <c r="AM139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -18055,6 +18475,9 @@
       <c r="AM140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -18180,6 +18603,9 @@
       <c r="AM141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -18305,6 +18731,9 @@
       <c r="AM142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -18430,6 +18859,9 @@
       <c r="AM143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -18555,6 +18987,9 @@
       <c r="AM144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AN144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -18680,6 +19115,9 @@
       <c r="AM145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AN145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -18805,6 +19243,9 @@
       <c r="AM146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AN146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -18930,6 +19371,9 @@
       <c r="AM147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AN147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -19055,6 +19499,9 @@
       <c r="AM148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AN148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -19180,6 +19627,9 @@
       <c r="AM149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AN149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -19305,6 +19755,9 @@
       <c r="AM150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AN150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -19430,6 +19883,9 @@
       <c r="AM151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AN151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -19555,6 +20011,9 @@
       <c r="AM152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AN152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -19680,6 +20139,9 @@
       <c r="AM153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AN153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -19805,6 +20267,9 @@
       <c r="AM154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AN154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -19930,6 +20395,9 @@
       <c r="AM155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AN155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -20055,6 +20523,9 @@
       <c r="AM156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AN156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -20180,6 +20651,9 @@
       <c r="AM157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AN157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -20305,6 +20779,9 @@
       <c r="AM158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AN158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -20430,6 +20907,9 @@
       <c r="AM159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AN159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -20555,6 +21035,9 @@
       <c r="AM160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AN160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -20680,6 +21163,9 @@
       <c r="AM161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AN161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -20805,6 +21291,9 @@
       <c r="AM162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AN162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -20930,6 +21419,9 @@
       <c r="AM163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AN163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -21055,6 +21547,9 @@
       <c r="AM164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AN164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -21081,9 +21576,12 @@
       <c r="AM165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AN165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM165"/>
+  <autoFilter ref="A1:AN165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AN$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AO$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN165"/>
+  <dimension ref="A1:AO165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -483,6 +483,7 @@
     <col width="16" customWidth="1" min="38" max="38"/>
     <col width="16" customWidth="1" min="39" max="39"/>
     <col width="16" customWidth="1" min="40" max="40"/>
+    <col width="16" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,6 +687,11 @@
           <t>2026-09-08 22:09</t>
         </is>
       </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -814,6 +820,9 @@
       <c r="AN2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AO2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -942,6 +951,9 @@
       <c r="AN3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AO3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1070,6 +1082,9 @@
       <c r="AN4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AO4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1198,6 +1213,9 @@
       <c r="AN5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AO5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1326,6 +1344,9 @@
       <c r="AN6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AO6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1454,6 +1475,9 @@
       <c r="AN7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AO7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1582,6 +1606,9 @@
       <c r="AN8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AO8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1710,6 +1737,9 @@
       <c r="AN9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AO9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1838,6 +1868,9 @@
       <c r="AN10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AO10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1966,6 +1999,9 @@
       <c r="AN11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AO11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2094,6 +2130,9 @@
       <c r="AN12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2222,6 +2261,9 @@
       <c r="AN13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AO13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2350,6 +2392,9 @@
       <c r="AN14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AO14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2478,6 +2523,9 @@
       <c r="AN15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AO15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2606,6 +2654,9 @@
       <c r="AN16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AO16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2734,6 +2785,9 @@
       <c r="AN17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AO17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2862,6 +2916,9 @@
       <c r="AN18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AO18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2990,6 +3047,9 @@
       <c r="AN19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AO19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3118,6 +3178,9 @@
       <c r="AN20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AO20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3246,6 +3309,9 @@
       <c r="AN21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AO21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3374,6 +3440,9 @@
       <c r="AN22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3502,6 +3571,9 @@
       <c r="AN23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AO23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3630,6 +3702,9 @@
       <c r="AN24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AO24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3758,6 +3833,9 @@
       <c r="AN25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3886,6 +3964,9 @@
       <c r="AN26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AO26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4014,6 +4095,9 @@
       <c r="AN27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AO27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4142,6 +4226,9 @@
       <c r="AN28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AO28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4270,6 +4357,9 @@
       <c r="AN29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AO29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4398,6 +4488,9 @@
       <c r="AN30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AO30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4526,6 +4619,9 @@
       <c r="AN31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AO31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4654,6 +4750,9 @@
       <c r="AN32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AO32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4782,6 +4881,9 @@
       <c r="AN33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4910,6 +5012,9 @@
       <c r="AN34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5038,6 +5143,9 @@
       <c r="AN35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AO35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5166,6 +5274,9 @@
       <c r="AN36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AO36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5294,6 +5405,9 @@
       <c r="AN37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AO37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5422,6 +5536,9 @@
       <c r="AN38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AO38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5550,6 +5667,9 @@
       <c r="AN39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AO39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5678,6 +5798,9 @@
       <c r="AN40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5806,6 +5929,9 @@
       <c r="AN41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5934,6 +6060,9 @@
       <c r="AN42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6062,6 +6191,9 @@
       <c r="AN43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6190,6 +6322,9 @@
       <c r="AN44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6318,6 +6453,9 @@
       <c r="AN45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6446,6 +6584,9 @@
       <c r="AN46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AO46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6574,6 +6715,9 @@
       <c r="AN47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AO47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6702,6 +6846,9 @@
       <c r="AN48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AO48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6830,6 +6977,9 @@
       <c r="AN49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AO49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6958,6 +7108,9 @@
       <c r="AN50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AO50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7086,6 +7239,9 @@
       <c r="AN51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AO51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7214,6 +7370,9 @@
       <c r="AN52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AO52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7342,6 +7501,9 @@
       <c r="AN53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AO53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7470,6 +7632,9 @@
       <c r="AN54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AO54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7598,6 +7763,9 @@
       <c r="AN55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AO55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7726,6 +7894,9 @@
       <c r="AN56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AO56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7854,6 +8025,9 @@
       <c r="AN57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7982,6 +8156,9 @@
       <c r="AN58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AO58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8110,6 +8287,9 @@
       <c r="AN59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AO59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8238,6 +8418,9 @@
       <c r="AN60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AO60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8366,6 +8549,9 @@
       <c r="AN61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8494,6 +8680,9 @@
       <c r="AN62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8622,6 +8811,9 @@
       <c r="AN63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8750,6 +8942,9 @@
       <c r="AN64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AO64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8878,6 +9073,9 @@
       <c r="AN65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -9006,6 +9204,9 @@
       <c r="AN66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -9134,6 +9335,9 @@
       <c r="AN67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9262,6 +9466,9 @@
       <c r="AN68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -9390,6 +9597,9 @@
       <c r="AN69" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AO69" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9518,6 +9728,9 @@
       <c r="AN70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9646,6 +9859,9 @@
       <c r="AN71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9774,6 +9990,9 @@
       <c r="AN72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9902,6 +10121,9 @@
       <c r="AN73" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AO73" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -10030,6 +10252,9 @@
       <c r="AN74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -10158,6 +10383,9 @@
       <c r="AN75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10286,6 +10514,9 @@
       <c r="AN76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -10414,6 +10645,9 @@
       <c r="AN77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -10542,6 +10776,9 @@
       <c r="AN78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -10670,6 +10907,9 @@
       <c r="AN79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -10798,6 +11038,9 @@
       <c r="AN80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -10926,6 +11169,9 @@
       <c r="AN81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -11054,6 +11300,9 @@
       <c r="AN82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -11182,6 +11431,9 @@
       <c r="AN83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11310,6 +11562,9 @@
       <c r="AN84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11438,6 +11693,9 @@
       <c r="AN85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AO85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11566,6 +11824,9 @@
       <c r="AN86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AO86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11694,6 +11955,9 @@
       <c r="AN87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11822,6 +12086,9 @@
       <c r="AN88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11950,6 +12217,9 @@
       <c r="AN89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -12078,6 +12348,9 @@
       <c r="AN90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -12206,6 +12479,9 @@
       <c r="AN91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -12334,6 +12610,9 @@
       <c r="AN92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -12462,6 +12741,9 @@
       <c r="AN93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AO93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12590,6 +12872,9 @@
       <c r="AN94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AO94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12718,6 +13003,9 @@
       <c r="AN95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AO95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -12846,6 +13134,9 @@
       <c r="AN96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AO96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -12974,6 +13265,9 @@
       <c r="AN97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AO97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -13102,6 +13396,9 @@
       <c r="AN98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AO98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -13230,6 +13527,9 @@
       <c r="AN99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13358,6 +13658,9 @@
       <c r="AN100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AO100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13486,6 +13789,9 @@
       <c r="AN101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AO101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -13614,6 +13920,9 @@
       <c r="AN102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AO102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -13742,6 +14051,9 @@
       <c r="AN103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AO103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -13870,6 +14182,9 @@
       <c r="AN104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AO104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -13998,6 +14313,9 @@
       <c r="AN105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AO105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -14126,6 +14444,9 @@
       <c r="AN106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AO106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -14254,6 +14575,9 @@
       <c r="AN107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AO107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -14382,6 +14706,9 @@
       <c r="AN108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -14510,6 +14837,9 @@
       <c r="AN109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -14638,6 +14968,9 @@
       <c r="AN110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AO110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -14766,6 +15099,9 @@
       <c r="AN111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AO111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -14894,6 +15230,9 @@
       <c r="AN112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AO112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -15022,6 +15361,9 @@
       <c r="AN113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AO113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -15150,6 +15492,9 @@
       <c r="AN114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AO114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -15278,6 +15623,9 @@
       <c r="AN115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AO115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15406,6 +15754,9 @@
       <c r="AN116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AO116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -15534,6 +15885,9 @@
       <c r="AN117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AO117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -15662,6 +16016,9 @@
       <c r="AN118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AO118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -15790,6 +16147,9 @@
       <c r="AN119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AO119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -15918,6 +16278,9 @@
       <c r="AN120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AO120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -16046,6 +16409,9 @@
       <c r="AN121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AO121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -16174,6 +16540,9 @@
       <c r="AN122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AO122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -16302,6 +16671,9 @@
       <c r="AN123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AO123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -16430,6 +16802,9 @@
       <c r="AN124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AO124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -16558,6 +16933,9 @@
       <c r="AN125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AO125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -16686,6 +17064,9 @@
       <c r="AN126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AO126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -16814,6 +17195,9 @@
       <c r="AN127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AO127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -16942,6 +17326,9 @@
       <c r="AN128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AO128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -17070,6 +17457,9 @@
       <c r="AN129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AO129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -17198,6 +17588,9 @@
       <c r="AN130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AO130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -17326,6 +17719,9 @@
       <c r="AN131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AO131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -17454,6 +17850,9 @@
       <c r="AN132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AO132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -17582,6 +17981,9 @@
       <c r="AN133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AO133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -17710,6 +18112,9 @@
       <c r="AN134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AO134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -17838,6 +18243,9 @@
       <c r="AN135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AO135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -17966,6 +18374,9 @@
       <c r="AN136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AO136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -18094,6 +18505,9 @@
       <c r="AN137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AO137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -18222,6 +18636,9 @@
       <c r="AN138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AO138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -18350,6 +18767,9 @@
       <c r="AN139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -18478,6 +18898,9 @@
       <c r="AN140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -18606,6 +19029,9 @@
       <c r="AN141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -18734,6 +19160,9 @@
       <c r="AN142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -18862,6 +19291,9 @@
       <c r="AN143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -18990,6 +19422,9 @@
       <c r="AN144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AO144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -19118,6 +19553,9 @@
       <c r="AN145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AO145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -19246,6 +19684,9 @@
       <c r="AN146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AO146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -19374,6 +19815,9 @@
       <c r="AN147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AO147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -19502,6 +19946,9 @@
       <c r="AN148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AO148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -19630,6 +20077,9 @@
       <c r="AN149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AO149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -19758,6 +20208,9 @@
       <c r="AN150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AO150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -19886,6 +20339,9 @@
       <c r="AN151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AO151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -20014,6 +20470,9 @@
       <c r="AN152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AO152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -20142,6 +20601,9 @@
       <c r="AN153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AO153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -20270,6 +20732,9 @@
       <c r="AN154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AO154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -20398,6 +20863,9 @@
       <c r="AN155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AO155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -20526,6 +20994,9 @@
       <c r="AN156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AO156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -20654,6 +21125,9 @@
       <c r="AN157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AO157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -20782,6 +21256,9 @@
       <c r="AN158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AO158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -20910,6 +21387,9 @@
       <c r="AN159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AO159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -21038,6 +21518,9 @@
       <c r="AN160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AO160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -21166,6 +21649,9 @@
       <c r="AN161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AO161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -21294,6 +21780,9 @@
       <c r="AN162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AO162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -21422,6 +21911,9 @@
       <c r="AN163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AO163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -21550,6 +22042,9 @@
       <c r="AN164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AO164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -21579,9 +22074,12 @@
       <c r="AN165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AO165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN165"/>
+  <autoFilter ref="A1:AO165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 09:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AO$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AP$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO165"/>
+  <dimension ref="A1:AP165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -484,6 +484,7 @@
     <col width="16" customWidth="1" min="39" max="39"/>
     <col width="16" customWidth="1" min="40" max="40"/>
     <col width="16" customWidth="1" min="41" max="41"/>
+    <col width="16" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -692,6 +693,11 @@
           <t>2026-09-09 01:12</t>
         </is>
       </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 04:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -823,6 +829,9 @@
       <c r="AO2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AP2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -954,6 +963,9 @@
       <c r="AO3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AP3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1085,6 +1097,9 @@
       <c r="AO4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AP4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1216,6 +1231,9 @@
       <c r="AO5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AP5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1347,6 +1365,9 @@
       <c r="AO6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AP6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1478,6 +1499,9 @@
       <c r="AO7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AP7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1609,6 +1633,9 @@
       <c r="AO8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AP8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1740,6 +1767,9 @@
       <c r="AO9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AP9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1871,6 +1901,9 @@
       <c r="AO10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AP10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2002,6 +2035,9 @@
       <c r="AO11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AP11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2133,6 +2169,9 @@
       <c r="AO12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2264,6 +2303,9 @@
       <c r="AO13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AP13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2395,6 +2437,9 @@
       <c r="AO14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AP14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2526,6 +2571,9 @@
       <c r="AO15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AP15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2657,6 +2705,9 @@
       <c r="AO16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AP16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2788,6 +2839,9 @@
       <c r="AO17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AP17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2919,6 +2973,9 @@
       <c r="AO18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AP18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3050,6 +3107,9 @@
       <c r="AO19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AP19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3181,6 +3241,9 @@
       <c r="AO20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AP20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3312,6 +3375,9 @@
       <c r="AO21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AP21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3443,6 +3509,9 @@
       <c r="AO22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3574,6 +3643,9 @@
       <c r="AO23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AP23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3705,6 +3777,9 @@
       <c r="AO24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AP24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3836,6 +3911,9 @@
       <c r="AO25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3967,6 +4045,9 @@
       <c r="AO26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AP26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4098,6 +4179,9 @@
       <c r="AO27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AP27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4229,6 +4313,9 @@
       <c r="AO28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AP28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4360,6 +4447,9 @@
       <c r="AO29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AP29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4491,6 +4581,9 @@
       <c r="AO30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AP30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4622,6 +4715,9 @@
       <c r="AO31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AP31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4753,6 +4849,9 @@
       <c r="AO32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AP32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4884,6 +4983,9 @@
       <c r="AO33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5015,6 +5117,9 @@
       <c r="AO34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5146,6 +5251,9 @@
       <c r="AO35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AP35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5277,6 +5385,9 @@
       <c r="AO36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AP36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5408,6 +5519,9 @@
       <c r="AO37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AP37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5539,6 +5653,9 @@
       <c r="AO38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AP38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5670,6 +5787,9 @@
       <c r="AO39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AP39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5801,6 +5921,9 @@
       <c r="AO40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5932,6 +6055,9 @@
       <c r="AO41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6063,6 +6189,9 @@
       <c r="AO42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6194,6 +6323,9 @@
       <c r="AO43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6325,6 +6457,9 @@
       <c r="AO44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6456,6 +6591,9 @@
       <c r="AO45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6587,6 +6725,9 @@
       <c r="AO46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AP46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6718,6 +6859,9 @@
       <c r="AO47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AP47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6849,6 +6993,9 @@
       <c r="AO48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AP48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6980,6 +7127,9 @@
       <c r="AO49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AP49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7111,6 +7261,9 @@
       <c r="AO50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AP50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7242,6 +7395,9 @@
       <c r="AO51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AP51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7373,6 +7529,9 @@
       <c r="AO52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AP52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7504,6 +7663,9 @@
       <c r="AO53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AP53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7635,6 +7797,9 @@
       <c r="AO54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AP54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7766,6 +7931,9 @@
       <c r="AO55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AP55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7897,6 +8065,9 @@
       <c r="AO56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AP56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8028,6 +8199,9 @@
       <c r="AO57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8159,6 +8333,9 @@
       <c r="AO58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AP58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8290,6 +8467,9 @@
       <c r="AO59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AP59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8421,6 +8601,9 @@
       <c r="AO60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AP60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8552,6 +8735,9 @@
       <c r="AO61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8683,6 +8869,9 @@
       <c r="AO62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8814,6 +9003,9 @@
       <c r="AO63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8945,6 +9137,9 @@
       <c r="AO64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AP64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -9076,6 +9271,9 @@
       <c r="AO65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -9207,6 +9405,9 @@
       <c r="AO66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -9338,6 +9539,9 @@
       <c r="AO67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9469,6 +9673,9 @@
       <c r="AO68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -9600,6 +9807,9 @@
       <c r="AO69" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AP69" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9731,6 +9941,9 @@
       <c r="AO70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9862,6 +10075,9 @@
       <c r="AO71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9993,6 +10209,9 @@
       <c r="AO72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -10124,6 +10343,9 @@
       <c r="AO73" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AP73" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -10255,6 +10477,9 @@
       <c r="AO74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -10386,6 +10611,9 @@
       <c r="AO75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10517,6 +10745,9 @@
       <c r="AO76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -10648,6 +10879,9 @@
       <c r="AO77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -10779,6 +11013,9 @@
       <c r="AO78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -10910,6 +11147,9 @@
       <c r="AO79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -11041,6 +11281,9 @@
       <c r="AO80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP80" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -11172,6 +11415,9 @@
       <c r="AO81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -11303,6 +11549,9 @@
       <c r="AO82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -11434,6 +11683,9 @@
       <c r="AO83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11565,6 +11817,9 @@
       <c r="AO84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11696,6 +11951,9 @@
       <c r="AO85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AP85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11827,6 +12085,9 @@
       <c r="AO86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AP86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11958,6 +12219,9 @@
       <c r="AO87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -12089,6 +12353,9 @@
       <c r="AO88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -12220,6 +12487,9 @@
       <c r="AO89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -12351,6 +12621,9 @@
       <c r="AO90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -12482,6 +12755,9 @@
       <c r="AO91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -12613,6 +12889,9 @@
       <c r="AO92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -12744,6 +13023,9 @@
       <c r="AO93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AP93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12875,6 +13157,9 @@
       <c r="AO94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AP94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -13006,6 +13291,9 @@
       <c r="AO95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AP95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -13137,6 +13425,9 @@
       <c r="AO96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AP96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -13268,6 +13559,9 @@
       <c r="AO97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AP97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -13399,6 +13693,9 @@
       <c r="AO98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AP98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -13530,6 +13827,9 @@
       <c r="AO99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13661,6 +13961,9 @@
       <c r="AO100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AP100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13792,6 +14095,9 @@
       <c r="AO101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AP101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -13923,6 +14229,9 @@
       <c r="AO102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AP102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -14054,6 +14363,9 @@
       <c r="AO103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AP103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -14185,6 +14497,9 @@
       <c r="AO104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AP104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -14316,6 +14631,9 @@
       <c r="AO105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AP105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -14447,6 +14765,9 @@
       <c r="AO106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AP106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -14578,6 +14899,9 @@
       <c r="AO107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AP107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -14709,6 +15033,9 @@
       <c r="AO108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -14840,6 +15167,9 @@
       <c r="AO109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -14971,6 +15301,9 @@
       <c r="AO110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AP110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -15102,6 +15435,9 @@
       <c r="AO111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AP111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -15233,6 +15569,9 @@
       <c r="AO112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AP112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -15364,6 +15703,9 @@
       <c r="AO113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AP113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -15495,6 +15837,9 @@
       <c r="AO114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AP114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -15626,6 +15971,9 @@
       <c r="AO115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AP115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15757,6 +16105,9 @@
       <c r="AO116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AP116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -15888,6 +16239,9 @@
       <c r="AO117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AP117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -16019,6 +16373,9 @@
       <c r="AO118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AP118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -16150,6 +16507,9 @@
       <c r="AO119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AP119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -16281,6 +16641,9 @@
       <c r="AO120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AP120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -16412,6 +16775,9 @@
       <c r="AO121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AP121" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -16543,6 +16909,9 @@
       <c r="AO122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AP122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -16674,6 +17043,9 @@
       <c r="AO123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AP123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -16805,6 +17177,9 @@
       <c r="AO124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AP124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -16936,6 +17311,9 @@
       <c r="AO125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AP125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -17067,6 +17445,9 @@
       <c r="AO126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AP126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -17198,6 +17579,9 @@
       <c r="AO127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AP127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -17329,6 +17713,9 @@
       <c r="AO128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AP128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -17460,6 +17847,9 @@
       <c r="AO129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AP129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -17591,6 +17981,9 @@
       <c r="AO130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AP130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -17722,6 +18115,9 @@
       <c r="AO131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AP131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -17853,6 +18249,9 @@
       <c r="AO132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AP132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -17984,6 +18383,9 @@
       <c r="AO133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AP133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -18115,6 +18517,9 @@
       <c r="AO134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AP134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -18246,6 +18651,9 @@
       <c r="AO135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AP135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -18377,6 +18785,9 @@
       <c r="AO136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AP136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -18508,6 +18919,9 @@
       <c r="AO137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AP137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -18639,6 +19053,9 @@
       <c r="AO138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AP138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -18770,6 +19187,9 @@
       <c r="AO139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -18901,6 +19321,9 @@
       <c r="AO140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -19032,6 +19455,9 @@
       <c r="AO141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -19163,6 +19589,9 @@
       <c r="AO142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -19294,6 +19723,9 @@
       <c r="AO143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -19425,6 +19857,9 @@
       <c r="AO144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AP144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -19556,6 +19991,9 @@
       <c r="AO145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AP145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -19687,6 +20125,9 @@
       <c r="AO146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AP146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -19818,6 +20259,9 @@
       <c r="AO147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AP147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -19949,6 +20393,9 @@
       <c r="AO148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AP148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -20080,6 +20527,9 @@
       <c r="AO149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AP149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -20211,6 +20661,9 @@
       <c r="AO150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AP150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -20342,6 +20795,9 @@
       <c r="AO151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AP151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -20473,6 +20929,9 @@
       <c r="AO152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AP152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -20604,6 +21063,9 @@
       <c r="AO153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AP153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -20735,6 +21197,9 @@
       <c r="AO154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AP154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -20866,6 +21331,9 @@
       <c r="AO155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AP155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -20997,6 +21465,9 @@
       <c r="AO156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AP156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -21128,6 +21599,9 @@
       <c r="AO157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AP157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -21259,6 +21733,9 @@
       <c r="AO158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AP158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -21390,6 +21867,9 @@
       <c r="AO159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AP159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -21521,6 +22001,9 @@
       <c r="AO160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AP160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -21652,6 +22135,9 @@
       <c r="AO161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AP161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -21783,6 +22269,9 @@
       <c r="AO162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AP162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -21914,6 +22403,9 @@
       <c r="AO163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AP163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -22045,6 +22537,9 @@
       <c r="AO164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AP164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -22077,9 +22572,12 @@
       <c r="AO165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AP165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO165"/>
+  <autoFilter ref="A1:AP165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AP$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AQ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP165"/>
+  <dimension ref="A1:AQ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,6 +485,7 @@
     <col width="16" customWidth="1" min="40" max="40"/>
     <col width="16" customWidth="1" min="41" max="41"/>
     <col width="16" customWidth="1" min="42" max="42"/>
+    <col width="16" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -698,6 +699,11 @@
           <t>2026-09-09 04:10</t>
         </is>
       </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 07:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -832,6 +838,9 @@
       <c r="AP2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AQ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -966,6 +975,9 @@
       <c r="AP3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AQ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1100,6 +1112,9 @@
       <c r="AP4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AQ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1234,6 +1249,9 @@
       <c r="AP5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AQ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1368,6 +1386,9 @@
       <c r="AP6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AQ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1502,6 +1523,9 @@
       <c r="AP7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AQ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1636,6 +1660,9 @@
       <c r="AP8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AQ8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1770,6 +1797,9 @@
       <c r="AP9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AQ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1904,6 +1934,9 @@
       <c r="AP10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AQ10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2038,6 +2071,9 @@
       <c r="AP11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AQ11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2172,6 +2208,9 @@
       <c r="AP12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2306,6 +2345,9 @@
       <c r="AP13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AQ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2440,6 +2482,9 @@
       <c r="AP14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AQ14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2574,6 +2619,9 @@
       <c r="AP15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AQ15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2708,6 +2756,9 @@
       <c r="AP16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AQ16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2842,6 +2893,9 @@
       <c r="AP17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AQ17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2976,6 +3030,9 @@
       <c r="AP18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AQ18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3110,6 +3167,9 @@
       <c r="AP19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AQ19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3244,6 +3304,9 @@
       <c r="AP20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AQ20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3378,6 +3441,9 @@
       <c r="AP21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AQ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3512,6 +3578,9 @@
       <c r="AP22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3646,6 +3715,9 @@
       <c r="AP23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AQ23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3780,6 +3852,9 @@
       <c r="AP24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AQ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3914,6 +3989,9 @@
       <c r="AP25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4048,6 +4126,9 @@
       <c r="AP26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AQ26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4182,6 +4263,9 @@
       <c r="AP27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AQ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4316,6 +4400,9 @@
       <c r="AP28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AQ28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4450,6 +4537,9 @@
       <c r="AP29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AQ29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4584,6 +4674,9 @@
       <c r="AP30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AQ30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4718,6 +4811,9 @@
       <c r="AP31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AQ31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4852,6 +4948,9 @@
       <c r="AP32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AQ32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4986,6 +5085,9 @@
       <c r="AP33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5120,6 +5222,9 @@
       <c r="AP34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5254,6 +5359,9 @@
       <c r="AP35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AQ35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5388,6 +5496,9 @@
       <c r="AP36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AQ36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5522,6 +5633,9 @@
       <c r="AP37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AQ37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5656,6 +5770,9 @@
       <c r="AP38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AQ38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5790,6 +5907,9 @@
       <c r="AP39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AQ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5924,6 +6044,9 @@
       <c r="AP40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6058,6 +6181,9 @@
       <c r="AP41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6192,6 +6318,9 @@
       <c r="AP42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6326,6 +6455,9 @@
       <c r="AP43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6460,6 +6592,9 @@
       <c r="AP44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6594,6 +6729,9 @@
       <c r="AP45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6728,6 +6866,9 @@
       <c r="AP46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AQ46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6862,6 +7003,9 @@
       <c r="AP47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AQ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6996,6 +7140,9 @@
       <c r="AP48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AQ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7130,6 +7277,9 @@
       <c r="AP49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AQ49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7264,6 +7414,9 @@
       <c r="AP50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AQ50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7398,6 +7551,9 @@
       <c r="AP51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AQ51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7532,6 +7688,9 @@
       <c r="AP52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AQ52" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7666,6 +7825,9 @@
       <c r="AP53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AQ53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7800,6 +7962,9 @@
       <c r="AP54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AQ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7934,6 +8099,9 @@
       <c r="AP55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AQ55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8068,6 +8236,9 @@
       <c r="AP56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AQ56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8202,6 +8373,9 @@
       <c r="AP57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8336,6 +8510,9 @@
       <c r="AP58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AQ58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8470,6 +8647,9 @@
       <c r="AP59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AQ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8604,6 +8784,9 @@
       <c r="AP60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AQ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8738,6 +8921,9 @@
       <c r="AP61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8872,6 +9058,9 @@
       <c r="AP62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9006,6 +9195,9 @@
       <c r="AP63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -9140,6 +9332,9 @@
       <c r="AP64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AQ64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -9274,6 +9469,9 @@
       <c r="AP65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -9408,6 +9606,9 @@
       <c r="AP66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -9542,6 +9743,9 @@
       <c r="AP67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9676,6 +9880,9 @@
       <c r="AP68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -9810,6 +10017,9 @@
       <c r="AP69" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AQ69" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9944,6 +10154,9 @@
       <c r="AP70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -10078,6 +10291,9 @@
       <c r="AP71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -10212,6 +10428,9 @@
       <c r="AP72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -10346,6 +10565,9 @@
       <c r="AP73" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AQ73" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -10480,6 +10702,9 @@
       <c r="AP74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ74" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -10614,6 +10839,9 @@
       <c r="AP75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10748,6 +10976,9 @@
       <c r="AP76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -10882,6 +11113,9 @@
       <c r="AP77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11016,6 +11250,9 @@
       <c r="AP78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -11150,6 +11387,9 @@
       <c r="AP79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -11284,6 +11524,9 @@
       <c r="AP80" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -11418,6 +11661,9 @@
       <c r="AP81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -11552,6 +11798,9 @@
       <c r="AP82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -11686,6 +11935,9 @@
       <c r="AP83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11820,6 +12072,9 @@
       <c r="AP84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ84" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11954,6 +12209,9 @@
       <c r="AP85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AQ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -12088,6 +12346,9 @@
       <c r="AP86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AQ86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -12222,6 +12483,9 @@
       <c r="AP87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -12356,6 +12620,9 @@
       <c r="AP88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -12490,6 +12757,9 @@
       <c r="AP89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -12624,6 +12894,9 @@
       <c r="AP90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -12758,6 +13031,9 @@
       <c r="AP91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -12892,6 +13168,9 @@
       <c r="AP92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -13026,6 +13305,9 @@
       <c r="AP93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AQ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -13160,6 +13442,9 @@
       <c r="AP94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AQ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -13294,6 +13579,9 @@
       <c r="AP95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AQ95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -13428,6 +13716,9 @@
       <c r="AP96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AQ96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -13562,6 +13853,9 @@
       <c r="AP97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AQ97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -13696,6 +13990,9 @@
       <c r="AP98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AQ98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -13830,6 +14127,9 @@
       <c r="AP99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13964,6 +14264,9 @@
       <c r="AP100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AQ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -14098,6 +14401,9 @@
       <c r="AP101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AQ101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -14232,6 +14538,9 @@
       <c r="AP102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AQ102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -14366,6 +14675,9 @@
       <c r="AP103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AQ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -14500,6 +14812,9 @@
       <c r="AP104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AQ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -14634,6 +14949,9 @@
       <c r="AP105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AQ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -14768,6 +15086,9 @@
       <c r="AP106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AQ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -14902,6 +15223,9 @@
       <c r="AP107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AQ107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -15036,6 +15360,9 @@
       <c r="AP108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -15170,6 +15497,9 @@
       <c r="AP109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -15304,6 +15634,9 @@
       <c r="AP110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AQ110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -15438,6 +15771,9 @@
       <c r="AP111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AQ111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -15572,6 +15908,9 @@
       <c r="AP112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AQ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -15706,6 +16045,9 @@
       <c r="AP113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AQ113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -15840,6 +16182,9 @@
       <c r="AP114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AQ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -15974,6 +16319,9 @@
       <c r="AP115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AQ115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -16108,6 +16456,9 @@
       <c r="AP116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AQ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -16242,6 +16593,9 @@
       <c r="AP117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AQ117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -16376,6 +16730,9 @@
       <c r="AP118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AQ118" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -16510,6 +16867,9 @@
       <c r="AP119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AQ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -16644,6 +17004,9 @@
       <c r="AP120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AQ120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -16778,6 +17141,9 @@
       <c r="AP121" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AQ121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -16912,6 +17278,9 @@
       <c r="AP122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AQ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -17046,6 +17415,9 @@
       <c r="AP123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AQ123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -17180,6 +17552,9 @@
       <c r="AP124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AQ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -17314,6 +17689,9 @@
       <c r="AP125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AQ125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -17448,6 +17826,9 @@
       <c r="AP126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AQ126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -17582,6 +17963,9 @@
       <c r="AP127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AQ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -17716,6 +18100,9 @@
       <c r="AP128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AQ128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -17850,6 +18237,9 @@
       <c r="AP129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AQ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -17984,6 +18374,9 @@
       <c r="AP130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AQ130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -18118,6 +18511,9 @@
       <c r="AP131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AQ131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -18252,6 +18648,9 @@
       <c r="AP132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AQ132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -18386,6 +18785,9 @@
       <c r="AP133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AQ133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -18520,6 +18922,9 @@
       <c r="AP134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AQ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -18654,6 +19059,9 @@
       <c r="AP135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AQ135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -18788,6 +19196,9 @@
       <c r="AP136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AQ136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -18922,6 +19333,9 @@
       <c r="AP137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AQ137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -19056,6 +19470,9 @@
       <c r="AP138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AQ138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -19190,6 +19607,9 @@
       <c r="AP139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -19324,6 +19744,9 @@
       <c r="AP140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -19458,6 +19881,9 @@
       <c r="AP141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -19592,6 +20018,9 @@
       <c r="AP142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -19726,6 +20155,9 @@
       <c r="AP143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -19860,6 +20292,9 @@
       <c r="AP144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AQ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -19994,6 +20429,9 @@
       <c r="AP145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AQ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -20128,6 +20566,9 @@
       <c r="AP146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AQ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -20262,6 +20703,9 @@
       <c r="AP147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AQ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -20396,6 +20840,9 @@
       <c r="AP148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AQ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -20530,6 +20977,9 @@
       <c r="AP149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AQ149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -20664,6 +21114,9 @@
       <c r="AP150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AQ150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -20798,6 +21251,9 @@
       <c r="AP151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AQ151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -20932,6 +21388,9 @@
       <c r="AP152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AQ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -21066,6 +21525,9 @@
       <c r="AP153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AQ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -21200,6 +21662,9 @@
       <c r="AP154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AQ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -21334,6 +21799,9 @@
       <c r="AP155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AQ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -21468,6 +21936,9 @@
       <c r="AP156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AQ156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -21602,6 +22073,9 @@
       <c r="AP157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AQ157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -21736,6 +22210,9 @@
       <c r="AP158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AQ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -21870,6 +22347,9 @@
       <c r="AP159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AQ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -22004,6 +22484,9 @@
       <c r="AP160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AQ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -22138,6 +22621,9 @@
       <c r="AP161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AQ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -22272,6 +22758,9 @@
       <c r="AP162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AQ162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -22406,6 +22895,9 @@
       <c r="AP163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AQ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -22540,6 +23032,9 @@
       <c r="AP164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AQ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -22575,9 +23070,12 @@
       <c r="AP165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AQ165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP165"/>
+  <autoFilter ref="A1:AQ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AQ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AR$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ165"/>
+  <dimension ref="A1:AR165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -486,6 +486,7 @@
     <col width="16" customWidth="1" min="41" max="41"/>
     <col width="16" customWidth="1" min="42" max="42"/>
     <col width="16" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -704,6 +705,11 @@
           <t>2026-09-09 07:11</t>
         </is>
       </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -841,6 +847,9 @@
       <c r="AQ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AR2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -978,6 +987,9 @@
       <c r="AQ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AR3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1115,6 +1127,9 @@
       <c r="AQ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AR4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1252,6 +1267,9 @@
       <c r="AQ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AR5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1389,6 +1407,9 @@
       <c r="AQ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AR6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1526,6 +1547,9 @@
       <c r="AQ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AR7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1663,6 +1687,9 @@
       <c r="AQ8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AR8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1800,6 +1827,9 @@
       <c r="AQ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AR9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1937,6 +1967,9 @@
       <c r="AQ10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AR10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2074,6 +2107,9 @@
       <c r="AQ11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AR11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2211,6 +2247,9 @@
       <c r="AQ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2348,6 +2387,9 @@
       <c r="AQ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AR13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2485,6 +2527,9 @@
       <c r="AQ14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AR14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2622,6 +2667,9 @@
       <c r="AQ15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AR15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2759,6 +2807,9 @@
       <c r="AQ16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AR16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2896,6 +2947,9 @@
       <c r="AQ17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AR17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3033,6 +3087,9 @@
       <c r="AQ18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AR18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3170,6 +3227,9 @@
       <c r="AQ19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AR19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3307,6 +3367,9 @@
       <c r="AQ20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AR20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3444,6 +3507,9 @@
       <c r="AQ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AR21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3581,6 +3647,9 @@
       <c r="AQ22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3718,6 +3787,9 @@
       <c r="AQ23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AR23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3855,6 +3927,9 @@
       <c r="AQ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AR24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3992,6 +4067,9 @@
       <c r="AQ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4129,6 +4207,9 @@
       <c r="AQ26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AR26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4266,6 +4347,9 @@
       <c r="AQ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AR27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4403,6 +4487,9 @@
       <c r="AQ28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AR28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4540,6 +4627,9 @@
       <c r="AQ29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AR29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4677,6 +4767,9 @@
       <c r="AQ30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AR30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4814,6 +4907,9 @@
       <c r="AQ31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AR31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4951,6 +5047,9 @@
       <c r="AQ32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AR32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5088,6 +5187,9 @@
       <c r="AQ33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5225,6 +5327,9 @@
       <c r="AQ34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5362,6 +5467,9 @@
       <c r="AQ35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AR35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5499,6 +5607,9 @@
       <c r="AQ36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AR36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5636,6 +5747,9 @@
       <c r="AQ37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AR37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5773,6 +5887,9 @@
       <c r="AQ38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AR38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5910,6 +6027,9 @@
       <c r="AQ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AR39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6047,6 +6167,9 @@
       <c r="AQ40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6184,6 +6307,9 @@
       <c r="AQ41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6321,6 +6447,9 @@
       <c r="AQ42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6458,6 +6587,9 @@
       <c r="AQ43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6595,6 +6727,9 @@
       <c r="AQ44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6732,6 +6867,9 @@
       <c r="AQ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6869,6 +7007,9 @@
       <c r="AQ46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AR46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7006,6 +7147,9 @@
       <c r="AQ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AR47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7143,6 +7287,9 @@
       <c r="AQ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AR48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7280,6 +7427,9 @@
       <c r="AQ49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AR49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7417,6 +7567,9 @@
       <c r="AQ50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AR50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7554,6 +7707,9 @@
       <c r="AQ51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AR51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7691,6 +7847,9 @@
       <c r="AQ52" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AR52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7828,6 +7987,9 @@
       <c r="AQ53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AR53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7965,6 +8127,9 @@
       <c r="AQ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AR54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8102,6 +8267,9 @@
       <c r="AQ55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AR55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8239,6 +8407,9 @@
       <c r="AQ56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AR56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8376,6 +8547,9 @@
       <c r="AQ57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8513,6 +8687,9 @@
       <c r="AQ58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AR58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8650,6 +8827,9 @@
       <c r="AQ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AR59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8787,6 +8967,9 @@
       <c r="AQ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AR60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8924,6 +9107,9 @@
       <c r="AQ61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR61" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -9061,6 +9247,9 @@
       <c r="AQ62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9198,6 +9387,9 @@
       <c r="AQ63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -9335,6 +9527,9 @@
       <c r="AQ64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AR64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -9472,6 +9667,9 @@
       <c r="AQ65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -9609,6 +9807,9 @@
       <c r="AQ66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -9746,6 +9947,9 @@
       <c r="AQ67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR67" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9883,6 +10087,9 @@
       <c r="AQ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10020,6 +10227,9 @@
       <c r="AQ69" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AR69" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -10157,6 +10367,9 @@
       <c r="AQ70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -10294,6 +10507,9 @@
       <c r="AQ71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -10431,6 +10647,9 @@
       <c r="AQ72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -10568,6 +10787,9 @@
       <c r="AQ73" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AR73" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -10705,6 +10927,9 @@
       <c r="AQ74" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR74" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -10842,6 +11067,9 @@
       <c r="AQ75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10979,6 +11207,9 @@
       <c r="AQ76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -11116,6 +11347,9 @@
       <c r="AQ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11253,6 +11487,9 @@
       <c r="AQ78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -11390,6 +11627,9 @@
       <c r="AQ79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -11527,6 +11767,9 @@
       <c r="AQ80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AR80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -11664,6 +11907,9 @@
       <c r="AQ81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -11801,6 +12047,9 @@
       <c r="AQ82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -11938,6 +12187,9 @@
       <c r="AQ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -12075,6 +12327,9 @@
       <c r="AQ84" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -12212,6 +12467,9 @@
       <c r="AQ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AR85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -12349,6 +12607,9 @@
       <c r="AQ86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AR86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -12486,6 +12747,9 @@
       <c r="AQ87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -12623,6 +12887,9 @@
       <c r="AQ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -12760,6 +13027,9 @@
       <c r="AQ89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -12897,6 +13167,9 @@
       <c r="AQ90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -13034,6 +13307,9 @@
       <c r="AQ91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -13171,6 +13447,9 @@
       <c r="AQ92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -13308,6 +13587,9 @@
       <c r="AQ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AR93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -13445,6 +13727,9 @@
       <c r="AQ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AR94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -13582,6 +13867,9 @@
       <c r="AQ95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AR95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -13719,6 +14007,9 @@
       <c r="AQ96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AR96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -13856,6 +14147,9 @@
       <c r="AQ97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AR97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -13993,6 +14287,9 @@
       <c r="AQ98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AR98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -14130,6 +14427,9 @@
       <c r="AQ99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -14267,6 +14567,9 @@
       <c r="AQ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AR100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -14404,6 +14707,9 @@
       <c r="AQ101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AR101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -14541,6 +14847,9 @@
       <c r="AQ102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AR102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -14678,6 +14987,9 @@
       <c r="AQ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AR103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -14815,6 +15127,9 @@
       <c r="AQ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AR104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -14952,6 +15267,9 @@
       <c r="AQ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AR105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -15089,6 +15407,9 @@
       <c r="AQ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AR106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -15226,6 +15547,9 @@
       <c r="AQ107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AR107" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -15363,6 +15687,9 @@
       <c r="AQ108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -15500,6 +15827,9 @@
       <c r="AQ109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -15637,6 +15967,9 @@
       <c r="AQ110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AR110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -15774,6 +16107,9 @@
       <c r="AQ111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AR111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -15911,6 +16247,9 @@
       <c r="AQ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AR112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -16048,6 +16387,9 @@
       <c r="AQ113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AR113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -16185,6 +16527,9 @@
       <c r="AQ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AR114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -16322,6 +16667,9 @@
       <c r="AQ115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AR115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -16459,6 +16807,9 @@
       <c r="AQ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AR116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -16596,6 +16947,9 @@
       <c r="AQ117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AR117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -16733,6 +17087,9 @@
       <c r="AQ118" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AR118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -16870,6 +17227,9 @@
       <c r="AQ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AR119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -17007,6 +17367,9 @@
       <c r="AQ120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AR120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -17144,6 +17507,9 @@
       <c r="AQ121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AR121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -17281,6 +17647,9 @@
       <c r="AQ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AR122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -17418,6 +17787,9 @@
       <c r="AQ123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AR123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -17555,6 +17927,9 @@
       <c r="AQ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AR124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -17692,6 +18067,9 @@
       <c r="AQ125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AR125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -17829,6 +18207,9 @@
       <c r="AQ126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AR126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -17966,6 +18347,9 @@
       <c r="AQ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AR127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -18103,6 +18487,9 @@
       <c r="AQ128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AR128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -18240,6 +18627,9 @@
       <c r="AQ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AR129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -18377,6 +18767,9 @@
       <c r="AQ130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AR130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -18514,6 +18907,9 @@
       <c r="AQ131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AR131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -18651,6 +19047,9 @@
       <c r="AQ132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AR132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -18788,6 +19187,9 @@
       <c r="AQ133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AR133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -18925,6 +19327,9 @@
       <c r="AQ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AR134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -19062,6 +19467,9 @@
       <c r="AQ135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AR135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -19199,6 +19607,9 @@
       <c r="AQ136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AR136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -19336,6 +19747,9 @@
       <c r="AQ137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AR137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -19473,6 +19887,9 @@
       <c r="AQ138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AR138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -19610,6 +20027,9 @@
       <c r="AQ139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -19747,6 +20167,9 @@
       <c r="AQ140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -19884,6 +20307,9 @@
       <c r="AQ141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -20021,6 +20447,9 @@
       <c r="AQ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -20158,6 +20587,9 @@
       <c r="AQ143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -20295,6 +20727,9 @@
       <c r="AQ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AR144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -20432,6 +20867,9 @@
       <c r="AQ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AR145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -20569,6 +21007,9 @@
       <c r="AQ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AR146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -20706,6 +21147,9 @@
       <c r="AQ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AR147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -20843,6 +21287,9 @@
       <c r="AQ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AR148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -20980,6 +21427,9 @@
       <c r="AQ149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AR149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -21117,6 +21567,9 @@
       <c r="AQ150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AR150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -21254,6 +21707,9 @@
       <c r="AQ151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AR151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -21391,6 +21847,9 @@
       <c r="AQ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AR152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -21528,6 +21987,9 @@
       <c r="AQ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AR153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -21665,6 +22127,9 @@
       <c r="AQ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AR154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -21802,6 +22267,9 @@
       <c r="AQ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AR155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -21939,6 +22407,9 @@
       <c r="AQ156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AR156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -22076,6 +22547,9 @@
       <c r="AQ157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AR157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -22213,6 +22687,9 @@
       <c r="AQ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AR158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -22350,6 +22827,9 @@
       <c r="AQ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AR159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -22487,6 +22967,9 @@
       <c r="AQ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AR160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -22624,6 +23107,9 @@
       <c r="AQ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AR161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -22761,6 +23247,9 @@
       <c r="AQ162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AR162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -22898,6 +23387,9 @@
       <c r="AQ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AR163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -23035,6 +23527,9 @@
       <c r="AQ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AR164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -23073,9 +23568,12 @@
       <c r="AQ165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AR165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AQ165"/>
+  <autoFilter ref="A1:AR165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 18:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AR$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AS$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR165"/>
+  <dimension ref="A1:AS165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,7 @@
     <col width="16" customWidth="1" min="42" max="42"/>
     <col width="16" customWidth="1" min="43" max="43"/>
     <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="16" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -710,6 +711,11 @@
           <t>2026-09-09 10:08</t>
         </is>
       </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -850,6 +856,9 @@
       <c r="AR2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AS2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -990,6 +999,9 @@
       <c r="AR3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AS3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1130,6 +1142,9 @@
       <c r="AR4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AS4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1270,6 +1285,9 @@
       <c r="AR5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AS5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1410,6 +1428,9 @@
       <c r="AR6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AS6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1550,6 +1571,9 @@
       <c r="AR7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AS7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1690,6 +1714,9 @@
       <c r="AR8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AS8" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1830,6 +1857,9 @@
       <c r="AR9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AS9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1970,6 +2000,9 @@
       <c r="AR10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AS10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2110,6 +2143,9 @@
       <c r="AR11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AS11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2250,6 +2286,9 @@
       <c r="AR12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2390,6 +2429,9 @@
       <c r="AR13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AS13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2530,6 +2572,9 @@
       <c r="AR14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AS14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2670,6 +2715,9 @@
       <c r="AR15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AS15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2810,6 +2858,9 @@
       <c r="AR16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AS16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2950,6 +3001,9 @@
       <c r="AR17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AS17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3090,6 +3144,9 @@
       <c r="AR18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AS18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3230,6 +3287,9 @@
       <c r="AR19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AS19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3370,6 +3430,9 @@
       <c r="AR20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AS20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3510,6 +3573,9 @@
       <c r="AR21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AS21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3650,6 +3716,9 @@
       <c r="AR22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3790,6 +3859,9 @@
       <c r="AR23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AS23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3930,6 +4002,9 @@
       <c r="AR24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AS24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4070,6 +4145,9 @@
       <c r="AR25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4210,6 +4288,9 @@
       <c r="AR26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AS26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4350,6 +4431,9 @@
       <c r="AR27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AS27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4490,6 +4574,9 @@
       <c r="AR28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AS28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4630,6 +4717,9 @@
       <c r="AR29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AS29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4770,6 +4860,9 @@
       <c r="AR30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AS30" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4910,6 +5003,9 @@
       <c r="AR31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AS31" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5050,6 +5146,9 @@
       <c r="AR32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AS32" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5190,6 +5289,9 @@
       <c r="AR33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5330,6 +5432,9 @@
       <c r="AR34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5470,6 +5575,9 @@
       <c r="AR35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AS35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5610,6 +5718,9 @@
       <c r="AR36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AS36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5750,6 +5861,9 @@
       <c r="AR37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AS37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5890,6 +6004,9 @@
       <c r="AR38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AS38" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6030,6 +6147,9 @@
       <c r="AR39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AS39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6170,6 +6290,9 @@
       <c r="AR40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6310,6 +6433,9 @@
       <c r="AR41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6450,6 +6576,9 @@
       <c r="AR42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6590,6 +6719,9 @@
       <c r="AR43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6730,6 +6862,9 @@
       <c r="AR44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6870,6 +7005,9 @@
       <c r="AR45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7010,6 +7148,9 @@
       <c r="AR46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AS46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7150,6 +7291,9 @@
       <c r="AR47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AS47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7290,6 +7434,9 @@
       <c r="AR48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AS48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7430,6 +7577,9 @@
       <c r="AR49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AS49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7570,6 +7720,9 @@
       <c r="AR50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AS50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7710,6 +7863,9 @@
       <c r="AR51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AS51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7850,6 +8006,9 @@
       <c r="AR52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AS52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7990,6 +8149,9 @@
       <c r="AR53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AS53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8130,6 +8292,9 @@
       <c r="AR54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AS54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8270,6 +8435,9 @@
       <c r="AR55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AS55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8410,6 +8578,9 @@
       <c r="AR56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AS56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8550,6 +8721,9 @@
       <c r="AR57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8690,6 +8864,9 @@
       <c r="AR58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AS58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8830,6 +9007,9 @@
       <c r="AR59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AS59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8970,6 +9150,9 @@
       <c r="AR60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AS60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -9110,6 +9293,9 @@
       <c r="AR61" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -9250,6 +9436,9 @@
       <c r="AR62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9390,6 +9579,9 @@
       <c r="AR63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -9530,6 +9722,9 @@
       <c r="AR64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AS64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -9670,6 +9865,9 @@
       <c r="AR65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -9810,6 +10008,9 @@
       <c r="AR66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -9950,6 +10151,9 @@
       <c r="AR67" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -10090,6 +10294,9 @@
       <c r="AR68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10230,6 +10437,9 @@
       <c r="AR69" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -10370,6 +10580,9 @@
       <c r="AR70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -10510,6 +10723,9 @@
       <c r="AR71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -10650,6 +10866,9 @@
       <c r="AR72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -10790,6 +11009,9 @@
       <c r="AR73" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -10930,6 +11152,9 @@
       <c r="AR74" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11070,6 +11295,9 @@
       <c r="AR75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -11210,6 +11438,9 @@
       <c r="AR76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -11350,6 +11581,9 @@
       <c r="AR77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11490,6 +11724,9 @@
       <c r="AR78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -11630,6 +11867,9 @@
       <c r="AR79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -11770,6 +12010,9 @@
       <c r="AR80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AS80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -11910,6 +12153,9 @@
       <c r="AR81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -12050,6 +12296,9 @@
       <c r="AR82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -12190,6 +12439,9 @@
       <c r="AR83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -12330,6 +12582,9 @@
       <c r="AR84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -12470,6 +12725,9 @@
       <c r="AR85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AS85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -12610,6 +12868,9 @@
       <c r="AR86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS86" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -12750,6 +13011,9 @@
       <c r="AR87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -12890,6 +13154,9 @@
       <c r="AR88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -13030,6 +13297,9 @@
       <c r="AR89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -13170,6 +13440,9 @@
       <c r="AR90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -13310,6 +13583,9 @@
       <c r="AR91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -13450,6 +13726,9 @@
       <c r="AR92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -13590,6 +13869,9 @@
       <c r="AR93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AS93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -13730,6 +14012,9 @@
       <c r="AR94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AS94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -13870,6 +14155,9 @@
       <c r="AR95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AS95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14010,6 +14298,9 @@
       <c r="AR96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AS96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -14150,6 +14441,9 @@
       <c r="AR97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AS97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -14290,6 +14584,9 @@
       <c r="AR98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AS98" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -14430,6 +14727,9 @@
       <c r="AR99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -14570,6 +14870,9 @@
       <c r="AR100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AS100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -14710,6 +15013,9 @@
       <c r="AR101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AS101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -14850,6 +15156,9 @@
       <c r="AR102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AS102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -14990,6 +15299,9 @@
       <c r="AR103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AS103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -15130,6 +15442,9 @@
       <c r="AR104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AS104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -15270,6 +15585,9 @@
       <c r="AR105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AS105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -15410,6 +15728,9 @@
       <c r="AR106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AS106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -15550,6 +15871,9 @@
       <c r="AR107" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AS107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -15690,6 +16014,9 @@
       <c r="AR108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -15830,6 +16157,9 @@
       <c r="AR109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -15970,6 +16300,9 @@
       <c r="AR110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AS110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -16110,6 +16443,9 @@
       <c r="AR111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AS111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -16250,6 +16586,9 @@
       <c r="AR112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AS112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -16390,6 +16729,9 @@
       <c r="AR113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AS113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -16530,6 +16872,9 @@
       <c r="AR114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AS114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -16670,6 +17015,9 @@
       <c r="AR115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AS115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -16810,6 +17158,9 @@
       <c r="AR116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AS116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -16950,6 +17301,9 @@
       <c r="AR117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AS117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -17090,6 +17444,9 @@
       <c r="AR118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AS118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -17230,6 +17587,9 @@
       <c r="AR119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AS119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -17370,6 +17730,9 @@
       <c r="AR120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AS120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -17510,6 +17873,9 @@
       <c r="AR121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AS121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -17650,6 +18016,9 @@
       <c r="AR122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AS122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -17790,6 +18159,9 @@
       <c r="AR123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AS123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -17930,6 +18302,9 @@
       <c r="AR124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AS124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -18070,6 +18445,9 @@
       <c r="AR125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AS125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -18210,6 +18588,9 @@
       <c r="AR126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AS126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -18350,6 +18731,9 @@
       <c r="AR127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AS127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -18490,6 +18874,9 @@
       <c r="AR128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AS128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -18630,6 +19017,9 @@
       <c r="AR129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AS129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -18770,6 +19160,9 @@
       <c r="AR130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AS130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -18910,6 +19303,9 @@
       <c r="AR131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AS131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -19050,6 +19446,9 @@
       <c r="AR132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AS132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -19190,6 +19589,9 @@
       <c r="AR133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AS133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -19330,6 +19732,9 @@
       <c r="AR134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AS134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -19470,6 +19875,9 @@
       <c r="AR135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AS135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -19610,6 +20018,9 @@
       <c r="AR136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AS136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -19750,6 +20161,9 @@
       <c r="AR137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AS137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -19890,6 +20304,9 @@
       <c r="AR138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AS138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -20030,6 +20447,9 @@
       <c r="AR139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -20170,6 +20590,9 @@
       <c r="AR140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -20310,6 +20733,9 @@
       <c r="AR141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -20450,6 +20876,9 @@
       <c r="AR142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -20590,6 +21019,9 @@
       <c r="AR143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -20730,6 +21162,9 @@
       <c r="AR144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AS144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -20870,6 +21305,9 @@
       <c r="AR145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AS145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -21010,6 +21448,9 @@
       <c r="AR146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AS146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -21150,6 +21591,9 @@
       <c r="AR147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AS147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -21290,6 +21734,9 @@
       <c r="AR148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AS148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -21430,6 +21877,9 @@
       <c r="AR149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AS149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -21570,6 +22020,9 @@
       <c r="AR150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AS150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -21710,6 +22163,9 @@
       <c r="AR151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AS151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -21850,6 +22306,9 @@
       <c r="AR152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AS152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -21990,6 +22449,9 @@
       <c r="AR153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AS153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -22130,6 +22592,9 @@
       <c r="AR154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AS154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -22270,6 +22735,9 @@
       <c r="AR155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AS155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -22410,6 +22878,9 @@
       <c r="AR156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AS156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -22550,6 +23021,9 @@
       <c r="AR157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AS157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -22690,6 +23164,9 @@
       <c r="AR158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AS158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -22830,6 +23307,9 @@
       <c r="AR159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AS159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -22970,6 +23450,9 @@
       <c r="AR160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AS160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -23110,6 +23593,9 @@
       <c r="AR161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AS161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -23250,6 +23736,9 @@
       <c r="AR162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AS162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -23390,6 +23879,9 @@
       <c r="AR163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AS163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -23530,6 +24022,9 @@
       <c r="AR164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AS164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -23571,9 +24066,12 @@
       <c r="AR165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AS165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AR165"/>
+  <autoFilter ref="A1:AS165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-09 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AS$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AT$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS165"/>
+  <dimension ref="A1:AT165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,7 @@
     <col width="16" customWidth="1" min="43" max="43"/>
     <col width="16" customWidth="1" min="44" max="44"/>
     <col width="16" customWidth="1" min="45" max="45"/>
+    <col width="16" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -716,6 +717,11 @@
           <t>2026-09-09 13:11</t>
         </is>
       </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -859,6 +865,9 @@
       <c r="AS2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AT2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1002,6 +1011,9 @@
       <c r="AS3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AT3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1145,6 +1157,9 @@
       <c r="AS4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AT4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1288,6 +1303,9 @@
       <c r="AS5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AT5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1431,6 +1449,9 @@
       <c r="AS6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AT6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1574,6 +1595,9 @@
       <c r="AS7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AT7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1717,6 +1741,9 @@
       <c r="AS8" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AT8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1860,6 +1887,9 @@
       <c r="AS9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AT9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2003,6 +2033,9 @@
       <c r="AS10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AT10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2146,6 +2179,9 @@
       <c r="AS11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AT11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2289,6 +2325,9 @@
       <c r="AS12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2432,6 +2471,9 @@
       <c r="AS13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AT13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2575,6 +2617,9 @@
       <c r="AS14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AT14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2718,6 +2763,9 @@
       <c r="AS15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AT15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2861,6 +2909,9 @@
       <c r="AS16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AT16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3004,6 +3055,9 @@
       <c r="AS17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AT17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3147,6 +3201,9 @@
       <c r="AS18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AT18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3290,6 +3347,9 @@
       <c r="AS19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AT19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3433,6 +3493,9 @@
       <c r="AS20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AT20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3576,6 +3639,9 @@
       <c r="AS21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AT21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3719,6 +3785,9 @@
       <c r="AS22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3862,6 +3931,9 @@
       <c r="AS23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AT23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4005,6 +4077,9 @@
       <c r="AS24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AT24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4148,6 +4223,9 @@
       <c r="AS25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4291,6 +4369,9 @@
       <c r="AS26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AT26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4434,6 +4515,9 @@
       <c r="AS27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AT27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4577,6 +4661,9 @@
       <c r="AS28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AT28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4720,6 +4807,9 @@
       <c r="AS29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AT29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4863,6 +4953,9 @@
       <c r="AS30" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AT30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5006,6 +5099,9 @@
       <c r="AS31" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AT31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5149,6 +5245,9 @@
       <c r="AS32" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AT32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5292,6 +5391,9 @@
       <c r="AS33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AT33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5435,6 +5537,9 @@
       <c r="AS34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5578,6 +5683,9 @@
       <c r="AS35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AT35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5721,6 +5829,9 @@
       <c r="AS36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AT36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5864,6 +5975,9 @@
       <c r="AS37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AT37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6007,6 +6121,9 @@
       <c r="AS38" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AT38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6150,6 +6267,9 @@
       <c r="AS39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AT39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6293,6 +6413,9 @@
       <c r="AS40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6436,6 +6559,9 @@
       <c r="AS41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6579,6 +6705,9 @@
       <c r="AS42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6722,6 +6851,9 @@
       <c r="AS43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AT43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6865,6 +6997,9 @@
       <c r="AS44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7008,6 +7143,9 @@
       <c r="AS45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7151,6 +7289,9 @@
       <c r="AS46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AT46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7294,6 +7435,9 @@
       <c r="AS47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AT47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7437,6 +7581,9 @@
       <c r="AS48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AT48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7580,6 +7727,9 @@
       <c r="AS49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AT49" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7723,6 +7873,9 @@
       <c r="AS50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AT50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -7866,6 +8019,9 @@
       <c r="AS51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AT51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8009,6 +8165,9 @@
       <c r="AS52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AT52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8152,6 +8311,9 @@
       <c r="AS53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AT53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8295,6 +8457,9 @@
       <c r="AS54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AT54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8438,6 +8603,9 @@
       <c r="AS55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AT55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8581,6 +8749,9 @@
       <c r="AS56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AT56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8724,6 +8895,9 @@
       <c r="AS57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8867,6 +9041,9 @@
       <c r="AS58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AT58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9010,6 +9187,9 @@
       <c r="AS59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AT59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -9153,6 +9333,9 @@
       <c r="AS60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AT60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -9296,6 +9479,9 @@
       <c r="AS61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AT61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -9439,6 +9625,9 @@
       <c r="AS62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AT62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9582,6 +9771,9 @@
       <c r="AS63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AT63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -9725,6 +9917,9 @@
       <c r="AS64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AT64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -9868,6 +10063,9 @@
       <c r="AS65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10011,6 +10209,9 @@
       <c r="AS66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -10154,6 +10355,9 @@
       <c r="AS67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AT67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -10297,6 +10501,9 @@
       <c r="AS68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10440,6 +10647,9 @@
       <c r="AS69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AT69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -10583,6 +10793,9 @@
       <c r="AS70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -10726,6 +10939,9 @@
       <c r="AS71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -10869,6 +11085,9 @@
       <c r="AS72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11012,6 +11231,9 @@
       <c r="AS73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AT73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -11155,6 +11377,9 @@
       <c r="AS74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AT74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11298,6 +11523,9 @@
       <c r="AS75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -11441,6 +11669,9 @@
       <c r="AS76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -11584,6 +11815,9 @@
       <c r="AS77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11727,6 +11961,9 @@
       <c r="AS78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -11870,6 +12107,9 @@
       <c r="AS79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -12013,6 +12253,9 @@
       <c r="AS80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AT80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -12156,6 +12399,9 @@
       <c r="AS81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -12299,6 +12545,9 @@
       <c r="AS82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -12442,6 +12691,9 @@
       <c r="AS83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -12585,6 +12837,9 @@
       <c r="AS84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AT84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -12728,6 +12983,9 @@
       <c r="AS85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AT85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -12871,6 +13129,9 @@
       <c r="AS86" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AT86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -13014,6 +13275,9 @@
       <c r="AS87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -13157,6 +13421,9 @@
       <c r="AS88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -13300,6 +13567,9 @@
       <c r="AS89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -13443,6 +13713,9 @@
       <c r="AS90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -13586,6 +13859,9 @@
       <c r="AS91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -13729,6 +14005,9 @@
       <c r="AS92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -13872,6 +14151,9 @@
       <c r="AS93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AT93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14015,6 +14297,9 @@
       <c r="AS94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AT94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -14158,6 +14443,9 @@
       <c r="AS95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AT95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14301,6 +14589,9 @@
       <c r="AS96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AT96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -14444,6 +14735,9 @@
       <c r="AS97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AT97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -14587,6 +14881,9 @@
       <c r="AS98" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AT98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -14730,6 +15027,9 @@
       <c r="AS99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -14873,6 +15173,9 @@
       <c r="AS100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AT100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -15016,6 +15319,9 @@
       <c r="AS101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AT101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -15159,6 +15465,9 @@
       <c r="AS102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AT102" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -15302,6 +15611,9 @@
       <c r="AS103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AT103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -15445,6 +15757,9 @@
       <c r="AS104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AT104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -15588,6 +15903,9 @@
       <c r="AS105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AT105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -15731,6 +16049,9 @@
       <c r="AS106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AT106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -15874,6 +16195,9 @@
       <c r="AS107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AT107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -16017,6 +16341,9 @@
       <c r="AS108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -16160,6 +16487,9 @@
       <c r="AS109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT109" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -16303,6 +16633,9 @@
       <c r="AS110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AT110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -16446,6 +16779,9 @@
       <c r="AS111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AT111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -16589,6 +16925,9 @@
       <c r="AS112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AT112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -16732,6 +17071,9 @@
       <c r="AS113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AT113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -16875,6 +17217,9 @@
       <c r="AS114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AT114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -17018,6 +17363,9 @@
       <c r="AS115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AT115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -17161,6 +17509,9 @@
       <c r="AS116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AT116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -17304,6 +17655,9 @@
       <c r="AS117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AT117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -17447,6 +17801,9 @@
       <c r="AS118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AT118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -17590,6 +17947,9 @@
       <c r="AS119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AT119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -17733,6 +18093,9 @@
       <c r="AS120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AT120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -17876,6 +18239,9 @@
       <c r="AS121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AT121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -18019,6 +18385,9 @@
       <c r="AS122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AT122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -18162,6 +18531,9 @@
       <c r="AS123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AT123" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -18305,6 +18677,9 @@
       <c r="AS124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AT124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -18448,6 +18823,9 @@
       <c r="AS125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AT125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -18591,6 +18969,9 @@
       <c r="AS126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AT126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -18734,6 +19115,9 @@
       <c r="AS127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AT127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -18877,6 +19261,9 @@
       <c r="AS128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AT128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -19020,6 +19407,9 @@
       <c r="AS129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AT129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -19163,6 +19553,9 @@
       <c r="AS130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AT130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -19306,6 +19699,9 @@
       <c r="AS131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AT131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -19449,6 +19845,9 @@
       <c r="AS132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AT132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -19592,6 +19991,9 @@
       <c r="AS133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AT133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -19735,6 +20137,9 @@
       <c r="AS134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AT134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -19878,6 +20283,9 @@
       <c r="AS135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AT135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -20021,6 +20429,9 @@
       <c r="AS136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AT136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -20164,6 +20575,9 @@
       <c r="AS137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AT137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -20307,6 +20721,9 @@
       <c r="AS138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AT138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -20450,6 +20867,9 @@
       <c r="AS139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -20593,6 +21013,9 @@
       <c r="AS140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -20736,6 +21159,9 @@
       <c r="AS141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -20879,6 +21305,9 @@
       <c r="AS142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -21022,6 +21451,9 @@
       <c r="AS143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -21165,6 +21597,9 @@
       <c r="AS144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AT144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -21308,6 +21743,9 @@
       <c r="AS145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AT145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -21451,6 +21889,9 @@
       <c r="AS146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AT146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -21594,6 +22035,9 @@
       <c r="AS147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AT147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -21737,6 +22181,9 @@
       <c r="AS148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AT148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -21880,6 +22327,9 @@
       <c r="AS149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AT149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -22023,6 +22473,9 @@
       <c r="AS150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AT150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -22166,6 +22619,9 @@
       <c r="AS151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AT151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -22309,6 +22765,9 @@
       <c r="AS152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AT152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -22452,6 +22911,9 @@
       <c r="AS153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AT153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -22595,6 +23057,9 @@
       <c r="AS154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AT154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -22738,6 +23203,9 @@
       <c r="AS155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AT155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -22881,6 +23349,9 @@
       <c r="AS156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AT156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -23024,6 +23495,9 @@
       <c r="AS157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AT157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -23167,6 +23641,9 @@
       <c r="AS158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AT158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -23310,6 +23787,9 @@
       <c r="AS159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AT159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -23453,6 +23933,9 @@
       <c r="AS160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AT160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -23596,6 +24079,9 @@
       <c r="AS161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AT161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -23739,6 +24225,9 @@
       <c r="AS162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AT162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -23882,6 +24371,9 @@
       <c r="AS163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AT163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -24025,6 +24517,9 @@
       <c r="AS164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AT164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -24069,9 +24564,12 @@
       <c r="AS165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AT165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AS165"/>
+  <autoFilter ref="A1:AT165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 00:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AT$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AU$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT165"/>
+  <dimension ref="A1:AU165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -489,6 +489,7 @@
     <col width="16" customWidth="1" min="44" max="44"/>
     <col width="16" customWidth="1" min="45" max="45"/>
     <col width="16" customWidth="1" min="46" max="46"/>
+    <col width="16" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -722,6 +723,11 @@
           <t>2026-09-09 16:08</t>
         </is>
       </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 19:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -868,6 +874,9 @@
       <c r="AT2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AU2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1014,6 +1023,9 @@
       <c r="AT3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AU3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1160,6 +1172,9 @@
       <c r="AT4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AU4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1306,6 +1321,9 @@
       <c r="AT5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AU5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1452,6 +1470,9 @@
       <c r="AT6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AU6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1598,6 +1619,9 @@
       <c r="AT7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AU7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1744,6 +1768,9 @@
       <c r="AT8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AU8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1890,6 +1917,9 @@
       <c r="AT9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AU9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2036,6 +2066,9 @@
       <c r="AT10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AU10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2182,6 +2215,9 @@
       <c r="AT11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AU11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2328,6 +2364,9 @@
       <c r="AT12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2474,6 +2513,9 @@
       <c r="AT13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AU13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2620,6 +2662,9 @@
       <c r="AT14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AU14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2766,6 +2811,9 @@
       <c r="AT15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AU15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2912,6 +2960,9 @@
       <c r="AT16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AU16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3058,6 +3109,9 @@
       <c r="AT17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AU17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3204,6 +3258,9 @@
       <c r="AT18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AU18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3350,6 +3407,9 @@
       <c r="AT19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AU19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3496,6 +3556,9 @@
       <c r="AT20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AU20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3642,6 +3705,9 @@
       <c r="AT21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AU21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3788,6 +3854,9 @@
       <c r="AT22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3934,6 +4003,9 @@
       <c r="AT23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AU23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4080,6 +4152,9 @@
       <c r="AT24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AU24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4226,6 +4301,9 @@
       <c r="AT25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4372,6 +4450,9 @@
       <c r="AT26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AU26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4518,6 +4599,9 @@
       <c r="AT27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AU27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4664,6 +4748,9 @@
       <c r="AT28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AU28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4810,6 +4897,9 @@
       <c r="AT29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AU29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4956,6 +5046,9 @@
       <c r="AT30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5102,6 +5195,9 @@
       <c r="AT31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5248,6 +5344,9 @@
       <c r="AT32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5394,6 +5493,9 @@
       <c r="AT33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5540,6 +5642,9 @@
       <c r="AT34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5686,6 +5791,9 @@
       <c r="AT35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AU35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5832,6 +5940,9 @@
       <c r="AT36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AU36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5978,6 +6089,9 @@
       <c r="AT37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AU37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6124,6 +6238,9 @@
       <c r="AT38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AU38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6270,6 +6387,9 @@
       <c r="AT39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AU39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6416,6 +6536,9 @@
       <c r="AT40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6562,6 +6685,9 @@
       <c r="AT41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6708,6 +6834,9 @@
       <c r="AT42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6854,6 +6983,9 @@
       <c r="AT43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7000,6 +7132,9 @@
       <c r="AT44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7146,6 +7281,9 @@
       <c r="AT45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7292,6 +7430,9 @@
       <c r="AT46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AU46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7438,6 +7579,9 @@
       <c r="AT47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AU47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7584,6 +7728,9 @@
       <c r="AT48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AU48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7730,6 +7877,9 @@
       <c r="AT49" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AU49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -7876,6 +8026,9 @@
       <c r="AT50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AU50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8022,6 +8175,9 @@
       <c r="AT51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AU51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8168,6 +8324,9 @@
       <c r="AT52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AU52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8314,6 +8473,9 @@
       <c r="AT53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AU53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8460,6 +8622,9 @@
       <c r="AT54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AU54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8606,6 +8771,9 @@
       <c r="AT55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AU55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8752,6 +8920,9 @@
       <c r="AT56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AU56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8898,6 +9069,9 @@
       <c r="AT57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AU57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9044,6 +9218,9 @@
       <c r="AT58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AU58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9190,6 +9367,9 @@
       <c r="AT59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AU59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -9336,6 +9516,9 @@
       <c r="AT60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AU60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -9482,6 +9665,9 @@
       <c r="AT61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AU61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -9628,6 +9814,9 @@
       <c r="AT62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9774,6 +9963,9 @@
       <c r="AT63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -9920,6 +10112,9 @@
       <c r="AT64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10066,6 +10261,9 @@
       <c r="AT65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10212,6 +10410,9 @@
       <c r="AT66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -10358,6 +10559,9 @@
       <c r="AT67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AU67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -10504,6 +10708,9 @@
       <c r="AT68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10650,6 +10857,9 @@
       <c r="AT69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AU69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -10796,6 +11006,9 @@
       <c r="AT70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -10942,6 +11155,9 @@
       <c r="AT71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11088,6 +11304,9 @@
       <c r="AT72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AU72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11234,6 +11453,9 @@
       <c r="AT73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AU73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -11380,6 +11602,9 @@
       <c r="AT74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AU74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11526,6 +11751,9 @@
       <c r="AT75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -11672,6 +11900,9 @@
       <c r="AT76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -11818,6 +12049,9 @@
       <c r="AT77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11964,6 +12198,9 @@
       <c r="AT78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -12110,6 +12347,9 @@
       <c r="AT79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -12256,6 +12496,9 @@
       <c r="AT80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AU80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -12402,6 +12645,9 @@
       <c r="AT81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -12548,6 +12794,9 @@
       <c r="AT82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -12694,6 +12943,9 @@
       <c r="AT83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -12840,6 +13092,9 @@
       <c r="AT84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AU84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -12986,6 +13241,9 @@
       <c r="AT85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AU85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -13132,6 +13390,9 @@
       <c r="AT86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AU86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -13278,6 +13539,9 @@
       <c r="AT87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -13424,6 +13688,9 @@
       <c r="AT88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -13570,6 +13837,9 @@
       <c r="AT89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -13716,6 +13986,9 @@
       <c r="AT90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -13862,6 +14135,9 @@
       <c r="AT91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14008,6 +14284,9 @@
       <c r="AT92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -14154,6 +14433,9 @@
       <c r="AT93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AU93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14300,6 +14582,9 @@
       <c r="AT94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AU94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -14446,6 +14731,9 @@
       <c r="AT95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AU95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14592,6 +14880,9 @@
       <c r="AT96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AU96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -14738,6 +15029,9 @@
       <c r="AT97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AU97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -14884,6 +15178,9 @@
       <c r="AT98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AU98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -15030,6 +15327,9 @@
       <c r="AT99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -15176,6 +15476,9 @@
       <c r="AT100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AU100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -15322,6 +15625,9 @@
       <c r="AT101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AU101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -15468,6 +15774,9 @@
       <c r="AT102" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AU102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -15614,6 +15923,9 @@
       <c r="AT103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AU103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -15760,6 +16072,9 @@
       <c r="AT104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AU104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -15906,6 +16221,9 @@
       <c r="AT105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AU105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -16052,6 +16370,9 @@
       <c r="AT106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AU106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -16198,6 +16519,9 @@
       <c r="AT107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AU107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -16344,6 +16668,9 @@
       <c r="AT108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -16490,6 +16817,9 @@
       <c r="AT109" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -16636,6 +16966,9 @@
       <c r="AT110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AU110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -16782,6 +17115,9 @@
       <c r="AT111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AU111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -16928,6 +17264,9 @@
       <c r="AT112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AU112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -17074,6 +17413,9 @@
       <c r="AT113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AU113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -17220,6 +17562,9 @@
       <c r="AT114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AU114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -17366,6 +17711,9 @@
       <c r="AT115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AU115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -17512,6 +17860,9 @@
       <c r="AT116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AU116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -17658,6 +18009,9 @@
       <c r="AT117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AU117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -17804,6 +18158,9 @@
       <c r="AT118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AU118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -17950,6 +18307,9 @@
       <c r="AT119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AU119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -18096,6 +18456,9 @@
       <c r="AT120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AU120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -18242,6 +18605,9 @@
       <c r="AT121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AU121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -18388,6 +18754,9 @@
       <c r="AT122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AU122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -18534,6 +18903,9 @@
       <c r="AT123" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AU123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -18680,6 +19052,9 @@
       <c r="AT124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AU124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -18826,6 +19201,9 @@
       <c r="AT125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AU125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -18972,6 +19350,9 @@
       <c r="AT126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AU126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -19118,6 +19499,9 @@
       <c r="AT127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AU127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -19264,6 +19648,9 @@
       <c r="AT128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AU128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -19410,6 +19797,9 @@
       <c r="AT129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AU129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -19556,6 +19946,9 @@
       <c r="AT130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AU130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -19702,6 +20095,9 @@
       <c r="AT131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AU131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -19848,6 +20244,9 @@
       <c r="AT132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AU132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -19994,6 +20393,9 @@
       <c r="AT133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AU133" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -20140,6 +20542,9 @@
       <c r="AT134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AU134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -20286,6 +20691,9 @@
       <c r="AT135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AU135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -20432,6 +20840,9 @@
       <c r="AT136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AU136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -20578,6 +20989,9 @@
       <c r="AT137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AU137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -20724,6 +21138,9 @@
       <c r="AT138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AU138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -20870,6 +21287,9 @@
       <c r="AT139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -21016,6 +21436,9 @@
       <c r="AT140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -21162,6 +21585,9 @@
       <c r="AT141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -21308,6 +21734,9 @@
       <c r="AT142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -21454,6 +21883,9 @@
       <c r="AT143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -21600,6 +22032,9 @@
       <c r="AT144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AU144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -21746,6 +22181,9 @@
       <c r="AT145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AU145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -21892,6 +22330,9 @@
       <c r="AT146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AU146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -22038,6 +22479,9 @@
       <c r="AT147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AU147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -22184,6 +22628,9 @@
       <c r="AT148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AU148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -22330,6 +22777,9 @@
       <c r="AT149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AU149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -22476,6 +22926,9 @@
       <c r="AT150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AU150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -22622,6 +23075,9 @@
       <c r="AT151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AU151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -22768,6 +23224,9 @@
       <c r="AT152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AU152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -22914,6 +23373,9 @@
       <c r="AT153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AU153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -23060,6 +23522,9 @@
       <c r="AT154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AU154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -23206,6 +23671,9 @@
       <c r="AT155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AU155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -23352,6 +23820,9 @@
       <c r="AT156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AU156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -23498,6 +23969,9 @@
       <c r="AT157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AU157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -23644,6 +24118,9 @@
       <c r="AT158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AU158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -23790,6 +24267,9 @@
       <c r="AT159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AU159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -23936,6 +24416,9 @@
       <c r="AT160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AU160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -24082,6 +24565,9 @@
       <c r="AT161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AU161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -24228,6 +24714,9 @@
       <c r="AT162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AU162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -24374,6 +24863,9 @@
       <c r="AT163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AU163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -24520,6 +25012,9 @@
       <c r="AT164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AU164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -24567,9 +25062,12 @@
       <c r="AT165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AU165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AT165"/>
+  <autoFilter ref="A1:AU165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 03:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AU$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AV$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU165"/>
+  <dimension ref="A1:AV165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -490,6 +490,7 @@
     <col width="16" customWidth="1" min="45" max="45"/>
     <col width="16" customWidth="1" min="46" max="46"/>
     <col width="16" customWidth="1" min="47" max="47"/>
+    <col width="16" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -728,6 +729,11 @@
           <t>2026-09-09 19:12</t>
         </is>
       </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -877,6 +883,9 @@
       <c r="AU2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AV2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1026,6 +1035,9 @@
       <c r="AU3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AV3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1175,6 +1187,9 @@
       <c r="AU4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AV4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1324,6 +1339,9 @@
       <c r="AU5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AV5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1473,6 +1491,9 @@
       <c r="AU6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AV6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1622,6 +1643,9 @@
       <c r="AU7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AV7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1771,6 +1795,9 @@
       <c r="AU8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AV8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1920,6 +1947,9 @@
       <c r="AU9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AV9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2069,6 +2099,9 @@
       <c r="AU10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AV10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2218,6 +2251,9 @@
       <c r="AU11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AV11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2367,6 +2403,9 @@
       <c r="AU12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2516,6 +2555,9 @@
       <c r="AU13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AV13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2665,6 +2707,9 @@
       <c r="AU14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AV14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2814,6 +2859,9 @@
       <c r="AU15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AV15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2963,6 +3011,9 @@
       <c r="AU16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AV16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3112,6 +3163,9 @@
       <c r="AU17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AV17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3261,6 +3315,9 @@
       <c r="AU18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AV18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3410,6 +3467,9 @@
       <c r="AU19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AV19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3559,6 +3619,9 @@
       <c r="AU20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AV20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3708,6 +3771,9 @@
       <c r="AU21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AV21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3857,6 +3923,9 @@
       <c r="AU22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4006,6 +4075,9 @@
       <c r="AU23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AV23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4155,6 +4227,9 @@
       <c r="AU24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AV24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4304,6 +4379,9 @@
       <c r="AU25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4453,6 +4531,9 @@
       <c r="AU26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AV26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4602,6 +4683,9 @@
       <c r="AU27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AV27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4751,6 +4835,9 @@
       <c r="AU28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AV28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4900,6 +4987,9 @@
       <c r="AU29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AV29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5049,6 +5139,9 @@
       <c r="AU30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5198,6 +5291,9 @@
       <c r="AU31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5347,6 +5443,9 @@
       <c r="AU32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5496,6 +5595,9 @@
       <c r="AU33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5645,6 +5747,9 @@
       <c r="AU34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5794,6 +5899,9 @@
       <c r="AU35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AV35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5943,6 +6051,9 @@
       <c r="AU36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AV36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6092,6 +6203,9 @@
       <c r="AU37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AV37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6241,6 +6355,9 @@
       <c r="AU38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AV38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6390,6 +6507,9 @@
       <c r="AU39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AV39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6539,6 +6659,9 @@
       <c r="AU40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6688,6 +6811,9 @@
       <c r="AU41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6837,6 +6963,9 @@
       <c r="AU42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -6986,6 +7115,9 @@
       <c r="AU43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7135,6 +7267,9 @@
       <c r="AU44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7284,6 +7419,9 @@
       <c r="AU45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7433,6 +7571,9 @@
       <c r="AU46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AV46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7582,6 +7723,9 @@
       <c r="AU47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AV47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7731,6 +7875,9 @@
       <c r="AU48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AV48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7880,6 +8027,9 @@
       <c r="AU49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AV49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8029,6 +8179,9 @@
       <c r="AU50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AV50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8178,6 +8331,9 @@
       <c r="AU51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AV51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8327,6 +8483,9 @@
       <c r="AU52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AV52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8476,6 +8635,9 @@
       <c r="AU53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AV53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8625,6 +8787,9 @@
       <c r="AU54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AV54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8774,6 +8939,9 @@
       <c r="AU55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AV55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8923,6 +9091,9 @@
       <c r="AU56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AV56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9072,6 +9243,9 @@
       <c r="AU57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AV57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9221,6 +9395,9 @@
       <c r="AU58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AV58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9370,6 +9547,9 @@
       <c r="AU59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AV59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -9519,6 +9699,9 @@
       <c r="AU60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AV60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -9668,6 +9851,9 @@
       <c r="AU61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AV61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -9817,6 +10003,9 @@
       <c r="AU62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -9966,6 +10155,9 @@
       <c r="AU63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10115,6 +10307,9 @@
       <c r="AU64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10264,6 +10459,9 @@
       <c r="AU65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10413,6 +10611,9 @@
       <c r="AU66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -10562,6 +10763,9 @@
       <c r="AU67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AV67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -10711,6 +10915,9 @@
       <c r="AU68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10860,6 +11067,9 @@
       <c r="AU69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AV69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11009,6 +11219,9 @@
       <c r="AU70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -11158,6 +11371,9 @@
       <c r="AU71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11307,6 +11523,9 @@
       <c r="AU72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AV72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11456,6 +11675,9 @@
       <c r="AU73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AV73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -11605,6 +11827,9 @@
       <c r="AU74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AV74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11754,6 +11979,9 @@
       <c r="AU75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -11903,6 +12131,9 @@
       <c r="AU76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -12052,6 +12283,9 @@
       <c r="AU77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -12201,6 +12435,9 @@
       <c r="AU78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -12350,6 +12587,9 @@
       <c r="AU79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -12499,6 +12739,9 @@
       <c r="AU80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AV80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -12648,6 +12891,9 @@
       <c r="AU81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -12797,6 +13043,9 @@
       <c r="AU82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -12946,6 +13195,9 @@
       <c r="AU83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13095,6 +13347,9 @@
       <c r="AU84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AV84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -13244,6 +13499,9 @@
       <c r="AU85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AV85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -13393,6 +13651,9 @@
       <c r="AU86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AV86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -13542,6 +13803,9 @@
       <c r="AU87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -13691,6 +13955,9 @@
       <c r="AU88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -13840,6 +14107,9 @@
       <c r="AU89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -13989,6 +14259,9 @@
       <c r="AU90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -14138,6 +14411,9 @@
       <c r="AU91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14287,6 +14563,9 @@
       <c r="AU92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -14436,6 +14715,9 @@
       <c r="AU93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AV93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14585,6 +14867,9 @@
       <c r="AU94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AV94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -14734,6 +15019,9 @@
       <c r="AU95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AV95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -14883,6 +15171,9 @@
       <c r="AU96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AV96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -15032,6 +15323,9 @@
       <c r="AU97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AV97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -15181,6 +15475,9 @@
       <c r="AU98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AV98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -15330,6 +15627,9 @@
       <c r="AU99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -15479,6 +15779,9 @@
       <c r="AU100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AV100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -15628,6 +15931,9 @@
       <c r="AU101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AV101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -15777,6 +16083,9 @@
       <c r="AU102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AV102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -15926,6 +16235,9 @@
       <c r="AU103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AV103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -16075,6 +16387,9 @@
       <c r="AU104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AV104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -16224,6 +16539,9 @@
       <c r="AU105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AV105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -16373,6 +16691,9 @@
       <c r="AU106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AV106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -16522,6 +16843,9 @@
       <c r="AU107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AV107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -16671,6 +16995,9 @@
       <c r="AU108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -16820,6 +17147,9 @@
       <c r="AU109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AV109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -16969,6 +17299,9 @@
       <c r="AU110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AV110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -17118,6 +17451,9 @@
       <c r="AU111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AV111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -17267,6 +17603,9 @@
       <c r="AU112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AV112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -17416,6 +17755,9 @@
       <c r="AU113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AV113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -17565,6 +17907,9 @@
       <c r="AU114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AV114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -17714,6 +18059,9 @@
       <c r="AU115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AV115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -17863,6 +18211,9 @@
       <c r="AU116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AV116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -18012,6 +18363,9 @@
       <c r="AU117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AV117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -18161,6 +18515,9 @@
       <c r="AU118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AV118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -18310,6 +18667,9 @@
       <c r="AU119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AV119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -18459,6 +18819,9 @@
       <c r="AU120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AV120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -18608,6 +18971,9 @@
       <c r="AU121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AV121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -18757,6 +19123,9 @@
       <c r="AU122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AV122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -18906,6 +19275,9 @@
       <c r="AU123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="AV123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -19055,6 +19427,9 @@
       <c r="AU124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AV124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -19204,6 +19579,9 @@
       <c r="AU125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AV125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -19353,6 +19731,9 @@
       <c r="AU126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AV126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -19502,6 +19883,9 @@
       <c r="AU127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AV127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -19651,6 +20035,9 @@
       <c r="AU128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AV128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -19800,6 +20187,9 @@
       <c r="AU129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AV129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -19949,6 +20339,9 @@
       <c r="AU130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AV130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -20098,6 +20491,9 @@
       <c r="AU131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AV131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -20247,6 +20643,9 @@
       <c r="AU132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AV132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -20396,6 +20795,9 @@
       <c r="AU133" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AV133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -20545,6 +20947,9 @@
       <c r="AU134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AV134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -20694,6 +21099,9 @@
       <c r="AU135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AV135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -20843,6 +21251,9 @@
       <c r="AU136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AV136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -20992,6 +21403,9 @@
       <c r="AU137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AV137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -21141,6 +21555,9 @@
       <c r="AU138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AV138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -21290,6 +21707,9 @@
       <c r="AU139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -21439,6 +21859,9 @@
       <c r="AU140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -21588,6 +22011,9 @@
       <c r="AU141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -21737,6 +22163,9 @@
       <c r="AU142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -21886,6 +22315,9 @@
       <c r="AU143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -22035,6 +22467,9 @@
       <c r="AU144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AV144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -22184,6 +22619,9 @@
       <c r="AU145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AV145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -22333,6 +22771,9 @@
       <c r="AU146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AV146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -22482,6 +22923,9 @@
       <c r="AU147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AV147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -22631,6 +23075,9 @@
       <c r="AU148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AV148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -22780,6 +23227,9 @@
       <c r="AU149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AV149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -22929,6 +23379,9 @@
       <c r="AU150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AV150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -23078,6 +23531,9 @@
       <c r="AU151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AV151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -23227,6 +23683,9 @@
       <c r="AU152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AV152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -23376,6 +23835,9 @@
       <c r="AU153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AV153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -23525,6 +23987,9 @@
       <c r="AU154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AV154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -23674,6 +24139,9 @@
       <c r="AU155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AV155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -23823,6 +24291,9 @@
       <c r="AU156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AV156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -23972,6 +24443,9 @@
       <c r="AU157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AV157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -24121,6 +24595,9 @@
       <c r="AU158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AV158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -24270,6 +24747,9 @@
       <c r="AU159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AV159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -24419,6 +24899,9 @@
       <c r="AU160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AV160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -24568,6 +25051,9 @@
       <c r="AU161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AV161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -24717,6 +25203,9 @@
       <c r="AU162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AV162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -24866,6 +25355,9 @@
       <c r="AU163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AV163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -25015,6 +25507,9 @@
       <c r="AU164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AV164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -25065,9 +25560,12 @@
       <c r="AU165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AV165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AU165"/>
+  <autoFilter ref="A1:AV165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 06:13 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AV$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AW$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV165"/>
+  <dimension ref="A1:AW165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -491,6 +491,7 @@
     <col width="16" customWidth="1" min="46" max="46"/>
     <col width="16" customWidth="1" min="47" max="47"/>
     <col width="16" customWidth="1" min="48" max="48"/>
+    <col width="16" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -734,6 +735,11 @@
           <t>2026-09-09 22:09</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -886,6 +892,9 @@
       <c r="AV2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AW2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1038,6 +1047,9 @@
       <c r="AV3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AW3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1190,6 +1202,9 @@
       <c r="AV4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AW4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1342,6 +1357,9 @@
       <c r="AV5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AW5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1494,6 +1512,9 @@
       <c r="AV6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AW6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1646,6 +1667,9 @@
       <c r="AV7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AW7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1798,6 +1822,9 @@
       <c r="AV8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AW8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1950,6 +1977,9 @@
       <c r="AV9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AW9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2102,6 +2132,9 @@
       <c r="AV10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AW10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2254,6 +2287,9 @@
       <c r="AV11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AW11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2406,6 +2442,9 @@
       <c r="AV12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2558,6 +2597,9 @@
       <c r="AV13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AW13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2710,6 +2752,9 @@
       <c r="AV14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AW14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2862,6 +2907,9 @@
       <c r="AV15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AW15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3014,6 +3062,9 @@
       <c r="AV16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AW16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3166,6 +3217,9 @@
       <c r="AV17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AW17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3318,6 +3372,9 @@
       <c r="AV18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AW18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3470,6 +3527,9 @@
       <c r="AV19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AW19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3622,6 +3682,9 @@
       <c r="AV20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AW20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3774,6 +3837,9 @@
       <c r="AV21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AW21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3926,6 +3992,9 @@
       <c r="AV22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4078,6 +4147,9 @@
       <c r="AV23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AW23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4230,6 +4302,9 @@
       <c r="AV24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AW24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4382,6 +4457,9 @@
       <c r="AV25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4534,6 +4612,9 @@
       <c r="AV26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AW26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4686,6 +4767,9 @@
       <c r="AV27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AW27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4838,6 +4922,9 @@
       <c r="AV28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AW28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4990,6 +5077,9 @@
       <c r="AV29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AW29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5142,6 +5232,9 @@
       <c r="AV30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5294,6 +5387,9 @@
       <c r="AV31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5446,6 +5542,9 @@
       <c r="AV32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5598,6 +5697,9 @@
       <c r="AV33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5750,6 +5852,9 @@
       <c r="AV34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -5902,6 +6007,9 @@
       <c r="AV35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AW35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6054,6 +6162,9 @@
       <c r="AV36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AW36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6206,6 +6317,9 @@
       <c r="AV37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AW37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6358,6 +6472,9 @@
       <c r="AV38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AW38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6510,6 +6627,9 @@
       <c r="AV39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AW39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6662,6 +6782,9 @@
       <c r="AV40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6814,6 +6937,9 @@
       <c r="AV41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -6966,6 +7092,9 @@
       <c r="AV42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7118,6 +7247,9 @@
       <c r="AV43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7270,6 +7402,9 @@
       <c r="AV44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7422,6 +7557,9 @@
       <c r="AV45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7574,6 +7712,9 @@
       <c r="AV46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AW46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7726,6 +7867,9 @@
       <c r="AV47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AW47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7878,6 +8022,9 @@
       <c r="AV48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AW48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8030,6 +8177,9 @@
       <c r="AV49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AW49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8182,6 +8332,9 @@
       <c r="AV50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AW50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8334,6 +8487,9 @@
       <c r="AV51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AW51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8486,6 +8642,9 @@
       <c r="AV52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AW52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8638,6 +8797,9 @@
       <c r="AV53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AW53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8790,6 +8952,9 @@
       <c r="AV54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AW54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8942,6 +9107,9 @@
       <c r="AV55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AW55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9094,6 +9262,9 @@
       <c r="AV56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AW56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9246,6 +9417,9 @@
       <c r="AV57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AW57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9398,6 +9572,9 @@
       <c r="AV58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AW58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9550,6 +9727,9 @@
       <c r="AV59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AW59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -9702,6 +9882,9 @@
       <c r="AV60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AW60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -9854,6 +10037,9 @@
       <c r="AV61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AW61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10006,6 +10192,9 @@
       <c r="AV62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10158,6 +10347,9 @@
       <c r="AV63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10310,6 +10502,9 @@
       <c r="AV64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10462,6 +10657,9 @@
       <c r="AV65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10614,6 +10812,9 @@
       <c r="AV66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -10766,6 +10967,9 @@
       <c r="AV67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AW67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -10918,6 +11122,9 @@
       <c r="AV68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -11070,6 +11277,9 @@
       <c r="AV69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AW69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11222,6 +11432,9 @@
       <c r="AV70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -11374,6 +11587,9 @@
       <c r="AV71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11526,6 +11742,9 @@
       <c r="AV72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AW72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11678,6 +11897,9 @@
       <c r="AV73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AW73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -11830,6 +12052,9 @@
       <c r="AV74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AW74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11982,6 +12207,9 @@
       <c r="AV75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -12134,6 +12362,9 @@
       <c r="AV76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -12286,6 +12517,9 @@
       <c r="AV77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -12438,6 +12672,9 @@
       <c r="AV78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -12590,6 +12827,9 @@
       <c r="AV79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -12742,6 +12982,9 @@
       <c r="AV80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AW80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -12894,6 +13137,9 @@
       <c r="AV81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13046,6 +13292,9 @@
       <c r="AV82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -13198,6 +13447,9 @@
       <c r="AV83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13350,6 +13602,9 @@
       <c r="AV84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AW84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -13502,6 +13757,9 @@
       <c r="AV85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AW85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -13654,6 +13912,9 @@
       <c r="AV86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AW86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -13806,6 +14067,9 @@
       <c r="AV87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -13958,6 +14222,9 @@
       <c r="AV88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -14110,6 +14377,9 @@
       <c r="AV89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -14262,6 +14532,9 @@
       <c r="AV90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -14414,6 +14687,9 @@
       <c r="AV91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14566,6 +14842,9 @@
       <c r="AV92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -14718,6 +14997,9 @@
       <c r="AV93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AW93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -14870,6 +15152,9 @@
       <c r="AV94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AW94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -15022,6 +15307,9 @@
       <c r="AV95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AW95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -15174,6 +15462,9 @@
       <c r="AV96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AW96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -15326,6 +15617,9 @@
       <c r="AV97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AW97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -15478,6 +15772,9 @@
       <c r="AV98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AW98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -15630,6 +15927,9 @@
       <c r="AV99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -15782,6 +16082,9 @@
       <c r="AV100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AW100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -15934,6 +16237,9 @@
       <c r="AV101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AW101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -16086,6 +16392,9 @@
       <c r="AV102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AW102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -16238,6 +16547,9 @@
       <c r="AV103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AW103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -16390,6 +16702,9 @@
       <c r="AV104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AW104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -16542,6 +16857,9 @@
       <c r="AV105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AW105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -16694,6 +17012,9 @@
       <c r="AV106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AW106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -16846,6 +17167,9 @@
       <c r="AV107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AW107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -16998,6 +17322,9 @@
       <c r="AV108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -17150,6 +17477,9 @@
       <c r="AV109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AW109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -17302,6 +17632,9 @@
       <c r="AV110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AW110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -17454,6 +17787,9 @@
       <c r="AV111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AW111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -17606,6 +17942,9 @@
       <c r="AV112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AW112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -17758,6 +18097,9 @@
       <c r="AV113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AW113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -17910,6 +18252,9 @@
       <c r="AV114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AW114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -18062,6 +18407,9 @@
       <c r="AV115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AW115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -18214,6 +18562,9 @@
       <c r="AV116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AW116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -18366,6 +18717,9 @@
       <c r="AV117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AW117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -18518,6 +18872,9 @@
       <c r="AV118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AW118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -18670,6 +19027,9 @@
       <c r="AV119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AW119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -18822,6 +19182,9 @@
       <c r="AV120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AW120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -18974,6 +19337,9 @@
       <c r="AV121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AW121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -19126,6 +19492,9 @@
       <c r="AV122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AW122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -19278,6 +19647,9 @@
       <c r="AV123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="AW123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -19430,6 +19802,9 @@
       <c r="AV124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AW124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -19582,6 +19957,9 @@
       <c r="AV125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AW125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -19734,6 +20112,9 @@
       <c r="AV126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AW126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -19886,6 +20267,9 @@
       <c r="AV127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AW127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -20038,6 +20422,9 @@
       <c r="AV128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AW128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -20190,6 +20577,9 @@
       <c r="AV129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AW129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -20342,6 +20732,9 @@
       <c r="AV130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AW130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -20494,6 +20887,9 @@
       <c r="AV131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AW131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -20646,6 +21042,9 @@
       <c r="AV132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AW132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -20798,6 +21197,9 @@
       <c r="AV133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AW133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -20950,6 +21352,9 @@
       <c r="AV134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AW134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -21102,6 +21507,9 @@
       <c r="AV135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AW135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -21254,6 +21662,9 @@
       <c r="AV136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AW136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -21406,6 +21817,9 @@
       <c r="AV137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AW137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -21558,6 +21972,9 @@
       <c r="AV138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AW138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -21710,6 +22127,9 @@
       <c r="AV139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -21862,6 +22282,9 @@
       <c r="AV140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -22014,6 +22437,9 @@
       <c r="AV141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -22166,6 +22592,9 @@
       <c r="AV142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -22318,6 +22747,9 @@
       <c r="AV143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -22470,6 +22902,9 @@
       <c r="AV144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AW144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -22622,6 +23057,9 @@
       <c r="AV145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AW145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -22774,6 +23212,9 @@
       <c r="AV146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AW146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -22926,6 +23367,9 @@
       <c r="AV147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AW147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -23078,6 +23522,9 @@
       <c r="AV148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AW148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -23230,6 +23677,9 @@
       <c r="AV149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AW149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -23382,6 +23832,9 @@
       <c r="AV150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AW150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -23534,6 +23987,9 @@
       <c r="AV151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AW151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -23686,6 +24142,9 @@
       <c r="AV152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AW152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -23838,6 +24297,9 @@
       <c r="AV153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AW153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -23990,6 +24452,9 @@
       <c r="AV154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AW154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -24142,6 +24607,9 @@
       <c r="AV155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AW155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -24294,6 +24762,9 @@
       <c r="AV156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AW156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -24446,6 +24917,9 @@
       <c r="AV157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AW157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -24598,6 +25072,9 @@
       <c r="AV158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AW158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -24750,6 +25227,9 @@
       <c r="AV159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AW159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -24902,6 +25382,9 @@
       <c r="AV160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AW160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -25054,6 +25537,9 @@
       <c r="AV161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AW161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -25206,6 +25692,9 @@
       <c r="AV162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AW162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -25358,6 +25847,9 @@
       <c r="AV163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AW163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -25510,6 +26002,9 @@
       <c r="AV164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AW164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -25563,9 +26058,12 @@
       <c r="AV165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AW165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV165"/>
+  <autoFilter ref="A1:AW165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AW$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AX$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW165"/>
+  <dimension ref="A1:AX165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -492,6 +492,7 @@
     <col width="16" customWidth="1" min="47" max="47"/>
     <col width="16" customWidth="1" min="48" max="48"/>
     <col width="16" customWidth="1" min="49" max="49"/>
+    <col width="16" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -740,6 +741,11 @@
           <t>2026-09-10 01:13</t>
         </is>
       </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -895,6 +901,9 @@
       <c r="AW2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AX2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1050,6 +1059,9 @@
       <c r="AW3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AX3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1205,6 +1217,9 @@
       <c r="AW4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AX4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1360,6 +1375,9 @@
       <c r="AW5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AX5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1515,6 +1533,9 @@
       <c r="AW6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AX6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1670,6 +1691,9 @@
       <c r="AW7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AX7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1825,6 +1849,9 @@
       <c r="AW8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AX8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1980,6 +2007,9 @@
       <c r="AW9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AX9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2135,6 +2165,9 @@
       <c r="AW10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AX10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2290,6 +2323,9 @@
       <c r="AW11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AX11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2445,6 +2481,9 @@
       <c r="AW12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2600,6 +2639,9 @@
       <c r="AW13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AX13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2755,6 +2797,9 @@
       <c r="AW14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AX14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2910,6 +2955,9 @@
       <c r="AW15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AX15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3065,6 +3113,9 @@
       <c r="AW16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AX16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3220,6 +3271,9 @@
       <c r="AW17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AX17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3375,6 +3429,9 @@
       <c r="AW18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AX18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3530,6 +3587,9 @@
       <c r="AW19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AX19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3685,6 +3745,9 @@
       <c r="AW20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AX20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3840,6 +3903,9 @@
       <c r="AW21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AX21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3995,6 +4061,9 @@
       <c r="AW22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4150,6 +4219,9 @@
       <c r="AW23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AX23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4305,6 +4377,9 @@
       <c r="AW24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AX24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4460,6 +4535,9 @@
       <c r="AW25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4615,6 +4693,9 @@
       <c r="AW26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AX26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4770,6 +4851,9 @@
       <c r="AW27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AX27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4925,6 +5009,9 @@
       <c r="AW28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AX28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5080,6 +5167,9 @@
       <c r="AW29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AX29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5235,6 +5325,9 @@
       <c r="AW30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5390,6 +5483,9 @@
       <c r="AW31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5545,6 +5641,9 @@
       <c r="AW32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5700,6 +5799,9 @@
       <c r="AW33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5855,6 +5957,9 @@
       <c r="AW34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6010,6 +6115,9 @@
       <c r="AW35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AX35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6165,6 +6273,9 @@
       <c r="AW36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AX36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6320,6 +6431,9 @@
       <c r="AW37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AX37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6475,6 +6589,9 @@
       <c r="AW38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AX38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6630,6 +6747,9 @@
       <c r="AW39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AX39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6785,6 +6905,9 @@
       <c r="AW40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -6940,6 +7063,9 @@
       <c r="AW41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7095,6 +7221,9 @@
       <c r="AW42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7250,6 +7379,9 @@
       <c r="AW43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7405,6 +7537,9 @@
       <c r="AW44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7560,6 +7695,9 @@
       <c r="AW45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7715,6 +7853,9 @@
       <c r="AW46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AX46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7870,6 +8011,9 @@
       <c r="AW47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AX47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8025,6 +8169,9 @@
       <c r="AW48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AX48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8180,6 +8327,9 @@
       <c r="AW49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AX49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8335,6 +8485,9 @@
       <c r="AW50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AX50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8490,6 +8643,9 @@
       <c r="AW51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AX51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8645,6 +8801,9 @@
       <c r="AW52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AX52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8800,6 +8959,9 @@
       <c r="AW53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AX53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8955,6 +9117,9 @@
       <c r="AW54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AX54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9110,6 +9275,9 @@
       <c r="AW55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AX55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9265,6 +9433,9 @@
       <c r="AW56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AX56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9420,6 +9591,9 @@
       <c r="AW57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AX57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9575,6 +9749,9 @@
       <c r="AW58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AX58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9730,6 +9907,9 @@
       <c r="AW59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AX59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -9885,6 +10065,9 @@
       <c r="AW60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AX60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10040,6 +10223,9 @@
       <c r="AW61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AX61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10195,6 +10381,9 @@
       <c r="AW62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10350,6 +10539,9 @@
       <c r="AW63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10505,6 +10697,9 @@
       <c r="AW64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10660,6 +10855,9 @@
       <c r="AW65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10815,6 +11013,9 @@
       <c r="AW66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -10970,6 +11171,9 @@
       <c r="AW67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AX67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11125,6 +11329,9 @@
       <c r="AW68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -11280,6 +11487,9 @@
       <c r="AW69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AX69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11435,6 +11645,9 @@
       <c r="AW70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -11590,6 +11803,9 @@
       <c r="AW71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11745,6 +11961,9 @@
       <c r="AW72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AX72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11900,6 +12119,9 @@
       <c r="AW73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AX73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -12055,6 +12277,9 @@
       <c r="AW74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AX74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -12210,6 +12435,9 @@
       <c r="AW75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -12365,6 +12593,9 @@
       <c r="AW76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -12520,6 +12751,9 @@
       <c r="AW77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -12675,6 +12909,9 @@
       <c r="AW78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -12830,6 +13067,9 @@
       <c r="AW79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -12985,6 +13225,9 @@
       <c r="AW80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AX80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -13140,6 +13383,9 @@
       <c r="AW81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13295,6 +13541,9 @@
       <c r="AW82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -13450,6 +13699,9 @@
       <c r="AW83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13605,6 +13857,9 @@
       <c r="AW84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AX84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -13760,6 +14015,9 @@
       <c r="AW85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AX85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -13915,6 +14173,9 @@
       <c r="AW86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AX86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -14070,6 +14331,9 @@
       <c r="AW87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -14225,6 +14489,9 @@
       <c r="AW88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -14380,6 +14647,9 @@
       <c r="AW89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -14535,6 +14805,9 @@
       <c r="AW90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -14690,6 +14963,9 @@
       <c r="AW91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -14845,6 +15121,9 @@
       <c r="AW92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -15000,6 +15279,9 @@
       <c r="AW93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AX93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -15155,6 +15437,9 @@
       <c r="AW94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AX94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -15310,6 +15595,9 @@
       <c r="AW95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AX95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -15465,6 +15753,9 @@
       <c r="AW96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AX96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -15620,6 +15911,9 @@
       <c r="AW97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AX97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -15775,6 +16069,9 @@
       <c r="AW98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AX98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -15930,6 +16227,9 @@
       <c r="AW99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -16085,6 +16385,9 @@
       <c r="AW100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AX100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -16240,6 +16543,9 @@
       <c r="AW101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AX101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -16395,6 +16701,9 @@
       <c r="AW102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AX102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -16550,6 +16859,9 @@
       <c r="AW103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AX103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -16705,6 +17017,9 @@
       <c r="AW104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AX104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -16860,6 +17175,9 @@
       <c r="AW105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AX105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -17015,6 +17333,9 @@
       <c r="AW106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AX106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -17170,6 +17491,9 @@
       <c r="AW107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AX107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -17325,6 +17649,9 @@
       <c r="AW108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -17480,6 +17807,9 @@
       <c r="AW109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AX109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -17635,6 +17965,9 @@
       <c r="AW110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AX110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -17790,6 +18123,9 @@
       <c r="AW111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AX111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -17945,6 +18281,9 @@
       <c r="AW112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AX112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -18100,6 +18439,9 @@
       <c r="AW113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AX113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -18255,6 +18597,9 @@
       <c r="AW114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AX114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -18410,6 +18755,9 @@
       <c r="AW115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AX115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -18565,6 +18913,9 @@
       <c r="AW116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AX116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -18720,6 +19071,9 @@
       <c r="AW117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AX117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -18875,6 +19229,9 @@
       <c r="AW118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AX118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -19030,6 +19387,9 @@
       <c r="AW119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AX119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -19185,6 +19545,9 @@
       <c r="AW120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AX120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -19340,6 +19703,9 @@
       <c r="AW121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AX121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -19495,6 +19861,9 @@
       <c r="AW122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AX122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -19650,6 +20019,9 @@
       <c r="AW123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="AX123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -19805,6 +20177,9 @@
       <c r="AW124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AX124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -19960,6 +20335,9 @@
       <c r="AW125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AX125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -20115,6 +20493,9 @@
       <c r="AW126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AX126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -20270,6 +20651,9 @@
       <c r="AW127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AX127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -20425,6 +20809,9 @@
       <c r="AW128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AX128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -20580,6 +20967,9 @@
       <c r="AW129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AX129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -20735,6 +21125,9 @@
       <c r="AW130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AX130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -20890,6 +21283,9 @@
       <c r="AW131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AX131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -21045,6 +21441,9 @@
       <c r="AW132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AX132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -21200,6 +21599,9 @@
       <c r="AW133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AX133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -21355,6 +21757,9 @@
       <c r="AW134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AX134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -21510,6 +21915,9 @@
       <c r="AW135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AX135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -21665,6 +22073,9 @@
       <c r="AW136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AX136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -21820,6 +22231,9 @@
       <c r="AW137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AX137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -21975,6 +22389,9 @@
       <c r="AW138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AX138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -22130,6 +22547,9 @@
       <c r="AW139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -22285,6 +22705,9 @@
       <c r="AW140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -22440,6 +22863,9 @@
       <c r="AW141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -22595,6 +23021,9 @@
       <c r="AW142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -22750,6 +23179,9 @@
       <c r="AW143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -22905,6 +23337,9 @@
       <c r="AW144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AX144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -23060,6 +23495,9 @@
       <c r="AW145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AX145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -23215,6 +23653,9 @@
       <c r="AW146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AX146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -23370,6 +23811,9 @@
       <c r="AW147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AX147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -23525,6 +23969,9 @@
       <c r="AW148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AX148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -23680,6 +24127,9 @@
       <c r="AW149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AX149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -23835,6 +24285,9 @@
       <c r="AW150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AX150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -23990,6 +24443,9 @@
       <c r="AW151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AX151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -24145,6 +24601,9 @@
       <c r="AW152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AX152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -24300,6 +24759,9 @@
       <c r="AW153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AX153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -24455,6 +24917,9 @@
       <c r="AW154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AX154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -24610,6 +25075,9 @@
       <c r="AW155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AX155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -24765,6 +25233,9 @@
       <c r="AW156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AX156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -24920,6 +25391,9 @@
       <c r="AW157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AX157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -25075,6 +25549,9 @@
       <c r="AW158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AX158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -25230,6 +25707,9 @@
       <c r="AW159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AX159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -25385,6 +25865,9 @@
       <c r="AW160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AX160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -25540,6 +26023,9 @@
       <c r="AW161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AX161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -25695,6 +26181,9 @@
       <c r="AW162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AX162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -25850,6 +26339,9 @@
       <c r="AW163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AX163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -26005,6 +26497,9 @@
       <c r="AW164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AX164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -26061,9 +26556,12 @@
       <c r="AW165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AX165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW165"/>
+  <autoFilter ref="A1:AX165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AX$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AY$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX165"/>
+  <dimension ref="A1:AY165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -493,6 +493,7 @@
     <col width="16" customWidth="1" min="48" max="48"/>
     <col width="16" customWidth="1" min="49" max="49"/>
     <col width="16" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -746,6 +747,11 @@
           <t>2026-09-10 04:09</t>
         </is>
       </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 07:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -904,6 +910,9 @@
       <c r="AX2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AY2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1062,6 +1071,9 @@
       <c r="AX3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AY3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1220,6 +1232,9 @@
       <c r="AX4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AY4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1378,6 +1393,9 @@
       <c r="AX5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AY5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1536,6 +1554,9 @@
       <c r="AX6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AY6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1694,6 +1715,9 @@
       <c r="AX7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AY7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1852,6 +1876,9 @@
       <c r="AX8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AY8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2010,6 +2037,9 @@
       <c r="AX9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AY9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2168,6 +2198,9 @@
       <c r="AX10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AY10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2326,6 +2359,9 @@
       <c r="AX11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AY11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2484,6 +2520,9 @@
       <c r="AX12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2642,6 +2681,9 @@
       <c r="AX13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AY13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2800,6 +2842,9 @@
       <c r="AX14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AY14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2958,6 +3003,9 @@
       <c r="AX15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AY15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3116,6 +3164,9 @@
       <c r="AX16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AY16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3274,6 +3325,9 @@
       <c r="AX17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AY17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3432,6 +3486,9 @@
       <c r="AX18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AY18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3590,6 +3647,9 @@
       <c r="AX19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AY19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3748,6 +3808,9 @@
       <c r="AX20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AY20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3906,6 +3969,9 @@
       <c r="AX21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AY21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4064,6 +4130,9 @@
       <c r="AX22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4222,6 +4291,9 @@
       <c r="AX23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AY23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4380,6 +4452,9 @@
       <c r="AX24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AY24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4538,6 +4613,9 @@
       <c r="AX25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4696,6 +4774,9 @@
       <c r="AX26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AY26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4854,6 +4935,9 @@
       <c r="AX27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AY27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5012,6 +5096,9 @@
       <c r="AX28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AY28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5170,6 +5257,9 @@
       <c r="AX29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AY29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5328,6 +5418,9 @@
       <c r="AX30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5486,6 +5579,9 @@
       <c r="AX31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5644,6 +5740,9 @@
       <c r="AX32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5802,6 +5901,9 @@
       <c r="AX33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -5960,6 +6062,9 @@
       <c r="AX34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6118,6 +6223,9 @@
       <c r="AX35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AY35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6276,6 +6384,9 @@
       <c r="AX36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AY36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6434,6 +6545,9 @@
       <c r="AX37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AY37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6592,6 +6706,9 @@
       <c r="AX38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AY38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6750,6 +6867,9 @@
       <c r="AX39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AY39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -6908,6 +7028,9 @@
       <c r="AX40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY40" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7066,6 +7189,9 @@
       <c r="AX41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7224,6 +7350,9 @@
       <c r="AX42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7382,6 +7511,9 @@
       <c r="AX43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7540,6 +7672,9 @@
       <c r="AX44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7698,6 +7833,9 @@
       <c r="AX45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7856,6 +7994,9 @@
       <c r="AX46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AY46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8014,6 +8155,9 @@
       <c r="AX47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AY47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8172,6 +8316,9 @@
       <c r="AX48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AY48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8330,6 +8477,9 @@
       <c r="AX49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AY49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8488,6 +8638,9 @@
       <c r="AX50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AY50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8646,6 +8799,9 @@
       <c r="AX51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AY51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8804,6 +8960,9 @@
       <c r="AX52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AY52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8962,6 +9121,9 @@
       <c r="AX53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AY53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9120,6 +9282,9 @@
       <c r="AX54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AY54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9278,6 +9443,9 @@
       <c r="AX55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AY55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9436,6 +9604,9 @@
       <c r="AX56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AY56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9594,6 +9765,9 @@
       <c r="AX57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AY57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9752,6 +9926,9 @@
       <c r="AX58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AY58" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -9910,6 +10087,9 @@
       <c r="AX59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AY59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10068,6 +10248,9 @@
       <c r="AX60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AY60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10226,6 +10409,9 @@
       <c r="AX61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AY61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10384,6 +10570,9 @@
       <c r="AX62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10542,6 +10731,9 @@
       <c r="AX63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY63" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10700,6 +10892,9 @@
       <c r="AX64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY64" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10858,6 +11053,9 @@
       <c r="AX65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -11016,6 +11214,9 @@
       <c r="AX66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11174,6 +11375,9 @@
       <c r="AX67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AY67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11332,6 +11536,9 @@
       <c r="AX68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -11490,6 +11697,9 @@
       <c r="AX69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AY69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11648,6 +11858,9 @@
       <c r="AX70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -11806,6 +12019,9 @@
       <c r="AX71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11964,6 +12180,9 @@
       <c r="AX72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AY72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -12122,6 +12341,9 @@
       <c r="AX73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AY73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -12280,6 +12502,9 @@
       <c r="AX74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AY74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -12438,6 +12663,9 @@
       <c r="AX75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -12596,6 +12824,9 @@
       <c r="AX76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -12754,6 +12985,9 @@
       <c r="AX77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -12912,6 +13146,9 @@
       <c r="AX78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -13070,6 +13307,9 @@
       <c r="AX79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -13228,6 +13468,9 @@
       <c r="AX80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AY80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -13386,6 +13629,9 @@
       <c r="AX81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13544,6 +13790,9 @@
       <c r="AX82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -13702,6 +13951,9 @@
       <c r="AX83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -13860,6 +14112,9 @@
       <c r="AX84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AY84" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -14018,6 +14273,9 @@
       <c r="AX85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AY85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -14176,6 +14434,9 @@
       <c r="AX86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AY86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -14334,6 +14595,9 @@
       <c r="AX87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -14492,6 +14756,9 @@
       <c r="AX88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -14650,6 +14917,9 @@
       <c r="AX89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -14808,6 +15078,9 @@
       <c r="AX90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -14966,6 +15239,9 @@
       <c r="AX91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -15124,6 +15400,9 @@
       <c r="AX92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -15282,6 +15561,9 @@
       <c r="AX93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AY93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -15440,6 +15722,9 @@
       <c r="AX94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AY94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -15598,6 +15883,9 @@
       <c r="AX95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AY95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -15756,6 +16044,9 @@
       <c r="AX96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AY96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -15914,6 +16205,9 @@
       <c r="AX97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AY97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -16072,6 +16366,9 @@
       <c r="AX98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AY98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -16230,6 +16527,9 @@
       <c r="AX99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -16388,6 +16688,9 @@
       <c r="AX100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AY100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -16546,6 +16849,9 @@
       <c r="AX101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AY101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -16704,6 +17010,9 @@
       <c r="AX102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AY102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -16862,6 +17171,9 @@
       <c r="AX103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AY103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -17020,6 +17332,9 @@
       <c r="AX104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AY104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -17178,6 +17493,9 @@
       <c r="AX105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AY105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -17336,6 +17654,9 @@
       <c r="AX106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AY106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -17494,6 +17815,9 @@
       <c r="AX107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AY107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -17652,6 +17976,9 @@
       <c r="AX108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -17810,6 +18137,9 @@
       <c r="AX109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AY109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -17968,6 +18298,9 @@
       <c r="AX110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AY110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -18126,6 +18459,9 @@
       <c r="AX111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AY111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -18284,6 +18620,9 @@
       <c r="AX112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AY112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -18442,6 +18781,9 @@
       <c r="AX113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AY113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -18600,6 +18942,9 @@
       <c r="AX114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AY114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -18758,6 +19103,9 @@
       <c r="AX115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AY115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -18916,6 +19264,9 @@
       <c r="AX116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AY116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -19074,6 +19425,9 @@
       <c r="AX117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AY117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -19232,6 +19586,9 @@
       <c r="AX118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AY118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -19390,6 +19747,9 @@
       <c r="AX119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AY119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -19548,6 +19908,9 @@
       <c r="AX120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AY120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -19706,6 +20069,9 @@
       <c r="AX121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AY121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -19864,6 +20230,9 @@
       <c r="AX122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AY122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -20022,6 +20391,9 @@
       <c r="AX123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="AY123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -20180,6 +20552,9 @@
       <c r="AX124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AY124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -20338,6 +20713,9 @@
       <c r="AX125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AY125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -20496,6 +20874,9 @@
       <c r="AX126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AY126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -20654,6 +21035,9 @@
       <c r="AX127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AY127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -20812,6 +21196,9 @@
       <c r="AX128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AY128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -20970,6 +21357,9 @@
       <c r="AX129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AY129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -21128,6 +21518,9 @@
       <c r="AX130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AY130" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -21286,6 +21679,9 @@
       <c r="AX131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AY131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -21444,6 +21840,9 @@
       <c r="AX132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AY132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -21602,6 +22001,9 @@
       <c r="AX133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AY133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -21760,6 +22162,9 @@
       <c r="AX134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AY134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -21918,6 +22323,9 @@
       <c r="AX135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AY135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -22076,6 +22484,9 @@
       <c r="AX136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AY136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -22234,6 +22645,9 @@
       <c r="AX137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AY137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -22392,6 +22806,9 @@
       <c r="AX138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AY138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -22550,6 +22967,9 @@
       <c r="AX139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -22708,6 +23128,9 @@
       <c r="AX140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -22866,6 +23289,9 @@
       <c r="AX141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -23024,6 +23450,9 @@
       <c r="AX142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -23182,6 +23611,9 @@
       <c r="AX143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -23340,6 +23772,9 @@
       <c r="AX144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AY144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -23498,6 +23933,9 @@
       <c r="AX145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AY145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -23656,6 +24094,9 @@
       <c r="AX146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AY146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -23814,6 +24255,9 @@
       <c r="AX147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AY147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -23972,6 +24416,9 @@
       <c r="AX148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AY148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -24130,6 +24577,9 @@
       <c r="AX149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AY149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -24288,6 +24738,9 @@
       <c r="AX150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AY150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -24446,6 +24899,9 @@
       <c r="AX151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AY151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -24604,6 +25060,9 @@
       <c r="AX152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AY152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -24762,6 +25221,9 @@
       <c r="AX153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AY153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -24920,6 +25382,9 @@
       <c r="AX154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AY154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -25078,6 +25543,9 @@
       <c r="AX155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AY155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -25236,6 +25704,9 @@
       <c r="AX156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AY156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -25394,6 +25865,9 @@
       <c r="AX157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AY157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -25552,6 +26026,9 @@
       <c r="AX158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AY158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -25710,6 +26187,9 @@
       <c r="AX159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AY159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -25868,6 +26348,9 @@
       <c r="AX160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AY160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -26026,6 +26509,9 @@
       <c r="AX161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AY161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -26184,6 +26670,9 @@
       <c r="AX162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AY162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -26342,6 +26831,9 @@
       <c r="AX163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AY163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -26500,6 +26992,9 @@
       <c r="AX164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AY164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -26559,9 +27054,12 @@
       <c r="AX165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AY165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AX165"/>
+  <autoFilter ref="A1:AY165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AY$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AZ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY165"/>
+  <dimension ref="A1:AZ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -494,6 +494,7 @@
     <col width="16" customWidth="1" min="49" max="49"/>
     <col width="16" customWidth="1" min="50" max="50"/>
     <col width="16" customWidth="1" min="51" max="51"/>
+    <col width="16" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -752,6 +753,11 @@
           <t>2026-09-10 07:12</t>
         </is>
       </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -913,6 +919,9 @@
       <c r="AY2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="AZ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1074,6 +1083,9 @@
       <c r="AY3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="AZ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1235,6 +1247,9 @@
       <c r="AY4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="AZ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1396,6 +1411,9 @@
       <c r="AY5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AZ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1557,6 +1575,9 @@
       <c r="AY6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="AZ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1718,6 +1739,9 @@
       <c r="AY7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="AZ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1879,6 +1903,9 @@
       <c r="AY8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="AZ8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2040,6 +2067,9 @@
       <c r="AY9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="AZ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2201,6 +2231,9 @@
       <c r="AY10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AZ10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2362,6 +2395,9 @@
       <c r="AY11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="AZ11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2523,6 +2559,9 @@
       <c r="AY12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2684,6 +2723,9 @@
       <c r="AY13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="AZ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2845,6 +2887,9 @@
       <c r="AY14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AZ14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3006,6 +3051,9 @@
       <c r="AY15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="AZ15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3167,6 +3215,9 @@
       <c r="AY16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AZ16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3328,6 +3379,9 @@
       <c r="AY17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AZ17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3489,6 +3543,9 @@
       <c r="AY18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AZ18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3650,6 +3707,9 @@
       <c r="AY19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="AZ19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3811,6 +3871,9 @@
       <c r="AY20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="AZ20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3972,6 +4035,9 @@
       <c r="AY21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="AZ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4133,6 +4199,9 @@
       <c r="AY22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4294,6 +4363,9 @@
       <c r="AY23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AZ23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4455,6 +4527,9 @@
       <c r="AY24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AZ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4616,6 +4691,9 @@
       <c r="AY25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4777,6 +4855,9 @@
       <c r="AY26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="AZ26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4938,6 +5019,9 @@
       <c r="AY27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AZ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5099,6 +5183,9 @@
       <c r="AY28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="AZ28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5260,6 +5347,9 @@
       <c r="AY29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="AZ29" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5421,6 +5511,9 @@
       <c r="AY30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5582,6 +5675,9 @@
       <c r="AY31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5743,6 +5839,9 @@
       <c r="AY32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -5904,6 +6003,9 @@
       <c r="AY33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6065,6 +6167,9 @@
       <c r="AY34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6226,6 +6331,9 @@
       <c r="AY35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AZ35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6387,6 +6495,9 @@
       <c r="AY36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AZ36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6548,6 +6659,9 @@
       <c r="AY37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="AZ37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6709,6 +6823,9 @@
       <c r="AY38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="AZ38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6870,6 +6987,9 @@
       <c r="AY39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="AZ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7031,6 +7151,9 @@
       <c r="AY40" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7192,6 +7315,9 @@
       <c r="AY41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7353,6 +7479,9 @@
       <c r="AY42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7514,6 +7643,9 @@
       <c r="AY43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7675,6 +7807,9 @@
       <c r="AY44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7836,6 +7971,9 @@
       <c r="AY45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7997,6 +8135,9 @@
       <c r="AY46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="AZ46" s="3" t="n">
+        <v>21.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8158,6 +8299,9 @@
       <c r="AY47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AZ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8319,6 +8463,9 @@
       <c r="AY48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="AZ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8480,6 +8627,9 @@
       <c r="AY49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AZ49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8641,6 +8791,9 @@
       <c r="AY50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AZ50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8802,6 +8955,9 @@
       <c r="AY51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="AZ51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8963,6 +9119,9 @@
       <c r="AY52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AZ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9124,6 +9283,9 @@
       <c r="AY53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AZ53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9285,6 +9447,9 @@
       <c r="AY54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="AZ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9446,6 +9611,9 @@
       <c r="AY55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AZ55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9607,6 +9775,9 @@
       <c r="AY56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AZ56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9768,6 +9939,9 @@
       <c r="AY57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="AZ57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -9929,6 +10103,9 @@
       <c r="AY58" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AZ58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10090,6 +10267,9 @@
       <c r="AY59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="AZ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10251,6 +10431,9 @@
       <c r="AY60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="AZ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10412,6 +10595,9 @@
       <c r="AY61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="AZ61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10573,6 +10759,9 @@
       <c r="AY62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10734,6 +10923,9 @@
       <c r="AY63" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10895,6 +11087,9 @@
       <c r="AY64" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -11056,6 +11251,9 @@
       <c r="AY65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -11217,6 +11415,9 @@
       <c r="AY66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11378,6 +11579,9 @@
       <c r="AY67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AZ67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11539,6 +11743,9 @@
       <c r="AY68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -11700,6 +11907,9 @@
       <c r="AY69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AZ69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11861,6 +12071,9 @@
       <c r="AY70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12022,6 +12235,9 @@
       <c r="AY71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -12183,6 +12399,9 @@
       <c r="AY72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="AZ72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -12344,6 +12563,9 @@
       <c r="AY73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AZ73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -12505,6 +12727,9 @@
       <c r="AY74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AZ74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -12666,6 +12891,9 @@
       <c r="AY75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -12827,6 +13055,9 @@
       <c r="AY76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -12988,6 +13219,9 @@
       <c r="AY77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13149,6 +13383,9 @@
       <c r="AY78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ78" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -13310,6 +13547,9 @@
       <c r="AY79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -13471,6 +13711,9 @@
       <c r="AY80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AZ80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -13632,6 +13875,9 @@
       <c r="AY81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -13793,6 +14039,9 @@
       <c r="AY82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -13954,6 +14203,9 @@
       <c r="AY83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -14115,6 +14367,9 @@
       <c r="AY84" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AZ84" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -14276,6 +14531,9 @@
       <c r="AY85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AZ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -14437,6 +14695,9 @@
       <c r="AY86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="AZ86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -14598,6 +14859,9 @@
       <c r="AY87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -14759,6 +15023,9 @@
       <c r="AY88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -14920,6 +15187,9 @@
       <c r="AY89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -15081,6 +15351,9 @@
       <c r="AY90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ90" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -15242,6 +15515,9 @@
       <c r="AY91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -15403,6 +15679,9 @@
       <c r="AY92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -15564,6 +15843,9 @@
       <c r="AY93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="AZ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -15725,6 +16007,9 @@
       <c r="AY94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AZ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -15886,6 +16171,9 @@
       <c r="AY95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AZ95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -16047,6 +16335,9 @@
       <c r="AY96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="AZ96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -16208,6 +16499,9 @@
       <c r="AY97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AZ97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -16369,6 +16663,9 @@
       <c r="AY98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="AZ98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -16530,6 +16827,9 @@
       <c r="AY99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -16691,6 +16991,9 @@
       <c r="AY100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AZ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -16852,6 +17155,9 @@
       <c r="AY101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AZ101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -17013,6 +17319,9 @@
       <c r="AY102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AZ102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -17174,6 +17483,9 @@
       <c r="AY103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="AZ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -17335,6 +17647,9 @@
       <c r="AY104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AZ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -17496,6 +17811,9 @@
       <c r="AY105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AZ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -17657,6 +17975,9 @@
       <c r="AY106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="AZ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -17818,6 +18139,9 @@
       <c r="AY107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="AZ107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -17979,6 +18303,9 @@
       <c r="AY108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -18140,6 +18467,9 @@
       <c r="AY109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AZ109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -18301,6 +18631,9 @@
       <c r="AY110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="AZ110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -18462,6 +18795,9 @@
       <c r="AY111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AZ111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -18623,6 +18959,9 @@
       <c r="AY112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AZ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -18784,6 +19123,9 @@
       <c r="AY113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AZ113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -18945,6 +19287,9 @@
       <c r="AY114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="AZ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -19106,6 +19451,9 @@
       <c r="AY115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="AZ115" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -19267,6 +19615,9 @@
       <c r="AY116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AZ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -19428,6 +19779,9 @@
       <c r="AY117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="AZ117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -19589,6 +19943,9 @@
       <c r="AY118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AZ118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -19750,6 +20107,9 @@
       <c r="AY119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AZ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -19911,6 +20271,9 @@
       <c r="AY120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="AZ120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -20072,6 +20435,9 @@
       <c r="AY121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="AZ121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -20233,6 +20599,9 @@
       <c r="AY122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="AZ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -20394,6 +20763,9 @@
       <c r="AY123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="AZ123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -20555,6 +20927,9 @@
       <c r="AY124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AZ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -20716,6 +21091,9 @@
       <c r="AY125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AZ125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -20877,6 +21255,9 @@
       <c r="AY126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AZ126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -21038,6 +21419,9 @@
       <c r="AY127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="AZ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -21199,6 +21583,9 @@
       <c r="AY128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AZ128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -21360,6 +21747,9 @@
       <c r="AY129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AZ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -21521,6 +21911,9 @@
       <c r="AY130" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AZ130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -21682,6 +22075,9 @@
       <c r="AY131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="AZ131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -21843,6 +22239,9 @@
       <c r="AY132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="AZ132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -22004,6 +22403,9 @@
       <c r="AY133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AZ133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -22165,6 +22567,9 @@
       <c r="AY134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="AZ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -22326,6 +22731,9 @@
       <c r="AY135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AZ135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -22487,6 +22895,9 @@
       <c r="AY136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AZ136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -22648,6 +23059,9 @@
       <c r="AY137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="AZ137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -22809,6 +23223,9 @@
       <c r="AY138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="AZ138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -22970,6 +23387,9 @@
       <c r="AY139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -23131,6 +23551,9 @@
       <c r="AY140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -23292,6 +23715,9 @@
       <c r="AY141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -23453,6 +23879,9 @@
       <c r="AY142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -23614,6 +24043,9 @@
       <c r="AY143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -23775,6 +24207,9 @@
       <c r="AY144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="AZ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -23936,6 +24371,9 @@
       <c r="AY145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="AZ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -24097,6 +24535,9 @@
       <c r="AY146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AZ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -24258,6 +24699,9 @@
       <c r="AY147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="AZ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -24419,6 +24863,9 @@
       <c r="AY148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="AZ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -24580,6 +25027,9 @@
       <c r="AY149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="AZ149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -24741,6 +25191,9 @@
       <c r="AY150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="AZ150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -24902,6 +25355,9 @@
       <c r="AY151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="AZ151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -25063,6 +25519,9 @@
       <c r="AY152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AZ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -25224,6 +25683,9 @@
       <c r="AY153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="AZ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -25385,6 +25847,9 @@
       <c r="AY154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="AZ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -25546,6 +26011,9 @@
       <c r="AY155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="AZ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -25707,6 +26175,9 @@
       <c r="AY156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AZ156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -25868,6 +26339,9 @@
       <c r="AY157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="AZ157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -26029,6 +26503,9 @@
       <c r="AY158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AZ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -26190,6 +26667,9 @@
       <c r="AY159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="AZ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -26351,6 +26831,9 @@
       <c r="AY160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AZ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -26512,6 +26995,9 @@
       <c r="AY161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="AZ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -26673,6 +27159,9 @@
       <c r="AY162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="AZ162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -26834,6 +27323,9 @@
       <c r="AY163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="AZ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -26995,6 +27487,9 @@
       <c r="AY164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="AZ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -27057,9 +27552,12 @@
       <c r="AY165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="AZ165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY165"/>
+  <autoFilter ref="A1:AZ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$AZ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BA$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ165"/>
+  <dimension ref="A1:BA165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -495,6 +495,7 @@
     <col width="16" customWidth="1" min="50" max="50"/>
     <col width="16" customWidth="1" min="51" max="51"/>
     <col width="16" customWidth="1" min="52" max="52"/>
+    <col width="16" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,6 +759,11 @@
           <t>2026-09-10 10:09</t>
         </is>
       </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -922,6 +928,9 @@
       <c r="AZ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BA2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1086,6 +1095,9 @@
       <c r="AZ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BA3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1250,6 +1262,9 @@
       <c r="AZ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BA4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1414,6 +1429,9 @@
       <c r="AZ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BA5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1578,6 +1596,9 @@
       <c r="AZ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BA6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1742,6 +1763,9 @@
       <c r="AZ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BA7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1906,6 +1930,9 @@
       <c r="AZ8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BA8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2070,6 +2097,9 @@
       <c r="AZ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BA9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2234,6 +2264,9 @@
       <c r="AZ10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BA10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2398,6 +2431,9 @@
       <c r="AZ11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="BA11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2562,6 +2598,9 @@
       <c r="AZ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2726,6 +2765,9 @@
       <c r="AZ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BA13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2890,6 +2932,9 @@
       <c r="AZ14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BA14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3054,6 +3099,9 @@
       <c r="AZ15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BA15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3218,6 +3266,9 @@
       <c r="AZ16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BA16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3382,6 +3433,9 @@
       <c r="AZ17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BA17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3546,6 +3600,9 @@
       <c r="AZ18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BA18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3710,6 +3767,9 @@
       <c r="AZ19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BA19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3874,6 +3934,9 @@
       <c r="AZ20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BA20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4038,6 +4101,9 @@
       <c r="AZ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BA21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4202,6 +4268,9 @@
       <c r="AZ22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4366,6 +4435,9 @@
       <c r="AZ23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BA23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4530,6 +4602,9 @@
       <c r="AZ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BA24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4694,6 +4769,9 @@
       <c r="AZ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4858,6 +4936,9 @@
       <c r="AZ26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BA26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5022,6 +5103,9 @@
       <c r="AZ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BA27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5186,6 +5270,9 @@
       <c r="AZ28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="BA28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5350,6 +5437,9 @@
       <c r="AZ29" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BA29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5514,6 +5604,9 @@
       <c r="AZ30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5678,6 +5771,9 @@
       <c r="AZ31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5842,6 +5938,9 @@
       <c r="AZ32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6006,6 +6105,9 @@
       <c r="AZ33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BA33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6170,6 +6272,9 @@
       <c r="AZ34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6334,6 +6439,9 @@
       <c r="AZ35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BA35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6498,6 +6606,9 @@
       <c r="AZ36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BA36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6662,6 +6773,9 @@
       <c r="AZ37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BA37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6826,6 +6940,9 @@
       <c r="AZ38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="BA38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -6990,6 +7107,9 @@
       <c r="AZ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BA39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7154,6 +7274,9 @@
       <c r="AZ40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7318,6 +7441,9 @@
       <c r="AZ41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BA41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7482,6 +7608,9 @@
       <c r="AZ42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BA42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7646,6 +7775,9 @@
       <c r="AZ43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BA43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7810,6 +7942,9 @@
       <c r="AZ44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BA44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7974,6 +8109,9 @@
       <c r="AZ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BA45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -8138,6 +8276,9 @@
       <c r="AZ46" s="3" t="n">
         <v>21.05</v>
       </c>
+      <c r="BA46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8302,6 +8443,9 @@
       <c r="AZ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BA47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8466,6 +8610,9 @@
       <c r="AZ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BA48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8630,6 +8777,9 @@
       <c r="AZ49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BA49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8794,6 +8944,9 @@
       <c r="AZ50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BA50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8958,6 +9111,9 @@
       <c r="AZ51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="BA51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -9122,6 +9278,9 @@
       <c r="AZ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BA52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9286,6 +9445,9 @@
       <c r="AZ53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BA53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9450,6 +9612,9 @@
       <c r="AZ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BA54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9614,6 +9779,9 @@
       <c r="AZ55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BA55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9778,6 +9946,9 @@
       <c r="AZ56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BA56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -9942,6 +10113,9 @@
       <c r="AZ57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BA57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10106,6 +10280,9 @@
       <c r="AZ58" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BA58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10270,6 +10447,9 @@
       <c r="AZ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BA59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10434,6 +10614,9 @@
       <c r="AZ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BA60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10598,6 +10781,9 @@
       <c r="AZ61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BA61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10762,6 +10948,9 @@
       <c r="AZ62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BA62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10926,6 +11115,9 @@
       <c r="AZ63" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="BA63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -11090,6 +11282,9 @@
       <c r="AZ64" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BA64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -11254,6 +11449,9 @@
       <c r="AZ65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -11418,6 +11616,9 @@
       <c r="AZ66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11582,6 +11783,9 @@
       <c r="AZ67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BA67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11746,6 +11950,9 @@
       <c r="AZ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -11910,6 +12117,9 @@
       <c r="AZ69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BA69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -12074,6 +12284,9 @@
       <c r="AZ70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12238,6 +12451,9 @@
       <c r="AZ71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -12402,6 +12618,9 @@
       <c r="AZ72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BA72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -12566,6 +12785,9 @@
       <c r="AZ73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BA73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -12730,6 +12952,9 @@
       <c r="AZ74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BA74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -12894,6 +13119,9 @@
       <c r="AZ75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13058,6 +13286,9 @@
       <c r="AZ76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -13222,6 +13453,9 @@
       <c r="AZ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13386,6 +13620,9 @@
       <c r="AZ78" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -13550,6 +13787,9 @@
       <c r="AZ79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -13714,6 +13954,9 @@
       <c r="AZ80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BA80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -13878,6 +14121,9 @@
       <c r="AZ81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -14042,6 +14288,9 @@
       <c r="AZ82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -14206,6 +14455,9 @@
       <c r="AZ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -14370,6 +14622,9 @@
       <c r="AZ84" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BA84" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -14534,6 +14789,9 @@
       <c r="AZ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BA85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -14698,6 +14956,9 @@
       <c r="AZ86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BA86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -14862,6 +15123,9 @@
       <c r="AZ87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -15026,6 +15290,9 @@
       <c r="AZ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -15190,6 +15457,9 @@
       <c r="AZ89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -15354,6 +15624,9 @@
       <c r="AZ90" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -15518,6 +15791,9 @@
       <c r="AZ91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -15682,6 +15958,9 @@
       <c r="AZ92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -15846,6 +16125,9 @@
       <c r="AZ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BA93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -16010,6 +16292,9 @@
       <c r="AZ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BA94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -16174,6 +16459,9 @@
       <c r="AZ95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BA95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -16338,6 +16626,9 @@
       <c r="AZ96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BA96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -16502,6 +16793,9 @@
       <c r="AZ97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BA97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -16666,6 +16960,9 @@
       <c r="AZ98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BA98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -16830,6 +17127,9 @@
       <c r="AZ99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -16994,6 +17294,9 @@
       <c r="AZ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BA100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -17158,6 +17461,9 @@
       <c r="AZ101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BA101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -17322,6 +17628,9 @@
       <c r="AZ102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BA102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -17486,6 +17795,9 @@
       <c r="AZ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BA103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -17650,6 +17962,9 @@
       <c r="AZ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BA104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -17814,6 +18129,9 @@
       <c r="AZ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BA105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -17978,6 +18296,9 @@
       <c r="AZ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BA106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -18142,6 +18463,9 @@
       <c r="AZ107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BA107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -18306,6 +18630,9 @@
       <c r="AZ108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -18470,6 +18797,9 @@
       <c r="AZ109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BA109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -18634,6 +18964,9 @@
       <c r="AZ110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BA110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -18798,6 +19131,9 @@
       <c r="AZ111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BA111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -18962,6 +19298,9 @@
       <c r="AZ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BA112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -19126,6 +19465,9 @@
       <c r="AZ113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BA113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -19290,6 +19632,9 @@
       <c r="AZ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BA114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -19454,6 +19799,9 @@
       <c r="AZ115" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BA115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -19618,6 +19966,9 @@
       <c r="AZ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BA116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -19782,6 +20133,9 @@
       <c r="AZ117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="BA117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -19946,6 +20300,9 @@
       <c r="AZ118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BA118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -20110,6 +20467,9 @@
       <c r="AZ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BA119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -20274,6 +20634,9 @@
       <c r="AZ120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BA120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -20438,6 +20801,9 @@
       <c r="AZ121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BA121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -20602,6 +20968,9 @@
       <c r="AZ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BA122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -20766,6 +21135,9 @@
       <c r="AZ123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BA123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -20930,6 +21302,9 @@
       <c r="AZ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BA124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -21094,6 +21469,9 @@
       <c r="AZ125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BA125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -21258,6 +21636,9 @@
       <c r="AZ126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BA126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -21422,6 +21803,9 @@
       <c r="AZ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BA127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -21586,6 +21970,9 @@
       <c r="AZ128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BA128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -21750,6 +22137,9 @@
       <c r="AZ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BA129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -21914,6 +22304,9 @@
       <c r="AZ130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BA130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -22078,6 +22471,9 @@
       <c r="AZ131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BA131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -22242,6 +22638,9 @@
       <c r="AZ132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BA132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -22406,6 +22805,9 @@
       <c r="AZ133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BA133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -22570,6 +22972,9 @@
       <c r="AZ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BA134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -22734,6 +23139,9 @@
       <c r="AZ135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BA135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -22898,6 +23306,9 @@
       <c r="AZ136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BA136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -23062,6 +23473,9 @@
       <c r="AZ137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BA137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -23226,6 +23640,9 @@
       <c r="AZ138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BA138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -23390,6 +23807,9 @@
       <c r="AZ139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -23554,6 +23974,9 @@
       <c r="AZ140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -23718,6 +24141,9 @@
       <c r="AZ141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -23882,6 +24308,9 @@
       <c r="AZ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -24046,6 +24475,9 @@
       <c r="AZ143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -24210,6 +24642,9 @@
       <c r="AZ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BA144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -24374,6 +24809,9 @@
       <c r="AZ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BA145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -24538,6 +24976,9 @@
       <c r="AZ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BA146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -24702,6 +25143,9 @@
       <c r="AZ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BA147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -24866,6 +25310,9 @@
       <c r="AZ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BA148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -25030,6 +25477,9 @@
       <c r="AZ149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BA149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -25194,6 +25644,9 @@
       <c r="AZ150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BA150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -25358,6 +25811,9 @@
       <c r="AZ151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="BA151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -25522,6 +25978,9 @@
       <c r="AZ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BA152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -25686,6 +26145,9 @@
       <c r="AZ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BA153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -25850,6 +26312,9 @@
       <c r="AZ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BA154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -26014,6 +26479,9 @@
       <c r="AZ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BA155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -26178,6 +26646,9 @@
       <c r="AZ156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BA156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -26342,6 +26813,9 @@
       <c r="AZ157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BA157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -26506,6 +26980,9 @@
       <c r="AZ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BA158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -26670,6 +27147,9 @@
       <c r="AZ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BA159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -26834,6 +27314,9 @@
       <c r="AZ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BA160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -26998,6 +27481,9 @@
       <c r="AZ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BA161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -27162,6 +27648,9 @@
       <c r="AZ162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="BA162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -27326,6 +27815,9 @@
       <c r="AZ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BA163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -27490,6 +27982,9 @@
       <c r="AZ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BA164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -27555,9 +28050,12 @@
       <c r="AZ165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BA165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ165"/>
+  <autoFilter ref="A1:BA165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-10 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BA$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BB$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA165"/>
+  <dimension ref="A1:BB165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,7 @@
     <col width="16" customWidth="1" min="51" max="51"/>
     <col width="16" customWidth="1" min="52" max="52"/>
     <col width="16" customWidth="1" min="53" max="53"/>
+    <col width="16" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -764,6 +765,11 @@
           <t>2026-09-10 13:10</t>
         </is>
       </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -931,6 +937,9 @@
       <c r="BA2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BB2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1098,6 +1107,9 @@
       <c r="BA3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BB3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1265,6 +1277,9 @@
       <c r="BA4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BB4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1432,6 +1447,9 @@
       <c r="BA5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BB5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1599,6 +1617,9 @@
       <c r="BA6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BB6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1766,6 +1787,9 @@
       <c r="BA7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BB7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1933,6 +1957,9 @@
       <c r="BA8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BB8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2100,6 +2127,9 @@
       <c r="BA9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BB9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2267,6 +2297,9 @@
       <c r="BA10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BB10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2434,6 +2467,9 @@
       <c r="BA11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="BB11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2601,6 +2637,9 @@
       <c r="BA12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2768,6 +2807,9 @@
       <c r="BA13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BB13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2935,6 +2977,9 @@
       <c r="BA14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BB14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3102,6 +3147,9 @@
       <c r="BA15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BB15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3269,6 +3317,9 @@
       <c r="BA16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BB16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3436,6 +3487,9 @@
       <c r="BA17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BB17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3603,6 +3657,9 @@
       <c r="BA18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BB18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3770,6 +3827,9 @@
       <c r="BA19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BB19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3937,6 +3997,9 @@
       <c r="BA20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BB20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4104,6 +4167,9 @@
       <c r="BA21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BB21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4271,6 +4337,9 @@
       <c r="BA22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4438,6 +4507,9 @@
       <c r="BA23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BB23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4605,6 +4677,9 @@
       <c r="BA24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BB24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4772,6 +4847,9 @@
       <c r="BA25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4939,6 +5017,9 @@
       <c r="BA26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BB26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5106,6 +5187,9 @@
       <c r="BA27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BB27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5273,6 +5357,9 @@
       <c r="BA28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="BB28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5440,6 +5527,9 @@
       <c r="BA29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BB29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5607,6 +5697,9 @@
       <c r="BA30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5774,6 +5867,9 @@
       <c r="BA31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -5941,6 +6037,9 @@
       <c r="BA32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6108,6 +6207,9 @@
       <c r="BA33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BB33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6275,6 +6377,9 @@
       <c r="BA34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6442,6 +6547,9 @@
       <c r="BA35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BB35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6609,6 +6717,9 @@
       <c r="BA36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BB36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6776,6 +6887,9 @@
       <c r="BA37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BB37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -6943,6 +7057,9 @@
       <c r="BA38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="BB38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7110,6 +7227,9 @@
       <c r="BA39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BB39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7277,6 +7397,9 @@
       <c r="BA40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7444,6 +7567,9 @@
       <c r="BA41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BB41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7611,6 +7737,9 @@
       <c r="BA42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BB42" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7778,6 +7907,9 @@
       <c r="BA43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BB43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7945,6 +8077,9 @@
       <c r="BA44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BB44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8112,6 +8247,9 @@
       <c r="BA45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BB45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -8279,6 +8417,9 @@
       <c r="BA46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BB46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8446,6 +8587,9 @@
       <c r="BA47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BB47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8613,6 +8757,9 @@
       <c r="BA48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BB48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8780,6 +8927,9 @@
       <c r="BA49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BB49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8947,6 +9097,9 @@
       <c r="BA50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BB50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -9114,6 +9267,9 @@
       <c r="BA51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="BB51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -9281,6 +9437,9 @@
       <c r="BA52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BB52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9448,6 +9607,9 @@
       <c r="BA53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BB53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9615,6 +9777,9 @@
       <c r="BA54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BB54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9782,6 +9947,9 @@
       <c r="BA55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BB55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -9949,6 +10117,9 @@
       <c r="BA56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BB56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10116,6 +10287,9 @@
       <c r="BA57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BB57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10283,6 +10457,9 @@
       <c r="BA58" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BB58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10450,6 +10627,9 @@
       <c r="BA59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BB59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10617,6 +10797,9 @@
       <c r="BA60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BB60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10784,6 +10967,9 @@
       <c r="BA61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BB61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10951,6 +11137,9 @@
       <c r="BA62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BB62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -11118,6 +11307,9 @@
       <c r="BA63" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="BB63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -11285,6 +11477,9 @@
       <c r="BA64" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BB64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -11452,6 +11647,9 @@
       <c r="BA65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -11619,6 +11817,9 @@
       <c r="BA66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11786,6 +11987,9 @@
       <c r="BA67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BB67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11953,6 +12157,9 @@
       <c r="BA68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12120,6 +12327,9 @@
       <c r="BA69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BB69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -12287,6 +12497,9 @@
       <c r="BA70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB70" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12454,6 +12667,9 @@
       <c r="BA71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -12621,6 +12837,9 @@
       <c r="BA72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BB72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -12788,6 +13007,9 @@
       <c r="BA73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BB73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -12955,6 +13177,9 @@
       <c r="BA74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BB74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13122,6 +13347,9 @@
       <c r="BA75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13289,6 +13517,9 @@
       <c r="BA76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -13456,6 +13687,9 @@
       <c r="BA77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13623,6 +13857,9 @@
       <c r="BA78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BB78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -13790,6 +14027,9 @@
       <c r="BA79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -13957,6 +14197,9 @@
       <c r="BA80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BB80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -14124,6 +14367,9 @@
       <c r="BA81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -14291,6 +14537,9 @@
       <c r="BA82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -14458,6 +14707,9 @@
       <c r="BA83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -14625,6 +14877,9 @@
       <c r="BA84" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BB84" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -14792,6 +15047,9 @@
       <c r="BA85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BB85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -14959,6 +15217,9 @@
       <c r="BA86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BB86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -15126,6 +15387,9 @@
       <c r="BA87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -15293,6 +15557,9 @@
       <c r="BA88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -15460,6 +15727,9 @@
       <c r="BA89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -15627,6 +15897,9 @@
       <c r="BA90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BB90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -15794,6 +16067,9 @@
       <c r="BA91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -15961,6 +16237,9 @@
       <c r="BA92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -16128,6 +16407,9 @@
       <c r="BA93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BB93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -16295,6 +16577,9 @@
       <c r="BA94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BB94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -16462,6 +16747,9 @@
       <c r="BA95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BB95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -16629,6 +16917,9 @@
       <c r="BA96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BB96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -16796,6 +17087,9 @@
       <c r="BA97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BB97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -16963,6 +17257,9 @@
       <c r="BA98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BB98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -17130,6 +17427,9 @@
       <c r="BA99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -17297,6 +17597,9 @@
       <c r="BA100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BB100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -17464,6 +17767,9 @@
       <c r="BA101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BB101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -17631,6 +17937,9 @@
       <c r="BA102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BB102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -17798,6 +18107,9 @@
       <c r="BA103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BB103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -17965,6 +18277,9 @@
       <c r="BA104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BB104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -18132,6 +18447,9 @@
       <c r="BA105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BB105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -18299,6 +18617,9 @@
       <c r="BA106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BB106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -18466,6 +18787,9 @@
       <c r="BA107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BB107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -18633,6 +18957,9 @@
       <c r="BA108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -18800,6 +19127,9 @@
       <c r="BA109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BB109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -18967,6 +19297,9 @@
       <c r="BA110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BB110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -19134,6 +19467,9 @@
       <c r="BA111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BB111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -19301,6 +19637,9 @@
       <c r="BA112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BB112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -19468,6 +19807,9 @@
       <c r="BA113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BB113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -19635,6 +19977,9 @@
       <c r="BA114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BB114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -19802,6 +20147,9 @@
       <c r="BA115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BB115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -19969,6 +20317,9 @@
       <c r="BA116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BB116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -20136,6 +20487,9 @@
       <c r="BA117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="BB117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -20303,6 +20657,9 @@
       <c r="BA118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BB118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -20470,6 +20827,9 @@
       <c r="BA119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BB119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -20637,6 +20997,9 @@
       <c r="BA120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BB120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -20804,6 +21167,9 @@
       <c r="BA121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BB121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -20971,6 +21337,9 @@
       <c r="BA122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BB122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -21138,6 +21507,9 @@
       <c r="BA123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BB123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -21305,6 +21677,9 @@
       <c r="BA124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BB124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -21472,6 +21847,9 @@
       <c r="BA125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BB125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -21639,6 +22017,9 @@
       <c r="BA126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BB126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -21806,6 +22187,9 @@
       <c r="BA127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BB127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -21973,6 +22357,9 @@
       <c r="BA128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BB128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -22140,6 +22527,9 @@
       <c r="BA129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BB129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -22307,6 +22697,9 @@
       <c r="BA130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BB130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -22474,6 +22867,9 @@
       <c r="BA131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BB131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -22641,6 +23037,9 @@
       <c r="BA132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BB132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -22808,6 +23207,9 @@
       <c r="BA133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BB133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -22975,6 +23377,9 @@
       <c r="BA134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BB134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -23142,6 +23547,9 @@
       <c r="BA135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BB135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -23309,6 +23717,9 @@
       <c r="BA136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BB136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -23476,6 +23887,9 @@
       <c r="BA137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BB137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -23643,6 +24057,9 @@
       <c r="BA138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BB138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -23810,6 +24227,9 @@
       <c r="BA139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -23977,6 +24397,9 @@
       <c r="BA140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -24144,6 +24567,9 @@
       <c r="BA141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -24311,6 +24737,9 @@
       <c r="BA142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -24478,6 +24907,9 @@
       <c r="BA143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -24645,6 +25077,9 @@
       <c r="BA144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BB144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -24812,6 +25247,9 @@
       <c r="BA145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BB145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -24979,6 +25417,9 @@
       <c r="BA146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BB146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -25146,6 +25587,9 @@
       <c r="BA147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BB147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -25313,6 +25757,9 @@
       <c r="BA148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BB148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -25480,6 +25927,9 @@
       <c r="BA149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BB149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -25647,6 +26097,9 @@
       <c r="BA150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BB150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -25814,6 +26267,9 @@
       <c r="BA151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="BB151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -25981,6 +26437,9 @@
       <c r="BA152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BB152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -26148,6 +26607,9 @@
       <c r="BA153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BB153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -26315,6 +26777,9 @@
       <c r="BA154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BB154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -26482,6 +26947,9 @@
       <c r="BA155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BB155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -26649,6 +27117,9 @@
       <c r="BA156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BB156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -26816,6 +27287,9 @@
       <c r="BA157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BB157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -26983,6 +27457,9 @@
       <c r="BA158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BB158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -27150,6 +27627,9 @@
       <c r="BA159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BB159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -27317,6 +27797,9 @@
       <c r="BA160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BB160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -27484,6 +27967,9 @@
       <c r="BA161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BB161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -27651,6 +28137,9 @@
       <c r="BA162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="BB162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -27818,6 +28307,9 @@
       <c r="BA163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BB163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -27985,6 +28477,9 @@
       <c r="BA164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BB164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -28053,9 +28548,12 @@
       <c r="BA165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BB165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BA165"/>
+  <autoFilter ref="A1:BB165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-11 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BB$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BC$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB165"/>
+  <dimension ref="A1:BC165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,7 @@
     <col width="16" customWidth="1" min="52" max="52"/>
     <col width="16" customWidth="1" min="53" max="53"/>
     <col width="16" customWidth="1" min="54" max="54"/>
+    <col width="16" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -770,6 +771,11 @@
           <t>2026-09-10 16:08</t>
         </is>
       </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-10 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -940,6 +946,9 @@
       <c r="BB2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BC2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1110,6 +1119,9 @@
       <c r="BB3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BC3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1280,6 +1292,9 @@
       <c r="BB4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BC4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1450,6 +1465,9 @@
       <c r="BB5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BC5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1620,6 +1638,9 @@
       <c r="BB6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BC6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1790,6 +1811,9 @@
       <c r="BB7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BC7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1960,6 +1984,9 @@
       <c r="BB8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BC8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2130,6 +2157,9 @@
       <c r="BB9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BC9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2300,6 +2330,9 @@
       <c r="BB10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BC10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2470,6 +2503,9 @@
       <c r="BB11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="BC11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2640,6 +2676,9 @@
       <c r="BB12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2810,6 +2849,9 @@
       <c r="BB13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BC13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2980,6 +3022,9 @@
       <c r="BB14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BC14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3150,6 +3195,9 @@
       <c r="BB15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BC15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3320,6 +3368,9 @@
       <c r="BB16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BC16" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3490,6 +3541,9 @@
       <c r="BB17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BC17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3660,6 +3714,9 @@
       <c r="BB18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BC18" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3830,6 +3887,9 @@
       <c r="BB19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BC19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4000,6 +4060,9 @@
       <c r="BB20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BC20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4170,6 +4233,9 @@
       <c r="BB21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BC21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4340,6 +4406,9 @@
       <c r="BB22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4510,6 +4579,9 @@
       <c r="BB23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BC23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4680,6 +4752,9 @@
       <c r="BB24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BC24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4850,6 +4925,9 @@
       <c r="BB25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5020,6 +5098,9 @@
       <c r="BB26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BC26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5190,6 +5271,9 @@
       <c r="BB27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BC27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5360,6 +5444,9 @@
       <c r="BB28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="BC28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5530,6 +5617,9 @@
       <c r="BB29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BC29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5700,6 +5790,9 @@
       <c r="BB30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5870,6 +5963,9 @@
       <c r="BB31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6040,6 +6136,9 @@
       <c r="BB32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6210,6 +6309,9 @@
       <c r="BB33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BC33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6380,6 +6482,9 @@
       <c r="BB34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6550,6 +6655,9 @@
       <c r="BB35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BC35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6720,6 +6828,9 @@
       <c r="BB36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BC36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6890,6 +7001,9 @@
       <c r="BB37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BC37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7060,6 +7174,9 @@
       <c r="BB38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="BC38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7230,6 +7347,9 @@
       <c r="BB39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BC39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7400,6 +7520,9 @@
       <c r="BB40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7570,6 +7693,9 @@
       <c r="BB41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BC41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7740,6 +7866,9 @@
       <c r="BB42" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BC42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7910,6 +8039,9 @@
       <c r="BB43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BC43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -8080,6 +8212,9 @@
       <c r="BB44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BC44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8250,6 +8385,9 @@
       <c r="BB45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BC45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -8420,6 +8558,9 @@
       <c r="BB46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BC46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8590,6 +8731,9 @@
       <c r="BB47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BC47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8760,6 +8904,9 @@
       <c r="BB48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BC48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -8930,6 +9077,9 @@
       <c r="BB49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BC49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -9100,6 +9250,9 @@
       <c r="BB50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BC50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -9270,6 +9423,9 @@
       <c r="BB51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="BC51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -9440,6 +9596,9 @@
       <c r="BB52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BC52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9610,6 +9769,9 @@
       <c r="BB53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BC53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9780,6 +9942,9 @@
       <c r="BB54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BC54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -9950,6 +10115,9 @@
       <c r="BB55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BC55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -10120,6 +10288,9 @@
       <c r="BB56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BC56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10290,6 +10461,9 @@
       <c r="BB57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BC57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10460,6 +10634,9 @@
       <c r="BB58" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BC58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10630,6 +10807,9 @@
       <c r="BB59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BC59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10800,6 +10980,9 @@
       <c r="BB60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BC60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10970,6 +11153,9 @@
       <c r="BB61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BC61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -11140,6 +11326,9 @@
       <c r="BB62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BC62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -11310,6 +11499,9 @@
       <c r="BB63" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="BC63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -11480,6 +11672,9 @@
       <c r="BB64" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BC64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -11650,6 +11845,9 @@
       <c r="BB65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -11820,6 +12018,9 @@
       <c r="BB66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11990,6 +12191,9 @@
       <c r="BB67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BC67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -12160,6 +12364,9 @@
       <c r="BB68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12330,6 +12537,9 @@
       <c r="BB69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BC69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -12500,6 +12710,9 @@
       <c r="BB70" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12670,6 +12883,9 @@
       <c r="BB71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -12840,6 +13056,9 @@
       <c r="BB72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BC72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -13010,6 +13229,9 @@
       <c r="BB73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BC73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -13180,6 +13402,9 @@
       <c r="BB74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BC74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13350,6 +13575,9 @@
       <c r="BB75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13520,6 +13748,9 @@
       <c r="BB76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -13690,6 +13921,9 @@
       <c r="BB77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -13860,6 +14094,9 @@
       <c r="BB78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BC78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -14030,6 +14267,9 @@
       <c r="BB79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -14200,6 +14440,9 @@
       <c r="BB80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BC80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -14370,6 +14613,9 @@
       <c r="BB81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -14540,6 +14786,9 @@
       <c r="BB82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -14710,6 +14959,9 @@
       <c r="BB83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -14880,6 +15132,9 @@
       <c r="BB84" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BC84" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -15050,6 +15305,9 @@
       <c r="BB85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BC85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -15220,6 +15478,9 @@
       <c r="BB86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BC86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -15390,6 +15651,9 @@
       <c r="BB87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -15560,6 +15824,9 @@
       <c r="BB88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -15730,6 +15997,9 @@
       <c r="BB89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -15900,6 +16170,9 @@
       <c r="BB90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BC90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -16070,6 +16343,9 @@
       <c r="BB91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -16240,6 +16516,9 @@
       <c r="BB92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -16410,6 +16689,9 @@
       <c r="BB93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BC93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -16580,6 +16862,9 @@
       <c r="BB94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BC94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -16750,6 +17035,9 @@
       <c r="BB95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BC95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -16920,6 +17208,9 @@
       <c r="BB96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BC96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -17090,6 +17381,9 @@
       <c r="BB97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BC97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -17260,6 +17554,9 @@
       <c r="BB98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BC98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -17430,6 +17727,9 @@
       <c r="BB99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -17600,6 +17900,9 @@
       <c r="BB100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BC100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -17770,6 +18073,9 @@
       <c r="BB101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BC101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -17940,6 +18246,9 @@
       <c r="BB102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BC102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -18110,6 +18419,9 @@
       <c r="BB103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BC103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -18280,6 +18592,9 @@
       <c r="BB104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BC104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -18450,6 +18765,9 @@
       <c r="BB105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BC105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -18620,6 +18938,9 @@
       <c r="BB106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BC106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -18790,6 +19111,9 @@
       <c r="BB107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BC107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -18960,6 +19284,9 @@
       <c r="BB108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -19130,6 +19457,9 @@
       <c r="BB109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BC109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -19300,6 +19630,9 @@
       <c r="BB110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BC110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -19470,6 +19803,9 @@
       <c r="BB111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BC111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -19640,6 +19976,9 @@
       <c r="BB112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BC112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -19810,6 +20149,9 @@
       <c r="BB113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BC113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -19980,6 +20322,9 @@
       <c r="BB114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BC114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -20150,6 +20495,9 @@
       <c r="BB115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BC115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -20320,6 +20668,9 @@
       <c r="BB116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BC116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -20490,6 +20841,9 @@
       <c r="BB117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="BC117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -20660,6 +21014,9 @@
       <c r="BB118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BC118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -20830,6 +21187,9 @@
       <c r="BB119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BC119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -21000,6 +21360,9 @@
       <c r="BB120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BC120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -21170,6 +21533,9 @@
       <c r="BB121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BC121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -21340,6 +21706,9 @@
       <c r="BB122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BC122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -21510,6 +21879,9 @@
       <c r="BB123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BC123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -21680,6 +22052,9 @@
       <c r="BB124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BC124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -21850,6 +22225,9 @@
       <c r="BB125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BC125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -22020,6 +22398,9 @@
       <c r="BB126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BC126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -22190,6 +22571,9 @@
       <c r="BB127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BC127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -22360,6 +22744,9 @@
       <c r="BB128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BC128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -22530,6 +22917,9 @@
       <c r="BB129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BC129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -22700,6 +23090,9 @@
       <c r="BB130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BC130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -22870,6 +23263,9 @@
       <c r="BB131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BC131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -23040,6 +23436,9 @@
       <c r="BB132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BC132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -23210,6 +23609,9 @@
       <c r="BB133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BC133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -23380,6 +23782,9 @@
       <c r="BB134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BC134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -23550,6 +23955,9 @@
       <c r="BB135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BC135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -23720,6 +24128,9 @@
       <c r="BB136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BC136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -23890,6 +24301,9 @@
       <c r="BB137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BC137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -24060,6 +24474,9 @@
       <c r="BB138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BC138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -24230,6 +24647,9 @@
       <c r="BB139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -24400,6 +24820,9 @@
       <c r="BB140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -24570,6 +24993,9 @@
       <c r="BB141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -24740,6 +25166,9 @@
       <c r="BB142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -24910,6 +25339,9 @@
       <c r="BB143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -25080,6 +25512,9 @@
       <c r="BB144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BC144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -25250,6 +25685,9 @@
       <c r="BB145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BC145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -25420,6 +25858,9 @@
       <c r="BB146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BC146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -25590,6 +26031,9 @@
       <c r="BB147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BC147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -25760,6 +26204,9 @@
       <c r="BB148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BC148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -25930,6 +26377,9 @@
       <c r="BB149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BC149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -26100,6 +26550,9 @@
       <c r="BB150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BC150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -26270,6 +26723,9 @@
       <c r="BB151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="BC151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -26440,6 +26896,9 @@
       <c r="BB152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BC152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -26610,6 +27069,9 @@
       <c r="BB153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BC153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -26780,6 +27242,9 @@
       <c r="BB154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BC154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -26950,6 +27415,9 @@
       <c r="BB155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BC155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -27120,6 +27588,9 @@
       <c r="BB156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BC156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -27290,6 +27761,9 @@
       <c r="BB157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BC157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -27460,6 +27934,9 @@
       <c r="BB158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BC158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -27630,6 +28107,9 @@
       <c r="BB159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BC159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -27800,6 +28280,9 @@
       <c r="BB160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BC160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -27970,6 +28453,9 @@
       <c r="BB161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BC161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -28140,6 +28626,9 @@
       <c r="BB162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="BC162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -28310,6 +28799,9 @@
       <c r="BB163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BC163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -28480,6 +28972,9 @@
       <c r="BB164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BC164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -28551,9 +29046,12 @@
       <c r="BB165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BC165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB165"/>
+  <autoFilter ref="A1:BC165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-11 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BC$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BD$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC165"/>
+  <dimension ref="A1:BD165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -498,6 +498,7 @@
     <col width="16" customWidth="1" min="53" max="53"/>
     <col width="16" customWidth="1" min="54" max="54"/>
     <col width="16" customWidth="1" min="55" max="55"/>
+    <col width="16" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -776,6 +777,11 @@
           <t>2026-09-10 22:09</t>
         </is>
       </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 01:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -949,6 +955,9 @@
       <c r="BC2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BD2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1122,6 +1131,9 @@
       <c r="BC3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BD3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1295,6 +1307,9 @@
       <c r="BC4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BD4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1468,6 +1483,9 @@
       <c r="BC5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BD5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1641,6 +1659,9 @@
       <c r="BC6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BD6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1814,6 +1835,9 @@
       <c r="BC7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BD7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1987,6 +2011,9 @@
       <c r="BC8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BD8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2160,6 +2187,9 @@
       <c r="BC9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BD9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2333,6 +2363,9 @@
       <c r="BC10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BD10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2506,6 +2539,9 @@
       <c r="BC11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="BD11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2679,6 +2715,9 @@
       <c r="BC12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2852,6 +2891,9 @@
       <c r="BC13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BD13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3025,6 +3067,9 @@
       <c r="BC14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BD14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3198,6 +3243,9 @@
       <c r="BC15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BD15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3371,6 +3419,9 @@
       <c r="BC16" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BD16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3544,6 +3595,9 @@
       <c r="BC17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BD17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3717,6 +3771,9 @@
       <c r="BC18" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BD18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3890,6 +3947,9 @@
       <c r="BC19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BD19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4063,6 +4123,9 @@
       <c r="BC20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BD20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4236,6 +4299,9 @@
       <c r="BC21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BD21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4409,6 +4475,9 @@
       <c r="BC22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4582,6 +4651,9 @@
       <c r="BC23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BD23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4755,6 +4827,9 @@
       <c r="BC24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BD24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4928,6 +5003,9 @@
       <c r="BC25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5101,6 +5179,9 @@
       <c r="BC26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BD26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5274,6 +5355,9 @@
       <c r="BC27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BD27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5447,6 +5531,9 @@
       <c r="BC28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="BD28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5620,6 +5707,9 @@
       <c r="BC29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BD29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5793,6 +5883,9 @@
       <c r="BC30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5966,6 +6059,9 @@
       <c r="BC31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6139,6 +6235,9 @@
       <c r="BC32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6312,6 +6411,9 @@
       <c r="BC33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BD33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6485,6 +6587,9 @@
       <c r="BC34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6658,6 +6763,9 @@
       <c r="BC35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BD35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6831,6 +6939,9 @@
       <c r="BC36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BD36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7004,6 +7115,9 @@
       <c r="BC37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BD37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7177,6 +7291,9 @@
       <c r="BC38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="BD38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7350,6 +7467,9 @@
       <c r="BC39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BD39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7523,6 +7643,9 @@
       <c r="BC40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7696,6 +7819,9 @@
       <c r="BC41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BD41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7869,6 +7995,9 @@
       <c r="BC42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -8042,6 +8171,9 @@
       <c r="BC43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BD43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -8215,6 +8347,9 @@
       <c r="BC44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BD44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8388,6 +8523,9 @@
       <c r="BC45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BD45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -8561,6 +8699,9 @@
       <c r="BC46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BD46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8734,6 +8875,9 @@
       <c r="BC47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BD47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -8907,6 +9051,9 @@
       <c r="BC48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BD48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -9080,6 +9227,9 @@
       <c r="BC49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BD49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -9253,6 +9403,9 @@
       <c r="BC50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BD50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -9426,6 +9579,9 @@
       <c r="BC51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="BD51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -9599,6 +9755,9 @@
       <c r="BC52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BD52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9772,6 +9931,9 @@
       <c r="BC53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BD53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -9945,6 +10107,9 @@
       <c r="BC54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BD54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -10118,6 +10283,9 @@
       <c r="BC55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BD55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -10291,6 +10459,9 @@
       <c r="BC56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BD56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10464,6 +10635,9 @@
       <c r="BC57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BD57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10637,6 +10811,9 @@
       <c r="BC58" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BD58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10810,6 +10987,9 @@
       <c r="BC59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BD59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10983,6 +11163,9 @@
       <c r="BC60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BD60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -11156,6 +11339,9 @@
       <c r="BC61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BD61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -11329,6 +11515,9 @@
       <c r="BC62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BD62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -11502,6 +11691,9 @@
       <c r="BC63" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="BD63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -11675,6 +11867,9 @@
       <c r="BC64" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BD64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -11848,6 +12043,9 @@
       <c r="BC65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -12021,6 +12219,9 @@
       <c r="BC66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -12194,6 +12395,9 @@
       <c r="BC67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BD67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -12367,6 +12571,9 @@
       <c r="BC68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12540,6 +12747,9 @@
       <c r="BC69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BD69" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -12713,6 +12923,9 @@
       <c r="BC70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -12886,6 +13099,9 @@
       <c r="BC71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -13059,6 +13275,9 @@
       <c r="BC72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BD72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -13232,6 +13451,9 @@
       <c r="BC73" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BD73" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -13405,6 +13627,9 @@
       <c r="BC74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BD74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13578,6 +13803,9 @@
       <c r="BC75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -13751,6 +13979,9 @@
       <c r="BC76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -13924,6 +14155,9 @@
       <c r="BC77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -14097,6 +14331,9 @@
       <c r="BC78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BD78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -14270,6 +14507,9 @@
       <c r="BC79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -14443,6 +14683,9 @@
       <c r="BC80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BD80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -14616,6 +14859,9 @@
       <c r="BC81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -14789,6 +15035,9 @@
       <c r="BC82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -14962,6 +15211,9 @@
       <c r="BC83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -15135,6 +15387,9 @@
       <c r="BC84" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BD84" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -15308,6 +15563,9 @@
       <c r="BC85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BD85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -15481,6 +15739,9 @@
       <c r="BC86" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BD86" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -15654,6 +15915,9 @@
       <c r="BC87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -15827,6 +16091,9 @@
       <c r="BC88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -16000,6 +16267,9 @@
       <c r="BC89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -16173,6 +16443,9 @@
       <c r="BC90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -16346,6 +16619,9 @@
       <c r="BC91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -16519,6 +16795,9 @@
       <c r="BC92" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD92" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -16692,6 +16971,9 @@
       <c r="BC93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BD93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -16865,6 +17147,9 @@
       <c r="BC94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BD94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -17038,6 +17323,9 @@
       <c r="BC95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BD95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -17211,6 +17499,9 @@
       <c r="BC96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BD96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -17384,6 +17675,9 @@
       <c r="BC97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BD97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -17557,6 +17851,9 @@
       <c r="BC98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BD98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -17730,6 +18027,9 @@
       <c r="BC99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -17903,6 +18203,9 @@
       <c r="BC100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BD100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -18076,6 +18379,9 @@
       <c r="BC101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BD101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -18249,6 +18555,9 @@
       <c r="BC102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BD102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -18422,6 +18731,9 @@
       <c r="BC103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BD103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -18595,6 +18907,9 @@
       <c r="BC104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BD104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -18768,6 +19083,9 @@
       <c r="BC105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BD105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -18941,6 +19259,9 @@
       <c r="BC106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BD106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -19114,6 +19435,9 @@
       <c r="BC107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BD107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -19287,6 +19611,9 @@
       <c r="BC108" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD108" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -19460,6 +19787,9 @@
       <c r="BC109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BD109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -19633,6 +19963,9 @@
       <c r="BC110" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BD110" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -19806,6 +20139,9 @@
       <c r="BC111" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BD111" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -19979,6 +20315,9 @@
       <c r="BC112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -20152,6 +20491,9 @@
       <c r="BC113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BD113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -20325,6 +20667,9 @@
       <c r="BC114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BD114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -20498,6 +20843,9 @@
       <c r="BC115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BD115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -20671,6 +21019,9 @@
       <c r="BC116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BD116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -20844,6 +21195,9 @@
       <c r="BC117" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="BD117" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -21017,6 +21371,9 @@
       <c r="BC118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BD118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -21190,6 +21547,9 @@
       <c r="BC119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BD119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -21363,6 +21723,9 @@
       <c r="BC120" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BD120" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -21536,6 +21899,9 @@
       <c r="BC121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BD121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -21709,6 +22075,9 @@
       <c r="BC122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BD122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -21882,6 +22251,9 @@
       <c r="BC123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BD123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -22055,6 +22427,9 @@
       <c r="BC124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BD124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -22228,6 +22603,9 @@
       <c r="BC125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -22401,6 +22779,9 @@
       <c r="BC126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -22574,6 +22955,9 @@
       <c r="BC127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BD127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -22747,6 +23131,9 @@
       <c r="BC128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BD128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -22920,6 +23307,9 @@
       <c r="BC129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BD129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -23093,6 +23483,9 @@
       <c r="BC130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BD130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -23266,6 +23659,9 @@
       <c r="BC131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BD131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -23439,6 +23835,9 @@
       <c r="BC132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BD132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -23612,6 +24011,9 @@
       <c r="BC133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BD133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -23785,6 +24187,9 @@
       <c r="BC134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BD134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -23958,6 +24363,9 @@
       <c r="BC135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BD135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -24131,6 +24539,9 @@
       <c r="BC136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BD136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -24304,6 +24715,9 @@
       <c r="BC137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BD137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -24477,6 +24891,9 @@
       <c r="BC138" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BD138" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -24650,6 +25067,9 @@
       <c r="BC139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -24823,6 +25243,9 @@
       <c r="BC140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -24996,6 +25419,9 @@
       <c r="BC141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -25169,6 +25595,9 @@
       <c r="BC142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -25342,6 +25771,9 @@
       <c r="BC143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -25515,6 +25947,9 @@
       <c r="BC144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BD144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -25688,6 +26123,9 @@
       <c r="BC145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BD145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -25861,6 +26299,9 @@
       <c r="BC146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BD146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -26034,6 +26475,9 @@
       <c r="BC147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BD147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -26207,6 +26651,9 @@
       <c r="BC148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BD148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -26380,6 +26827,9 @@
       <c r="BC149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BD149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -26553,6 +27003,9 @@
       <c r="BC150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BD150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -26726,6 +27179,9 @@
       <c r="BC151" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="BD151" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -26899,6 +27355,9 @@
       <c r="BC152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BD152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -27072,6 +27531,9 @@
       <c r="BC153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BD153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -27245,6 +27707,9 @@
       <c r="BC154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BD154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -27418,6 +27883,9 @@
       <c r="BC155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BD155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -27591,6 +28059,9 @@
       <c r="BC156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BD156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -27764,6 +28235,9 @@
       <c r="BC157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BD157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -27937,6 +28411,9 @@
       <c r="BC158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BD158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -28110,6 +28587,9 @@
       <c r="BC159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BD159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -28283,6 +28763,9 @@
       <c r="BC160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BD160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -28456,6 +28939,9 @@
       <c r="BC161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BD161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -28629,6 +29115,9 @@
       <c r="BC162" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="BD162" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -28802,6 +29291,9 @@
       <c r="BC163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BD163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -28975,6 +29467,9 @@
       <c r="BC164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BD164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -29049,9 +29544,12 @@
       <c r="BC165" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BD165" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC165"/>
+  <autoFilter ref="A1:BD165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-11 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BD$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BE$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD165"/>
+  <dimension ref="A1:BE165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,7 @@
     <col width="16" customWidth="1" min="54" max="54"/>
     <col width="16" customWidth="1" min="55" max="55"/>
     <col width="16" customWidth="1" min="56" max="56"/>
+    <col width="16" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -782,6 +783,11 @@
           <t>2026-09-11 01:11</t>
         </is>
       </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -958,6 +964,9 @@
       <c r="BD2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BE2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1134,6 +1143,9 @@
       <c r="BD3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BE3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1310,6 +1322,9 @@
       <c r="BD4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BE4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1486,6 +1501,9 @@
       <c r="BD5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BE5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1662,6 +1680,9 @@
       <c r="BD6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BE6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1838,6 +1859,9 @@
       <c r="BD7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BE7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2014,6 +2038,9 @@
       <c r="BD8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BE8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2190,6 +2217,9 @@
       <c r="BD9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BE9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2366,6 +2396,9 @@
       <c r="BD10" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BE10" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2542,6 +2575,9 @@
       <c r="BD11" s="3" t="n">
         <v>20.19</v>
       </c>
+      <c r="BE11" s="3" t="n">
+        <v>20.19</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2718,6 +2754,9 @@
       <c r="BD12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2894,6 +2933,9 @@
       <c r="BD13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BE13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3070,6 +3112,9 @@
       <c r="BD14" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BE14" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3246,6 +3291,9 @@
       <c r="BD15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BE15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3422,6 +3470,9 @@
       <c r="BD16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BE16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3598,6 +3649,9 @@
       <c r="BD17" s="3" t="n">
         <v>20.75</v>
       </c>
+      <c r="BE17" s="3" t="n">
+        <v>20.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3774,6 +3828,9 @@
       <c r="BD18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BE18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3950,6 +4007,9 @@
       <c r="BD19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BE19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4126,6 +4186,9 @@
       <c r="BD20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BE20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4302,6 +4365,9 @@
       <c r="BD21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BE21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4478,6 +4544,9 @@
       <c r="BD22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BE22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4654,6 +4723,9 @@
       <c r="BD23" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BE23" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4830,6 +4902,9 @@
       <c r="BD24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BE24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5006,6 +5081,9 @@
       <c r="BD25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -5182,6 +5260,9 @@
       <c r="BD26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BE26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5358,6 +5439,9 @@
       <c r="BD27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BE27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5534,6 +5618,9 @@
       <c r="BD28" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="BE28" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -5710,6 +5797,9 @@
       <c r="BD29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BE29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -5886,6 +5976,9 @@
       <c r="BD30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -6062,6 +6155,9 @@
       <c r="BD31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -6238,6 +6334,9 @@
       <c r="BD32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -6414,6 +6513,9 @@
       <c r="BD33" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BE33" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -6590,6 +6692,9 @@
       <c r="BD34" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE34" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -6766,6 +6871,9 @@
       <c r="BD35" s="3" t="n">
         <v>20.39</v>
       </c>
+      <c r="BE35" s="3" t="n">
+        <v>20.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -6942,6 +7050,9 @@
       <c r="BD36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BE36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7118,6 +7229,9 @@
       <c r="BD37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BE37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7294,6 +7408,9 @@
       <c r="BD38" s="3" t="n">
         <v>20.88</v>
       </c>
+      <c r="BE38" s="3" t="n">
+        <v>20.88</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7470,6 +7587,9 @@
       <c r="BD39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BE39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7646,6 +7766,9 @@
       <c r="BD40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7822,6 +7945,9 @@
       <c r="BD41" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BE41" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7998,6 +8124,9 @@
       <c r="BD42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -8174,6 +8303,9 @@
       <c r="BD43" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BE43" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -8350,6 +8482,9 @@
       <c r="BD44" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BE44" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8526,6 +8661,9 @@
       <c r="BD45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BE45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -8702,6 +8840,9 @@
       <c r="BD46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BE46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8878,6 +9019,9 @@
       <c r="BD47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BE47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -9054,6 +9198,9 @@
       <c r="BD48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BE48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -9230,6 +9377,9 @@
       <c r="BD49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BE49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -9406,6 +9556,9 @@
       <c r="BD50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BE50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -9582,6 +9735,9 @@
       <c r="BD51" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="BE51" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -9758,6 +9914,9 @@
       <c r="BD52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BE52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -9934,6 +10093,9 @@
       <c r="BD53" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BE53" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -10110,6 +10272,9 @@
       <c r="BD54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BE54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -10286,6 +10451,9 @@
       <c r="BD55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BE55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -10462,6 +10630,9 @@
       <c r="BD56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BE56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10638,6 +10809,9 @@
       <c r="BD57" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BE57" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10814,6 +10988,9 @@
       <c r="BD58" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BE58" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10990,6 +11167,9 @@
       <c r="BD59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BE59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -11166,6 +11346,9 @@
       <c r="BD60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BE60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -11342,6 +11525,9 @@
       <c r="BD61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BE61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -11518,6 +11704,9 @@
       <c r="BD62" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BE62" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -11694,6 +11883,9 @@
       <c r="BD63" s="3" t="n">
         <v>21.25</v>
       </c>
+      <c r="BE63" s="3" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -11870,6 +12062,9 @@
       <c r="BD64" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BE64" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -12046,6 +12241,9 @@
       <c r="BD65" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE65" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -12222,6 +12420,9 @@
       <c r="BD66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -12398,6 +12599,9 @@
       <c r="BD67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BE67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -12574,6 +12778,9 @@
       <c r="BD68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BE68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -12750,6 +12957,9 @@
       <c r="BD69" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BE6